<commit_message>
Add episode 11 "다리가 부러진 영웅"
The family says Taeo rarely plays with his toy whose leg is broken.
Episode 11 turns that around: the green hero with a broken leg waits
in the corner of the toy box, then Taeo twists his own ankle kicking.
Everyone still plays with him (Dad as his legs, Jaei with the board
game, the grandparents with food), and that night he puts a plaster on
the green hero and takes it on the mission and to bed.

New broken toy, bandage and toy box props. The Excel sheet adds
episodes 10-11 and notes the idea came from the family. Cache v161.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -16,11 +16,11 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$149</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$189</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -701,7 +701,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>누나 머리끈 뺏기, 흉내 내기… 누나 괴롭히기가 취미인 막내. 사실은 누나가 좋아서 그래요. “맛있는 거 죠!”가 입버릇이고, 어벤져스를 사랑해서 영웅 이름도 태오식으로 불러요(블루베리, 스테잌로저…).</t>
+          <t>누나 괴롭히기가 취미인 막내(사실은 누나가 좋아서). 혼자 노는 것 같아도 가족 말을 다 듣고 있고, 틀려도 일단 소리 지르며 우기다가 들키면 머리를 긁적긁적. “맛있는 거 죠!”가 입버릇이고, 어벤져스 영웅도 태오식으로 불러요(블루베리, 쉬터맨, 스테잌로저…). 블랙 위도우랑 수가 제일 예쁘대요.</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1230,35 +1230,95 @@
       <c r="A13" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
-      <c r="F13" s="7" t="n"/>
-      <c r="G13" s="7" t="n"/>
-      <c r="H13" s="7" t="n"/>
-      <c r="I13" s="7" t="n"/>
-      <c r="J13" s="7" t="inlineStr">
-        <is>
-          <t>기획 중</t>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>혼자 노는 줄만 알았던 태오. 그런데 어른들이 소곤소곤 한 말까지 다 듣고 있었다. “왜 놀려! 놀리지 마!”</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>재이, 엄마, 아빠, 태오</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>“패드로 어벤져스 게임 하자!” (보드게임) / “늘어나는 애 이름 뭐야?” 또 묻기 / “오구마꼬치 맞아!!” 우기다 긁적긁적</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>속삭인 말도 다 듣는 태오 / “글씨는 몰라도 가족 마음 읽는 건 1등이야.”</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>아이는 혼자 노는 것 같아도 다 듣고 있어요. 그러니 아이 곁에서는 따뜻한 말을.</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>오늘 가족에게 들은 말 중에 제일 기분 좋았던 말은 뭐예요?</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>완성</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="n">
+      <c r="A14" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
-      <c r="F14" s="7" t="n"/>
-      <c r="G14" s="7" t="n"/>
-      <c r="H14" s="7" t="n"/>
-      <c r="I14" s="7" t="n"/>
-      <c r="J14" s="7" t="inlineStr">
-        <is>
-          <t>기획 중</t>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>다리가 부러진 영웅</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>장난감 영웅이 잔뜩인 태오. 그런데 다리가 부러진 초록 영웅은 늘 상자 구석에만 있다. 그러던 어느 날, 태오 다리가 삐끗했다.</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>재이, 할머니, 엄마, 아빠, 할아버지, 태오</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>“블루베리 출동! 쉬터맨도 출동!” / 태권도 발차기하다 삐끗</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>다리 부러진 초록 영웅에게 반창고를 붙여 주는 태오 / “다리 아파도 영웅이야!”</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>다리가 아파도, 모양이 달라져도 소중한 친구예요. 아플 때 곁에 있어 주는 게 진짜 영웅이에요.</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>우리 집에 오래 안 가지고 논 장난감이 있나요? 그 장난감에게 한마디 해 줄까요?</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>완성</t>
         </is>
       </c>
     </row>
@@ -1280,13 +1340,49 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="7" t="n"/>
+      <c r="I16" s="7" t="n"/>
+      <c r="J16" s="7" t="inlineStr">
+        <is>
+          <t>기획 중</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="7" t="n"/>
+      <c r="C17" s="7" t="n"/>
+      <c r="D17" s="7" t="n"/>
+      <c r="E17" s="7" t="n"/>
+      <c r="F17" s="7" t="n"/>
+      <c r="G17" s="7" t="n"/>
+      <c r="H17" s="7" t="n"/>
+      <c r="I17" s="7" t="n"/>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>기획 중</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:J12"/>
+  <autoFilter ref="A3:J14"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"아이디어,기획 중,콘티,완성"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1300,7 +1396,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H149"/>
+  <dimension ref="A1:H189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6067,8 +6163,1275 @@
       <c r="G149" s="6" t="inlineStr"/>
       <c r="H149" s="6" t="inlineStr"/>
     </row>
+    <row r="150">
+      <c r="A150" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B150" s="4" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D150" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E150" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F150" s="4" t="inlineStr">
+        <is>
+          <t>태오는 혼자서도 잘 논다.</t>
+        </is>
+      </c>
+      <c r="G150" s="4" t="inlineStr"/>
+      <c r="H150" s="4" t="inlineStr">
+        <is>
+          <t>슈웅~ 쾅!</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B151" s="6" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C151" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D151" s="6" t="inlineStr">
+        <is>
+          <t>부엌</t>
+        </is>
+      </c>
+      <c r="E151" s="6" t="inlineStr">
+        <is>
+          <t>아빠, 엄마</t>
+        </is>
+      </c>
+      <c r="F151" s="6" t="inlineStr"/>
+      <c r="G151" s="6" t="inlineStr">
+        <is>
+          <t>태오 요즘 혼자서도 잘 노네.
+응. 우리 말은 하나도 안 듣는 것 같아.</t>
+        </is>
+      </c>
+      <c r="H151" s="6" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B152" s="4" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D152" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E152" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F152" s="4" t="inlineStr"/>
+      <c r="G152" s="4" t="inlineStr">
+        <is>
+          <t>(생각) (다 듣고 있지롱.)</t>
+        </is>
+      </c>
+      <c r="H152" s="4" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B153" s="6" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C153" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D153" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E153" s="6" t="inlineStr">
+        <is>
+          <t>태오, 아빠</t>
+        </is>
+      </c>
+      <c r="F153" s="6" t="inlineStr"/>
+      <c r="G153" s="6" t="inlineStr">
+        <is>
+          <t>아빠! 패드로 어벤져스 게임 하자!
+패드? 이 태블릿?</t>
+        </is>
+      </c>
+      <c r="H153" s="6" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B154" s="4" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D154" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E154" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F154" s="4" t="inlineStr"/>
+      <c r="G154" s="4" t="inlineStr">
+        <is>
+          <t>아니! 이거!</t>
+        </is>
+      </c>
+      <c r="H154" s="4" t="inlineStr">
+        <is>
+          <t>짠!</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B155" s="6" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C155" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D155" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E155" s="6" t="inlineStr">
+        <is>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F155" s="6" t="inlineStr"/>
+      <c r="G155" s="6" t="inlineStr">
+        <is>
+          <t>…이게 패드야?</t>
+        </is>
+      </c>
+      <c r="H155" s="6" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B156" s="4" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D156" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E156" s="4" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="F156" s="4" t="inlineStr"/>
+      <c r="G156" s="4" t="inlineStr">
+        <is>
+          <t>나는 블랙 위도우랑 수! 제일 예뻐!
+그럼 누나는 쉬터맨…아니, 스파이더맨!</t>
+        </is>
+      </c>
+      <c r="H156" s="4" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B157" s="6" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C157" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D157" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E157" s="6" t="inlineStr">
+        <is>
+          <t>태오, 아빠</t>
+        </is>
+      </c>
+      <c r="F157" s="6" t="inlineStr"/>
+      <c r="G157" s="6" t="inlineStr">
+        <is>
+          <t>아빠, 늘어나는 애 이름 뭐야?
+리드.</t>
+        </is>
+      </c>
+      <c r="H157" s="6" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B158" s="4" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D158" s="4" t="inlineStr">
+        <is>
+          <t>효과: 속도선</t>
+        </is>
+      </c>
+      <c r="E158" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F158" s="4" t="inlineStr">
+        <is>
+          <t>3분 뒤.</t>
+        </is>
+      </c>
+      <c r="G158" s="4" t="inlineStr">
+        <is>
+          <t>아빠, 늘어나는 애 이름 뭐야?</t>
+        </is>
+      </c>
+      <c r="H158" s="4" t="inlineStr">
+        <is>
+          <t>또?!</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B159" s="6" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C159" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D159" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E159" s="6" t="inlineStr">
+        <is>
+          <t>아빠, 태오, 재이, 엄마</t>
+        </is>
+      </c>
+      <c r="F159" s="6" t="inlineStr"/>
+      <c r="G159" s="6" t="inlineStr">
+        <is>
+          <t>카드에 적힌 숫자만큼 가는 거야. 태오 이거 읽을 수 있어?</t>
+        </is>
+      </c>
+      <c r="H159" s="6" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B160" s="4" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D160" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E160" s="4" t="inlineStr">
+        <is>
+          <t>아빠, 엄마</t>
+        </is>
+      </c>
+      <c r="F160" s="4" t="inlineStr"/>
+      <c r="G160" s="4" t="inlineStr">
+        <is>
+          <t>(속삭임) (태오는 아직 글씨랑 숫자 잘 모르잖아~)</t>
+        </is>
+      </c>
+      <c r="H160" s="4" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B161" s="6" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C161" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D161" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E161" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F161" s="6" t="inlineStr"/>
+      <c r="G161" s="6" t="inlineStr">
+        <is>
+          <t>왜 놀려! 놀리지 마!!</t>
+        </is>
+      </c>
+      <c r="H161" s="6" t="inlineStr">
+        <is>
+          <t>삿대질!</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B162" s="4" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="D162" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E162" s="4" t="inlineStr">
+        <is>
+          <t>아빠, 재이</t>
+        </is>
+      </c>
+      <c r="F162" s="4" t="inlineStr"/>
+      <c r="G162" s="4" t="inlineStr">
+        <is>
+          <t>어떻게 들었지? 속삭였는데…
+아빠, 태오는 다 들어!</t>
+        </is>
+      </c>
+      <c r="H162" s="4" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B163" s="6" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C163" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="D163" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E163" s="6" t="inlineStr">
+        <is>
+          <t>엄마, 태오</t>
+        </is>
+      </c>
+      <c r="F163" s="6" t="inlineStr"/>
+      <c r="G163" s="6" t="inlineStr">
+        <is>
+          <t>그럼 우리 태오가 제일 잘하는 놀이 하자!
+오구마꼬치 피었습니다!</t>
+        </is>
+      </c>
+      <c r="H163" s="6" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B164" s="4" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C164" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="D164" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E164" s="4" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F164" s="4" t="inlineStr"/>
+      <c r="G164" s="4" t="inlineStr">
+        <is>
+          <t>…오구마꼬치? 무궁화 꽃이 피었습니다겠지.</t>
+        </is>
+      </c>
+      <c r="H164" s="4" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B165" s="6" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C165" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="D165" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E165" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F165" s="6" t="inlineStr"/>
+      <c r="G165" s="6" t="inlineStr">
+        <is>
+          <t>아니야! 오구마꼬치 맞아!! 어린이집에서도 그렇게 해!!</t>
+        </is>
+      </c>
+      <c r="H165" s="6" t="inlineStr">
+        <is>
+          <t>빡빡</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B166" s="4" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C166" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="D166" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E166" s="4" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F166" s="4" t="inlineStr"/>
+      <c r="G166" s="4" t="inlineStr">
+        <is>
+          <t>여기 책에도 ‘무궁화 꽃이’라고 쓰여 있는데?</t>
+        </is>
+      </c>
+      <c r="H166" s="4" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B167" s="6" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C167" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="D167" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E167" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F167" s="6" t="inlineStr"/>
+      <c r="G167" s="6" t="inlineStr">
+        <is>
+          <t>…헤헤. 무궁…꼬치?</t>
+        </is>
+      </c>
+      <c r="H167" s="6" t="inlineStr">
+        <is>
+          <t>긁적긁적</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B168" s="4" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C168" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="D168" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E168" s="4" t="inlineStr">
+        <is>
+          <t>태오, 아빠, 엄마, 재이</t>
+        </is>
+      </c>
+      <c r="F168" s="4" t="inlineStr"/>
+      <c r="G168" s="4" t="inlineStr">
+        <is>
+          <t>오구마꼬치~ 피었습니다!</t>
+        </is>
+      </c>
+      <c r="H168" s="4" t="inlineStr">
+        <is>
+          <t>얼음!</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B169" s="6" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C169" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="D169" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E169" s="6" t="inlineStr">
+        <is>
+          <t>태오, 아빠</t>
+        </is>
+      </c>
+      <c r="F169" s="6" t="inlineStr"/>
+      <c r="G169" s="6" t="inlineStr">
+        <is>
+          <t>아빠 움직였다! 아빠 아웃!</t>
+        </is>
+      </c>
+      <c r="H169" s="6" t="inlineStr">
+        <is>
+          <t>하하하</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B170" s="4" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C170" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="D170" s="4" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E170" s="4" t="inlineStr">
+        <is>
+          <t>엄마, 아빠</t>
+        </is>
+      </c>
+      <c r="F170" s="4" t="inlineStr">
+        <is>
+          <t>그날 밤, 거실.</t>
+        </is>
+      </c>
+      <c r="G170" s="4" t="inlineStr">
+        <is>
+          <t>(속삭임) (태오가 글씨 모른다는 말에 속상했나 봐.)
+(속삭임) (그러게. 아빠가 너무 쉽게 말했네.)</t>
+        </is>
+      </c>
+      <c r="H170" s="4" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B171" s="6" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C171" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="D171" s="6" t="inlineStr">
+        <is>
+          <t>방(밤)</t>
+        </is>
+      </c>
+      <c r="E171" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F171" s="6" t="inlineStr"/>
+      <c r="G171" s="6" t="inlineStr">
+        <is>
+          <t>(생각) (…다 들린다.)</t>
+        </is>
+      </c>
+      <c r="H171" s="6" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B172" s="4" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C172" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="D172" s="4" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E172" s="4" t="inlineStr">
+        <is>
+          <t>엄마, 아빠</t>
+        </is>
+      </c>
+      <c r="F172" s="4" t="inlineStr"/>
+      <c r="G172" s="4" t="inlineStr">
+        <is>
+          <t>(속삭임) 그래도 우리 태오는 글씨는 몰라도, 가족 마음 읽는 건 1등이야.
+(속삭임) 오구마꼬치도 세계 1등이고.</t>
+        </is>
+      </c>
+      <c r="H172" s="4" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B173" s="6" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C173" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="D173" s="6" t="inlineStr">
+        <is>
+          <t>방(밤)</t>
+        </is>
+      </c>
+      <c r="E173" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F173" s="6" t="inlineStr">
+        <is>
+          <t>태오는 오늘도 다 듣고 있다.</t>
+        </is>
+      </c>
+      <c r="G173" s="6" t="inlineStr"/>
+      <c r="H173" s="6" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B174" s="4" t="inlineStr">
+        <is>
+          <t>태오는 다 듣고 있다</t>
+        </is>
+      </c>
+      <c r="C174" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="D174" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E174" s="4" t="inlineStr"/>
+      <c r="F174" s="4" t="inlineStr">
+        <is>
+          <t>그래서 우리는, 좋은 말만 들려주기로 했다.</t>
+        </is>
+      </c>
+      <c r="G174" s="4" t="inlineStr"/>
+      <c r="H174" s="4" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B175" s="6" t="inlineStr">
+        <is>
+          <t>다리가 부러진 영웅</t>
+        </is>
+      </c>
+      <c r="C175" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D175" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E175" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F175" s="6" t="inlineStr">
+        <is>
+          <t>태오에게는 장난감 영웅이 잔뜩 있다.</t>
+        </is>
+      </c>
+      <c r="G175" s="6" t="inlineStr">
+        <is>
+          <t>블루베리 출동! 쉬터맨도 출동!</t>
+        </is>
+      </c>
+      <c r="H175" s="6" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B176" s="4" t="inlineStr">
+        <is>
+          <t>다리가 부러진 영웅</t>
+        </is>
+      </c>
+      <c r="C176" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D176" s="4" t="inlineStr">
+        <is>
+          <t>효과: 어두움</t>
+        </is>
+      </c>
+      <c r="E176" s="4" t="inlineStr"/>
+      <c r="F176" s="4" t="inlineStr">
+        <is>
+          <t>그런데 상자 구석, 다리가 부러진 초록 영웅은… / 오늘도 출동하지 못했다.</t>
+        </is>
+      </c>
+      <c r="G176" s="4" t="inlineStr"/>
+      <c r="H176" s="4" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B177" s="6" t="inlineStr">
+        <is>
+          <t>다리가 부러진 영웅</t>
+        </is>
+      </c>
+      <c r="C177" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D177" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E177" s="6" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F177" s="6" t="inlineStr"/>
+      <c r="G177" s="6" t="inlineStr">
+        <is>
+          <t>태오야, 초록 영웅은 왜 안 데리고 놀아?
+걔는 다리 부러졌잖아. 못 뛰어.</t>
+        </is>
+      </c>
+      <c r="H177" s="6" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B178" s="4" t="inlineStr">
+        <is>
+          <t>다리가 부러진 영웅</t>
+        </is>
+      </c>
+      <c r="C178" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D178" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E178" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F178" s="4" t="inlineStr">
+        <is>
+          <t>그다음 날, 태권도 발차기 연습을 하다가…</t>
+        </is>
+      </c>
+      <c r="G178" s="4" t="inlineStr"/>
+      <c r="H178" s="4" t="inlineStr">
+        <is>
+          <t>얍!, 삐끗!</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B179" s="6" t="inlineStr">
+        <is>
+          <t>다리가 부러진 영웅</t>
+        </is>
+      </c>
+      <c r="C179" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D179" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E179" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F179" s="6" t="inlineStr"/>
+      <c r="G179" s="6" t="inlineStr">
+        <is>
+          <t>으아앙~ 다리 아파!</t>
+        </is>
+      </c>
+      <c r="H179" s="6" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B180" s="4" t="inlineStr">
+        <is>
+          <t>다리가 부러진 영웅</t>
+        </is>
+      </c>
+      <c r="C180" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D180" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E180" s="4" t="inlineStr">
+        <is>
+          <t>태오, 엄마</t>
+        </is>
+      </c>
+      <c r="F180" s="4" t="inlineStr"/>
+      <c r="G180" s="4" t="inlineStr">
+        <is>
+          <t>살짝 삐었네. 며칠은 뛰면 안 돼.
+그럼 나 이제 못 놀아?</t>
+        </is>
+      </c>
+      <c r="H180" s="4" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B181" s="6" t="inlineStr">
+        <is>
+          <t>다리가 부러진 영웅</t>
+        </is>
+      </c>
+      <c r="C181" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="D181" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E181" s="6" t="inlineStr">
+        <is>
+          <t>아빠, 태오</t>
+        </is>
+      </c>
+      <c r="F181" s="6" t="inlineStr"/>
+      <c r="G181" s="6" t="inlineStr">
+        <is>
+          <t>무슨 소리! 오늘은 아빠가 태오 다리다!</t>
+        </is>
+      </c>
+      <c r="H181" s="6" t="inlineStr">
+        <is>
+          <t>번쩍!</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B182" s="4" t="inlineStr">
+        <is>
+          <t>다리가 부러진 영웅</t>
+        </is>
+      </c>
+      <c r="C182" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D182" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E182" s="4" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F182" s="4" t="inlineStr"/>
+      <c r="G182" s="4" t="inlineStr">
+        <is>
+          <t>누나는 앉아서 하는 패드 게임 해 줄게!</t>
+        </is>
+      </c>
+      <c r="H182" s="4" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B183" s="6" t="inlineStr">
+        <is>
+          <t>다리가 부러진 영웅</t>
+        </is>
+      </c>
+      <c r="C183" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="D183" s="6" t="inlineStr">
+        <is>
+          <t>할머니 댁</t>
+        </is>
+      </c>
+      <c r="E183" s="6" t="inlineStr">
+        <is>
+          <t>할머니, 할아버지</t>
+        </is>
+      </c>
+      <c r="F183" s="6" t="inlineStr">
+        <is>
+          <t>할머니 할아버지도 달려오셨다.</t>
+        </is>
+      </c>
+      <c r="G183" s="6" t="inlineStr">
+        <is>
+          <t>아이고 우리 강아지, 할머니가 맛있는 거 해 왔다.</t>
+        </is>
+      </c>
+      <c r="H183" s="6" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B184" s="4" t="inlineStr">
+        <is>
+          <t>다리가 부러진 영웅</t>
+        </is>
+      </c>
+      <c r="C184" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D184" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E184" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F184" s="4" t="inlineStr"/>
+      <c r="G184" s="4" t="inlineStr">
+        <is>
+          <t>다리 아파도… 다들 나랑 놀아 주네.</t>
+        </is>
+      </c>
+      <c r="H184" s="4" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B185" s="6" t="inlineStr">
+        <is>
+          <t>다리가 부러진 영웅</t>
+        </is>
+      </c>
+      <c r="C185" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="D185" s="6" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E185" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F185" s="6" t="inlineStr">
+        <is>
+          <t>그날 밤, 장난감 상자를 보다가.</t>
+        </is>
+      </c>
+      <c r="G185" s="6" t="inlineStr">
+        <is>
+          <t>(생각) (…너도 심심했지?)</t>
+        </is>
+      </c>
+      <c r="H185" s="6" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B186" s="4" t="inlineStr">
+        <is>
+          <t>다리가 부러진 영웅</t>
+        </is>
+      </c>
+      <c r="C186" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D186" s="4" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E186" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F186" s="4" t="inlineStr"/>
+      <c r="G186" s="4" t="inlineStr">
+        <is>
+          <t>내가 반창고 붙여 줄게. 이제 너도 출동이야!</t>
+        </is>
+      </c>
+      <c r="H186" s="4" t="inlineStr">
+        <is>
+          <t>찰칵</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B187" s="6" t="inlineStr">
+        <is>
+          <t>다리가 부러진 영웅</t>
+        </is>
+      </c>
+      <c r="C187" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="D187" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E187" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F187" s="6" t="inlineStr"/>
+      <c r="G187" s="6" t="inlineStr">
+        <is>
+          <t>다리 아파도 영웅이야! 제일 용감한 초록 영웅!</t>
+        </is>
+      </c>
+      <c r="H187" s="6" t="inlineStr"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B188" s="4" t="inlineStr">
+        <is>
+          <t>다리가 부러진 영웅</t>
+        </is>
+      </c>
+      <c r="C188" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="D188" s="4" t="inlineStr">
+        <is>
+          <t>방(밤)</t>
+        </is>
+      </c>
+      <c r="E188" s="4" t="inlineStr">
+        <is>
+          <t>재이, 엄마</t>
+        </is>
+      </c>
+      <c r="F188" s="4" t="inlineStr"/>
+      <c r="G188" s="4" t="inlineStr">
+        <is>
+          <t>(속삭임) (태오가… 초록 영웅이랑 자네.)
+(속삭임) (아파 보니까 알았나 봐.)</t>
+        </is>
+      </c>
+      <c r="H188" s="4" t="inlineStr"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B189" s="6" t="inlineStr">
+        <is>
+          <t>다리가 부러진 영웅</t>
+        </is>
+      </c>
+      <c r="C189" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="D189" s="6" t="inlineStr">
+        <is>
+          <t>방(밤)</t>
+        </is>
+      </c>
+      <c r="E189" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F189" s="6" t="inlineStr">
+        <is>
+          <t>아플 때 곁에 있어 주는 게 진짜 영웅이다.</t>
+        </is>
+      </c>
+      <c r="G189" s="6" t="inlineStr"/>
+      <c r="H189" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:H149"/>
+  <autoFilter ref="A3:H189"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -6082,7 +7445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -6356,9 +7719,21 @@
       <c r="A14" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="4" t="inlineStr"/>
-      <c r="C14" s="4" t="inlineStr"/>
-      <c r="D14" s="4" t="inlineStr"/>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>오구마꼬치 피었습니다</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>무궁화 꽃이 피었습니다</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>술래 놀이</t>
+        </is>
+      </c>
       <c r="E14" s="4" t="inlineStr"/>
       <c r="F14" s="4" t="inlineStr"/>
     </row>
@@ -6366,9 +7741,21 @@
       <c r="A15" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="6" t="inlineStr"/>
-      <c r="C15" s="6" t="inlineStr"/>
-      <c r="D15" s="6" t="inlineStr"/>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>패드</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>마블 5분 보드게임</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>“패드로 어벤져스 게임 하자!”</t>
+        </is>
+      </c>
       <c r="E15" s="6" t="inlineStr"/>
       <c r="F15" s="6" t="inlineStr"/>
     </row>
@@ -6376,9 +7763,21 @@
       <c r="A16" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="4" t="inlineStr"/>
-      <c r="C16" s="4" t="inlineStr"/>
-      <c r="D16" s="4" t="inlineStr"/>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>쉬터맨</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>스파이더맨</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>거미 영웅</t>
+        </is>
+      </c>
       <c r="E16" s="4" t="inlineStr"/>
       <c r="F16" s="4" t="inlineStr"/>
     </row>
@@ -6386,9 +7785,21 @@
       <c r="A17" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="6" t="inlineStr"/>
-      <c r="C17" s="6" t="inlineStr"/>
-      <c r="D17" s="6" t="inlineStr"/>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>아이엠둔</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>닥터 둠</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>판타스틱 4의 악당</t>
+        </is>
+      </c>
       <c r="E17" s="6" t="inlineStr"/>
       <c r="F17" s="6" t="inlineStr"/>
     </row>
@@ -6396,9 +7807,21 @@
       <c r="A18" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="4" t="inlineStr"/>
-      <c r="C18" s="4" t="inlineStr"/>
-      <c r="D18" s="4" t="inlineStr"/>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>늘어나는 애</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>리드 (판타스틱 4)</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>이름을 자꾸 까먹어서 “늘어나는 애 이름 뭐야?”</t>
+        </is>
+      </c>
       <c r="E18" s="4" t="inlineStr"/>
       <c r="F18" s="4" t="inlineStr"/>
     </row>
@@ -6552,8 +7975,58 @@
       <c r="E33" s="6" t="inlineStr"/>
       <c r="F33" s="6" t="inlineStr"/>
     </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" s="4" t="inlineStr"/>
+      <c r="C34" s="4" t="inlineStr"/>
+      <c r="D34" s="4" t="inlineStr"/>
+      <c r="E34" s="4" t="inlineStr"/>
+      <c r="F34" s="4" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="B35" s="6" t="inlineStr"/>
+      <c r="C35" s="6" t="inlineStr"/>
+      <c r="D35" s="6" t="inlineStr"/>
+      <c r="E35" s="6" t="inlineStr"/>
+      <c r="F35" s="6" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B36" s="4" t="inlineStr"/>
+      <c r="C36" s="4" t="inlineStr"/>
+      <c r="D36" s="4" t="inlineStr"/>
+      <c r="E36" s="4" t="inlineStr"/>
+      <c r="F36" s="4" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="B37" s="6" t="inlineStr"/>
+      <c r="C37" s="6" t="inlineStr"/>
+      <c r="D37" s="6" t="inlineStr"/>
+      <c r="E37" s="6" t="inlineStr"/>
+      <c r="F37" s="6" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="B38" s="4" t="inlineStr"/>
+      <c r="C38" s="4" t="inlineStr"/>
+      <c r="D38" s="4" t="inlineStr"/>
+      <c r="E38" s="4" t="inlineStr"/>
+      <c r="F38" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F33"/>
+  <autoFilter ref="A3:F38"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -6567,7 +8040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -6733,18 +8206,18 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>김태오!</t>
+          <t>늘어나는 애 이름 뭐야?</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr"/>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+          <t>판타스틱 4 리드 이름이 또 생각 안 날 때</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr"/>
@@ -6755,22 +8228,18 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>짐방</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>김서방</t>
-        </is>
-      </c>
+          <t>블랙 위도우랑 수가 제일 예뻐!</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr"/>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+          <t>영웅 이야기만 나오면</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr"/>
@@ -6779,30 +8248,70 @@
       <c r="A11" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="6" t="inlineStr"/>
-      <c r="C11" s="6" t="inlineStr"/>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>태오 입버릇</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>왜 놀려! 놀리지 마!</t>
+        </is>
+      </c>
       <c r="D11" s="6" t="inlineStr"/>
-      <c r="E11" s="6" t="inlineStr"/>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>“태오는 글씨·숫자 잘 몰라” 소리를 들으면 (손가락질하며)</t>
+        </is>
+      </c>
       <c r="F11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="4" t="inlineStr"/>
-      <c r="C12" s="4" t="inlineStr"/>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>재이 입버릇</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>김태오!</t>
+        </is>
+      </c>
       <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="4" t="inlineStr"/>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+        </is>
+      </c>
       <c r="F12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="6" t="inlineStr"/>
-      <c r="C13" s="6" t="inlineStr"/>
-      <c r="D13" s="6" t="inlineStr"/>
-      <c r="E13" s="6" t="inlineStr"/>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>짐방</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>김서방</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+        </is>
+      </c>
       <c r="F13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
@@ -6925,8 +8434,38 @@
       <c r="E25" s="6" t="inlineStr"/>
       <c r="F25" s="6" t="inlineStr"/>
     </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="4" t="inlineStr"/>
+      <c r="C26" s="4" t="inlineStr"/>
+      <c r="D26" s="4" t="inlineStr"/>
+      <c r="E26" s="4" t="inlineStr"/>
+      <c r="F26" s="4" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="6" t="inlineStr"/>
+      <c r="C27" s="6" t="inlineStr"/>
+      <c r="D27" s="6" t="inlineStr"/>
+      <c r="E27" s="6" t="inlineStr"/>
+      <c r="F27" s="6" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" s="4" t="inlineStr"/>
+      <c r="C28" s="4" t="inlineStr"/>
+      <c r="D28" s="4" t="inlineStr"/>
+      <c r="E28" s="4" t="inlineStr"/>
+      <c r="F28" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F25"/>
+  <autoFilter ref="A3:F28"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -6945,7 +8484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6992,7 +8531,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>태권도 승급 심사</t>
+          <t>다리가 부러진 장난감</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -7002,39 +8541,35 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>긴장한 태오가 심사장에서 넘어진다. 가족 응원석에선 할아버지가 제일 크게 “메가랩터킥!”을 외치고…</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>넘어져도 다시 일어나면 그게 진짜 실력이에요.</t>
-        </is>
-      </c>
+          <t>(가족 제보) 태오는 다리가 부러진 장난감은 잘 안 가지고 논다 → 11화로 만듦</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr"/>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>아이디어</t>
+          <t>완성</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>할머니의 파마 대작전</t>
+          <t>태권도 승급 심사</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>할머니, 재이</t>
+          <t>태오</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>재이가 미용실 놀이로 할머니 머리를 ‘펴’ 드리겠다고 나섰다. 결과는 더 뽀글뽀글?</t>
+          <t>긴장한 태오가 심사장에서 넘어진다. 가족 응원석에선 할아버지가 제일 크게 “메가랩터킥!”을 외치고…</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>있는 그대로의 모습이 가장 예뻐요.</t>
+          <t>넘어져도 다시 일어나면 그게 진짜 실력이에요.</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -7046,22 +8581,22 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>아빠의 비밀 요리</t>
+          <t>할머니의 파마 대작전</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>아빠, 태오</t>
+          <t>할머니, 재이</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>엄마 생일, 아빠와 태오가 몰래 미역국을 끓인다. 미역이 냄비 밖으로 넘쳐 나오는데…</t>
+          <t>재이가 미용실 놀이로 할머니 머리를 ‘펴’ 드리겠다고 나섰다. 결과는 더 뽀글뽀글?</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>마음을 담으면 서툴러도 최고의 선물이에요.</t>
+          <t>있는 그대로의 모습이 가장 예뻐요.</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -7073,36 +8608,56 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
+          <t>아빠의 비밀 요리</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>아빠, 태오</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>엄마 생일, 아빠와 태오가 몰래 미역국을 끓인다. 미역이 냄비 밖으로 넘쳐 나오는데…</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>마음을 담으면 서툴러도 최고의 선물이에요.</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>아이디어</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
           <t>누나 대신 태오</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>태오, 재이</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>누나가 아파서 학교에 못 간 날, 태오가 누나의 ‘하루 비서’가 된다.</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>도움을 받던 사람도 도움을 줄 수 있어요.</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>아이디어</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr"/>
-      <c r="B8" s="4" t="inlineStr"/>
-      <c r="C8" s="4" t="inlineStr"/>
-      <c r="D8" s="4" t="inlineStr"/>
-      <c r="E8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr"/>
@@ -7111,8 +8666,15 @@
       <c r="D9" s="6" t="inlineStr"/>
       <c r="E9" s="6" t="inlineStr"/>
     </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr"/>
+      <c r="B10" s="4" t="inlineStr"/>
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:E9"/>
+  <autoFilter ref="A3:E10"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add episode 12 "어벤져스에 가년~"
Taeo plays the "시장에 가면" chain game as "어벤져스에 가년~", listing
who is in the Avengers. It joins Taeo's dictionary, and episode 12 has
the whole family play it: Taeo insists it is 가년, Dad is out for saying
Steve Rogers instead of 스테잌로저, Mom asks who the stretchy one is,
Grandpa passes by guessing 우엉, and Grandma, not knowing any heroes,
says "어벤져스에 가면… 우리 태오도 있고!" so the game ends with all six
of the family. Excel sheet adds episode 12. Cache v162.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -16,9 +16,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$189</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$208</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$10</definedName>
   </definedNames>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1326,17 +1326,47 @@
       <c r="A15" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="7" t="n"/>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
-      <c r="F15" s="7" t="n"/>
-      <c r="G15" s="7" t="n"/>
-      <c r="H15" s="7" t="n"/>
-      <c r="I15" s="7" t="n"/>
-      <c r="J15" s="7" t="inlineStr">
-        <is>
-          <t>기획 중</t>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>“어벤져스에 가년~ 블루베리도 있고!” 태오가 만든 놀이에 온 가족이 모였다. 그런데 태오어를 모르면 바로 땡!</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>재이, 할머니, 엄마, 아빠, 할아버지, 태오</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>“어벤져스는 가년이야!!” 우기기 / 아빠 “스티브 로저스” → “땡! 스테잌로저야!” / 할아버지 얼떨결에 “우엉?” 정답</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>할머니 “어벤져스에 가면… 우리 태오도 있고!” / 우리 집 어벤져스는 여섯 명</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>우리 가족이 바로, 서로를 지켜 주는 어벤져스예요.</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>‘우리 집에 가면~’ 놀이를 해 볼까요? 우리 가족에게 있는 것을 하나씩 이어 말해 봐요.</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>완성</t>
         </is>
       </c>
     </row>
@@ -1376,13 +1406,31 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="7" t="n"/>
+      <c r="D18" s="7" t="n"/>
+      <c r="E18" s="7" t="n"/>
+      <c r="F18" s="7" t="n"/>
+      <c r="G18" s="7" t="n"/>
+      <c r="H18" s="7" t="n"/>
+      <c r="I18" s="7" t="n"/>
+      <c r="J18" s="7" t="inlineStr">
+        <is>
+          <t>기획 중</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:J14"/>
+  <autoFilter ref="A3:J15"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"아이디어,기획 중,콘티,완성"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1396,7 +1444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H189"/>
+  <dimension ref="A1:H208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7430,8 +7478,593 @@
       <c r="G189" s="6" t="inlineStr"/>
       <c r="H189" s="6" t="inlineStr"/>
     </row>
+    <row r="190">
+      <c r="A190" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B190" s="4" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C190" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D190" s="4" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E190" s="4" t="inlineStr">
+        <is>
+          <t>재이, 할머니, 엄마, 아빠, 할아버지, 태오</t>
+        </is>
+      </c>
+      <c r="F190" s="4" t="inlineStr">
+        <is>
+          <t>저녁을 먹고, 온 가족이 거실에 모였다.</t>
+        </is>
+      </c>
+      <c r="G190" s="4" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년 놀이 하자!</t>
+        </is>
+      </c>
+      <c r="H190" s="4" t="inlineStr"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B191" s="6" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C191" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D191" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E191" s="6" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F191" s="6" t="inlineStr"/>
+      <c r="G191" s="6" t="inlineStr">
+        <is>
+          <t>…가년? ‘시장에 가면’ 놀이 말하는 거지? ‘가면’이야.</t>
+        </is>
+      </c>
+      <c r="H191" s="6" t="inlineStr"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B192" s="4" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C192" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D192" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E192" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F192" s="4" t="inlineStr"/>
+      <c r="G192" s="4" t="inlineStr">
+        <is>
+          <t>가년 맞아!! 어벤져스는 가년이야!!</t>
+        </is>
+      </c>
+      <c r="H192" s="4" t="inlineStr"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B193" s="6" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C193" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D193" s="6" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E193" s="6" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F193" s="6" t="inlineStr"/>
+      <c r="G193" s="6" t="inlineStr">
+        <is>
+          <t>그래, 가년 하자~
+어벤져스에 가년~ 블루베리도 있고!</t>
+        </is>
+      </c>
+      <c r="H193" s="6" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B194" s="4" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C194" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D194" s="4" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E194" s="4" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F194" s="4" t="inlineStr"/>
+      <c r="G194" s="4" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~ 블루베리도 있고, 쉬터맨도 있고!</t>
+        </is>
+      </c>
+      <c r="H194" s="4" t="inlineStr"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B195" s="6" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C195" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D195" s="6" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E195" s="6" t="inlineStr">
+        <is>
+          <t>아빠, 태오</t>
+        </is>
+      </c>
+      <c r="F195" s="6" t="inlineStr"/>
+      <c r="G195" s="6" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~ 블루베리도 있고, 쉬터맨도 있고, 스티브 로저스도 있고!</t>
+        </is>
+      </c>
+      <c r="H195" s="6" t="inlineStr"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B196" s="4" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C196" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D196" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E196" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F196" s="4" t="inlineStr"/>
+      <c r="G196" s="4" t="inlineStr">
+        <is>
+          <t>땡!! 스테잌로저야!!</t>
+        </is>
+      </c>
+      <c r="H196" s="4" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B197" s="6" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C197" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D197" s="6" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E197" s="6" t="inlineStr">
+        <is>
+          <t>아빠, 재이</t>
+        </is>
+      </c>
+      <c r="F197" s="6" t="inlineStr"/>
+      <c r="G197" s="6" t="inlineStr">
+        <is>
+          <t>아… 스테잌로저…</t>
+        </is>
+      </c>
+      <c r="H197" s="6" t="inlineStr">
+        <is>
+          <t>긁적긁적, 깔깔깔</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B198" s="4" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C198" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D198" s="4" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E198" s="4" t="inlineStr">
+        <is>
+          <t>엄마, 태오</t>
+        </is>
+      </c>
+      <c r="F198" s="4" t="inlineStr"/>
+      <c r="G198" s="4" t="inlineStr">
+        <is>
+          <t>…스테잌로저도 있고, 늘어나는 애도 있고!
+엄마 잘한다!</t>
+        </is>
+      </c>
+      <c r="H198" s="4" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B199" s="6" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C199" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D199" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E199" s="6" t="inlineStr">
+        <is>
+          <t>태오, 엄마</t>
+        </is>
+      </c>
+      <c r="F199" s="6" t="inlineStr"/>
+      <c r="G199" s="6" t="inlineStr">
+        <is>
+          <t>근데 엄마, 늘어나는 애 이름 뭐야?
+…너도 몰라?</t>
+        </is>
+      </c>
+      <c r="H199" s="6" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B200" s="4" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C200" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D200" s="4" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E200" s="4" t="inlineStr">
+        <is>
+          <t>할아버지, 태오</t>
+        </is>
+      </c>
+      <c r="F200" s="4" t="inlineStr"/>
+      <c r="G200" s="4" t="inlineStr">
+        <is>
+          <t>허허, 할아버지 차례구나. 어벤져스에 가면… 우… 우엉?</t>
+        </is>
+      </c>
+      <c r="H200" s="4" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B201" s="6" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C201" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D201" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E201" s="6" t="inlineStr">
+        <is>
+          <t>태오, 할아버지</t>
+        </is>
+      </c>
+      <c r="F201" s="6" t="inlineStr"/>
+      <c r="G201" s="6" t="inlineStr">
+        <is>
+          <t>맞아!! 우엉 있어! 할아버지 통과!</t>
+        </is>
+      </c>
+      <c r="H201" s="6" t="inlineStr">
+        <is>
+          <t>얼떨결에 정답</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B202" s="4" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C202" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="D202" s="4" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E202" s="4" t="inlineStr">
+        <is>
+          <t>할머니, 태오</t>
+        </is>
+      </c>
+      <c r="F202" s="4" t="inlineStr"/>
+      <c r="G202" s="4" t="inlineStr">
+        <is>
+          <t>어벤져스에 가면… 블루…베리도 있고… 에고, 할머니는 모르겠다.</t>
+        </is>
+      </c>
+      <c r="H202" s="4" t="inlineStr"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B203" s="6" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C203" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="D203" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E203" s="6" t="inlineStr">
+        <is>
+          <t>할머니</t>
+        </is>
+      </c>
+      <c r="F203" s="6" t="inlineStr"/>
+      <c r="G203" s="6" t="inlineStr">
+        <is>
+          <t>어벤져스에 가면… 우리 태오도 있고!</t>
+        </is>
+      </c>
+      <c r="H203" s="6" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B204" s="4" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C204" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="D204" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E204" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F204" s="4" t="inlineStr"/>
+      <c r="G204" s="4" t="inlineStr">
+        <is>
+          <t>나도 어벤져스야?</t>
+        </is>
+      </c>
+      <c r="H204" s="4" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B205" s="6" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C205" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="D205" s="6" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E205" s="6" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F205" s="6" t="inlineStr"/>
+      <c r="G205" s="6" t="inlineStr">
+        <is>
+          <t>그럼! 누나 괴롭히는 힘은 우주 최강이지.</t>
+        </is>
+      </c>
+      <c r="H205" s="6" t="inlineStr">
+        <is>
+          <t>헤헤</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B206" s="4" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C206" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="D206" s="4" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E206" s="4" t="inlineStr">
+        <is>
+          <t>재이, 할머니, 엄마, 아빠, 할아버지, 태오</t>
+        </is>
+      </c>
+      <c r="F206" s="4" t="inlineStr"/>
+      <c r="G206" s="4" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~ 할머니도 있고, 할아버지도 있고, 엄마도, 아빠도, 누나도 있고!</t>
+        </is>
+      </c>
+      <c r="H206" s="4" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B207" s="6" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C207" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="D207" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E207" s="6" t="inlineStr">
+        <is>
+          <t>재이, 할머니, 엄마, 아빠, 할아버지, 태오</t>
+        </is>
+      </c>
+      <c r="F207" s="6" t="inlineStr"/>
+      <c r="G207" s="6" t="inlineStr">
+        <is>
+          <t>…그리고 나도 있고!</t>
+        </is>
+      </c>
+      <c r="H207" s="6" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B208" s="4" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C208" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="D208" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E208" s="4" t="inlineStr"/>
+      <c r="F208" s="4" t="inlineStr">
+        <is>
+          <t>우리 집 어벤져스는 오늘도 여섯 명이다.</t>
+        </is>
+      </c>
+      <c r="G208" s="4" t="inlineStr"/>
+      <c r="H208" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:H189"/>
+  <autoFilter ref="A3:H208"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -7445,7 +8078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -7829,9 +8462,21 @@
       <c r="A19" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="6" t="inlineStr"/>
-      <c r="C19" s="6" t="inlineStr"/>
-      <c r="D19" s="6" t="inlineStr"/>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>어벤져스에 가면~</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>‘시장에 가면’ 놀이의 태오판. 누구누구 있는지 이어 말하기</t>
+        </is>
+      </c>
       <c r="E19" s="6" t="inlineStr"/>
       <c r="F19" s="6" t="inlineStr"/>
     </row>
@@ -8025,8 +8670,18 @@
       <c r="E38" s="4" t="inlineStr"/>
       <c r="F38" s="4" t="inlineStr"/>
     </row>
+    <row r="39">
+      <c r="A39" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" s="6" t="inlineStr"/>
+      <c r="C39" s="6" t="inlineStr"/>
+      <c r="D39" s="6" t="inlineStr"/>
+      <c r="E39" s="6" t="inlineStr"/>
+      <c r="F39" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F38"/>
+  <autoFilter ref="A3:F39"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add episode 13 "아빠 레몬 먹어!"
Taeo tells Dad "아빠 레몬 먹어!!", and when Dad says no he answers with
Dad's own line: "싫어하는 것도 먹어야 튼튼해지고 근육도 생겨!".
Episode 13 sets it up with Dad telling Taeo that over broccoli the night
before; the family laughs that Taeo hears everything, Dad eats the lemon
first, flexes, and Taeo then tries his broccoli, before offering the
lemon to Jaei and running from "김태오!!".

The saying joins Taeo's list; new lemon and broccoli props; Excel adds
episode 13. Cache v163.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$208</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$224</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$39</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1371,20 +1371,50 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="n">
+      <c r="A16" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="7" t="n"/>
-      <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
-      <c r="F16" s="7" t="n"/>
-      <c r="G16" s="7" t="n"/>
-      <c r="H16" s="7" t="n"/>
-      <c r="I16" s="7" t="n"/>
-      <c r="J16" s="7" t="inlineStr">
-        <is>
-          <t>기획 중</t>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>아빠 레몬 먹어!</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>“싫어하는 것도 먹어야 튼튼해지고 근육도 생겨.” 아빠가 태오에게 한 말이, 레몬이 되어 아빠에게 돌아왔다.</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>재이, 엄마, 아빠, 태오</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>“아빠 레몬 먹어!!” “싫어!” “싫어하는 것도 먹어야 튼튼해지고 근육도 생겨!” — 아빠 말 그대로 돌려주기 / 시큼!!! 부르르</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>아빠가 먼저 레몬을 먹자 태오도 브로콜리 도전 / 그리고 “누나 레몬 먹어!” → “김태오!!”</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>내가 한 말은 아이가 그대로 돌려줘요. 먼저 해 보이는 게 최고의 잔소리예요.</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>우리 가족이 제일 싫어하는 음식은 뭐예요? 오늘 한 입씩 같이 도전해 볼까요?</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>완성</t>
         </is>
       </c>
     </row>
@@ -1424,13 +1454,31 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="7" t="n"/>
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="7" t="n"/>
+      <c r="G19" s="7" t="n"/>
+      <c r="H19" s="7" t="n"/>
+      <c r="I19" s="7" t="n"/>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>기획 중</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:J15"/>
+  <autoFilter ref="A3:J16"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"아이디어,기획 중,콘티,완성"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1444,7 +1492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H208"/>
+  <dimension ref="A1:H224"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -8063,8 +8111,526 @@
       <c r="G208" s="4" t="inlineStr"/>
       <c r="H208" s="4" t="inlineStr"/>
     </row>
+    <row r="209">
+      <c r="A209" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B209" s="6" t="inlineStr">
+        <is>
+          <t>아빠 레몬 먹어!</t>
+        </is>
+      </c>
+      <c r="C209" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D209" s="6" t="inlineStr">
+        <is>
+          <t>부엌</t>
+        </is>
+      </c>
+      <c r="E209" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F209" s="6" t="inlineStr">
+        <is>
+          <t>저녁 식탁. 태오 접시엔 초록 나무가 세 그루.</t>
+        </is>
+      </c>
+      <c r="G209" s="6" t="inlineStr">
+        <is>
+          <t>브로콜리 싫어!</t>
+        </is>
+      </c>
+      <c r="H209" s="6" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B210" s="4" t="inlineStr">
+        <is>
+          <t>아빠 레몬 먹어!</t>
+        </is>
+      </c>
+      <c r="C210" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D210" s="4" t="inlineStr">
+        <is>
+          <t>부엌</t>
+        </is>
+      </c>
+      <c r="E210" s="4" t="inlineStr">
+        <is>
+          <t>아빠, 태오</t>
+        </is>
+      </c>
+      <c r="F210" s="4" t="inlineStr"/>
+      <c r="G210" s="4" t="inlineStr">
+        <is>
+          <t>태오야, 싫어하는 것도 먹어야 튼튼해지고 근육도 생겨.</t>
+        </is>
+      </c>
+      <c r="H210" s="4" t="inlineStr">
+        <is>
+          <t>불끈</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B211" s="6" t="inlineStr">
+        <is>
+          <t>아빠 레몬 먹어!</t>
+        </is>
+      </c>
+      <c r="C211" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D211" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E211" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F211" s="6" t="inlineStr"/>
+      <c r="G211" s="6" t="inlineStr"/>
+      <c r="H211" s="6" t="inlineStr">
+        <is>
+          <t>우웩…, 꿀꺽</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B212" s="4" t="inlineStr">
+        <is>
+          <t>아빠 레몬 먹어!</t>
+        </is>
+      </c>
+      <c r="C212" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D212" s="4" t="inlineStr">
+        <is>
+          <t>부엌</t>
+        </is>
+      </c>
+      <c r="E212" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F212" s="4" t="inlineStr">
+        <is>
+          <t>다음 날, 과일 바구니에서 태오가 발견한 것.</t>
+        </is>
+      </c>
+      <c r="G212" s="4" t="inlineStr">
+        <is>
+          <t>(생각) (흐흐흐…)</t>
+        </is>
+      </c>
+      <c r="H212" s="4" t="inlineStr">
+        <is>
+          <t>반짝</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B213" s="6" t="inlineStr">
+        <is>
+          <t>아빠 레몬 먹어!</t>
+        </is>
+      </c>
+      <c r="C213" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D213" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E213" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F213" s="6" t="inlineStr"/>
+      <c r="G213" s="6" t="inlineStr">
+        <is>
+          <t>아빠 레몬 먹어!!</t>
+        </is>
+      </c>
+      <c r="H213" s="6" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B214" s="4" t="inlineStr">
+        <is>
+          <t>아빠 레몬 먹어!</t>
+        </is>
+      </c>
+      <c r="C214" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D214" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E214" s="4" t="inlineStr">
+        <is>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F214" s="4" t="inlineStr"/>
+      <c r="G214" s="4" t="inlineStr">
+        <is>
+          <t>싫어! 그건 너무 시잖아!</t>
+        </is>
+      </c>
+      <c r="H214" s="4" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B215" s="6" t="inlineStr">
+        <is>
+          <t>아빠 레몬 먹어!</t>
+        </is>
+      </c>
+      <c r="C215" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="D215" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E215" s="6" t="inlineStr">
+        <is>
+          <t>태오, 아빠</t>
+        </is>
+      </c>
+      <c r="F215" s="6" t="inlineStr"/>
+      <c r="G215" s="6" t="inlineStr">
+        <is>
+          <t>싫어하는 것도 먹어야 튼튼해지고 근육도 생겨!</t>
+        </is>
+      </c>
+      <c r="H215" s="6" t="inlineStr">
+        <is>
+          <t>똑같이!</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B216" s="4" t="inlineStr">
+        <is>
+          <t>아빠 레몬 먹어!</t>
+        </is>
+      </c>
+      <c r="C216" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D216" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E216" s="4" t="inlineStr">
+        <is>
+          <t>재이, 엄마</t>
+        </is>
+      </c>
+      <c r="F216" s="4" t="inlineStr"/>
+      <c r="G216" s="4" t="inlineStr">
+        <is>
+          <t>아빠가 어제 한 말이랑 똑같아!
+태오는 다 듣고 있다니까~</t>
+        </is>
+      </c>
+      <c r="H216" s="4" t="inlineStr">
+        <is>
+          <t>깔깔깔</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B217" s="6" t="inlineStr">
+        <is>
+          <t>아빠 레몬 먹어!</t>
+        </is>
+      </c>
+      <c r="C217" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="D217" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E217" s="6" t="inlineStr">
+        <is>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F217" s="6" t="inlineStr"/>
+      <c r="G217" s="6" t="inlineStr">
+        <is>
+          <t>…그래. 아빠가 한 말이니까 아빠가 먼저 먹어야지.</t>
+        </is>
+      </c>
+      <c r="H217" s="6" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B218" s="4" t="inlineStr">
+        <is>
+          <t>아빠 레몬 먹어!</t>
+        </is>
+      </c>
+      <c r="C218" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D218" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E218" s="4" t="inlineStr">
+        <is>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F218" s="4" t="inlineStr"/>
+      <c r="G218" s="4" t="inlineStr"/>
+      <c r="H218" s="4" t="inlineStr">
+        <is>
+          <t>시큼!!!, 부르르, 부르르</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B219" s="6" t="inlineStr">
+        <is>
+          <t>아빠 레몬 먹어!</t>
+        </is>
+      </c>
+      <c r="C219" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="D219" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E219" s="6" t="inlineStr">
+        <is>
+          <t>아빠, 태오</t>
+        </is>
+      </c>
+      <c r="F219" s="6" t="inlineStr"/>
+      <c r="G219" s="6" t="inlineStr">
+        <is>
+          <t>크으… 아빠 근육 생겼다!
+진짜?!</t>
+        </is>
+      </c>
+      <c r="H219" s="6" t="inlineStr">
+        <is>
+          <t>불끈불끈</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B220" s="4" t="inlineStr">
+        <is>
+          <t>아빠 레몬 먹어!</t>
+        </is>
+      </c>
+      <c r="C220" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D220" s="4" t="inlineStr">
+        <is>
+          <t>부엌</t>
+        </is>
+      </c>
+      <c r="E220" s="4" t="inlineStr">
+        <is>
+          <t>태오, 아빠</t>
+        </is>
+      </c>
+      <c r="F220" s="4" t="inlineStr">
+        <is>
+          <t>그날 저녁.</t>
+        </is>
+      </c>
+      <c r="G220" s="4" t="inlineStr">
+        <is>
+          <t>그럼 나도! 브로콜리 먹을래!</t>
+        </is>
+      </c>
+      <c r="H220" s="4" t="inlineStr"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B221" s="6" t="inlineStr">
+        <is>
+          <t>아빠 레몬 먹어!</t>
+        </is>
+      </c>
+      <c r="C221" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="D221" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E221" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F221" s="6" t="inlineStr"/>
+      <c r="G221" s="6" t="inlineStr">
+        <is>
+          <t>나 근육 생겼어?</t>
+        </is>
+      </c>
+      <c r="H221" s="6" t="inlineStr">
+        <is>
+          <t>우물우물</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B222" s="4" t="inlineStr">
+        <is>
+          <t>아빠 레몬 먹어!</t>
+        </is>
+      </c>
+      <c r="C222" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="D222" s="4" t="inlineStr">
+        <is>
+          <t>부엌</t>
+        </is>
+      </c>
+      <c r="E222" s="4" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="F222" s="4" t="inlineStr"/>
+      <c r="G222" s="4" t="inlineStr">
+        <is>
+          <t>이제 누나 차례! 누나 레몬 먹어!</t>
+        </is>
+      </c>
+      <c r="H222" s="4" t="inlineStr"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B223" s="6" t="inlineStr">
+        <is>
+          <t>아빠 레몬 먹어!</t>
+        </is>
+      </c>
+      <c r="C223" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="D223" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E223" s="6" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F223" s="6" t="inlineStr"/>
+      <c r="G223" s="6" t="inlineStr">
+        <is>
+          <t>김태오!!</t>
+        </is>
+      </c>
+      <c r="H223" s="6" t="inlineStr">
+        <is>
+          <t>도망!</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B224" s="4" t="inlineStr">
+        <is>
+          <t>아빠 레몬 먹어!</t>
+        </is>
+      </c>
+      <c r="C224" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="D224" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E224" s="4" t="inlineStr"/>
+      <c r="F224" s="4" t="inlineStr">
+        <is>
+          <t>아빠가 한 말은 태오가 다 기억한다. / 그래서 아빠는 오늘도 먼저 한 입 먹는다.</t>
+        </is>
+      </c>
+      <c r="G224" s="4" t="inlineStr"/>
+      <c r="H224" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:H208"/>
+  <autoFilter ref="A3:H224"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -8695,7 +9261,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8910,13 +9476,13 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>왜 놀려! 놀리지 마!</t>
+          <t>아빠 레몬 먹어!! 싫어하는 것도 먹어야 튼튼해지고 근육도 생겨!</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr"/>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>“태오는 글씨·숫자 잘 몰라” 소리를 들으면 (손가락질하며)</t>
+          <t>아빠가 해 준 말을 그대로 돌려줄 때</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr"/>
@@ -8927,18 +9493,18 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>김태오!</t>
+          <t>왜 놀려! 놀리지 마!</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr"/>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+          <t>“태오는 글씨·숫자 잘 몰라” 소리를 들으면 (손가락질하며)</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr"/>
@@ -8949,22 +9515,18 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>짐방</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>김서방</t>
-        </is>
-      </c>
+          <t>김태오!</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr"/>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr"/>
@@ -8973,10 +9535,26 @@
       <c r="A14" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="4" t="inlineStr"/>
-      <c r="C14" s="4" t="inlineStr"/>
-      <c r="D14" s="4" t="inlineStr"/>
-      <c r="E14" s="4" t="inlineStr"/>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>짐방</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>김서방</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+        </is>
+      </c>
       <c r="F14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
@@ -9119,8 +9697,18 @@
       <c r="E28" s="4" t="inlineStr"/>
       <c r="F28" s="4" t="inlineStr"/>
     </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" s="6" t="inlineStr"/>
+      <c r="C29" s="6" t="inlineStr"/>
+      <c r="D29" s="6" t="inlineStr"/>
+      <c r="E29" s="6" t="inlineStr"/>
+      <c r="F29" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F28"/>
+  <autoFilter ref="A3:F29"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add episode 15 "타노스 나와라!"
More of Taeo: whenever the TV goes on he shouts "내꺼 틀어 줘!", when
bored he asks for something tasty, and then "싸우자!" His favourite game
is fighting Thanos with the Avengers. The three sayings join his list
and his bio.

Episode 15: Dad's news turns into Taeo's cartoon, snack requests ten
minutes after dinner, then Dad plays Thanos with Mom's purple rubber
glove and loses ten times with Jaei joining as Black Widow. Seeing Dad
worn out, Taeo takes the Thanos role and loses on purpose so Dad can
win; next morning it is "내꺼 틀어 줘!" again. Thanos is only named;
new TV and glove props. Excel adds episode 15. Cache v166.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$241</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$260</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$40</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>누나 괴롭히기가 취미인 막내(사실은 누나가 좋아서). 혼자 노는 것 같아도 가족 말을 다 듣고 있고, 틀려도 일단 소리 지르며 우기다가 들키면 머리를 긁적긁적. “맛있는 거 죠!”가 입버릇이고, 어벤져스 영웅도 태오식으로 불러요(블루베리, 쉬터맨, 스테잌로저…). 블랙 위도우랑 수가 제일 예쁘대요.</t>
+          <t>누나 괴롭히기가 취미인 막내(사실은 누나가 좋아서). 혼자 노는 것 같아도 가족 말을 다 듣고 있고, 틀려도 일단 소리 지르며 우기다가 들키면 머리를 긁적긁적. “맛있는 거 죠!”가 입버릇이고, 어벤져스 영웅도 태오식으로 불러요(블루베리, 쉬터맨, 스테잌로저…). 블랙 위도우랑 수가 제일 예쁘대요. 제일 좋아하는 놀이는 어벤져스로 타노스랑 싸우기!</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1467,20 +1467,50 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="n">
+      <c r="A18" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="7" t="n"/>
-      <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
-      <c r="F18" s="7" t="n"/>
-      <c r="G18" s="7" t="n"/>
-      <c r="H18" s="7" t="n"/>
-      <c r="I18" s="7" t="n"/>
-      <c r="J18" s="7" t="inlineStr">
-        <is>
-          <t>기획 중</t>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>티비만 틀면 “내꺼 틀어 줘!”, 심심하면 “맛있는 거 줘!”, 그리고 마지막은 언제나 “싸우자!” 오늘도 아빠는 타노스가 된다.</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>재이, 엄마, 아빠, 태오</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>아빠가 티비 켜자마자 “내꺼 틀어 줘!!” / 밥 먹고 10분 뒤 “심심해~ 맛있는 거 줘!” / “싸우자!” 엄마 고무장갑 낀 타노스 아빠</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>열 번 진 아빠를 보고 태오가 타노스를 맡아 일부러 져 준다 / “아빠 맨날 졌잖아. 오늘은 아빠가 이겨.”</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>매일 져 주는 사람이 있어요. 가끔은 우리가 그 사람을 쉬게 해 줘요.</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>우리 집에서 악당 역할을 제일 많이 해 준 사람은 누구예요? 오늘은 그 사람에게 뭐라고 말해 줄까요?</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>완성</t>
         </is>
       </c>
     </row>
@@ -1520,13 +1550,31 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="7" t="n"/>
+      <c r="C21" s="7" t="n"/>
+      <c r="D21" s="7" t="n"/>
+      <c r="E21" s="7" t="n"/>
+      <c r="F21" s="7" t="n"/>
+      <c r="G21" s="7" t="n"/>
+      <c r="H21" s="7" t="n"/>
+      <c r="I21" s="7" t="n"/>
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t>기획 중</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:J17"/>
+  <autoFilter ref="A3:J18"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"아이디어,기획 중,콘티,완성"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1540,7 +1588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H241"/>
+  <dimension ref="A1:H260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -9206,8 +9254,625 @@
       <c r="G241" s="6" t="inlineStr"/>
       <c r="H241" s="6" t="inlineStr"/>
     </row>
+    <row r="242">
+      <c r="A242" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B242" s="4" t="inlineStr">
+        <is>
+          <t>타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="C242" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D242" s="4" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E242" s="4" t="inlineStr">
+        <is>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F242" s="4" t="inlineStr">
+        <is>
+          <t>퇴근한 아빠, 오늘은 뉴스 좀 보려는데…</t>
+        </is>
+      </c>
+      <c r="G242" s="4" t="inlineStr"/>
+      <c r="H242" s="4" t="inlineStr">
+        <is>
+          <t>띡</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B243" s="6" t="inlineStr">
+        <is>
+          <t>타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="C243" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D243" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E243" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F243" s="6" t="inlineStr"/>
+      <c r="G243" s="6" t="inlineStr">
+        <is>
+          <t>내꺼 틀어 줘!!</t>
+        </is>
+      </c>
+      <c r="H243" s="6" t="inlineStr">
+        <is>
+          <t>0.1초</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B244" s="4" t="inlineStr">
+        <is>
+          <t>타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="C244" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D244" s="4" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E244" s="4" t="inlineStr">
+        <is>
+          <t>아빠, 태오</t>
+        </is>
+      </c>
+      <c r="F244" s="4" t="inlineStr"/>
+      <c r="G244" s="4" t="inlineStr">
+        <is>
+          <t>(속삭임) …아빠 뉴스는 내일 보지 뭐.</t>
+        </is>
+      </c>
+      <c r="H244" s="4" t="inlineStr"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B245" s="6" t="inlineStr">
+        <is>
+          <t>타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="C245" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D245" s="6" t="inlineStr">
+        <is>
+          <t>부엌</t>
+        </is>
+      </c>
+      <c r="E245" s="6" t="inlineStr">
+        <is>
+          <t>태오, 엄마</t>
+        </is>
+      </c>
+      <c r="F245" s="6" t="inlineStr">
+        <is>
+          <t>만화가 끝나고 10분 뒤.</t>
+        </is>
+      </c>
+      <c r="G245" s="6" t="inlineStr">
+        <is>
+          <t>엄마~ 심심해. 맛있는 거 줘!
+…밥 먹은 지 10분 됐어.</t>
+        </is>
+      </c>
+      <c r="H245" s="6" t="inlineStr"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B246" s="4" t="inlineStr">
+        <is>
+          <t>타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="C246" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D246" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E246" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F246" s="4" t="inlineStr"/>
+      <c r="G246" s="4" t="inlineStr">
+        <is>
+          <t>그럼 싸우자!!</t>
+        </is>
+      </c>
+      <c r="H246" s="4" t="inlineStr">
+        <is>
+          <t>번쩍</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B247" s="6" t="inlineStr">
+        <is>
+          <t>타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="C247" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D247" s="6" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E247" s="6" t="inlineStr">
+        <is>
+          <t>태오, 아빠</t>
+        </is>
+      </c>
+      <c r="F247" s="6" t="inlineStr"/>
+      <c r="G247" s="6" t="inlineStr">
+        <is>
+          <t>나는 어벤져스! 아빠는 타노스!
+또 아빠가 타노스야?</t>
+        </is>
+      </c>
+      <c r="H247" s="6" t="inlineStr"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B248" s="4" t="inlineStr">
+        <is>
+          <t>타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="C248" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D248" s="4" t="inlineStr">
+        <is>
+          <t>효과: 어두움</t>
+        </is>
+      </c>
+      <c r="E248" s="4" t="inlineStr">
+        <is>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F248" s="4" t="inlineStr"/>
+      <c r="G248" s="4" t="inlineStr">
+        <is>
+          <t>크크크… 나는 타노스다!</t>
+        </is>
+      </c>
+      <c r="H248" s="4" t="inlineStr">
+        <is>
+          <t>엄마 고무장갑</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B249" s="6" t="inlineStr">
+        <is>
+          <t>타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="C249" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D249" s="6" t="inlineStr">
+        <is>
+          <t>효과: 속도선</t>
+        </is>
+      </c>
+      <c r="E249" s="6" t="inlineStr">
+        <is>
+          <t>태오, 아빠</t>
+        </is>
+      </c>
+      <c r="F249" s="6" t="inlineStr"/>
+      <c r="G249" s="6" t="inlineStr">
+        <is>
+          <t>블루베리 펀치! 쉬터맨 거미줄! 스테잌로저 방패!</t>
+        </is>
+      </c>
+      <c r="H249" s="6" t="inlineStr">
+        <is>
+          <t>퍽!</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B250" s="4" t="inlineStr">
+        <is>
+          <t>타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="C250" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D250" s="4" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E250" s="4" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F250" s="4" t="inlineStr"/>
+      <c r="G250" s="4" t="inlineStr">
+        <is>
+          <t>블랙 위도우도 출동!
+누나 제일 예뻐!!</t>
+        </is>
+      </c>
+      <c r="H250" s="4" t="inlineStr"/>
+    </row>
+    <row r="251">
+      <c r="A251" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B251" s="6" t="inlineStr">
+        <is>
+          <t>타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="C251" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D251" s="6" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E251" s="6" t="inlineStr">
+        <is>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F251" s="6" t="inlineStr"/>
+      <c r="G251" s="6" t="inlineStr">
+        <is>
+          <t>으악… 타노스가 졌다…</t>
+        </is>
+      </c>
+      <c r="H251" s="6" t="inlineStr">
+        <is>
+          <t>쿵!</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B252" s="4" t="inlineStr">
+        <is>
+          <t>타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="C252" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D252" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E252" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F252" s="4" t="inlineStr"/>
+      <c r="G252" s="4" t="inlineStr">
+        <is>
+          <t>또 해! 또 해!!</t>
+        </is>
+      </c>
+      <c r="H252" s="4" t="inlineStr"/>
+    </row>
+    <row r="253">
+      <c r="A253" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B253" s="6" t="inlineStr">
+        <is>
+          <t>타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="C253" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D253" s="6" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E253" s="6" t="inlineStr">
+        <is>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F253" s="6" t="inlineStr">
+        <is>
+          <t>그렇게 타노스는 열 번 졌다.</t>
+        </is>
+      </c>
+      <c r="G253" s="6" t="inlineStr"/>
+      <c r="H253" s="6" t="inlineStr">
+        <is>
+          <t>헥헥</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B254" s="4" t="inlineStr">
+        <is>
+          <t>타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="C254" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="D254" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E254" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F254" s="4" t="inlineStr"/>
+      <c r="G254" s="4" t="inlineStr">
+        <is>
+          <t>(생각) (…아빠 힘든가?)</t>
+        </is>
+      </c>
+      <c r="H254" s="4" t="inlineStr"/>
+    </row>
+    <row r="255">
+      <c r="A255" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B255" s="6" t="inlineStr">
+        <is>
+          <t>타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="C255" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="D255" s="6" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E255" s="6" t="inlineStr">
+        <is>
+          <t>태오, 아빠</t>
+        </is>
+      </c>
+      <c r="F255" s="6" t="inlineStr"/>
+      <c r="G255" s="6" t="inlineStr">
+        <is>
+          <t>이번엔 내가 타노스 할게. 아빠가 어벤져스 해.</t>
+        </is>
+      </c>
+      <c r="H255" s="6" t="inlineStr"/>
+    </row>
+    <row r="256">
+      <c r="A256" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B256" s="4" t="inlineStr">
+        <is>
+          <t>타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="C256" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="D256" s="4" t="inlineStr">
+        <is>
+          <t>효과: 속도선</t>
+        </is>
+      </c>
+      <c r="E256" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F256" s="4" t="inlineStr"/>
+      <c r="G256" s="4" t="inlineStr">
+        <is>
+          <t>으악~ 타노스 졌다~ 아빠가 이겼다!</t>
+        </is>
+      </c>
+      <c r="H256" s="4" t="inlineStr">
+        <is>
+          <t>털썩</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B257" s="6" t="inlineStr">
+        <is>
+          <t>타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="C257" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="D257" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E257" s="6" t="inlineStr">
+        <is>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F257" s="6" t="inlineStr"/>
+      <c r="G257" s="6" t="inlineStr">
+        <is>
+          <t>태오야… 일부러 져 준 거야?</t>
+        </is>
+      </c>
+      <c r="H257" s="6" t="inlineStr"/>
+    </row>
+    <row r="258">
+      <c r="A258" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B258" s="4" t="inlineStr">
+        <is>
+          <t>타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="C258" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="D258" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E258" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F258" s="4" t="inlineStr"/>
+      <c r="G258" s="4" t="inlineStr">
+        <is>
+          <t>아빠 맨날 졌잖아. 오늘은 아빠가 이겨.</t>
+        </is>
+      </c>
+      <c r="H258" s="4" t="inlineStr"/>
+    </row>
+    <row r="259">
+      <c r="A259" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B259" s="6" t="inlineStr">
+        <is>
+          <t>타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="C259" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="D259" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E259" s="6" t="inlineStr">
+        <is>
+          <t>태오, 아빠</t>
+        </is>
+      </c>
+      <c r="F259" s="6" t="inlineStr">
+        <is>
+          <t>아빠 배터리, 다시 100%.</t>
+        </is>
+      </c>
+      <c r="G259" s="6" t="inlineStr"/>
+      <c r="H259" s="6" t="inlineStr"/>
+    </row>
+    <row r="260">
+      <c r="A260" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B260" s="4" t="inlineStr">
+        <is>
+          <t>타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="C260" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="D260" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E260" s="4" t="inlineStr">
+        <is>
+          <t>태오, 아빠</t>
+        </is>
+      </c>
+      <c r="F260" s="4" t="inlineStr">
+        <is>
+          <t>다음 날 아침.</t>
+        </is>
+      </c>
+      <c r="G260" s="4" t="inlineStr">
+        <is>
+          <t>내꺼 틀어 줘!!</t>
+        </is>
+      </c>
+      <c r="H260" s="4" t="inlineStr">
+        <is>
+          <t>…역시</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:H241"/>
+  <autoFilter ref="A3:H260"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -9860,7 +10525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -10119,13 +10784,13 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>왜 놀려! 놀리지 마!</t>
+          <t>내꺼 틀어 줘!</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr"/>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>“태오는 글씨·숫자 잘 몰라” 소리를 들으면 (손가락질하며)</t>
+          <t>누가 티비만 틀면</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr"/>
@@ -10136,18 +10801,18 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>김태오!</t>
+          <t>심심해~ 맛있는 거 줘!</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr"/>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+          <t>심심할 때마다</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr"/>
@@ -10158,22 +10823,18 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>짐방</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>김서방</t>
-        </is>
-      </c>
+          <t>싸우자! 타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr"/>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+          <t>어벤져스로 타노스랑 싸우는 놀이가 제일 좋을 때</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr"/>
@@ -10182,30 +10843,70 @@
       <c r="A16" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="4" t="inlineStr"/>
-      <c r="C16" s="4" t="inlineStr"/>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>태오 입버릇</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>왜 놀려! 놀리지 마!</t>
+        </is>
+      </c>
       <c r="D16" s="4" t="inlineStr"/>
-      <c r="E16" s="4" t="inlineStr"/>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>“태오는 글씨·숫자 잘 몰라” 소리를 들으면 (손가락질하며)</t>
+        </is>
+      </c>
       <c r="F16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="6" t="inlineStr"/>
-      <c r="C17" s="6" t="inlineStr"/>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>재이 입버릇</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>김태오!</t>
+        </is>
+      </c>
       <c r="D17" s="6" t="inlineStr"/>
-      <c r="E17" s="6" t="inlineStr"/>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+        </is>
+      </c>
       <c r="F17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="4" t="inlineStr"/>
-      <c r="C18" s="4" t="inlineStr"/>
-      <c r="D18" s="4" t="inlineStr"/>
-      <c r="E18" s="4" t="inlineStr"/>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>짐방</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>김서방</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+        </is>
+      </c>
       <c r="F18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
@@ -10328,8 +11029,38 @@
       <c r="E30" s="4" t="inlineStr"/>
       <c r="F30" s="4" t="inlineStr"/>
     </row>
+    <row r="31">
+      <c r="A31" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" s="6" t="inlineStr"/>
+      <c r="C31" s="6" t="inlineStr"/>
+      <c r="D31" s="6" t="inlineStr"/>
+      <c r="E31" s="6" t="inlineStr"/>
+      <c r="F31" s="6" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" s="4" t="inlineStr"/>
+      <c r="C32" s="4" t="inlineStr"/>
+      <c r="D32" s="4" t="inlineStr"/>
+      <c r="E32" s="4" t="inlineStr"/>
+      <c r="F32" s="4" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" s="6" t="inlineStr"/>
+      <c r="C33" s="6" t="inlineStr"/>
+      <c r="D33" s="6" t="inlineStr"/>
+      <c r="E33" s="6" t="inlineStr"/>
+      <c r="F33" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F30"/>
+  <autoFilter ref="A3:F33"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Note that Dad always plays Thanos
The family confirmed that in Taeo's favourite Avengers game Dad is
always Thanos. Dad's bio and Taeo's "싸우자! 타노스 나와라!" saying say
so, and the Excel sheet is regenerated. Cache v167.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -641,7 +641,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>아재개그 담당, 목말 태우기 전문. 방귀는 아빠가 원조라는 소문이 있어요.</t>
+          <t>아재개그 담당, 목말 태우기 전문. 방귀는 아빠가 원조라는 소문이 있어요. 태오랑 놀 때는 언제나 타노스 역을 맡아요.</t>
         </is>
       </c>
     </row>
@@ -10834,7 +10834,7 @@
       <c r="D15" s="6" t="inlineStr"/>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>어벤져스로 타노스랑 싸우는 놀이가 제일 좋을 때</t>
+          <t>제일 좋아하는 놀이, 어벤져스로 타노스랑 싸우기 (타노스는 늘 아빠)</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr"/>

</xml_diff>

<commit_message>
Give Dad's Thanos a gauntlet and add 인에터블 and 꿍끙이
The family filled in the details: Dad plays Thanos wearing an Infinity
Gauntlet and says "아임 인에비터블", which Taeo repeats as "아임
인에터블". Jaei called 방귀대장 뿡뿡이 "꿍끙이".

Episode 15 now uses a gold gauntlet toy instead of the invented rubber
glove; Dad says the line, a new panel has Taeo shout "아임 인에터블!!"
with Jaei whispering the right word, and Taeo says it again when he
takes the Thanos role. 인에터블 joins Taeo's dictionary, 꿍끙이 joins
Jaei's baby words and appears in Mom's notebook in episode 6. Excel
regenerated. Cache v168.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -17,9 +17,9 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$260</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$40</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$261</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1055,7 +1055,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>블루베리·스테잌로저·미스테리 / 우엉조림을 보고 “우엉은 마법사잖아!” / 할머니께 “쓰구미!” / 아기 재이의 “짐방!”</t>
+          <t>블루베리·스테잌로저·미스테리 / 우엉조림을 보고 “우엉은 마법사잖아!” / 할머니께 “쓰구미!” / 아기 재이의 “짐방!” (공책엔 꿍끙이 = 뿡뿡이도)</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -1477,7 +1477,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>티비만 틀면 “내꺼 틀어 줘!”, 심심하면 “맛있는 거 줘!”, 그리고 마지막은 언제나 “싸우자!” 오늘도 아빠는 타노스가 된다.</t>
+          <t>티비만 틀면 “내꺼 틀어 줘!”, 심심하면 “맛있는 거 줘!”, 그리고 마지막은 언제나 “싸우자!” 오늘도 아빠는 건틀렛을 끼고 타노스가 된다.</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -1487,7 +1487,7 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>아빠가 티비 켜자마자 “내꺼 틀어 줘!!” / 밥 먹고 10분 뒤 “심심해~ 맛있는 거 줘!” / “싸우자!” 엄마 고무장갑 낀 타노스 아빠</t>
+          <t>아빠가 티비 켜자마자 “내꺼 틀어 줘!!” / 밥 먹고 10분 뒤 “심심해~ 맛있는 거 줘!” / “싸우자!” 건틀렛 낀 타노스 아빠 “아임 인에비터블!” → 태오 “아임 인에터블!!”</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1506,7 +1506,7 @@
         </is>
       </c>
       <c r="I18" s="3" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
@@ -1588,7 +1588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H260"/>
+  <dimension ref="A1:H261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -9477,12 +9477,12 @@
       <c r="F248" s="4" t="inlineStr"/>
       <c r="G248" s="4" t="inlineStr">
         <is>
-          <t>크크크… 나는 타노스다!</t>
+          <t>아임… 인에비터블!</t>
         </is>
       </c>
       <c r="H248" s="4" t="inlineStr">
         <is>
-          <t>엄마 고무장갑</t>
+          <t>번쩍</t>
         </is>
       </c>
     </row>
@@ -9500,25 +9500,22 @@
       </c>
       <c r="D249" s="6" t="inlineStr">
         <is>
-          <t>효과: 속도선</t>
+          <t>효과: 집중선</t>
         </is>
       </c>
       <c r="E249" s="6" t="inlineStr">
         <is>
-          <t>태오, 아빠</t>
+          <t>태오, 재이</t>
         </is>
       </c>
       <c r="F249" s="6" t="inlineStr"/>
       <c r="G249" s="6" t="inlineStr">
         <is>
-          <t>블루베리 펀치! 쉬터맨 거미줄! 스테잌로저 방패!</t>
-        </is>
-      </c>
-      <c r="H249" s="6" t="inlineStr">
-        <is>
-          <t>퍽!</t>
-        </is>
-      </c>
+          <t>아임 인에터블!!
+(속삭임) (…인에비터블이야.)</t>
+        </is>
+      </c>
+      <c r="H249" s="6" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" s="3" t="n">
@@ -9534,22 +9531,25 @@
       </c>
       <c r="D250" s="4" t="inlineStr">
         <is>
-          <t>거실(밤)</t>
+          <t>효과: 속도선</t>
         </is>
       </c>
       <c r="E250" s="4" t="inlineStr">
         <is>
-          <t>재이, 태오</t>
+          <t>태오, 아빠</t>
         </is>
       </c>
       <c r="F250" s="4" t="inlineStr"/>
       <c r="G250" s="4" t="inlineStr">
         <is>
-          <t>블랙 위도우도 출동!
-누나 제일 예뻐!!</t>
-        </is>
-      </c>
-      <c r="H250" s="4" t="inlineStr"/>
+          <t>블루베리 펀치! 쉬터맨 거미줄! 스테잌로저 방패!</t>
+        </is>
+      </c>
+      <c r="H250" s="4" t="inlineStr">
+        <is>
+          <t>퍽!</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="5" t="n">
@@ -9570,20 +9570,17 @@
       </c>
       <c r="E251" s="6" t="inlineStr">
         <is>
-          <t>아빠</t>
+          <t>재이, 태오</t>
         </is>
       </c>
       <c r="F251" s="6" t="inlineStr"/>
       <c r="G251" s="6" t="inlineStr">
         <is>
-          <t>으악… 타노스가 졌다…</t>
-        </is>
-      </c>
-      <c r="H251" s="6" t="inlineStr">
-        <is>
-          <t>쿵!</t>
-        </is>
-      </c>
+          <t>블랙 위도우도 출동!
+누나 제일 예뻐!!</t>
+        </is>
+      </c>
+      <c r="H251" s="6" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" s="3" t="n">
@@ -9599,21 +9596,25 @@
       </c>
       <c r="D252" s="4" t="inlineStr">
         <is>
-          <t>효과: 집중선</t>
+          <t>거실(밤)</t>
         </is>
       </c>
       <c r="E252" s="4" t="inlineStr">
         <is>
-          <t>태오</t>
+          <t>아빠</t>
         </is>
       </c>
       <c r="F252" s="4" t="inlineStr"/>
       <c r="G252" s="4" t="inlineStr">
         <is>
-          <t>또 해! 또 해!!</t>
-        </is>
-      </c>
-      <c r="H252" s="4" t="inlineStr"/>
+          <t>으악… 타노스가 졌다…</t>
+        </is>
+      </c>
+      <c r="H252" s="4" t="inlineStr">
+        <is>
+          <t>쿵!</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="5" t="n">
@@ -9629,25 +9630,21 @@
       </c>
       <c r="D253" s="6" t="inlineStr">
         <is>
-          <t>거실(밤)</t>
+          <t>효과: 집중선</t>
         </is>
       </c>
       <c r="E253" s="6" t="inlineStr">
         <is>
-          <t>아빠</t>
-        </is>
-      </c>
-      <c r="F253" s="6" t="inlineStr">
-        <is>
-          <t>그렇게 타노스는 열 번 졌다.</t>
-        </is>
-      </c>
-      <c r="G253" s="6" t="inlineStr"/>
-      <c r="H253" s="6" t="inlineStr">
-        <is>
-          <t>헥헥</t>
-        </is>
-      </c>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F253" s="6" t="inlineStr"/>
+      <c r="G253" s="6" t="inlineStr">
+        <is>
+          <t>또 해! 또 해!!</t>
+        </is>
+      </c>
+      <c r="H253" s="6" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" s="3" t="n">
@@ -9663,21 +9660,25 @@
       </c>
       <c r="D254" s="4" t="inlineStr">
         <is>
-          <t>효과: 반짝</t>
+          <t>거실(밤)</t>
         </is>
       </c>
       <c r="E254" s="4" t="inlineStr">
         <is>
-          <t>태오</t>
-        </is>
-      </c>
-      <c r="F254" s="4" t="inlineStr"/>
-      <c r="G254" s="4" t="inlineStr">
-        <is>
-          <t>(생각) (…아빠 힘든가?)</t>
-        </is>
-      </c>
-      <c r="H254" s="4" t="inlineStr"/>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F254" s="4" t="inlineStr">
+        <is>
+          <t>그렇게 타노스는 열 번 졌다.</t>
+        </is>
+      </c>
+      <c r="G254" s="4" t="inlineStr"/>
+      <c r="H254" s="4" t="inlineStr">
+        <is>
+          <t>헥헥</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="5" t="n">
@@ -9693,18 +9694,18 @@
       </c>
       <c r="D255" s="6" t="inlineStr">
         <is>
-          <t>거실(밤)</t>
+          <t>효과: 반짝</t>
         </is>
       </c>
       <c r="E255" s="6" t="inlineStr">
         <is>
-          <t>태오, 아빠</t>
+          <t>태오</t>
         </is>
       </c>
       <c r="F255" s="6" t="inlineStr"/>
       <c r="G255" s="6" t="inlineStr">
         <is>
-          <t>이번엔 내가 타노스 할게. 아빠가 어벤져스 해.</t>
+          <t>(생각) (…아빠 힘든가?)</t>
         </is>
       </c>
       <c r="H255" s="6" t="inlineStr"/>
@@ -9723,25 +9724,21 @@
       </c>
       <c r="D256" s="4" t="inlineStr">
         <is>
-          <t>효과: 속도선</t>
+          <t>거실(밤)</t>
         </is>
       </c>
       <c r="E256" s="4" t="inlineStr">
         <is>
-          <t>태오</t>
+          <t>태오, 아빠</t>
         </is>
       </c>
       <c r="F256" s="4" t="inlineStr"/>
       <c r="G256" s="4" t="inlineStr">
         <is>
-          <t>으악~ 타노스 졌다~ 아빠가 이겼다!</t>
-        </is>
-      </c>
-      <c r="H256" s="4" t="inlineStr">
-        <is>
-          <t>털썩</t>
-        </is>
-      </c>
+          <t>이번엔 내가 타노스 할게. 아임 인에터블!</t>
+        </is>
+      </c>
+      <c r="H256" s="4" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" s="5" t="n">
@@ -9757,21 +9754,25 @@
       </c>
       <c r="D257" s="6" t="inlineStr">
         <is>
-          <t>효과: 반짝</t>
+          <t>효과: 속도선</t>
         </is>
       </c>
       <c r="E257" s="6" t="inlineStr">
         <is>
-          <t>아빠</t>
+          <t>태오</t>
         </is>
       </c>
       <c r="F257" s="6" t="inlineStr"/>
       <c r="G257" s="6" t="inlineStr">
         <is>
-          <t>태오야… 일부러 져 준 거야?</t>
-        </is>
-      </c>
-      <c r="H257" s="6" t="inlineStr"/>
+          <t>으악~ 타노스 졌다~ 아빠가 이겼다!</t>
+        </is>
+      </c>
+      <c r="H257" s="6" t="inlineStr">
+        <is>
+          <t>털썩</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="3" t="n">
@@ -9792,13 +9793,13 @@
       </c>
       <c r="E258" s="4" t="inlineStr">
         <is>
-          <t>태오</t>
+          <t>아빠</t>
         </is>
       </c>
       <c r="F258" s="4" t="inlineStr"/>
       <c r="G258" s="4" t="inlineStr">
         <is>
-          <t>아빠 맨날 졌잖아. 오늘은 아빠가 이겨.</t>
+          <t>태오야… 일부러 져 준 거야?</t>
         </is>
       </c>
       <c r="H258" s="4" t="inlineStr"/>
@@ -9822,15 +9823,15 @@
       </c>
       <c r="E259" s="6" t="inlineStr">
         <is>
-          <t>태오, 아빠</t>
-        </is>
-      </c>
-      <c r="F259" s="6" t="inlineStr">
-        <is>
-          <t>아빠 배터리, 다시 100%.</t>
-        </is>
-      </c>
-      <c r="G259" s="6" t="inlineStr"/>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F259" s="6" t="inlineStr"/>
+      <c r="G259" s="6" t="inlineStr">
+        <is>
+          <t>아빠 맨날 졌잖아. 오늘은 아빠가 이겨.</t>
+        </is>
+      </c>
       <c r="H259" s="6" t="inlineStr"/>
     </row>
     <row r="260">
@@ -9847,32 +9848,62 @@
       </c>
       <c r="D260" s="4" t="inlineStr">
         <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E260" s="4" t="inlineStr">
+        <is>
+          <t>태오, 아빠</t>
+        </is>
+      </c>
+      <c r="F260" s="4" t="inlineStr">
+        <is>
+          <t>아빠 배터리, 다시 100%.</t>
+        </is>
+      </c>
+      <c r="G260" s="4" t="inlineStr"/>
+      <c r="H260" s="4" t="inlineStr"/>
+    </row>
+    <row r="261">
+      <c r="A261" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B261" s="6" t="inlineStr">
+        <is>
+          <t>타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="C261" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="D261" s="6" t="inlineStr">
+        <is>
           <t>거실</t>
         </is>
       </c>
-      <c r="E260" s="4" t="inlineStr">
+      <c r="E261" s="6" t="inlineStr">
         <is>
           <t>태오, 아빠</t>
         </is>
       </c>
-      <c r="F260" s="4" t="inlineStr">
+      <c r="F261" s="6" t="inlineStr">
         <is>
           <t>다음 날 아침.</t>
         </is>
       </c>
-      <c r="G260" s="4" t="inlineStr">
+      <c r="G261" s="6" t="inlineStr">
         <is>
           <t>내꺼 틀어 줘!!</t>
         </is>
       </c>
-      <c r="H260" s="4" t="inlineStr">
+      <c r="H261" s="6" t="inlineStr">
         <is>
           <t>…역시</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:H260"/>
+  <autoFilter ref="A3:H261"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -9886,7 +9917,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -10294,17 +10325,17 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>어벤져스에 가년~</t>
+          <t>아임 인에터블</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>어벤져스에 가면~</t>
+          <t>아임 인에비터블 (I am inevitable)</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>‘시장에 가면’ 놀이의 태오판. 누구누구 있는지 이어 말하기</t>
+          <t>아빠 타노스가 건틀렛 끼고 하는 대사를 따라 할 때</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr"/>
@@ -10314,9 +10345,21 @@
       <c r="A21" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="6" t="inlineStr"/>
-      <c r="C21" s="6" t="inlineStr"/>
-      <c r="D21" s="6" t="inlineStr"/>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>어벤져스에 가면~</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>‘시장에 가면’ 놀이의 태오판. 누구누구 있는지 이어 말하기</t>
+        </is>
+      </c>
       <c r="E21" s="6" t="inlineStr"/>
       <c r="F21" s="6" t="inlineStr"/>
     </row>
@@ -10510,8 +10553,18 @@
       <c r="E40" s="4" t="inlineStr"/>
       <c r="F40" s="4" t="inlineStr"/>
     </row>
+    <row r="41">
+      <c r="A41" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" s="6" t="inlineStr"/>
+      <c r="C41" s="6" t="inlineStr"/>
+      <c r="D41" s="6" t="inlineStr"/>
+      <c r="E41" s="6" t="inlineStr"/>
+      <c r="F41" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F40"/>
+  <autoFilter ref="A3:F41"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -10525,7 +10578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -10834,7 +10887,7 @@
       <c r="D15" s="6" t="inlineStr"/>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>제일 좋아하는 놀이, 어벤져스로 타노스랑 싸우기 (타노스는 늘 아빠)</t>
+          <t>제일 좋아하는 놀이, 어벤져스로 타노스랑 싸우기 (타노스는 늘 아빠, 건틀렛 끼고 “아임 인에비터블”)</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr"/>
@@ -10913,10 +10966,26 @@
       <c r="A19" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="6" t="inlineStr"/>
-      <c r="C19" s="6" t="inlineStr"/>
-      <c r="D19" s="6" t="inlineStr"/>
-      <c r="E19" s="6" t="inlineStr"/>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>꿍끙이</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>뿡뿡이</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+        </is>
+      </c>
       <c r="F19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
@@ -11059,8 +11128,18 @@
       <c r="E33" s="6" t="inlineStr"/>
       <c r="F33" s="6" t="inlineStr"/>
     </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" s="4" t="inlineStr"/>
+      <c r="C34" s="4" t="inlineStr"/>
+      <c r="D34" s="4" t="inlineStr"/>
+      <c r="E34" s="4" t="inlineStr"/>
+      <c r="F34" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F33"/>
+  <autoFilter ref="A3:F34"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Taeo loves sour fruit: rework episode 13 around it
The family says Taeo loves lemons and other sour fruit like plums and
pineapple. His bio says so, and episode 13 now shows it: he finds his
favourite lemon, plum and pineapple in the fruit basket and eats lemon
happily before offering it to Dad, and after Dad's "시큼!!!" he asks
"뭐가 셔? 맛있는데." New sour fruit basket prop; Excel regenerated.
Cache v169.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$261</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$263</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$10</definedName>
@@ -696,12 +696,12 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>파란 윗옷·바지 (태권도복: 파란띠에 초록 줄)</t>
+          <t>파란 윗옷·바지 (태권도복: 파란띠에 초록 줄) · 좋아하는 것: 레몬·자두·파인애플 같은 신 과일</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>누나 괴롭히기가 취미인 막내(사실은 누나가 좋아서). 혼자 노는 것 같아도 가족 말을 다 듣고 있고, 틀려도 일단 소리 지르며 우기다가 들키면 머리를 긁적긁적. “맛있는 거 죠!”가 입버릇이고, 어벤져스 영웅도 태오식으로 불러요(블루베리, 쉬터맨, 스테잌로저…). 블랙 위도우랑 수가 제일 예쁘대요. 제일 좋아하는 놀이는 어벤져스로 타노스랑 싸우기!</t>
+          <t>누나 괴롭히기가 취미인 막내(사실은 누나가 좋아서). 혼자 노는 것 같아도 가족 말을 다 듣고 있고, 틀려도 일단 소리 지르며 우기다가 들키면 머리를 긁적긁적. “맛있는 거 죠!”가 입버릇이고, 어벤져스 영웅도 태오식으로 불러요(블루베리, 쉬터맨, 스테잌로저…). 블랙 위도우랑 수가 제일 예쁘대요. 제일 좋아하는 놀이는 어벤져스로 타노스랑 싸우기! 레몬·자두·파인애플처럼 신 과일을 제일 좋아해요.</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1381,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>“싫어하는 것도 먹어야 튼튼해지고 근육도 생겨.” 아빠가 태오에게 한 말이, 레몬이 되어 아빠에게 돌아왔다.</t>
+          <t>“싫어하는 것도 먹어야 튼튼해지고 근육도 생겨.” 아빠가 태오에게 한 말이, 태오가 제일 좋아하는 레몬이 되어 아빠에게 돌아왔다.</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -1391,7 +1391,7 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>“아빠 레몬 먹어!!” “싫어!” “싫어하는 것도 먹어야 튼튼해지고 근육도 생겨!” — 아빠 말 그대로 돌려주기 / 시큼!!! 부르르</t>
+          <t>태오가 제일 좋아하는 레몬·자두·파인애플 / “아빠 레몬 먹어!!” “싫어!” “싫어하는 것도 먹어야 튼튼해지고 근육도 생겨!” — 아빠 말 그대로 돌려주기 / 시큼!!! 부르르 → 태오 “뭐가 셔? 맛있는데.”</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -1410,7 +1410,7 @@
         </is>
       </c>
       <c r="I16" s="3" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
@@ -1588,7 +1588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H261"/>
+  <dimension ref="A1:H263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -8329,19 +8329,15 @@
       </c>
       <c r="F212" s="4" t="inlineStr">
         <is>
-          <t>다음 날, 과일 바구니에서 태오가 발견한 것.</t>
+          <t>다음 날, 과일 바구니. 태오가 제일 좋아하는 신 과일들!</t>
         </is>
       </c>
       <c r="G212" s="4" t="inlineStr">
         <is>
-          <t>(생각) (흐흐흐…)</t>
-        </is>
-      </c>
-      <c r="H212" s="4" t="inlineStr">
-        <is>
-          <t>반짝</t>
-        </is>
-      </c>
+          <t>레몬! 자두! 파인애플!</t>
+        </is>
+      </c>
+      <c r="H212" s="4" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" s="5" t="n">
@@ -8357,7 +8353,7 @@
       </c>
       <c r="D213" s="6" t="inlineStr">
         <is>
-          <t>효과: 집중선</t>
+          <t>효과: 반짝</t>
         </is>
       </c>
       <c r="E213" s="6" t="inlineStr">
@@ -8368,10 +8364,14 @@
       <c r="F213" s="6" t="inlineStr"/>
       <c r="G213" s="6" t="inlineStr">
         <is>
-          <t>아빠 레몬 먹어!!</t>
-        </is>
-      </c>
-      <c r="H213" s="6" t="inlineStr"/>
+          <t>음~ 새콤해! 레몬이 제일 맛있어!</t>
+        </is>
+      </c>
+      <c r="H213" s="6" t="inlineStr">
+        <is>
+          <t>쪽쪽</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="3" t="n">
@@ -8392,13 +8392,13 @@
       </c>
       <c r="E214" s="4" t="inlineStr">
         <is>
-          <t>아빠</t>
+          <t>태오</t>
         </is>
       </c>
       <c r="F214" s="4" t="inlineStr"/>
       <c r="G214" s="4" t="inlineStr">
         <is>
-          <t>싫어! 그건 너무 시잖아!</t>
+          <t>아빠 레몬 먹어!!</t>
         </is>
       </c>
       <c r="H214" s="4" t="inlineStr"/>
@@ -8417,25 +8417,21 @@
       </c>
       <c r="D215" s="6" t="inlineStr">
         <is>
-          <t>거실</t>
+          <t>효과: 집중선</t>
         </is>
       </c>
       <c r="E215" s="6" t="inlineStr">
         <is>
-          <t>태오, 아빠</t>
+          <t>아빠</t>
         </is>
       </c>
       <c r="F215" s="6" t="inlineStr"/>
       <c r="G215" s="6" t="inlineStr">
         <is>
-          <t>싫어하는 것도 먹어야 튼튼해지고 근육도 생겨!</t>
-        </is>
-      </c>
-      <c r="H215" s="6" t="inlineStr">
-        <is>
-          <t>똑같이!</t>
-        </is>
-      </c>
+          <t>싫어! 그건 너무 시잖아!</t>
+        </is>
+      </c>
+      <c r="H215" s="6" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" s="3" t="n">
@@ -8456,19 +8452,18 @@
       </c>
       <c r="E216" s="4" t="inlineStr">
         <is>
-          <t>재이, 엄마</t>
+          <t>태오, 아빠</t>
         </is>
       </c>
       <c r="F216" s="4" t="inlineStr"/>
       <c r="G216" s="4" t="inlineStr">
         <is>
-          <t>아빠가 어제 한 말이랑 똑같아!
-태오는 다 듣고 있다니까~</t>
+          <t>싫어하는 것도 먹어야 튼튼해지고 근육도 생겨!</t>
         </is>
       </c>
       <c r="H216" s="4" t="inlineStr">
         <is>
-          <t>깔깔깔</t>
+          <t>똑같이!</t>
         </is>
       </c>
     </row>
@@ -8486,21 +8481,26 @@
       </c>
       <c r="D217" s="6" t="inlineStr">
         <is>
-          <t>효과: 반짝</t>
+          <t>거실</t>
         </is>
       </c>
       <c r="E217" s="6" t="inlineStr">
         <is>
-          <t>아빠</t>
+          <t>재이, 엄마</t>
         </is>
       </c>
       <c r="F217" s="6" t="inlineStr"/>
       <c r="G217" s="6" t="inlineStr">
         <is>
-          <t>…그래. 아빠가 한 말이니까 아빠가 먼저 먹어야지.</t>
-        </is>
-      </c>
-      <c r="H217" s="6" t="inlineStr"/>
+          <t>아빠가 어제 한 말이랑 똑같아!
+태오는 다 듣고 있다니까~</t>
+        </is>
+      </c>
+      <c r="H217" s="6" t="inlineStr">
+        <is>
+          <t>깔깔깔</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="3" t="n">
@@ -8516,7 +8516,7 @@
       </c>
       <c r="D218" s="4" t="inlineStr">
         <is>
-          <t>효과: 집중선</t>
+          <t>효과: 반짝</t>
         </is>
       </c>
       <c r="E218" s="4" t="inlineStr">
@@ -8525,12 +8525,12 @@
         </is>
       </c>
       <c r="F218" s="4" t="inlineStr"/>
-      <c r="G218" s="4" t="inlineStr"/>
-      <c r="H218" s="4" t="inlineStr">
-        <is>
-          <t>시큼!!!, 부르르, 부르르</t>
-        </is>
-      </c>
+      <c r="G218" s="4" t="inlineStr">
+        <is>
+          <t>…그래. 아빠가 한 말이니까 아빠가 먼저 먹어야지.</t>
+        </is>
+      </c>
+      <c r="H218" s="4" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" s="5" t="n">
@@ -8546,24 +8546,19 @@
       </c>
       <c r="D219" s="6" t="inlineStr">
         <is>
-          <t>거실</t>
+          <t>효과: 집중선</t>
         </is>
       </c>
       <c r="E219" s="6" t="inlineStr">
         <is>
-          <t>아빠, 태오</t>
+          <t>아빠</t>
         </is>
       </c>
       <c r="F219" s="6" t="inlineStr"/>
-      <c r="G219" s="6" t="inlineStr">
-        <is>
-          <t>크으… 아빠 근육 생겼다!
-진짜?!</t>
-        </is>
-      </c>
+      <c r="G219" s="6" t="inlineStr"/>
       <c r="H219" s="6" t="inlineStr">
         <is>
-          <t>불끈불끈</t>
+          <t>시큼!!!, 부르르, 부르르</t>
         </is>
       </c>
     </row>
@@ -8581,22 +8576,18 @@
       </c>
       <c r="D220" s="4" t="inlineStr">
         <is>
-          <t>부엌</t>
+          <t>효과: 반짝</t>
         </is>
       </c>
       <c r="E220" s="4" t="inlineStr">
         <is>
-          <t>태오, 아빠</t>
-        </is>
-      </c>
-      <c r="F220" s="4" t="inlineStr">
-        <is>
-          <t>그날 저녁.</t>
-        </is>
-      </c>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F220" s="4" t="inlineStr"/>
       <c r="G220" s="4" t="inlineStr">
         <is>
-          <t>그럼 나도! 브로콜리 먹을래!</t>
+          <t>뭐가 셔? 맛있는데.</t>
         </is>
       </c>
       <c r="H220" s="4" t="inlineStr"/>
@@ -8615,23 +8606,24 @@
       </c>
       <c r="D221" s="6" t="inlineStr">
         <is>
-          <t>효과: 반짝</t>
+          <t>거실</t>
         </is>
       </c>
       <c r="E221" s="6" t="inlineStr">
         <is>
-          <t>태오</t>
+          <t>아빠, 태오</t>
         </is>
       </c>
       <c r="F221" s="6" t="inlineStr"/>
       <c r="G221" s="6" t="inlineStr">
         <is>
-          <t>나 근육 생겼어?</t>
+          <t>크으… 아빠 근육 생겼다!
+진짜?!</t>
         </is>
       </c>
       <c r="H221" s="6" t="inlineStr">
         <is>
-          <t>우물우물</t>
+          <t>불끈불끈</t>
         </is>
       </c>
     </row>
@@ -8654,13 +8646,17 @@
       </c>
       <c r="E222" s="4" t="inlineStr">
         <is>
-          <t>태오, 재이</t>
-        </is>
-      </c>
-      <c r="F222" s="4" t="inlineStr"/>
+          <t>태오, 아빠</t>
+        </is>
+      </c>
+      <c r="F222" s="4" t="inlineStr">
+        <is>
+          <t>그날 저녁.</t>
+        </is>
+      </c>
       <c r="G222" s="4" t="inlineStr">
         <is>
-          <t>이제 누나 차례! 누나 레몬 먹어!</t>
+          <t>그럼 나도! 브로콜리 먹을래!</t>
         </is>
       </c>
       <c r="H222" s="4" t="inlineStr"/>
@@ -8679,23 +8675,23 @@
       </c>
       <c r="D223" s="6" t="inlineStr">
         <is>
-          <t>효과: 집중선</t>
+          <t>효과: 반짝</t>
         </is>
       </c>
       <c r="E223" s="6" t="inlineStr">
         <is>
-          <t>재이</t>
+          <t>태오</t>
         </is>
       </c>
       <c r="F223" s="6" t="inlineStr"/>
       <c r="G223" s="6" t="inlineStr">
         <is>
-          <t>김태오!!</t>
+          <t>나 근육 생겼어?</t>
         </is>
       </c>
       <c r="H223" s="6" t="inlineStr">
         <is>
-          <t>도망!</t>
+          <t>우물우물</t>
         </is>
       </c>
     </row>
@@ -8713,81 +8709,80 @@
       </c>
       <c r="D224" s="4" t="inlineStr">
         <is>
-          <t>효과: 반짝</t>
-        </is>
-      </c>
-      <c r="E224" s="4" t="inlineStr"/>
-      <c r="F224" s="4" t="inlineStr">
-        <is>
-          <t>아빠가 한 말은 태오가 다 기억한다. / 그래서 아빠는 오늘도 먼저 한 입 먹는다.</t>
-        </is>
-      </c>
-      <c r="G224" s="4" t="inlineStr"/>
+          <t>부엌</t>
+        </is>
+      </c>
+      <c r="E224" s="4" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="F224" s="4" t="inlineStr"/>
+      <c r="G224" s="4" t="inlineStr">
+        <is>
+          <t>이제 누나 차례! 누나 레몬 먹어!</t>
+        </is>
+      </c>
       <c r="H224" s="4" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" s="5" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B225" s="6" t="inlineStr">
         <is>
-          <t>아빠 레스테스통 알아?</t>
+          <t>아빠 레몬 먹어!</t>
         </is>
       </c>
       <c r="C225" s="5" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="D225" s="6" t="inlineStr">
         <is>
-          <t>거실</t>
+          <t>효과: 집중선</t>
         </is>
       </c>
       <c r="E225" s="6" t="inlineStr">
         <is>
-          <t>태오</t>
-        </is>
-      </c>
-      <c r="F225" s="6" t="inlineStr">
-        <is>
-          <t>냠냠히어로 수퍼잭을 보고 난 태오.</t>
-        </is>
-      </c>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F225" s="6" t="inlineStr"/>
       <c r="G225" s="6" t="inlineStr">
         <is>
-          <t>레스테스통이 있어야 변신할 수 있어!</t>
-        </is>
-      </c>
-      <c r="H225" s="6" t="inlineStr"/>
+          <t>김태오!!</t>
+        </is>
+      </c>
+      <c r="H225" s="6" t="inlineStr">
+        <is>
+          <t>도망!</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="3" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B226" s="4" t="inlineStr">
         <is>
-          <t>아빠 레스테스통 알아?</t>
+          <t>아빠 레몬 먹어!</t>
         </is>
       </c>
       <c r="C226" s="3" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="D226" s="4" t="inlineStr">
         <is>
-          <t>거실</t>
-        </is>
-      </c>
-      <c r="E226" s="4" t="inlineStr">
-        <is>
-          <t>태오, 아빠</t>
-        </is>
-      </c>
-      <c r="F226" s="4" t="inlineStr"/>
-      <c r="G226" s="4" t="inlineStr">
-        <is>
-          <t>아빠 레스테스통 알아?
-레스…테스…통?</t>
-        </is>
-      </c>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E226" s="4" t="inlineStr"/>
+      <c r="F226" s="4" t="inlineStr">
+        <is>
+          <t>아빠가 한 말은 태오가 다 기억한다. / 그래서 아빠는 오늘도 먼저 한 입 먹는다.</t>
+        </is>
+      </c>
+      <c r="G226" s="4" t="inlineStr"/>
       <c r="H226" s="4" t="inlineStr"/>
     </row>
     <row r="227">
@@ -8800,22 +8795,26 @@
         </is>
       </c>
       <c r="C227" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D227" s="6" t="inlineStr">
         <is>
-          <t>효과: 집중선</t>
+          <t>거실</t>
         </is>
       </c>
       <c r="E227" s="6" t="inlineStr">
         <is>
-          <t>아빠</t>
-        </is>
-      </c>
-      <c r="F227" s="6" t="inlineStr"/>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F227" s="6" t="inlineStr">
+        <is>
+          <t>냠냠히어로 수퍼잭을 보고 난 태오.</t>
+        </is>
+      </c>
       <c r="G227" s="6" t="inlineStr">
         <is>
-          <t>…레스토랑? 테스트? 아빠 머리통?</t>
+          <t>레스테스통이 있어야 변신할 수 있어!</t>
         </is>
       </c>
       <c r="H227" s="6" t="inlineStr"/>
@@ -8830,22 +8829,23 @@
         </is>
       </c>
       <c r="C228" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D228" s="4" t="inlineStr">
         <is>
-          <t>효과: 집중선</t>
+          <t>거실</t>
         </is>
       </c>
       <c r="E228" s="4" t="inlineStr">
         <is>
-          <t>태오</t>
+          <t>태오, 아빠</t>
         </is>
       </c>
       <c r="F228" s="4" t="inlineStr"/>
       <c r="G228" s="4" t="inlineStr">
         <is>
-          <t>아니! 레스테스통!! 아빠 그것도 몰라?!</t>
+          <t>아빠 레스테스통 알아?
+레스…테스…통?</t>
         </is>
       </c>
       <c r="H228" s="4" t="inlineStr"/>
@@ -8860,29 +8860,25 @@
         </is>
       </c>
       <c r="C229" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D229" s="6" t="inlineStr">
         <is>
-          <t>거실</t>
+          <t>효과: 집중선</t>
         </is>
       </c>
       <c r="E229" s="6" t="inlineStr">
         <is>
-          <t>재이, 아빠</t>
+          <t>아빠</t>
         </is>
       </c>
       <c r="F229" s="6" t="inlineStr"/>
       <c r="G229" s="6" t="inlineStr">
         <is>
-          <t>아빠, 레시피 스톤! 냠냠히어로가 변신할 때 쓰는 돌이야.</t>
-        </is>
-      </c>
-      <c r="H229" s="6" t="inlineStr">
-        <is>
-          <t>통역 완료</t>
-        </is>
-      </c>
+          <t>…레스토랑? 테스트? 아빠 머리통?</t>
+        </is>
+      </c>
+      <c r="H229" s="6" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" s="3" t="n">
@@ -8894,11 +8890,11 @@
         </is>
       </c>
       <c r="C230" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D230" s="4" t="inlineStr">
         <is>
-          <t>효과: 반짝</t>
+          <t>효과: 집중선</t>
         </is>
       </c>
       <c r="E230" s="4" t="inlineStr">
@@ -8909,14 +8905,10 @@
       <c r="F230" s="4" t="inlineStr"/>
       <c r="G230" s="4" t="inlineStr">
         <is>
-          <t>그니까! 레스테스통!</t>
-        </is>
-      </c>
-      <c r="H230" s="4" t="inlineStr">
-        <is>
-          <t>당당</t>
-        </is>
-      </c>
+          <t>아니! 레스테스통!! 아빠 그것도 몰라?!</t>
+        </is>
+      </c>
+      <c r="H230" s="4" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" s="5" t="n">
@@ -8928,7 +8920,7 @@
         </is>
       </c>
       <c r="C231" s="5" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D231" s="6" t="inlineStr">
         <is>
@@ -8937,18 +8929,18 @@
       </c>
       <c r="E231" s="6" t="inlineStr">
         <is>
-          <t>태오</t>
-        </is>
-      </c>
-      <c r="F231" s="6" t="inlineStr">
-        <is>
-          <t>그날부터 태오의 레스테스통 찾기가 시작됐다.</t>
-        </is>
-      </c>
-      <c r="G231" s="6" t="inlineStr"/>
+          <t>재이, 아빠</t>
+        </is>
+      </c>
+      <c r="F231" s="6" t="inlineStr"/>
+      <c r="G231" s="6" t="inlineStr">
+        <is>
+          <t>아빠, 레시피 스톤! 냠냠히어로가 변신할 때 쓰는 돌이야.</t>
+        </is>
+      </c>
       <c r="H231" s="6" t="inlineStr">
         <is>
-          <t>뒤적뒤적</t>
+          <t>통역 완료</t>
         </is>
       </c>
     </row>
@@ -8962,11 +8954,11 @@
         </is>
       </c>
       <c r="C232" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D232" s="4" t="inlineStr">
         <is>
-          <t>효과: 어두움</t>
+          <t>효과: 반짝</t>
         </is>
       </c>
       <c r="E232" s="4" t="inlineStr">
@@ -8977,10 +8969,14 @@
       <c r="F232" s="4" t="inlineStr"/>
       <c r="G232" s="4" t="inlineStr">
         <is>
-          <t>레스테스통 없어… 나 변신 못 해…</t>
-        </is>
-      </c>
-      <c r="H232" s="4" t="inlineStr"/>
+          <t>그니까! 레스테스통!</t>
+        </is>
+      </c>
+      <c r="H232" s="4" t="inlineStr">
+        <is>
+          <t>당당</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="5" t="n">
@@ -8992,25 +8988,29 @@
         </is>
       </c>
       <c r="C233" s="5" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D233" s="6" t="inlineStr">
         <is>
-          <t>할머니 댁</t>
+          <t>거실</t>
         </is>
       </c>
       <c r="E233" s="6" t="inlineStr">
         <is>
-          <t>할머니, 태오</t>
-        </is>
-      </c>
-      <c r="F233" s="6" t="inlineStr"/>
-      <c r="G233" s="6" t="inlineStr">
-        <is>
-          <t>태오야, 할머니한테 레시피 스톤 있지.</t>
-        </is>
-      </c>
-      <c r="H233" s="6" t="inlineStr"/>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F233" s="6" t="inlineStr">
+        <is>
+          <t>그날부터 태오의 레스테스통 찾기가 시작됐다.</t>
+        </is>
+      </c>
+      <c r="G233" s="6" t="inlineStr"/>
+      <c r="H233" s="6" t="inlineStr">
+        <is>
+          <t>뒤적뒤적</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="3" t="n">
@@ -9022,11 +9022,11 @@
         </is>
       </c>
       <c r="C234" s="3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D234" s="4" t="inlineStr">
         <is>
-          <t>효과: 집중선</t>
+          <t>효과: 어두움</t>
         </is>
       </c>
       <c r="E234" s="4" t="inlineStr">
@@ -9037,7 +9037,7 @@
       <c r="F234" s="4" t="inlineStr"/>
       <c r="G234" s="4" t="inlineStr">
         <is>
-          <t>진짜?! 할머니도 냠냠히어로야?!</t>
+          <t>레스테스통 없어… 나 변신 못 해…</t>
         </is>
       </c>
       <c r="H234" s="4" t="inlineStr"/>
@@ -9052,20 +9052,24 @@
         </is>
       </c>
       <c r="C235" s="5" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D235" s="6" t="inlineStr">
         <is>
-          <t>효과: 반짝</t>
-        </is>
-      </c>
-      <c r="E235" s="6" t="inlineStr"/>
-      <c r="F235" s="6" t="inlineStr">
-        <is>
-          <t>할머니의 레시피 스톤은, 오래된 요리 공책이었다.</t>
-        </is>
-      </c>
-      <c r="G235" s="6" t="inlineStr"/>
+          <t>할머니 댁</t>
+        </is>
+      </c>
+      <c r="E235" s="6" t="inlineStr">
+        <is>
+          <t>할머니, 태오</t>
+        </is>
+      </c>
+      <c r="F235" s="6" t="inlineStr"/>
+      <c r="G235" s="6" t="inlineStr">
+        <is>
+          <t>태오야, 할머니한테 레시피 스톤 있지.</t>
+        </is>
+      </c>
       <c r="H235" s="6" t="inlineStr"/>
     </row>
     <row r="236">
@@ -9078,23 +9082,22 @@
         </is>
       </c>
       <c r="C236" s="3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D236" s="4" t="inlineStr">
         <is>
-          <t>부엌</t>
+          <t>효과: 집중선</t>
         </is>
       </c>
       <c r="E236" s="4" t="inlineStr">
         <is>
-          <t>할머니, 태오, 재이</t>
+          <t>태오</t>
         </is>
       </c>
       <c r="F236" s="4" t="inlineStr"/>
       <c r="G236" s="4" t="inlineStr">
         <is>
-          <t>그럼~ 싫어하는 것도 먹어야 튼튼해지지.
-시금치도 넣어야 해?</t>
+          <t>진짜?! 할머니도 냠냠히어로야?!</t>
         </is>
       </c>
       <c r="H236" s="4" t="inlineStr"/>
@@ -9109,29 +9112,21 @@
         </is>
       </c>
       <c r="C237" s="5" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D237" s="6" t="inlineStr">
         <is>
-          <t>효과: 집중선</t>
-        </is>
-      </c>
-      <c r="E237" s="6" t="inlineStr">
-        <is>
-          <t>태오</t>
-        </is>
-      </c>
-      <c r="F237" s="6" t="inlineStr"/>
-      <c r="G237" s="6" t="inlineStr">
-        <is>
-          <t>…그거 아빠가 한 말인데?</t>
-        </is>
-      </c>
-      <c r="H237" s="6" t="inlineStr">
-        <is>
-          <t>또 들었다</t>
-        </is>
-      </c>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E237" s="6" t="inlineStr"/>
+      <c r="F237" s="6" t="inlineStr">
+        <is>
+          <t>할머니의 레시피 스톤은, 오래된 요리 공책이었다.</t>
+        </is>
+      </c>
+      <c r="G237" s="6" t="inlineStr"/>
+      <c r="H237" s="6" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" s="3" t="n">
@@ -9143,7 +9138,7 @@
         </is>
       </c>
       <c r="C238" s="3" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D238" s="4" t="inlineStr">
         <is>
@@ -9152,16 +9147,17 @@
       </c>
       <c r="E238" s="4" t="inlineStr">
         <is>
-          <t>태오, 아빠</t>
+          <t>할머니, 태오, 재이</t>
         </is>
       </c>
       <c r="F238" s="4" t="inlineStr"/>
-      <c r="G238" s="4" t="inlineStr"/>
-      <c r="H238" s="4" t="inlineStr">
-        <is>
-          <t>냠냠, 냠냠</t>
-        </is>
-      </c>
+      <c r="G238" s="4" t="inlineStr">
+        <is>
+          <t>그럼~ 싫어하는 것도 먹어야 튼튼해지지.
+시금치도 넣어야 해?</t>
+        </is>
+      </c>
+      <c r="H238" s="4" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" s="5" t="n">
@@ -9173,11 +9169,11 @@
         </is>
       </c>
       <c r="C239" s="5" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D239" s="6" t="inlineStr">
         <is>
-          <t>효과: 반짝</t>
+          <t>효과: 집중선</t>
         </is>
       </c>
       <c r="E239" s="6" t="inlineStr">
@@ -9188,12 +9184,12 @@
       <c r="F239" s="6" t="inlineStr"/>
       <c r="G239" s="6" t="inlineStr">
         <is>
-          <t>냠냠히어로 태오, 변신 완료!!</t>
+          <t>…그거 아빠가 한 말인데?</t>
         </is>
       </c>
       <c r="H239" s="6" t="inlineStr">
         <is>
-          <t>번쩍!, 번쩍!</t>
+          <t>또 들었다</t>
         </is>
       </c>
     </row>
@@ -9207,7 +9203,7 @@
         </is>
       </c>
       <c r="C240" s="3" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D240" s="4" t="inlineStr">
         <is>
@@ -9216,17 +9212,16 @@
       </c>
       <c r="E240" s="4" t="inlineStr">
         <is>
-          <t>아빠, 할머니</t>
+          <t>태오, 아빠</t>
         </is>
       </c>
       <c r="F240" s="4" t="inlineStr"/>
-      <c r="G240" s="4" t="inlineStr">
-        <is>
-          <t>장모님, 레스테스통 덕분에 태오가 시금치를 다 먹네요.
-김서방, 그건 레스테스통이 아니라 할미 사랑이여~</t>
-        </is>
-      </c>
-      <c r="H240" s="4" t="inlineStr"/>
+      <c r="G240" s="4" t="inlineStr"/>
+      <c r="H240" s="4" t="inlineStr">
+        <is>
+          <t>냠냠, 냠냠</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="5" t="n">
@@ -9238,89 +9233,86 @@
         </is>
       </c>
       <c r="C241" s="5" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D241" s="6" t="inlineStr">
         <is>
           <t>효과: 반짝</t>
         </is>
       </c>
-      <c r="E241" s="6" t="inlineStr"/>
-      <c r="F241" s="6" t="inlineStr">
-        <is>
-          <t>진짜 레스테스통은 할머니 공책 속에 있었다. / 그리고 오늘, 태오 배 속에도.</t>
-        </is>
-      </c>
-      <c r="G241" s="6" t="inlineStr"/>
-      <c r="H241" s="6" t="inlineStr"/>
+      <c r="E241" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F241" s="6" t="inlineStr"/>
+      <c r="G241" s="6" t="inlineStr">
+        <is>
+          <t>냠냠히어로 태오, 변신 완료!!</t>
+        </is>
+      </c>
+      <c r="H241" s="6" t="inlineStr">
+        <is>
+          <t>번쩍!, 번쩍!</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="3" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B242" s="4" t="inlineStr">
         <is>
-          <t>타노스 나와라!</t>
+          <t>아빠 레스테스통 알아?</t>
         </is>
       </c>
       <c r="C242" s="3" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="D242" s="4" t="inlineStr">
         <is>
-          <t>거실(밤)</t>
+          <t>부엌</t>
         </is>
       </c>
       <c r="E242" s="4" t="inlineStr">
         <is>
-          <t>아빠</t>
-        </is>
-      </c>
-      <c r="F242" s="4" t="inlineStr">
-        <is>
-          <t>퇴근한 아빠, 오늘은 뉴스 좀 보려는데…</t>
-        </is>
-      </c>
-      <c r="G242" s="4" t="inlineStr"/>
-      <c r="H242" s="4" t="inlineStr">
-        <is>
-          <t>띡</t>
-        </is>
-      </c>
+          <t>아빠, 할머니</t>
+        </is>
+      </c>
+      <c r="F242" s="4" t="inlineStr"/>
+      <c r="G242" s="4" t="inlineStr">
+        <is>
+          <t>장모님, 레스테스통 덕분에 태오가 시금치를 다 먹네요.
+김서방, 그건 레스테스통이 아니라 할미 사랑이여~</t>
+        </is>
+      </c>
+      <c r="H242" s="4" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" s="5" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B243" s="6" t="inlineStr">
         <is>
-          <t>타노스 나와라!</t>
+          <t>아빠 레스테스통 알아?</t>
         </is>
       </c>
       <c r="C243" s="5" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="D243" s="6" t="inlineStr">
         <is>
-          <t>효과: 집중선</t>
-        </is>
-      </c>
-      <c r="E243" s="6" t="inlineStr">
-        <is>
-          <t>태오</t>
-        </is>
-      </c>
-      <c r="F243" s="6" t="inlineStr"/>
-      <c r="G243" s="6" t="inlineStr">
-        <is>
-          <t>내꺼 틀어 줘!!</t>
-        </is>
-      </c>
-      <c r="H243" s="6" t="inlineStr">
-        <is>
-          <t>0.1초</t>
-        </is>
-      </c>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E243" s="6" t="inlineStr"/>
+      <c r="F243" s="6" t="inlineStr">
+        <is>
+          <t>진짜 레스테스통은 할머니 공책 속에 있었다. / 그리고 오늘, 태오 배 속에도.</t>
+        </is>
+      </c>
+      <c r="G243" s="6" t="inlineStr"/>
+      <c r="H243" s="6" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" s="3" t="n">
@@ -9332,7 +9324,7 @@
         </is>
       </c>
       <c r="C244" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D244" s="4" t="inlineStr">
         <is>
@@ -9341,16 +9333,20 @@
       </c>
       <c r="E244" s="4" t="inlineStr">
         <is>
-          <t>아빠, 태오</t>
-        </is>
-      </c>
-      <c r="F244" s="4" t="inlineStr"/>
-      <c r="G244" s="4" t="inlineStr">
-        <is>
-          <t>(속삭임) …아빠 뉴스는 내일 보지 뭐.</t>
-        </is>
-      </c>
-      <c r="H244" s="4" t="inlineStr"/>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F244" s="4" t="inlineStr">
+        <is>
+          <t>퇴근한 아빠, 오늘은 뉴스 좀 보려는데…</t>
+        </is>
+      </c>
+      <c r="G244" s="4" t="inlineStr"/>
+      <c r="H244" s="4" t="inlineStr">
+        <is>
+          <t>띡</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="5" t="n">
@@ -9362,30 +9358,29 @@
         </is>
       </c>
       <c r="C245" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D245" s="6" t="inlineStr">
         <is>
-          <t>부엌</t>
+          <t>효과: 집중선</t>
         </is>
       </c>
       <c r="E245" s="6" t="inlineStr">
         <is>
-          <t>태오, 엄마</t>
-        </is>
-      </c>
-      <c r="F245" s="6" t="inlineStr">
-        <is>
-          <t>만화가 끝나고 10분 뒤.</t>
-        </is>
-      </c>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F245" s="6" t="inlineStr"/>
       <c r="G245" s="6" t="inlineStr">
         <is>
-          <t>엄마~ 심심해. 맛있는 거 줘!
-…밥 먹은 지 10분 됐어.</t>
-        </is>
-      </c>
-      <c r="H245" s="6" t="inlineStr"/>
+          <t>내꺼 틀어 줘!!</t>
+        </is>
+      </c>
+      <c r="H245" s="6" t="inlineStr">
+        <is>
+          <t>0.1초</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="3" t="n">
@@ -9397,29 +9392,25 @@
         </is>
       </c>
       <c r="C246" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D246" s="4" t="inlineStr">
         <is>
-          <t>효과: 집중선</t>
+          <t>거실(밤)</t>
         </is>
       </c>
       <c r="E246" s="4" t="inlineStr">
         <is>
-          <t>태오</t>
+          <t>아빠, 태오</t>
         </is>
       </c>
       <c r="F246" s="4" t="inlineStr"/>
       <c r="G246" s="4" t="inlineStr">
         <is>
-          <t>그럼 싸우자!!</t>
-        </is>
-      </c>
-      <c r="H246" s="4" t="inlineStr">
-        <is>
-          <t>번쩍</t>
-        </is>
-      </c>
+          <t>(속삭임) …아빠 뉴스는 내일 보지 뭐.</t>
+        </is>
+      </c>
+      <c r="H246" s="4" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" s="5" t="n">
@@ -9431,23 +9422,27 @@
         </is>
       </c>
       <c r="C247" s="5" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D247" s="6" t="inlineStr">
         <is>
-          <t>거실(밤)</t>
+          <t>부엌</t>
         </is>
       </c>
       <c r="E247" s="6" t="inlineStr">
         <is>
-          <t>태오, 아빠</t>
-        </is>
-      </c>
-      <c r="F247" s="6" t="inlineStr"/>
+          <t>태오, 엄마</t>
+        </is>
+      </c>
+      <c r="F247" s="6" t="inlineStr">
+        <is>
+          <t>만화가 끝나고 10분 뒤.</t>
+        </is>
+      </c>
       <c r="G247" s="6" t="inlineStr">
         <is>
-          <t>나는 어벤져스! 아빠는 타노스!
-또 아빠가 타노스야?</t>
+          <t>엄마~ 심심해. 맛있는 거 줘!
+…밥 먹은 지 10분 됐어.</t>
         </is>
       </c>
       <c r="H247" s="6" t="inlineStr"/>
@@ -9462,22 +9457,22 @@
         </is>
       </c>
       <c r="C248" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D248" s="4" t="inlineStr">
         <is>
-          <t>효과: 어두움</t>
+          <t>효과: 집중선</t>
         </is>
       </c>
       <c r="E248" s="4" t="inlineStr">
         <is>
-          <t>아빠</t>
+          <t>태오</t>
         </is>
       </c>
       <c r="F248" s="4" t="inlineStr"/>
       <c r="G248" s="4" t="inlineStr">
         <is>
-          <t>아임… 인에비터블!</t>
+          <t>그럼 싸우자!!</t>
         </is>
       </c>
       <c r="H248" s="4" t="inlineStr">
@@ -9496,23 +9491,23 @@
         </is>
       </c>
       <c r="C249" s="5" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D249" s="6" t="inlineStr">
         <is>
-          <t>효과: 집중선</t>
+          <t>거실(밤)</t>
         </is>
       </c>
       <c r="E249" s="6" t="inlineStr">
         <is>
-          <t>태오, 재이</t>
+          <t>태오, 아빠</t>
         </is>
       </c>
       <c r="F249" s="6" t="inlineStr"/>
       <c r="G249" s="6" t="inlineStr">
         <is>
-          <t>아임 인에터블!!
-(속삭임) (…인에비터블이야.)</t>
+          <t>나는 어벤져스! 아빠는 타노스!
+또 아빠가 타노스야?</t>
         </is>
       </c>
       <c r="H249" s="6" t="inlineStr"/>
@@ -9527,27 +9522,27 @@
         </is>
       </c>
       <c r="C250" s="3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D250" s="4" t="inlineStr">
         <is>
-          <t>효과: 속도선</t>
+          <t>효과: 어두움</t>
         </is>
       </c>
       <c r="E250" s="4" t="inlineStr">
         <is>
-          <t>태오, 아빠</t>
+          <t>아빠</t>
         </is>
       </c>
       <c r="F250" s="4" t="inlineStr"/>
       <c r="G250" s="4" t="inlineStr">
         <is>
-          <t>블루베리 펀치! 쉬터맨 거미줄! 스테잌로저 방패!</t>
+          <t>아임… 인에비터블!</t>
         </is>
       </c>
       <c r="H250" s="4" t="inlineStr">
         <is>
-          <t>퍽!</t>
+          <t>번쩍</t>
         </is>
       </c>
     </row>
@@ -9561,23 +9556,23 @@
         </is>
       </c>
       <c r="C251" s="5" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D251" s="6" t="inlineStr">
         <is>
-          <t>거실(밤)</t>
+          <t>효과: 집중선</t>
         </is>
       </c>
       <c r="E251" s="6" t="inlineStr">
         <is>
-          <t>재이, 태오</t>
+          <t>태오, 재이</t>
         </is>
       </c>
       <c r="F251" s="6" t="inlineStr"/>
       <c r="G251" s="6" t="inlineStr">
         <is>
-          <t>블랙 위도우도 출동!
-누나 제일 예뻐!!</t>
+          <t>아임 인에터블!!
+(속삭임) (…인에비터블이야.)</t>
         </is>
       </c>
       <c r="H251" s="6" t="inlineStr"/>
@@ -9592,27 +9587,27 @@
         </is>
       </c>
       <c r="C252" s="3" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D252" s="4" t="inlineStr">
         <is>
-          <t>거실(밤)</t>
+          <t>효과: 속도선</t>
         </is>
       </c>
       <c r="E252" s="4" t="inlineStr">
         <is>
-          <t>아빠</t>
+          <t>태오, 아빠</t>
         </is>
       </c>
       <c r="F252" s="4" t="inlineStr"/>
       <c r="G252" s="4" t="inlineStr">
         <is>
-          <t>으악… 타노스가 졌다…</t>
+          <t>블루베리 펀치! 쉬터맨 거미줄! 스테잌로저 방패!</t>
         </is>
       </c>
       <c r="H252" s="4" t="inlineStr">
         <is>
-          <t>쿵!</t>
+          <t>퍽!</t>
         </is>
       </c>
     </row>
@@ -9626,22 +9621,23 @@
         </is>
       </c>
       <c r="C253" s="5" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D253" s="6" t="inlineStr">
         <is>
-          <t>효과: 집중선</t>
+          <t>거실(밤)</t>
         </is>
       </c>
       <c r="E253" s="6" t="inlineStr">
         <is>
-          <t>태오</t>
+          <t>재이, 태오</t>
         </is>
       </c>
       <c r="F253" s="6" t="inlineStr"/>
       <c r="G253" s="6" t="inlineStr">
         <is>
-          <t>또 해! 또 해!!</t>
+          <t>블랙 위도우도 출동!
+누나 제일 예뻐!!</t>
         </is>
       </c>
       <c r="H253" s="6" t="inlineStr"/>
@@ -9656,7 +9652,7 @@
         </is>
       </c>
       <c r="C254" s="3" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D254" s="4" t="inlineStr">
         <is>
@@ -9668,15 +9664,15 @@
           <t>아빠</t>
         </is>
       </c>
-      <c r="F254" s="4" t="inlineStr">
-        <is>
-          <t>그렇게 타노스는 열 번 졌다.</t>
-        </is>
-      </c>
-      <c r="G254" s="4" t="inlineStr"/>
+      <c r="F254" s="4" t="inlineStr"/>
+      <c r="G254" s="4" t="inlineStr">
+        <is>
+          <t>으악… 타노스가 졌다…</t>
+        </is>
+      </c>
       <c r="H254" s="4" t="inlineStr">
         <is>
-          <t>헥헥</t>
+          <t>쿵!</t>
         </is>
       </c>
     </row>
@@ -9690,11 +9686,11 @@
         </is>
       </c>
       <c r="C255" s="5" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D255" s="6" t="inlineStr">
         <is>
-          <t>효과: 반짝</t>
+          <t>효과: 집중선</t>
         </is>
       </c>
       <c r="E255" s="6" t="inlineStr">
@@ -9705,7 +9701,7 @@
       <c r="F255" s="6" t="inlineStr"/>
       <c r="G255" s="6" t="inlineStr">
         <is>
-          <t>(생각) (…아빠 힘든가?)</t>
+          <t>또 해! 또 해!!</t>
         </is>
       </c>
       <c r="H255" s="6" t="inlineStr"/>
@@ -9720,7 +9716,7 @@
         </is>
       </c>
       <c r="C256" s="3" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D256" s="4" t="inlineStr">
         <is>
@@ -9729,16 +9725,20 @@
       </c>
       <c r="E256" s="4" t="inlineStr">
         <is>
-          <t>태오, 아빠</t>
-        </is>
-      </c>
-      <c r="F256" s="4" t="inlineStr"/>
-      <c r="G256" s="4" t="inlineStr">
-        <is>
-          <t>이번엔 내가 타노스 할게. 아임 인에터블!</t>
-        </is>
-      </c>
-      <c r="H256" s="4" t="inlineStr"/>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F256" s="4" t="inlineStr">
+        <is>
+          <t>그렇게 타노스는 열 번 졌다.</t>
+        </is>
+      </c>
+      <c r="G256" s="4" t="inlineStr"/>
+      <c r="H256" s="4" t="inlineStr">
+        <is>
+          <t>헥헥</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="5" t="n">
@@ -9750,11 +9750,11 @@
         </is>
       </c>
       <c r="C257" s="5" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D257" s="6" t="inlineStr">
         <is>
-          <t>효과: 속도선</t>
+          <t>효과: 반짝</t>
         </is>
       </c>
       <c r="E257" s="6" t="inlineStr">
@@ -9765,14 +9765,10 @@
       <c r="F257" s="6" t="inlineStr"/>
       <c r="G257" s="6" t="inlineStr">
         <is>
-          <t>으악~ 타노스 졌다~ 아빠가 이겼다!</t>
-        </is>
-      </c>
-      <c r="H257" s="6" t="inlineStr">
-        <is>
-          <t>털썩</t>
-        </is>
-      </c>
+          <t>(생각) (…아빠 힘든가?)</t>
+        </is>
+      </c>
+      <c r="H257" s="6" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" s="3" t="n">
@@ -9784,22 +9780,22 @@
         </is>
       </c>
       <c r="C258" s="3" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D258" s="4" t="inlineStr">
         <is>
-          <t>효과: 반짝</t>
+          <t>거실(밤)</t>
         </is>
       </c>
       <c r="E258" s="4" t="inlineStr">
         <is>
-          <t>아빠</t>
+          <t>태오, 아빠</t>
         </is>
       </c>
       <c r="F258" s="4" t="inlineStr"/>
       <c r="G258" s="4" t="inlineStr">
         <is>
-          <t>태오야… 일부러 져 준 거야?</t>
+          <t>이번엔 내가 타노스 할게. 아임 인에터블!</t>
         </is>
       </c>
       <c r="H258" s="4" t="inlineStr"/>
@@ -9814,11 +9810,11 @@
         </is>
       </c>
       <c r="C259" s="5" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D259" s="6" t="inlineStr">
         <is>
-          <t>효과: 반짝</t>
+          <t>효과: 속도선</t>
         </is>
       </c>
       <c r="E259" s="6" t="inlineStr">
@@ -9829,10 +9825,14 @@
       <c r="F259" s="6" t="inlineStr"/>
       <c r="G259" s="6" t="inlineStr">
         <is>
-          <t>아빠 맨날 졌잖아. 오늘은 아빠가 이겨.</t>
-        </is>
-      </c>
-      <c r="H259" s="6" t="inlineStr"/>
+          <t>으악~ 타노스 졌다~ 아빠가 이겼다!</t>
+        </is>
+      </c>
+      <c r="H259" s="6" t="inlineStr">
+        <is>
+          <t>털썩</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="3" t="n">
@@ -9844,7 +9844,7 @@
         </is>
       </c>
       <c r="C260" s="3" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D260" s="4" t="inlineStr">
         <is>
@@ -9853,15 +9853,15 @@
       </c>
       <c r="E260" s="4" t="inlineStr">
         <is>
-          <t>태오, 아빠</t>
-        </is>
-      </c>
-      <c r="F260" s="4" t="inlineStr">
-        <is>
-          <t>아빠 배터리, 다시 100%.</t>
-        </is>
-      </c>
-      <c r="G260" s="4" t="inlineStr"/>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F260" s="4" t="inlineStr"/>
+      <c r="G260" s="4" t="inlineStr">
+        <is>
+          <t>태오야… 일부러 져 준 거야?</t>
+        </is>
+      </c>
       <c r="H260" s="4" t="inlineStr"/>
     </row>
     <row r="261">
@@ -9874,36 +9874,96 @@
         </is>
       </c>
       <c r="C261" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="D261" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E261" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F261" s="6" t="inlineStr"/>
+      <c r="G261" s="6" t="inlineStr">
+        <is>
+          <t>아빠 맨날 졌잖아. 오늘은 아빠가 이겨.</t>
+        </is>
+      </c>
+      <c r="H261" s="6" t="inlineStr"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B262" s="4" t="inlineStr">
+        <is>
+          <t>타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="C262" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="D262" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E262" s="4" t="inlineStr">
+        <is>
+          <t>태오, 아빠</t>
+        </is>
+      </c>
+      <c r="F262" s="4" t="inlineStr">
+        <is>
+          <t>아빠 배터리, 다시 100%.</t>
+        </is>
+      </c>
+      <c r="G262" s="4" t="inlineStr"/>
+      <c r="H262" s="4" t="inlineStr"/>
+    </row>
+    <row r="263">
+      <c r="A263" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B263" s="6" t="inlineStr">
+        <is>
+          <t>타노스 나와라!</t>
+        </is>
+      </c>
+      <c r="C263" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="D261" s="6" t="inlineStr">
+      <c r="D263" s="6" t="inlineStr">
         <is>
           <t>거실</t>
         </is>
       </c>
-      <c r="E261" s="6" t="inlineStr">
+      <c r="E263" s="6" t="inlineStr">
         <is>
           <t>태오, 아빠</t>
         </is>
       </c>
-      <c r="F261" s="6" t="inlineStr">
+      <c r="F263" s="6" t="inlineStr">
         <is>
           <t>다음 날 아침.</t>
         </is>
       </c>
-      <c r="G261" s="6" t="inlineStr">
+      <c r="G263" s="6" t="inlineStr">
         <is>
           <t>내꺼 틀어 줘!!</t>
         </is>
       </c>
-      <c r="H261" s="6" t="inlineStr">
+      <c r="H263" s="6" t="inlineStr">
         <is>
           <t>…역시</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:H261"/>
+  <autoFilter ref="A3:H263"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Make the half lemon Taeo's trademark
The family suggested Taeo always carry half a lemon and lick it. The art
engine now draws a cut half lemon in Taeo's hand in every panel: in his
left hand normally, at his mouth with the new "lick" pose, and not at
all when his hand is on his face or he is lying down (nl: true skips it
for a panel). Episode 13's "새콤해!" panel uses the lick pose with
"할짝할짝", his bio and tag lead with the lemon, the cast card shows a
lemon badge, and the hub cover is re-rendered. README documents it;
Excel regenerated. Cache v171.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -686,7 +686,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>태권도 파란띠 · 누나 괴롭히기 선수</t>
+          <t>반쪽 레몬 · 누나 괴롭히기 선수</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -696,12 +696,12 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>파란 윗옷·바지 (태권도복: 파란띠에 초록 줄) · 좋아하는 것: 레몬·자두·파인애플 같은 신 과일</t>
+          <t>파란 윗옷·바지 (태권도복: 파란띠에 초록 줄) · 트레이드마크: 늘 들고 다니며 핥아 먹는 반쪽 레몬 (신 과일을 제일 좋아함)</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>누나 괴롭히기가 취미인 막내(사실은 누나가 좋아서). 혼자 노는 것 같아도 가족 말을 다 듣고 있고, 틀려도 일단 소리 지르며 우기다가 들키면 머리를 긁적긁적. “맛있는 거 죠!”가 입버릇이고, 어벤져스 영웅도 태오식으로 불러요(블루베리, 쉬터맨, 스테잌로저…). 블랙 위도우랑 수가 제일 예쁘대요. 제일 좋아하는 놀이는 어벤져스로 타노스랑 싸우기! 레몬·자두·파인애플처럼 신 과일을 제일 좋아해요. 모든 호칭은 태오 기준이라, 누가 “재이야” 하면 “재이 누나야!” 하고 고쳐 줘요.</t>
+          <t>반쪽 레몬을 늘 손에 들고 다니며 할짝할짝 핥아 먹는 막내(레몬·자두·파인애플처럼 신 과일이 제일 좋아요). 누나 괴롭히기가 취미인 막내(사실은 누나가 좋아서). 혼자 노는 것 같아도 가족 말을 다 듣고 있고, 틀려도 일단 소리 지르며 우기다가 들키면 머리를 긁적긁적. “맛있는 거 죠!”가 입버릇이고, 어벤져스 영웅도 태오식으로 불러요(블루베리, 쉬터맨, 스테잌로저…). 블랙 위도우랑 수가 제일 예쁘대요. 제일 좋아하는 놀이는 어벤져스로 타노스랑 싸우기! 모든 호칭은 태오 기준이라, 누가 “재이야” 하면 “재이 누나야!” 하고 고쳐 줘요.</t>
         </is>
       </c>
     </row>
@@ -8417,7 +8417,7 @@
       </c>
       <c r="H213" s="6" t="inlineStr">
         <is>
-          <t>쪽쪽</t>
+          <t>할짝할짝</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Jaei's traits and episode 17 "아니야, 치즈는 극혐!"
The family described Jaei: "아니야!" is her most used word, offered
food she says "맛있는데 지금은 먹기 싫어.", she dislikes cheese and
can't stand its smell, likes her room tidy and finishes homework early
before playing, and both kids like 티니핑 and 위시캣. Her bio, tag and
sayings follow.

Episode 17: homework done on Friday, Taeo spills toys into her tidy
room ("아니야! 아니야! 아니야!"), Mom's new dish gets "맛있는데 지금은
먹기 싫어", the kids watch both shows, and Dad's cheesy pizza makes Jaei
flee the smell until Taeo asks for a cheese-free half because he
remembers what she hates. The shows are only named. New pizza, smell and
desk props; Excel adds episode 17. Cache v172.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$284</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$303</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -536,7 +536,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>초등학생 · 참을성 만렙 누나</t>
+          <t>초등학생 · “아니야!” 정리왕 누나</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -546,12 +546,12 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>분홍 원피스, 흰 동그란 깃</t>
+          <t>분홍 원피스, 흰 동그란 깃 · 입버릇 “아니야!” · 정리왕, 숙제 미리 끝 · 치즈 극혐</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>동생이 아무리 괴롭혀도 참고 또 참는 누나. 태오가 혼나면 제일 먼저 달려가 안아 줘요. 하지만 참다 참다 폭발하면… “김태오!” 엉덩이 찰싹! 그림 그리기를 제일 좋아해요.</t>
+          <t>“아니야!”가 입버릇인 누나. 방은 늘 반듯하게 정리해 두고, 학교 숙제는 미리 다 해 놓고 노는 게 좋아요. 음식을 권하면 “맛있는데 지금은 먹기 싫어.” 치즈는 싫고 치즈 냄새는 극혐! 티니핑이랑 위시캣은 태오랑 둘 다 좋아해요. 동생이 괴롭혀도 참고 또 참다가, 폭발하면… “김태오!” 엉덩이 찰싹!</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1563,20 +1563,50 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="n">
+      <c r="A20" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="7" t="n"/>
-      <c r="C20" s="7" t="n"/>
-      <c r="D20" s="7" t="n"/>
-      <c r="E20" s="7" t="n"/>
-      <c r="F20" s="7" t="n"/>
-      <c r="G20" s="7" t="n"/>
-      <c r="H20" s="7" t="n"/>
-      <c r="I20" s="7" t="n"/>
-      <c r="J20" s="7" t="inlineStr">
-        <is>
-          <t>기획 중</t>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>아니야, 치즈는 극혐!</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>숙제는 미리 끝, 방은 반듯하게 정리 끝. 완벽한 토요일을 준비한 재이 누나. 그런데 아빠가 오늘 저녁은 치즈 듬뿍 피자라고…?</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>재이, 엄마, 아빠, 태오</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>숙제 미리 끝, 방 정리 끝 → 태오가 와르르 “아니야! 아니야! 아니야!” / “맛있는데… 지금은 먹기 싫어.” / 치즈 듬뿍 피자 “치즈 냄새!! 극혐!!” / “아니야인데 고마워?”</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>태오가 “누나 쪽은 치즈 빼 줘!” — 누나가 싫어하는 걸 다 기억한 동생 / 티니핑도 위시캣도 둘 다</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>좋아하는 건 달라도 괜찮아요. 서로 싫어하는 걸 기억해 주는 게 가족이에요.</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>우리 가족이 제일 싫어하는 음식은 뭐예요? 서로 알고 있나요?</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>완성</t>
         </is>
       </c>
     </row>
@@ -1616,13 +1646,31 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="7" t="n"/>
+      <c r="C23" s="7" t="n"/>
+      <c r="D23" s="7" t="n"/>
+      <c r="E23" s="7" t="n"/>
+      <c r="F23" s="7" t="n"/>
+      <c r="G23" s="7" t="n"/>
+      <c r="H23" s="7" t="n"/>
+      <c r="I23" s="7" t="n"/>
+      <c r="J23" s="7" t="inlineStr">
+        <is>
+          <t>기획 중</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:J19"/>
+  <autoFilter ref="A3:J20"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"아이디어,기획 중,콘티,완성"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1636,7 +1684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H284"/>
+  <dimension ref="A1:H303"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -10666,8 +10714,622 @@
         </is>
       </c>
     </row>
+    <row r="285">
+      <c r="A285" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B285" s="6" t="inlineStr">
+        <is>
+          <t>아니야, 치즈는 극혐!</t>
+        </is>
+      </c>
+      <c r="C285" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D285" s="6" t="inlineStr">
+        <is>
+          <t>방</t>
+        </is>
+      </c>
+      <c r="E285" s="6" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F285" s="6" t="inlineStr">
+        <is>
+          <t>금요일 저녁. 재이 누나는 벌써 숙제를 다 끝냈다.</t>
+        </is>
+      </c>
+      <c r="G285" s="6" t="inlineStr">
+        <is>
+          <t>숙제 끝! 이제 주말엔 실컷 놀 수 있어.</t>
+        </is>
+      </c>
+      <c r="H285" s="6" t="inlineStr">
+        <is>
+          <t>반듯반듯</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B286" s="4" t="inlineStr">
+        <is>
+          <t>아니야, 치즈는 극혐!</t>
+        </is>
+      </c>
+      <c r="C286" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D286" s="4" t="inlineStr">
+        <is>
+          <t>방</t>
+        </is>
+      </c>
+      <c r="E286" s="4" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="F286" s="4" t="inlineStr"/>
+      <c r="G286" s="4" t="inlineStr">
+        <is>
+          <t>누나 방에서 놀자~!
+아니야!! 방금 정리했단 말이야!</t>
+        </is>
+      </c>
+      <c r="H286" s="4" t="inlineStr">
+        <is>
+          <t>와르르</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B287" s="6" t="inlineStr">
+        <is>
+          <t>아니야, 치즈는 극혐!</t>
+        </is>
+      </c>
+      <c r="C287" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D287" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E287" s="6" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F287" s="6" t="inlineStr"/>
+      <c r="G287" s="6" t="inlineStr">
+        <is>
+          <t>아니야! 아니야! 아니야!</t>
+        </is>
+      </c>
+      <c r="H287" s="6" t="inlineStr"/>
+    </row>
+    <row r="288">
+      <c r="A288" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B288" s="4" t="inlineStr">
+        <is>
+          <t>아니야, 치즈는 극혐!</t>
+        </is>
+      </c>
+      <c r="C288" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D288" s="4" t="inlineStr">
+        <is>
+          <t>방</t>
+        </is>
+      </c>
+      <c r="E288" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F288" s="4" t="inlineStr">
+        <is>
+          <t>(그래도 정리는 태오가 했다.)</t>
+        </is>
+      </c>
+      <c r="G288" s="4" t="inlineStr"/>
+      <c r="H288" s="4" t="inlineStr">
+        <is>
+          <t>낑낑</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B289" s="6" t="inlineStr">
+        <is>
+          <t>아니야, 치즈는 극혐!</t>
+        </is>
+      </c>
+      <c r="C289" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D289" s="6" t="inlineStr">
+        <is>
+          <t>부엌</t>
+        </is>
+      </c>
+      <c r="E289" s="6" t="inlineStr">
+        <is>
+          <t>엄마, 재이</t>
+        </is>
+      </c>
+      <c r="F289" s="6" t="inlineStr">
+        <is>
+          <t>토요일 아침.</t>
+        </is>
+      </c>
+      <c r="G289" s="6" t="inlineStr">
+        <is>
+          <t>재이야, 이거 새로 만든 건데 먹어 볼래?</t>
+        </is>
+      </c>
+      <c r="H289" s="6" t="inlineStr"/>
+    </row>
+    <row r="290">
+      <c r="A290" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B290" s="4" t="inlineStr">
+        <is>
+          <t>아니야, 치즈는 극혐!</t>
+        </is>
+      </c>
+      <c r="C290" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D290" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E290" s="4" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F290" s="4" t="inlineStr"/>
+      <c r="G290" s="4" t="inlineStr">
+        <is>
+          <t>맛있는데… 지금은 먹기 싫어.</t>
+        </is>
+      </c>
+      <c r="H290" s="4" t="inlineStr"/>
+    </row>
+    <row r="291">
+      <c r="A291" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B291" s="6" t="inlineStr">
+        <is>
+          <t>아니야, 치즈는 극혐!</t>
+        </is>
+      </c>
+      <c r="C291" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="D291" s="6" t="inlineStr">
+        <is>
+          <t>부엌</t>
+        </is>
+      </c>
+      <c r="E291" s="6" t="inlineStr">
+        <is>
+          <t>엄마, 태오</t>
+        </is>
+      </c>
+      <c r="F291" s="6" t="inlineStr"/>
+      <c r="G291" s="6" t="inlineStr">
+        <is>
+          <t>…아직 안 먹어 봤잖아.
+나 줘! 나 줘!</t>
+        </is>
+      </c>
+      <c r="H291" s="6" t="inlineStr">
+        <is>
+          <t>할짝</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B292" s="4" t="inlineStr">
+        <is>
+          <t>아니야, 치즈는 극혐!</t>
+        </is>
+      </c>
+      <c r="C292" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D292" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E292" s="4" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F292" s="4" t="inlineStr">
+        <is>
+          <t>숙제는 미리 끝냈으니까, 오늘은 실컷!</t>
+        </is>
+      </c>
+      <c r="G292" s="4" t="inlineStr">
+        <is>
+          <t>티니핑!
+위시캣!</t>
+        </is>
+      </c>
+      <c r="H292" s="4" t="inlineStr"/>
+    </row>
+    <row r="293">
+      <c r="A293" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B293" s="6" t="inlineStr">
+        <is>
+          <t>아니야, 치즈는 극혐!</t>
+        </is>
+      </c>
+      <c r="C293" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="D293" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E293" s="6" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F293" s="6" t="inlineStr"/>
+      <c r="G293" s="6" t="inlineStr">
+        <is>
+          <t>둘 다 보자!</t>
+        </is>
+      </c>
+      <c r="H293" s="6" t="inlineStr">
+        <is>
+          <t>찰떡</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B294" s="4" t="inlineStr">
+        <is>
+          <t>아니야, 치즈는 극혐!</t>
+        </is>
+      </c>
+      <c r="C294" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D294" s="4" t="inlineStr">
+        <is>
+          <t>부엌</t>
+        </is>
+      </c>
+      <c r="E294" s="4" t="inlineStr">
+        <is>
+          <t>아빠, 태오</t>
+        </is>
+      </c>
+      <c r="F294" s="4" t="inlineStr">
+        <is>
+          <t>저녁. 아빠의 서프라이즈.</t>
+        </is>
+      </c>
+      <c r="G294" s="4" t="inlineStr">
+        <is>
+          <t>짜잔! 치즈 듬뿍 피자!</t>
+        </is>
+      </c>
+      <c r="H294" s="4" t="inlineStr"/>
+    </row>
+    <row r="295">
+      <c r="A295" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B295" s="6" t="inlineStr">
+        <is>
+          <t>아니야, 치즈는 극혐!</t>
+        </is>
+      </c>
+      <c r="C295" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="D295" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E295" s="6" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F295" s="6" t="inlineStr"/>
+      <c r="G295" s="6" t="inlineStr">
+        <is>
+          <t>으엑! 치즈 냄새!! 극혐!!</t>
+        </is>
+      </c>
+      <c r="H295" s="6" t="inlineStr"/>
+    </row>
+    <row r="296">
+      <c r="A296" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B296" s="4" t="inlineStr">
+        <is>
+          <t>아니야, 치즈는 극혐!</t>
+        </is>
+      </c>
+      <c r="C296" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D296" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E296" s="4" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F296" s="4" t="inlineStr"/>
+      <c r="G296" s="4" t="inlineStr">
+        <is>
+          <t>방 문 닫을 거야!</t>
+        </is>
+      </c>
+      <c r="H296" s="4" t="inlineStr">
+        <is>
+          <t>후다닥!</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B297" s="6" t="inlineStr">
+        <is>
+          <t>아니야, 치즈는 극혐!</t>
+        </is>
+      </c>
+      <c r="C297" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="D297" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E297" s="6" t="inlineStr">
+        <is>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F297" s="6" t="inlineStr"/>
+      <c r="G297" s="6" t="inlineStr">
+        <is>
+          <t>…아차. 재이는 치즈 싫어하지.</t>
+        </is>
+      </c>
+      <c r="H297" s="6" t="inlineStr"/>
+    </row>
+    <row r="298">
+      <c r="A298" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B298" s="4" t="inlineStr">
+        <is>
+          <t>아니야, 치즈는 극혐!</t>
+        </is>
+      </c>
+      <c r="C298" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="D298" s="4" t="inlineStr">
+        <is>
+          <t>부엌</t>
+        </is>
+      </c>
+      <c r="E298" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F298" s="4" t="inlineStr"/>
+      <c r="G298" s="4" t="inlineStr">
+        <is>
+          <t>아빠, 누나 쪽은 치즈 빼 줘! 누나는 치즈 냄새 싫어해.</t>
+        </is>
+      </c>
+      <c r="H298" s="4" t="inlineStr"/>
+    </row>
+    <row r="299">
+      <c r="A299" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B299" s="6" t="inlineStr">
+        <is>
+          <t>아니야, 치즈는 극혐!</t>
+        </is>
+      </c>
+      <c r="C299" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="D299" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E299" s="6" t="inlineStr">
+        <is>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F299" s="6" t="inlineStr"/>
+      <c r="G299" s="6" t="inlineStr">
+        <is>
+          <t>태오가 그걸 다 기억하네?</t>
+        </is>
+      </c>
+      <c r="H299" s="6" t="inlineStr"/>
+    </row>
+    <row r="300">
+      <c r="A300" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B300" s="4" t="inlineStr">
+        <is>
+          <t>아니야, 치즈는 극혐!</t>
+        </is>
+      </c>
+      <c r="C300" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="D300" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E300" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F300" s="4" t="inlineStr"/>
+      <c r="G300" s="4" t="inlineStr">
+        <is>
+          <t>누나가 맨날 ‘아니야!’ 해서 다 알아.</t>
+        </is>
+      </c>
+      <c r="H300" s="4" t="inlineStr"/>
+    </row>
+    <row r="301">
+      <c r="A301" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B301" s="6" t="inlineStr">
+        <is>
+          <t>아니야, 치즈는 극혐!</t>
+        </is>
+      </c>
+      <c r="C301" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="D301" s="6" t="inlineStr">
+        <is>
+          <t>부엌</t>
+        </is>
+      </c>
+      <c r="E301" s="6" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F301" s="6" t="inlineStr"/>
+      <c r="G301" s="6" t="inlineStr">
+        <is>
+          <t>누나! 치즈 없는 쪽!
+…아니야, 고마워.</t>
+        </is>
+      </c>
+      <c r="H301" s="6" t="inlineStr"/>
+    </row>
+    <row r="302">
+      <c r="A302" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B302" s="4" t="inlineStr">
+        <is>
+          <t>아니야, 치즈는 극혐!</t>
+        </is>
+      </c>
+      <c r="C302" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="D302" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E302" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F302" s="4" t="inlineStr"/>
+      <c r="G302" s="4" t="inlineStr">
+        <is>
+          <t>아니야인데 고마워?</t>
+        </is>
+      </c>
+      <c r="H302" s="4" t="inlineStr"/>
+    </row>
+    <row r="303">
+      <c r="A303" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B303" s="6" t="inlineStr">
+        <is>
+          <t>아니야, 치즈는 극혐!</t>
+        </is>
+      </c>
+      <c r="C303" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="D303" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E303" s="6" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F303" s="6" t="inlineStr">
+        <is>
+          <t>그날 밤, 누나는 치즈 없는 피자를, / 태오는 레몬을 핥으며 티니핑을 봤다.</t>
+        </is>
+      </c>
+      <c r="G303" s="6" t="inlineStr"/>
+      <c r="H303" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:H284"/>
+  <autoFilter ref="A3:H303"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -11342,7 +12004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11733,13 +12395,13 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>김태오!</t>
+          <t>아니야!</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr"/>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+          <t>하루에도 제일 많이 하는 말</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr"/>
@@ -11750,22 +12412,18 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>짐방</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>김서방</t>
-        </is>
-      </c>
+          <t>맛있는데 지금은 먹기 싫어.</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr"/>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+          <t>누가 음식을 권하면</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr"/>
@@ -11776,22 +12434,18 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>꿍끙이</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>뿡뿡이</t>
-        </is>
-      </c>
+          <t>치즈 냄새 극혐!</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr"/>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+          <t>치즈만 보면 (냄새는 더더욱)</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr"/>
@@ -11800,30 +12454,74 @@
       <c r="A22" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="B22" s="4" t="inlineStr"/>
-      <c r="C22" s="4" t="inlineStr"/>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>재이 입버릇</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>김태오!</t>
+        </is>
+      </c>
       <c r="D22" s="4" t="inlineStr"/>
-      <c r="E22" s="4" t="inlineStr"/>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+        </is>
+      </c>
       <c r="F22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="B23" s="6" t="inlineStr"/>
-      <c r="C23" s="6" t="inlineStr"/>
-      <c r="D23" s="6" t="inlineStr"/>
-      <c r="E23" s="6" t="inlineStr"/>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>짐방</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>김서방</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+        </is>
+      </c>
       <c r="F23" s="6" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="4" t="inlineStr"/>
-      <c r="C24" s="4" t="inlineStr"/>
-      <c r="D24" s="4" t="inlineStr"/>
-      <c r="E24" s="4" t="inlineStr"/>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>꿍끙이</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>뿡뿡이</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+        </is>
+      </c>
       <c r="F24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
@@ -11946,8 +12644,38 @@
       <c r="E36" s="4" t="inlineStr"/>
       <c r="F36" s="4" t="inlineStr"/>
     </row>
+    <row r="37">
+      <c r="A37" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="B37" s="6" t="inlineStr"/>
+      <c r="C37" s="6" t="inlineStr"/>
+      <c r="D37" s="6" t="inlineStr"/>
+      <c r="E37" s="6" t="inlineStr"/>
+      <c r="F37" s="6" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="B38" s="4" t="inlineStr"/>
+      <c r="C38" s="4" t="inlineStr"/>
+      <c r="D38" s="4" t="inlineStr"/>
+      <c r="E38" s="4" t="inlineStr"/>
+      <c r="F38" s="4" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" s="6" t="inlineStr"/>
+      <c r="C39" s="6" t="inlineStr"/>
+      <c r="D39" s="6" t="inlineStr"/>
+      <c r="E39" s="6" t="inlineStr"/>
+      <c r="F39" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F36"/>
+  <autoFilter ref="A3:F39"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Note that both kids love Marvel
Jaei and Taeo both like Marvel heroes: Spider-Man, the Fantastic Four
and the Avengers. Both bios now say so, and the Excel cast sheet is
regenerated. Cache v173.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -546,12 +546,12 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>분홍 원피스, 흰 동그란 깃 · 입버릇 “아니야!” · 정리왕, 숙제 미리 끝 · 치즈 극혐</t>
+          <t>분홍 원피스, 흰 동그란 깃 · 입버릇 “아니야!” · 정리왕, 숙제 미리 끝 · 치즈 극혐 · 태오랑 같이 마블(스파이더맨·판타스틱 4·어벤져스) 좋아함</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>“아니야!”가 입버릇인 누나. 방은 늘 반듯하게 정리해 두고, 학교 숙제는 미리 다 해 놓고 노는 게 좋아요. 음식을 권하면 “맛있는데 지금은 먹기 싫어.” 치즈는 싫고 치즈 냄새는 극혐! 티니핑이랑 위시캣은 태오랑 둘 다 좋아해요. 동생이 괴롭혀도 참고 또 참다가, 폭발하면… “김태오!” 엉덩이 찰싹!</t>
+          <t>“아니야!”가 입버릇인 누나. 방은 늘 반듯하게 정리해 두고, 학교 숙제는 미리 다 해 놓고 노는 게 좋아요. 음식을 권하면 “맛있는데 지금은 먹기 싫어.” 치즈는 싫고 치즈 냄새는 극혐! 티니핑, 위시캣, 그리고 스파이더맨·판타스틱 4·어벤져스 같은 마블 영웅은 태오랑 둘 다 좋아해요. 동생이 괴롭혀도 참고 또 참다가, 폭발하면… “김태오!” 엉덩이 찰싹!</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>반쪽 레몬을 늘 손에 들고 다니며 할짝할짝 핥아 먹는 막내(레몬·자두·파인애플처럼 신 과일이 제일 좋아요). 누나 괴롭히기가 취미인 막내(사실은 누나가 좋아서). 혼자 노는 것 같아도 가족 말을 다 듣고 있고, 틀려도 일단 소리 지르며 우기다가 들키면 머리를 긁적긁적. “맛있는 거 죠!”가 입버릇이고, 어벤져스 영웅도 태오식으로 불러요(블루베리, 쉬터맨, 스테잌로저…). 블랙 위도우랑 수가 제일 예쁘대요. 제일 좋아하는 놀이는 어벤져스로 타노스랑 싸우기! 모든 호칭은 태오 기준이라, 누가 “재이야” 하면 “재이 누나야!” 하고 고쳐 줘요.</t>
+          <t>반쪽 레몬을 늘 손에 들고 다니며 할짝할짝 핥아 먹는 막내(레몬·자두·파인애플처럼 신 과일이 제일 좋아요). 누나 괴롭히기가 취미인 막내(사실은 누나가 좋아서). 혼자 노는 것 같아도 가족 말을 다 듣고 있고, 틀려도 일단 소리 지르며 우기다가 들키면 머리를 긁적긁적. “맛있는 거 죠!”가 입버릇이고, 누나랑 같이 좋아하는 마블 영웅(스파이더맨, 판타스틱 4, 어벤져스)도 태오식으로 불러요(블루베리, 쉬터맨, 스테잌로저…). 블랙 위도우랑 수가 제일 예쁘대요. 제일 좋아하는 놀이는 어벤져스로 타노스랑 싸우기! 모든 호칭은 태오 기준이라, 누가 “재이야” 하면 “재이 누나야!” 하고 고쳐 줘요.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 시치민 · 선샘민 to Taeo's dictionary
Taeo calls his teacher "시치민" or "선샘민". It joins his dictionary,
and in episode 10 he now insists "오구마꼬치 맞아!! 선샘민도 그랬어!!".
Excel regenerated. Cache v174.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$303</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$10</definedName>
   </definedNames>
@@ -1247,7 +1247,7 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>“패드로 어벤져스 게임 하자!” (보드게임) / “늘어나는 애 이름 뭐야?” 또 묻기 / “오구마꼬치 맞아!!” 우기다 긁적긁적</t>
+          <t>“패드로 어벤져스 게임 하자!” (보드게임) / “늘어나는 애 이름 뭐야?” 또 묻기 / “오구마꼬치 맞아!! 선샘민도 그랬어!!” 우기다 긁적긁적</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -6952,7 +6952,7 @@
       <c r="F165" s="6" t="inlineStr"/>
       <c r="G165" s="6" t="inlineStr">
         <is>
-          <t>아니야! 오구마꼬치 맞아!! 어린이집에서도 그렇게 해!!</t>
+          <t>아니야! 오구마꼬치 맞아!! 선샘민도 그랬어!!</t>
         </is>
       </c>
       <c r="H165" s="6" t="inlineStr">
@@ -11343,7 +11343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11773,17 +11773,17 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>어벤져스에 가년~</t>
+          <t>시치민 · 선샘민</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>어벤져스에 가면~</t>
+          <t>선생님</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>‘시장에 가면’ 놀이의 태오판. 누구누구 있는지 이어 말하기</t>
+          <t>어린이집 선생님을 부르는 말</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr"/>
@@ -11793,9 +11793,21 @@
       <c r="A22" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="B22" s="4" t="inlineStr"/>
-      <c r="C22" s="4" t="inlineStr"/>
-      <c r="D22" s="4" t="inlineStr"/>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>어벤져스에 가면~</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>‘시장에 가면’ 놀이의 태오판. 누구누구 있는지 이어 말하기</t>
+        </is>
+      </c>
       <c r="E22" s="4" t="inlineStr"/>
       <c r="F22" s="4" t="inlineStr"/>
     </row>
@@ -11989,8 +12001,18 @@
       <c r="E41" s="6" t="inlineStr"/>
       <c r="F41" s="6" t="inlineStr"/>
     </row>
+    <row r="42">
+      <c r="A42" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" s="4" t="inlineStr"/>
+      <c r="C42" s="4" t="inlineStr"/>
+      <c r="D42" s="4" t="inlineStr"/>
+      <c r="E42" s="4" t="inlineStr"/>
+      <c r="F42" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F41"/>
+  <autoFilter ref="A3:F42"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Split 시치민 and 선샘민 in Taeo's dictionary
The family clarified that Taeo said "시치민" when he was younger and
says "선샘민" now, so they are two entries showing the step up.
Excel regenerated. Cache v175.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$303</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$10</definedName>
   </definedNames>
@@ -11343,7 +11343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11773,7 +11773,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>시치민 · 선샘민</t>
+          <t>시치민</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -11783,7 +11783,7 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>어린이집 선생님을 부르는 말</t>
+          <t>더 어릴 때 선생님을 부르던 말</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr"/>
@@ -11795,17 +11795,17 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>어벤져스에 가년~</t>
+          <t>선샘민</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>어벤져스에 가면~</t>
+          <t>선생님</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>‘시장에 가면’ 놀이의 태오판. 누구누구 있는지 이어 말하기</t>
+          <t>요즘 어린이집 선생님을 부르는 말 (시치민에서 한 단계 성장!)</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr"/>
@@ -11815,9 +11815,21 @@
       <c r="A23" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="B23" s="6" t="inlineStr"/>
-      <c r="C23" s="6" t="inlineStr"/>
-      <c r="D23" s="6" t="inlineStr"/>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>어벤져스에 가면~</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>‘시장에 가면’ 놀이의 태오판. 누구누구 있는지 이어 말하기</t>
+        </is>
+      </c>
       <c r="E23" s="6" t="inlineStr"/>
       <c r="F23" s="6" t="inlineStr"/>
     </row>
@@ -12011,8 +12023,18 @@
       <c r="E42" s="4" t="inlineStr"/>
       <c r="F42" s="4" t="inlineStr"/>
     </row>
+    <row r="43">
+      <c r="A43" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" s="6" t="inlineStr"/>
+      <c r="C43" s="6" t="inlineStr"/>
+      <c r="D43" s="6" t="inlineStr"/>
+      <c r="E43" s="6" t="inlineStr"/>
+      <c r="F43" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F42"/>
+  <autoFilter ref="A3:F43"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add episode 18 "말 화살"
The family says Taeo has grown more aggressive lately, throwing words
like "침 뱉을 거야", "때릴 거야", "바보야" and "피노키오야". Episode 18
shows those words as grey arrows that fly out when he loses a board
game and stick in Jaei. Mom does not scold; she names the feeling ("화
났구나, 화나는 건 괜찮아"), explains that words stick like arrows, and
gives him a family spell: say "나 화났어!", punch a pillow, breathe out.
He apologises ("누나는 바보 아니야, 블랙 위도우야"), a kind word flies
as a pink heart-tipped arrow, and Jaei answers "아니야, 괜찮아."

The rougher phrases stay in the episode only, not in the word
collections. Taeo's bio notes he is practising the spell. New word
arrow prop; Excel adds episode 18. Cache v177.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -16,8 +16,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$303</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$322</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$10</definedName>
@@ -701,7 +701,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>반쪽 레몬을 늘 손에 들고 다니며 할짝할짝 핥아 먹는 막내(레몬·자두·파인애플처럼 신 과일이 제일 좋아요). 누나 괴롭히기가 취미인 막내(사실은 누나가 좋아서). 혼자 노는 것 같아도 가족 말을 다 듣고 있고, 틀려도 일단 소리 지르며 우기다가 들키면 머리를 긁적긁적. “맛있는 거 죠!”가 입버릇이고, 누나랑 같이 좋아하는 마블 영웅(스파이더맨, 판타스틱 4, 어벤져스)도 태오식으로 불러요(블루베리, 쉬터맨, 스테잌로저…). 블랙 위도우랑 수가 제일 예쁘대요. 제일 좋아하는 놀이는 어벤져스로 타노스랑 싸우기! 모든 호칭은 태오 기준이라, 누가 “재이야” 하면 “재이 누나야!” 하고 고쳐 줘요.</t>
+          <t>반쪽 레몬을 늘 손에 들고 다니며 할짝할짝 핥아 먹는 막내(레몬·자두·파인애플처럼 신 과일이 제일 좋아요). 누나 괴롭히기가 취미인 막내(사실은 누나가 좋아서). 혼자 노는 것 같아도 가족 말을 다 듣고 있고, 틀려도 일단 소리 지르며 우기다가 들키면 머리를 긁적긁적. “맛있는 거 죠!”가 입버릇이고, 누나랑 같이 좋아하는 마블 영웅(스파이더맨, 판타스틱 4, 어벤져스)도 태오식으로 불러요(블루베리, 쉬터맨, 스테잌로저…). 블랙 위도우랑 수가 제일 예쁘대요. 제일 좋아하는 놀이는 어벤져스로 타노스랑 싸우기! 모든 호칭은 태오 기준이라, 누가 “재이야” 하면 “재이 누나야!” 하고 고쳐 줘요. 요즘은 화가 나면 뾰족한 말이 튀어나오지만, “나 화났어!” 주문을 연습 중이에요.</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1614,17 +1614,47 @@
       <c r="A21" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="7" t="n"/>
-      <c r="C21" s="7" t="n"/>
-      <c r="D21" s="7" t="n"/>
-      <c r="E21" s="7" t="n"/>
-      <c r="F21" s="7" t="n"/>
-      <c r="G21" s="7" t="n"/>
-      <c r="H21" s="7" t="n"/>
-      <c r="I21" s="7" t="n"/>
-      <c r="J21" s="7" t="inlineStr">
-        <is>
-          <t>기획 중</t>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>말 화살</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>“바보야! 피노키오야! 때릴 거야! 침 뱉을 거야!” 요즘 태오 입에서 뾰족한 말이 날아다닌다. 그 말이 누나 마음에 꽂힌 날.</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>재이, 엄마, 아빠, 태오</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>게임에 진 태오의 “바보야! 피노키오야! 때릴 거야! 침 뱉을 거야!”가 화살이 되어 날아간다 / 베개 펀치 “쾅쾅” / 아빠 “나도 피노키오 아니지?” “아빠는… 타노스야.”</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>혼내는 대신 “화났구나, 화나는 건 괜찮아.” / 우리 집 주문 “나 화났어!” 후~ / “누나는 바보 아니야, 블랙 위도우야.”</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>화난 마음은 괜찮아요. 하지만 말은 화살처럼 마음에 꽂혀요. 화날 땐 “나 화났어!”라고 말해요.</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>화가 날 때 나만의 진정 방법은 뭐예요? 우리 가족 ‘화날 때 주문’을 정해 볼까요?</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="J21" s="6" t="inlineStr">
+        <is>
+          <t>완성</t>
         </is>
       </c>
     </row>
@@ -1664,13 +1694,31 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" s="7" t="n"/>
+      <c r="C24" s="7" t="n"/>
+      <c r="D24" s="7" t="n"/>
+      <c r="E24" s="7" t="n"/>
+      <c r="F24" s="7" t="n"/>
+      <c r="G24" s="7" t="n"/>
+      <c r="H24" s="7" t="n"/>
+      <c r="I24" s="7" t="n"/>
+      <c r="J24" s="7" t="inlineStr">
+        <is>
+          <t>기획 중</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:J20"/>
+  <autoFilter ref="A3:J21"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"아이디어,기획 중,콘티,완성"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1684,7 +1732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H303"/>
+  <dimension ref="A1:H322"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -11328,8 +11376,605 @@
       <c r="G303" s="6" t="inlineStr"/>
       <c r="H303" s="6" t="inlineStr"/>
     </row>
+    <row r="304">
+      <c r="A304" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B304" s="4" t="inlineStr">
+        <is>
+          <t>말 화살</t>
+        </is>
+      </c>
+      <c r="C304" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D304" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E304" s="4" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="F304" s="4" t="inlineStr">
+        <is>
+          <t>요즘 태오는 싸움 놀이가 한창이다.</t>
+        </is>
+      </c>
+      <c r="G304" s="4" t="inlineStr">
+        <is>
+          <t>누나, 영웅 게임 하자!</t>
+        </is>
+      </c>
+      <c r="H304" s="4" t="inlineStr"/>
+    </row>
+    <row r="305">
+      <c r="A305" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B305" s="6" t="inlineStr">
+        <is>
+          <t>말 화살</t>
+        </is>
+      </c>
+      <c r="C305" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D305" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E305" s="6" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F305" s="6" t="inlineStr"/>
+      <c r="G305" s="6" t="inlineStr">
+        <is>
+          <t>누나가 이겼다~!</t>
+        </is>
+      </c>
+      <c r="H305" s="6" t="inlineStr"/>
+    </row>
+    <row r="306">
+      <c r="A306" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B306" s="4" t="inlineStr">
+        <is>
+          <t>말 화살</t>
+        </is>
+      </c>
+      <c r="C306" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D306" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E306" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F306" s="4" t="inlineStr"/>
+      <c r="G306" s="4" t="inlineStr">
+        <is>
+          <t>누나 바보야!! 피노키오야!!</t>
+        </is>
+      </c>
+      <c r="H306" s="4" t="inlineStr"/>
+    </row>
+    <row r="307">
+      <c r="A307" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B307" s="6" t="inlineStr">
+        <is>
+          <t>말 화살</t>
+        </is>
+      </c>
+      <c r="C307" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D307" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E307" s="6" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="F307" s="6" t="inlineStr"/>
+      <c r="G307" s="6" t="inlineStr"/>
+      <c r="H307" s="6" t="inlineStr">
+        <is>
+          <t>슝!, 슝!</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B308" s="4" t="inlineStr">
+        <is>
+          <t>말 화살</t>
+        </is>
+      </c>
+      <c r="C308" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D308" s="4" t="inlineStr">
+        <is>
+          <t>효과: 어두움</t>
+        </is>
+      </c>
+      <c r="E308" s="4" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F308" s="4" t="inlineStr">
+        <is>
+          <t>말이 화살처럼 꽂혔다.</t>
+        </is>
+      </c>
+      <c r="G308" s="4" t="inlineStr">
+        <is>
+          <t>…</t>
+        </is>
+      </c>
+      <c r="H308" s="4" t="inlineStr"/>
+    </row>
+    <row r="309">
+      <c r="A309" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B309" s="6" t="inlineStr">
+        <is>
+          <t>말 화살</t>
+        </is>
+      </c>
+      <c r="C309" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D309" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E309" s="6" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F309" s="6" t="inlineStr"/>
+      <c r="G309" s="6" t="inlineStr">
+        <is>
+          <t>누나는 태오랑 놀아 준 건데…</t>
+        </is>
+      </c>
+      <c r="H309" s="6" t="inlineStr"/>
+    </row>
+    <row r="310">
+      <c r="A310" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B310" s="4" t="inlineStr">
+        <is>
+          <t>말 화살</t>
+        </is>
+      </c>
+      <c r="C310" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D310" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E310" s="4" t="inlineStr">
+        <is>
+          <t>엄마, 태오</t>
+        </is>
+      </c>
+      <c r="F310" s="4" t="inlineStr"/>
+      <c r="G310" s="4" t="inlineStr">
+        <is>
+          <t>태오야.
+(생각) (혼날 거야…)</t>
+        </is>
+      </c>
+      <c r="H310" s="4" t="inlineStr"/>
+    </row>
+    <row r="311">
+      <c r="A311" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B311" s="6" t="inlineStr">
+        <is>
+          <t>말 화살</t>
+        </is>
+      </c>
+      <c r="C311" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D311" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E311" s="6" t="inlineStr">
+        <is>
+          <t>엄마</t>
+        </is>
+      </c>
+      <c r="F311" s="6" t="inlineStr"/>
+      <c r="G311" s="6" t="inlineStr">
+        <is>
+          <t>태오, 게임에 져서 많이 화났구나. 화나는 건 괜찮아.</t>
+        </is>
+      </c>
+      <c r="H311" s="6" t="inlineStr"/>
+    </row>
+    <row r="312">
+      <c r="A312" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B312" s="4" t="inlineStr">
+        <is>
+          <t>말 화살</t>
+        </is>
+      </c>
+      <c r="C312" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D312" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E312" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F312" s="4" t="inlineStr"/>
+      <c r="G312" s="4" t="inlineStr">
+        <is>
+          <t>…안 혼내?</t>
+        </is>
+      </c>
+      <c r="H312" s="4" t="inlineStr"/>
+    </row>
+    <row r="313">
+      <c r="A313" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B313" s="6" t="inlineStr">
+        <is>
+          <t>말 화살</t>
+        </is>
+      </c>
+      <c r="C313" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D313" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E313" s="6" t="inlineStr">
+        <is>
+          <t>엄마, 재이</t>
+        </is>
+      </c>
+      <c r="F313" s="6" t="inlineStr"/>
+      <c r="G313" s="6" t="inlineStr">
+        <is>
+          <t>그런데 말은 화살 같아서, 한 번 날아가면 누나 마음에 콕 꽂혀.</t>
+        </is>
+      </c>
+      <c r="H313" s="6" t="inlineStr"/>
+    </row>
+    <row r="314">
+      <c r="A314" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B314" s="4" t="inlineStr">
+        <is>
+          <t>말 화살</t>
+        </is>
+      </c>
+      <c r="C314" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D314" s="4" t="inlineStr">
+        <is>
+          <t>효과: 어두움</t>
+        </is>
+      </c>
+      <c r="E314" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F314" s="4" t="inlineStr"/>
+      <c r="G314" s="4" t="inlineStr">
+        <is>
+          <t>(생각) (누나 울어…)</t>
+        </is>
+      </c>
+      <c r="H314" s="4" t="inlineStr"/>
+    </row>
+    <row r="315">
+      <c r="A315" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B315" s="6" t="inlineStr">
+        <is>
+          <t>말 화살</t>
+        </is>
+      </c>
+      <c r="C315" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D315" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E315" s="6" t="inlineStr">
+        <is>
+          <t>엄마, 태오</t>
+        </is>
+      </c>
+      <c r="F315" s="6" t="inlineStr"/>
+      <c r="G315" s="6" t="inlineStr">
+        <is>
+          <t>화날 땐 화살 대신 이렇게 말하는 거야. ‘나 화났어!’
+그리고 숨을 후~</t>
+        </is>
+      </c>
+      <c r="H315" s="6" t="inlineStr"/>
+    </row>
+    <row r="316">
+      <c r="A316" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B316" s="4" t="inlineStr">
+        <is>
+          <t>말 화살</t>
+        </is>
+      </c>
+      <c r="C316" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="D316" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E316" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F316" s="4" t="inlineStr"/>
+      <c r="G316" s="4" t="inlineStr">
+        <is>
+          <t>나… 화났어!!</t>
+        </is>
+      </c>
+      <c r="H316" s="4" t="inlineStr">
+        <is>
+          <t>베개 펀치!, 쾅쾅</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B317" s="6" t="inlineStr">
+        <is>
+          <t>말 화살</t>
+        </is>
+      </c>
+      <c r="C317" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="D317" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E317" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F317" s="6" t="inlineStr">
+        <is>
+          <t>레몬 한 번 핥고, 숨 한 번 후~</t>
+        </is>
+      </c>
+      <c r="G317" s="6" t="inlineStr">
+        <is>
+          <t>후우~</t>
+        </is>
+      </c>
+      <c r="H317" s="6" t="inlineStr">
+        <is>
+          <t>할짝</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B318" s="4" t="inlineStr">
+        <is>
+          <t>말 화살</t>
+        </is>
+      </c>
+      <c r="C318" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="D318" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E318" s="4" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="F318" s="4" t="inlineStr"/>
+      <c r="G318" s="4" t="inlineStr">
+        <is>
+          <t>누나… 바보 아니야. 누나는 블랙 위도우야.</t>
+        </is>
+      </c>
+      <c r="H318" s="4" t="inlineStr"/>
+    </row>
+    <row r="319">
+      <c r="A319" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B319" s="6" t="inlineStr">
+        <is>
+          <t>말 화살</t>
+        </is>
+      </c>
+      <c r="C319" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="D319" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E319" s="6" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F319" s="6" t="inlineStr"/>
+      <c r="G319" s="6" t="inlineStr">
+        <is>
+          <t>…아니야, 괜찮아.</t>
+        </is>
+      </c>
+      <c r="H319" s="6" t="inlineStr"/>
+    </row>
+    <row r="320">
+      <c r="A320" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B320" s="4" t="inlineStr">
+        <is>
+          <t>말 화살</t>
+        </is>
+      </c>
+      <c r="C320" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="D320" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E320" s="4" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="F320" s="4" t="inlineStr"/>
+      <c r="G320" s="4" t="inlineStr">
+        <is>
+          <t>좋은 말도 화살처럼 콕 꽂히네.</t>
+        </is>
+      </c>
+      <c r="H320" s="4" t="inlineStr"/>
+    </row>
+    <row r="321">
+      <c r="A321" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B321" s="6" t="inlineStr">
+        <is>
+          <t>말 화살</t>
+        </is>
+      </c>
+      <c r="C321" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="D321" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E321" s="6" t="inlineStr">
+        <is>
+          <t>아빠, 태오</t>
+        </is>
+      </c>
+      <c r="F321" s="6" t="inlineStr">
+        <is>
+          <t>그날 저녁.</t>
+        </is>
+      </c>
+      <c r="G321" s="6" t="inlineStr">
+        <is>
+          <t>그럼 아빠도 피노키오 아니지?
+아빠는… 타노스야.</t>
+        </is>
+      </c>
+      <c r="H321" s="6" t="inlineStr">
+        <is>
+          <t>…그건 맞지</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B322" s="4" t="inlineStr">
+        <is>
+          <t>말 화살</t>
+        </is>
+      </c>
+      <c r="C322" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="D322" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E322" s="4" t="inlineStr"/>
+      <c r="F322" s="4" t="inlineStr">
+        <is>
+          <t>우리 집 새 주문: “나 화났어!” 그리고 후~</t>
+        </is>
+      </c>
+      <c r="G322" s="4" t="inlineStr"/>
+      <c r="H322" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:H303"/>
+  <autoFilter ref="A3:H322"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add 인누와 and episode 19 "엄마 인누와"
Taeo often wakes at night and calls "엄마 인누와" ("come here") until
Mom lies down beside him. 인누와 joins his dictionary and sayings.

Episode 19: the 2 a.m. call, Mom stumbling over night after night until
Dad says she has panda eyes and offers to go instead, only to be turned
away ("아니! 엄마!! 인누와!!"). Mom realises this word will soon be
gone, goes to him, and Taeo offers to pat her to sleep; that night she
falls asleep first. A new "sleepers" prop shows the drawn faces side by
side on pillows under a blanket instead of rotated bodies. Excel adds
episode 19. Cache v178.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$322</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$43</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$338</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1659,20 +1659,50 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="n">
+      <c r="A22" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="B22" s="7" t="n"/>
-      <c r="C22" s="7" t="n"/>
-      <c r="D22" s="7" t="n"/>
-      <c r="E22" s="7" t="n"/>
-      <c r="F22" s="7" t="n"/>
-      <c r="G22" s="7" t="n"/>
-      <c r="H22" s="7" t="n"/>
-      <c r="I22" s="7" t="n"/>
-      <c r="J22" s="7" t="inlineStr">
-        <is>
-          <t>기획 중</t>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>엄마 인누와</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>새벽 2시, 어둠 속에서 들려오는 작은 목소리. “엄마… 인누와~” 오늘 밤도 엄마는 태오 옆으로 간다.</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>엄마, 아빠, 태오</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>새벽 2시 “엄마… 인누와~” / 엄마 눈 밑이 판다 / 아빠가 대신 갔다가 “아니! 엄마!! 인누와!!” → 아빠 탈락</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>‘인누와’도 곧 사라질 말 / “엄마 피곤하지? 이번엔 내가 토닥토닥 해 줄게.” — 그날 밤은 엄마가 먼저 잠들었다</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>“인누와”는 금방 사라질 말이에요. 오늘 밤, 부를 때 옆에 있어 주세요.</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>잠이 안 올 때 누가 옆에 있으면 좋아요? 우리 가족 ‘잠 주문’을 만들어 볼까요?</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>완성</t>
         </is>
       </c>
     </row>
@@ -1712,13 +1742,31 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" s="7" t="n"/>
+      <c r="C25" s="7" t="n"/>
+      <c r="D25" s="7" t="n"/>
+      <c r="E25" s="7" t="n"/>
+      <c r="F25" s="7" t="n"/>
+      <c r="G25" s="7" t="n"/>
+      <c r="H25" s="7" t="n"/>
+      <c r="I25" s="7" t="n"/>
+      <c r="J25" s="7" t="inlineStr">
+        <is>
+          <t>기획 중</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:J21"/>
+  <autoFilter ref="A3:J22"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"아이디어,기획 중,콘티,완성"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1732,7 +1780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H322"/>
+  <dimension ref="A1:H338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -11973,8 +12021,509 @@
       <c r="G322" s="4" t="inlineStr"/>
       <c r="H322" s="4" t="inlineStr"/>
     </row>
+    <row r="323">
+      <c r="A323" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B323" s="6" t="inlineStr">
+        <is>
+          <t>엄마 인누와</t>
+        </is>
+      </c>
+      <c r="C323" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D323" s="6" t="inlineStr">
+        <is>
+          <t>방(밤)</t>
+        </is>
+      </c>
+      <c r="E323" s="6" t="inlineStr"/>
+      <c r="F323" s="6" t="inlineStr">
+        <is>
+          <t>새벽 2시.</t>
+        </is>
+      </c>
+      <c r="G323" s="6" t="inlineStr"/>
+      <c r="H323" s="6" t="inlineStr">
+        <is>
+          <t>쿨쿨</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B324" s="4" t="inlineStr">
+        <is>
+          <t>엄마 인누와</t>
+        </is>
+      </c>
+      <c r="C324" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D324" s="4" t="inlineStr">
+        <is>
+          <t>효과: 어두움</t>
+        </is>
+      </c>
+      <c r="E324" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F324" s="4" t="inlineStr"/>
+      <c r="G324" s="4" t="inlineStr">
+        <is>
+          <t>(속삭임) …엄마… 인누와~</t>
+        </is>
+      </c>
+      <c r="H324" s="4" t="inlineStr"/>
+    </row>
+    <row r="325">
+      <c r="A325" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B325" s="6" t="inlineStr">
+        <is>
+          <t>엄마 인누와</t>
+        </is>
+      </c>
+      <c r="C325" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D325" s="6" t="inlineStr">
+        <is>
+          <t>방(밤)</t>
+        </is>
+      </c>
+      <c r="E325" s="6" t="inlineStr"/>
+      <c r="F325" s="6" t="inlineStr">
+        <is>
+          <t>안방.</t>
+        </is>
+      </c>
+      <c r="G325" s="6" t="inlineStr">
+        <is>
+          <t>(속삭임) …또 부른다.</t>
+        </is>
+      </c>
+      <c r="H325" s="6" t="inlineStr">
+        <is>
+          <t>드르렁</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B326" s="4" t="inlineStr">
+        <is>
+          <t>엄마 인누와</t>
+        </is>
+      </c>
+      <c r="C326" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D326" s="4" t="inlineStr">
+        <is>
+          <t>방(밤)</t>
+        </is>
+      </c>
+      <c r="E326" s="4" t="inlineStr">
+        <is>
+          <t>엄마</t>
+        </is>
+      </c>
+      <c r="F326" s="4" t="inlineStr"/>
+      <c r="G326" s="4" t="inlineStr">
+        <is>
+          <t>(속삭임) 그래… 엄마 간다…</t>
+        </is>
+      </c>
+      <c r="H326" s="4" t="inlineStr">
+        <is>
+          <t>비틀비틀</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B327" s="6" t="inlineStr">
+        <is>
+          <t>엄마 인누와</t>
+        </is>
+      </c>
+      <c r="C327" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D327" s="6" t="inlineStr">
+        <is>
+          <t>방(밤)</t>
+        </is>
+      </c>
+      <c r="E327" s="6" t="inlineStr"/>
+      <c r="F327" s="6" t="inlineStr"/>
+      <c r="G327" s="6" t="inlineStr">
+        <is>
+          <t>(속삭임) 헤헤… 엄마 냄새.</t>
+        </is>
+      </c>
+      <c r="H327" s="6" t="inlineStr">
+        <is>
+          <t>토닥토닥</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B328" s="4" t="inlineStr">
+        <is>
+          <t>엄마 인누와</t>
+        </is>
+      </c>
+      <c r="C328" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D328" s="4" t="inlineStr">
+        <is>
+          <t>부엌</t>
+        </is>
+      </c>
+      <c r="E328" s="4" t="inlineStr">
+        <is>
+          <t>엄마, 아빠</t>
+        </is>
+      </c>
+      <c r="F328" s="4" t="inlineStr">
+        <is>
+          <t>다음 날 아침. 그다음 날도. 또 그다음 날도.</t>
+        </is>
+      </c>
+      <c r="G328" s="4" t="inlineStr">
+        <is>
+          <t>여보… 눈 밑이 판다야.</t>
+        </is>
+      </c>
+      <c r="H328" s="4" t="inlineStr">
+        <is>
+          <t>하아암</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B329" s="6" t="inlineStr">
+        <is>
+          <t>엄마 인누와</t>
+        </is>
+      </c>
+      <c r="C329" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="D329" s="6" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E329" s="6" t="inlineStr">
+        <is>
+          <t>아빠, 엄마</t>
+        </is>
+      </c>
+      <c r="F329" s="6" t="inlineStr"/>
+      <c r="G329" s="6" t="inlineStr">
+        <is>
+          <t>오늘 밤은 아빠가 갈게. 당신은 푹 자!</t>
+        </is>
+      </c>
+      <c r="H329" s="6" t="inlineStr"/>
+    </row>
+    <row r="330">
+      <c r="A330" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B330" s="4" t="inlineStr">
+        <is>
+          <t>엄마 인누와</t>
+        </is>
+      </c>
+      <c r="C330" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D330" s="4" t="inlineStr">
+        <is>
+          <t>효과: 어두움</t>
+        </is>
+      </c>
+      <c r="E330" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F330" s="4" t="inlineStr">
+        <is>
+          <t>그날 새벽.</t>
+        </is>
+      </c>
+      <c r="G330" s="4" t="inlineStr">
+        <is>
+          <t>(속삭임) 엄마… 인누와~</t>
+        </is>
+      </c>
+      <c r="H330" s="4" t="inlineStr"/>
+    </row>
+    <row r="331">
+      <c r="A331" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B331" s="6" t="inlineStr">
+        <is>
+          <t>엄마 인누와</t>
+        </is>
+      </c>
+      <c r="C331" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="D331" s="6" t="inlineStr">
+        <is>
+          <t>방(밤)</t>
+        </is>
+      </c>
+      <c r="E331" s="6" t="inlineStr">
+        <is>
+          <t>아빠, 태오</t>
+        </is>
+      </c>
+      <c r="F331" s="6" t="inlineStr"/>
+      <c r="G331" s="6" t="inlineStr">
+        <is>
+          <t>아빠 왔다~!
+아니! 엄마!! 인누와!!</t>
+        </is>
+      </c>
+      <c r="H331" s="6" t="inlineStr"/>
+    </row>
+    <row r="332">
+      <c r="A332" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B332" s="4" t="inlineStr">
+        <is>
+          <t>엄마 인누와</t>
+        </is>
+      </c>
+      <c r="C332" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D332" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E332" s="4" t="inlineStr">
+        <is>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F332" s="4" t="inlineStr"/>
+      <c r="G332" s="4" t="inlineStr">
+        <is>
+          <t>…아빠 탈락.</t>
+        </is>
+      </c>
+      <c r="H332" s="4" t="inlineStr">
+        <is>
+          <t>삐빅</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B333" s="6" t="inlineStr">
+        <is>
+          <t>엄마 인누와</t>
+        </is>
+      </c>
+      <c r="C333" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="D333" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E333" s="6" t="inlineStr">
+        <is>
+          <t>엄마</t>
+        </is>
+      </c>
+      <c r="F333" s="6" t="inlineStr">
+        <is>
+          <t>문 뒤에서 듣던 엄마는 생각했다.</t>
+        </is>
+      </c>
+      <c r="G333" s="6" t="inlineStr">
+        <is>
+          <t>(생각) (언젠가는 안 부르겠지. ‘인누와’도 곧 사라질 말이겠지.)</t>
+        </is>
+      </c>
+      <c r="H333" s="6" t="inlineStr"/>
+    </row>
+    <row r="334">
+      <c r="A334" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B334" s="4" t="inlineStr">
+        <is>
+          <t>엄마 인누와</t>
+        </is>
+      </c>
+      <c r="C334" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D334" s="4" t="inlineStr">
+        <is>
+          <t>방(밤)</t>
+        </is>
+      </c>
+      <c r="E334" s="4" t="inlineStr">
+        <is>
+          <t>엄마, 태오</t>
+        </is>
+      </c>
+      <c r="F334" s="4" t="inlineStr"/>
+      <c r="G334" s="4" t="inlineStr">
+        <is>
+          <t>엄마 여기 있어.</t>
+        </is>
+      </c>
+      <c r="H334" s="4" t="inlineStr"/>
+    </row>
+    <row r="335">
+      <c r="A335" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B335" s="6" t="inlineStr">
+        <is>
+          <t>엄마 인누와</t>
+        </is>
+      </c>
+      <c r="C335" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="D335" s="6" t="inlineStr">
+        <is>
+          <t>방(밤)</t>
+        </is>
+      </c>
+      <c r="E335" s="6" t="inlineStr"/>
+      <c r="F335" s="6" t="inlineStr"/>
+      <c r="G335" s="6" t="inlineStr">
+        <is>
+          <t>(속삭임) 엄마 피곤하지? 이번엔 내가 토닥토닥 해 줄게.</t>
+        </is>
+      </c>
+      <c r="H335" s="6" t="inlineStr"/>
+    </row>
+    <row r="336">
+      <c r="A336" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B336" s="4" t="inlineStr">
+        <is>
+          <t>엄마 인누와</t>
+        </is>
+      </c>
+      <c r="C336" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="D336" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E336" s="4" t="inlineStr">
+        <is>
+          <t>엄마</t>
+        </is>
+      </c>
+      <c r="F336" s="4" t="inlineStr"/>
+      <c r="G336" s="4" t="inlineStr"/>
+      <c r="H336" s="4" t="inlineStr">
+        <is>
+          <t>토닥… 토닥…</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B337" s="6" t="inlineStr">
+        <is>
+          <t>엄마 인누와</t>
+        </is>
+      </c>
+      <c r="C337" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="D337" s="6" t="inlineStr">
+        <is>
+          <t>방(밤)</t>
+        </is>
+      </c>
+      <c r="E337" s="6" t="inlineStr"/>
+      <c r="F337" s="6" t="inlineStr">
+        <is>
+          <t>그날 밤은 엄마가 먼저 잠들었다.</t>
+        </is>
+      </c>
+      <c r="G337" s="6" t="inlineStr"/>
+      <c r="H337" s="6" t="inlineStr">
+        <is>
+          <t>쿨쿨</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B338" s="4" t="inlineStr">
+        <is>
+          <t>엄마 인누와</t>
+        </is>
+      </c>
+      <c r="C338" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="D338" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E338" s="4" t="inlineStr"/>
+      <c r="F338" s="4" t="inlineStr">
+        <is>
+          <t>“인누와”라고 불러 주는 밤이, / 사실은 엄마에게도 선물이었다.</t>
+        </is>
+      </c>
+      <c r="G338" s="4" t="inlineStr"/>
+      <c r="H338" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:H322"/>
+  <autoFilter ref="A3:H338"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -11988,7 +12537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -12462,17 +13011,17 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>어벤져스에 가년~</t>
+          <t>인누와</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>어벤져스에 가면~</t>
+          <t>이리 와</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>‘시장에 가면’ 놀이의 태오판. 누구누구 있는지 이어 말하기</t>
+          <t>“엄마 인누와~” 밤에 깨서 옆에서 재워 달라고 부를 때</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr"/>
@@ -12482,9 +13031,21 @@
       <c r="A24" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="4" t="inlineStr"/>
-      <c r="C24" s="4" t="inlineStr"/>
-      <c r="D24" s="4" t="inlineStr"/>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>어벤져스에 가면~</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>‘시장에 가면’ 놀이의 태오판. 누구누구 있는지 이어 말하기</t>
+        </is>
+      </c>
       <c r="E24" s="4" t="inlineStr"/>
       <c r="F24" s="4" t="inlineStr"/>
     </row>
@@ -12678,8 +13239,18 @@
       <c r="E43" s="6" t="inlineStr"/>
       <c r="F43" s="6" t="inlineStr"/>
     </row>
+    <row r="44">
+      <c r="A44" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" s="4" t="inlineStr"/>
+      <c r="C44" s="4" t="inlineStr"/>
+      <c r="D44" s="4" t="inlineStr"/>
+      <c r="E44" s="4" t="inlineStr"/>
+      <c r="F44" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F43"/>
+  <autoFilter ref="A3:F44"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -12693,7 +13264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -13062,13 +13633,13 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>왜 놀려! 놀리지 마!</t>
+          <t>엄마 인누와~</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr"/>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>“태오는 글씨·숫자 잘 몰라” 소리를 들으면 (손가락질하며)</t>
+          <t>밤에 자다 깨서 (엄마가 옆에서 재워 줄 때까지)</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr"/>
@@ -13079,18 +13650,18 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>아니야!</t>
+          <t>왜 놀려! 놀리지 마!</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr"/>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>하루에도 제일 많이 하는 말</t>
+          <t>“태오는 글씨·숫자 잘 몰라” 소리를 들으면 (손가락질하며)</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr"/>
@@ -13106,13 +13677,13 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>맛있는데 지금은 먹기 싫어.</t>
+          <t>아니야!</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr"/>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>누가 음식을 권하면</t>
+          <t>하루에도 제일 많이 하는 말</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr"/>
@@ -13128,13 +13699,13 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>치즈 냄새 극혐!</t>
+          <t>맛있는데 지금은 먹기 싫어.</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr"/>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>치즈만 보면 (냄새는 더더욱)</t>
+          <t>누가 음식을 권하면</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr"/>
@@ -13150,13 +13721,13 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>김태오!</t>
+          <t>치즈 냄새 극혐!</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr"/>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+          <t>치즈만 보면 (냄새는 더더욱)</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr"/>
@@ -13167,22 +13738,18 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>짐방</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>김서방</t>
-        </is>
-      </c>
+          <t>김태오!</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr"/>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr"/>
@@ -13198,17 +13765,17 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>꿍끙이</t>
+          <t>짐방</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>뿡뿡이</t>
+          <t>김서방</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr"/>
@@ -13217,10 +13784,26 @@
       <c r="A25" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="B25" s="6" t="inlineStr"/>
-      <c r="C25" s="6" t="inlineStr"/>
-      <c r="D25" s="6" t="inlineStr"/>
-      <c r="E25" s="6" t="inlineStr"/>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>꿍끙이</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>뿡뿡이</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+        </is>
+      </c>
       <c r="F25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
@@ -13363,8 +13946,18 @@
       <c r="E39" s="6" t="inlineStr"/>
       <c r="F39" s="6" t="inlineStr"/>
     </row>
+    <row r="40">
+      <c r="A40" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" s="4" t="inlineStr"/>
+      <c r="C40" s="4" t="inlineStr"/>
+      <c r="D40" s="4" t="inlineStr"/>
+      <c r="E40" s="4" t="inlineStr"/>
+      <c r="F40" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F39"/>
+  <autoFilter ref="A3:F40"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add "거짓말! 아니야!" and episode 20
Jaei says "거짓말! 아니야!" when she feels bad or does not want to do
something. It joins her sayings and bio.

Episode 20: at hair-washing time she answers "거짓말! 아니야!", even
blaming the clock, and Taeo copies it for brushing teeth ("이거 내
말이야!"). Mom asks what is hidden behind the words and Jaei admits she
fears water in her eyes; Dad covers her eyes with a towel, Taeo cheers
her on with his lemon, and she finds it was not scary. That night Taeo
uses her line on her and she shouts "김태오!". New bathroom background,
shampoo and foam props. Excel adds episode 20. Cache v179.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$338</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$356</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$44</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -551,7 +551,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>“아니야!”가 입버릇인 누나. 방은 늘 반듯하게 정리해 두고, 학교 숙제는 미리 다 해 놓고 노는 게 좋아요. 음식을 권하면 “맛있는데 지금은 먹기 싫어.” 치즈는 싫고 치즈 냄새는 극혐! 티니핑, 위시캣, 그리고 스파이더맨·판타스틱 4·어벤져스 같은 마블 영웅은 태오랑 둘 다 좋아해요. 동생이 괴롭혀도 참고 또 참다가, 폭발하면… “김태오!” 엉덩이 찰싹!</t>
+          <t>“아니야!”가 입버릇인 누나. 방은 늘 반듯하게 정리해 두고, 학교 숙제는 미리 다 해 놓고 노는 게 좋아요. 음식을 권하면 “맛있는데 지금은 먹기 싫어.” 치즈는 싫고 치즈 냄새는 극혐! 티니핑, 위시캣, 그리고 스파이더맨·판타스틱 4·어벤져스 같은 마블 영웅은 태오랑 둘 다 좋아해요. 동생이 괴롭혀도 참고 또 참다가, 폭발하면… “김태오!” 엉덩이 찰싹! 기분 나쁘거나 하기 싫을 때는 “거짓말! 아니야!”</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1710,17 +1710,47 @@
       <c r="A23" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="B23" s="7" t="n"/>
-      <c r="C23" s="7" t="n"/>
-      <c r="D23" s="7" t="n"/>
-      <c r="E23" s="7" t="n"/>
-      <c r="F23" s="7" t="n"/>
-      <c r="G23" s="7" t="n"/>
-      <c r="H23" s="7" t="n"/>
-      <c r="I23" s="7" t="n"/>
-      <c r="J23" s="7" t="inlineStr">
-        <is>
-          <t>기획 중</t>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>거짓말! 아니야!</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>“머리 감을 시간이야.” “거짓말! 아니야!” 재이 누나가 기분 나쁘거나 하기 싫을 때 꺼내는 말. 그 뒤에 숨은 진짜 마음은 뭐였을까?</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>재이, 엄마, 아빠, 태오</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>“머리 감을 시간이야.” “거짓말! 아니야!” “시계가 거짓말이야!” / 태오도 “거짓말! 아니야!” 따라 하고 “이거 내 말이야!” / 마지막엔 태오가 누나 말을 도로 가져가 “김태오!”</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>‘아니야’ 뒤에 숨은 마음: 눈에 물 들어가는 게 무서워 / 엄마 ‘말해 줘서 고마워’, 아빠 수건으로 눈 가리기, 태오 레몬 냄새 응원</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>“아니야” 뒤에는 마음이 숨어 있어요. 이유를 말하면 가족이 도와줄 수 있어요.</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>나는 하기 싫을 때 어떤 말을 하나요? 그 말 뒤에는 어떤 마음이 숨어 있을까요?</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="J23" s="6" t="inlineStr">
+        <is>
+          <t>완성</t>
         </is>
       </c>
     </row>
@@ -1760,13 +1790,31 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="7" t="n"/>
+      <c r="C26" s="7" t="n"/>
+      <c r="D26" s="7" t="n"/>
+      <c r="E26" s="7" t="n"/>
+      <c r="F26" s="7" t="n"/>
+      <c r="G26" s="7" t="n"/>
+      <c r="H26" s="7" t="n"/>
+      <c r="I26" s="7" t="n"/>
+      <c r="J26" s="7" t="inlineStr">
+        <is>
+          <t>기획 중</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:J22"/>
+  <autoFilter ref="A3:J23"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"아이디어,기획 중,콘티,완성"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1780,7 +1828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H338"/>
+  <dimension ref="A1:H356"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -12522,8 +12570,567 @@
       <c r="G338" s="4" t="inlineStr"/>
       <c r="H338" s="4" t="inlineStr"/>
     </row>
+    <row r="339">
+      <c r="A339" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B339" s="6" t="inlineStr">
+        <is>
+          <t>거짓말! 아니야!</t>
+        </is>
+      </c>
+      <c r="C339" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D339" s="6" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E339" s="6" t="inlineStr">
+        <is>
+          <t>엄마, 재이</t>
+        </is>
+      </c>
+      <c r="F339" s="6" t="inlineStr">
+        <is>
+          <t>저녁 8시.</t>
+        </is>
+      </c>
+      <c r="G339" s="6" t="inlineStr">
+        <is>
+          <t>재이야, 머리 감을 시간이야.</t>
+        </is>
+      </c>
+      <c r="H339" s="6" t="inlineStr"/>
+    </row>
+    <row r="340">
+      <c r="A340" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B340" s="4" t="inlineStr">
+        <is>
+          <t>거짓말! 아니야!</t>
+        </is>
+      </c>
+      <c r="C340" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D340" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E340" s="4" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F340" s="4" t="inlineStr"/>
+      <c r="G340" s="4" t="inlineStr">
+        <is>
+          <t>거짓말! 아니야!!</t>
+        </is>
+      </c>
+      <c r="H340" s="4" t="inlineStr"/>
+    </row>
+    <row r="341">
+      <c r="A341" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B341" s="6" t="inlineStr">
+        <is>
+          <t>거짓말! 아니야!</t>
+        </is>
+      </c>
+      <c r="C341" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D341" s="6" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E341" s="6" t="inlineStr">
+        <is>
+          <t>엄마, 재이</t>
+        </is>
+      </c>
+      <c r="F341" s="6" t="inlineStr"/>
+      <c r="G341" s="6" t="inlineStr">
+        <is>
+          <t>거짓말 아니야. 시계 봐. 8시야.
+아니야! 시계가 거짓말이야!</t>
+        </is>
+      </c>
+      <c r="H341" s="6" t="inlineStr"/>
+    </row>
+    <row r="342">
+      <c r="A342" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B342" s="4" t="inlineStr">
+        <is>
+          <t>거짓말! 아니야!</t>
+        </is>
+      </c>
+      <c r="C342" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D342" s="4" t="inlineStr">
+        <is>
+          <t>부엌</t>
+        </is>
+      </c>
+      <c r="E342" s="4" t="inlineStr">
+        <is>
+          <t>아빠, 태오</t>
+        </is>
+      </c>
+      <c r="F342" s="4" t="inlineStr"/>
+      <c r="G342" s="4" t="inlineStr">
+        <is>
+          <t>태오야, 이 닦자~</t>
+        </is>
+      </c>
+      <c r="H342" s="4" t="inlineStr"/>
+    </row>
+    <row r="343">
+      <c r="A343" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B343" s="6" t="inlineStr">
+        <is>
+          <t>거짓말! 아니야!</t>
+        </is>
+      </c>
+      <c r="C343" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D343" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E343" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F343" s="6" t="inlineStr"/>
+      <c r="G343" s="6" t="inlineStr">
+        <is>
+          <t>거짓말! 아니야!!</t>
+        </is>
+      </c>
+      <c r="H343" s="6" t="inlineStr"/>
+    </row>
+    <row r="344">
+      <c r="A344" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B344" s="4" t="inlineStr">
+        <is>
+          <t>거짓말! 아니야!</t>
+        </is>
+      </c>
+      <c r="C344" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D344" s="4" t="inlineStr">
+        <is>
+          <t>부엌</t>
+        </is>
+      </c>
+      <c r="E344" s="4" t="inlineStr">
+        <is>
+          <t>아빠, 태오</t>
+        </is>
+      </c>
+      <c r="F344" s="4" t="inlineStr"/>
+      <c r="G344" s="4" t="inlineStr">
+        <is>
+          <t>누나 따라 하지 마~
+따라 아니야! 이거 내 말이야!</t>
+        </is>
+      </c>
+      <c r="H344" s="4" t="inlineStr"/>
+    </row>
+    <row r="345">
+      <c r="A345" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B345" s="6" t="inlineStr">
+        <is>
+          <t>거짓말! 아니야!</t>
+        </is>
+      </c>
+      <c r="C345" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="D345" s="6" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E345" s="6" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F345" s="6" t="inlineStr">
+        <is>
+          <t>하지만 재이 누나는 알고 있었다.</t>
+        </is>
+      </c>
+      <c r="G345" s="6" t="inlineStr">
+        <is>
+          <t>(생각) (사실은 내 말이 맞는데…)</t>
+        </is>
+      </c>
+      <c r="H345" s="6" t="inlineStr"/>
+    </row>
+    <row r="346">
+      <c r="A346" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B346" s="4" t="inlineStr">
+        <is>
+          <t>거짓말! 아니야!</t>
+        </is>
+      </c>
+      <c r="C346" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D346" s="4" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E346" s="4" t="inlineStr">
+        <is>
+          <t>엄마, 재이</t>
+        </is>
+      </c>
+      <c r="F346" s="4" t="inlineStr"/>
+      <c r="G346" s="4" t="inlineStr">
+        <is>
+          <t>재이가 하기 싫을 때 ‘거짓말! 아니야!’ 하는 거, 엄마 알아.</t>
+        </is>
+      </c>
+      <c r="H346" s="4" t="inlineStr"/>
+    </row>
+    <row r="347">
+      <c r="A347" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B347" s="6" t="inlineStr">
+        <is>
+          <t>거짓말! 아니야!</t>
+        </is>
+      </c>
+      <c r="C347" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="D347" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E347" s="6" t="inlineStr">
+        <is>
+          <t>엄마</t>
+        </is>
+      </c>
+      <c r="F347" s="6" t="inlineStr"/>
+      <c r="G347" s="6" t="inlineStr">
+        <is>
+          <t>그 말 뒤에 뭐가 숨어 있는지 말해 줄 수 있어?</t>
+        </is>
+      </c>
+      <c r="H347" s="6" t="inlineStr"/>
+    </row>
+    <row r="348">
+      <c r="A348" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B348" s="4" t="inlineStr">
+        <is>
+          <t>거짓말! 아니야!</t>
+        </is>
+      </c>
+      <c r="C348" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D348" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E348" s="4" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F348" s="4" t="inlineStr"/>
+      <c r="G348" s="4" t="inlineStr">
+        <is>
+          <t>(속삭임) …머리 헹굴 때 눈에 물 들어가는 게 무서워.</t>
+        </is>
+      </c>
+      <c r="H348" s="4" t="inlineStr"/>
+    </row>
+    <row r="349">
+      <c r="A349" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B349" s="6" t="inlineStr">
+        <is>
+          <t>거짓말! 아니야!</t>
+        </is>
+      </c>
+      <c r="C349" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="D349" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E349" s="6" t="inlineStr">
+        <is>
+          <t>엄마</t>
+        </is>
+      </c>
+      <c r="F349" s="6" t="inlineStr"/>
+      <c r="G349" s="6" t="inlineStr">
+        <is>
+          <t>아, 그래서 그랬구나. 말해 줘서 고마워. 같이 방법을 찾아보자.</t>
+        </is>
+      </c>
+      <c r="H349" s="6" t="inlineStr"/>
+    </row>
+    <row r="350">
+      <c r="A350" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B350" s="4" t="inlineStr">
+        <is>
+          <t>거짓말! 아니야!</t>
+        </is>
+      </c>
+      <c r="C350" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D350" s="4" t="inlineStr">
+        <is>
+          <t>bath</t>
+        </is>
+      </c>
+      <c r="E350" s="4" t="inlineStr">
+        <is>
+          <t>재이, 아빠, 태오</t>
+        </is>
+      </c>
+      <c r="F350" s="4" t="inlineStr"/>
+      <c r="G350" s="4" t="inlineStr">
+        <is>
+          <t>아빠가 수건으로 눈 가려 줄게. 절대 안 들어가!</t>
+        </is>
+      </c>
+      <c r="H350" s="4" t="inlineStr"/>
+    </row>
+    <row r="351">
+      <c r="A351" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B351" s="6" t="inlineStr">
+        <is>
+          <t>거짓말! 아니야!</t>
+        </is>
+      </c>
+      <c r="C351" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="D351" s="6" t="inlineStr">
+        <is>
+          <t>bath</t>
+        </is>
+      </c>
+      <c r="E351" s="6" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="F351" s="6" t="inlineStr"/>
+      <c r="G351" s="6" t="inlineStr">
+        <is>
+          <t>누나! 내 레몬 냄새 맡아 봐. 무서운 거 다 없어져!</t>
+        </is>
+      </c>
+      <c r="H351" s="6" t="inlineStr"/>
+    </row>
+    <row r="352">
+      <c r="A352" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B352" s="4" t="inlineStr">
+        <is>
+          <t>거짓말! 아니야!</t>
+        </is>
+      </c>
+      <c r="C352" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="D352" s="4" t="inlineStr">
+        <is>
+          <t>bath</t>
+        </is>
+      </c>
+      <c r="E352" s="4" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F352" s="4" t="inlineStr"/>
+      <c r="G352" s="4" t="inlineStr">
+        <is>
+          <t>하나, 둘, 셋… 후~</t>
+        </is>
+      </c>
+      <c r="H352" s="4" t="inlineStr">
+        <is>
+          <t>쏴아~</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B353" s="6" t="inlineStr">
+        <is>
+          <t>거짓말! 아니야!</t>
+        </is>
+      </c>
+      <c r="C353" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="D353" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E353" s="6" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F353" s="6" t="inlineStr"/>
+      <c r="G353" s="6" t="inlineStr">
+        <is>
+          <t>…어? 안 무서웠어!</t>
+        </is>
+      </c>
+      <c r="H353" s="6" t="inlineStr"/>
+    </row>
+    <row r="354">
+      <c r="A354" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B354" s="4" t="inlineStr">
+        <is>
+          <t>거짓말! 아니야!</t>
+        </is>
+      </c>
+      <c r="C354" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="D354" s="4" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E354" s="4" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F354" s="4" t="inlineStr">
+        <is>
+          <t>그날 밤.</t>
+        </is>
+      </c>
+      <c r="G354" s="4" t="inlineStr">
+        <is>
+          <t>진짜야! 하나도 안 무서웠어!
+거짓말! 아니야!</t>
+        </is>
+      </c>
+      <c r="H354" s="4" t="inlineStr"/>
+    </row>
+    <row r="355">
+      <c r="A355" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B355" s="6" t="inlineStr">
+        <is>
+          <t>거짓말! 아니야!</t>
+        </is>
+      </c>
+      <c r="C355" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="D355" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E355" s="6" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F355" s="6" t="inlineStr"/>
+      <c r="G355" s="6" t="inlineStr">
+        <is>
+          <t>김태오!! 그건 내 말이야!!</t>
+        </is>
+      </c>
+      <c r="H355" s="6" t="inlineStr">
+        <is>
+          <t>도망!</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B356" s="4" t="inlineStr">
+        <is>
+          <t>거짓말! 아니야!</t>
+        </is>
+      </c>
+      <c r="C356" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="D356" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E356" s="4" t="inlineStr"/>
+      <c r="F356" s="4" t="inlineStr">
+        <is>
+          <t>“아니야” 뒤에 숨은 마음을, / 이제 우리 집은 함께 찾아낸다.</t>
+        </is>
+      </c>
+      <c r="G356" s="4" t="inlineStr"/>
+      <c r="H356" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:H338"/>
+  <autoFilter ref="A3:H356"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -13264,7 +13871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -13699,13 +14306,13 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>맛있는데 지금은 먹기 싫어.</t>
+          <t>거짓말! 아니야!</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr"/>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>누가 음식을 권하면</t>
+          <t>기분 나쁘거나 하기 싫을 때</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr"/>
@@ -13721,13 +14328,13 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>치즈 냄새 극혐!</t>
+          <t>맛있는데 지금은 먹기 싫어.</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr"/>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>치즈만 보면 (냄새는 더더욱)</t>
+          <t>누가 음식을 권하면</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr"/>
@@ -13743,13 +14350,13 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>김태오!</t>
+          <t>치즈 냄새 극혐!</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr"/>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+          <t>치즈만 보면 (냄새는 더더욱)</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr"/>
@@ -13760,22 +14367,18 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>짐방</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>김서방</t>
-        </is>
-      </c>
+          <t>김태오!</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr"/>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr"/>
@@ -13791,17 +14394,17 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>꿍끙이</t>
+          <t>짐방</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>뿡뿡이</t>
+          <t>김서방</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr"/>
@@ -13810,10 +14413,26 @@
       <c r="A26" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="B26" s="4" t="inlineStr"/>
-      <c r="C26" s="4" t="inlineStr"/>
-      <c r="D26" s="4" t="inlineStr"/>
-      <c r="E26" s="4" t="inlineStr"/>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>꿍끙이</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>뿡뿡이</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+        </is>
+      </c>
       <c r="F26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
@@ -13956,8 +14575,18 @@
       <c r="E40" s="4" t="inlineStr"/>
       <c r="F40" s="4" t="inlineStr"/>
     </row>
+    <row r="41">
+      <c r="A41" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" s="6" t="inlineStr"/>
+      <c r="C41" s="6" t="inlineStr"/>
+      <c r="D41" s="6" t="inlineStr"/>
+      <c r="E41" s="6" t="inlineStr"/>
+      <c r="F41" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F40"/>
+  <autoFilter ref="A3:F41"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Fix episode 20 to match Jaei and Taeo, add episode 21
The family corrected the water fear: Jaei learned to dive and does not
mind water in her eyes, while Taeo is terrified of it. He also hates
brushing his teeth most, runs away, crawls along the floor and makes
Mom and Dad struggle morning and evening.

Episode 20 is rewritten: Jaei's "거짓말! 아니야!" now hides that she
wants to finish her drawing (Mom gives her ten more minutes), and in
the bathroom Jaei shows off her diving and holds Taeo's hand while Dad
covers his eyes with a towel and Taeo smells his lemon. Episode 21
"이 닦기 대작전": Taeo flees at 7:30 a.m. and again at 8:30 p.m.,
crawling under the sofa and table, until Dad turns brushing into the
game of beating Thanos hiding in his teeth. Bios and sayings updated;
new crawling Taeo and toothbrush props. Excel updated. Cache v180.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$356</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$374</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$44</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -551,7 +551,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>“아니야!”가 입버릇인 누나. 방은 늘 반듯하게 정리해 두고, 학교 숙제는 미리 다 해 놓고 노는 게 좋아요. 음식을 권하면 “맛있는데 지금은 먹기 싫어.” 치즈는 싫고 치즈 냄새는 극혐! 티니핑, 위시캣, 그리고 스파이더맨·판타스틱 4·어벤져스 같은 마블 영웅은 태오랑 둘 다 좋아해요. 동생이 괴롭혀도 참고 또 참다가, 폭발하면… “김태오!” 엉덩이 찰싹! 기분 나쁘거나 하기 싫을 때는 “거짓말! 아니야!”</t>
+          <t>“아니야!”가 입버릇인 누나. 방은 늘 반듯하게 정리해 두고, 학교 숙제는 미리 다 해 놓고 노는 게 좋아요. 음식을 권하면 “맛있는데 지금은 먹기 싫어.” 치즈는 싫고 치즈 냄새는 극혐! 티니핑, 위시캣, 그리고 스파이더맨·판타스틱 4·어벤져스 같은 마블 영웅은 태오랑 둘 다 좋아해요. 동생이 괴롭혀도 참고 또 참다가, 폭발하면… “김태오!” 엉덩이 찰싹! 기분 나쁘거나 하기 싫을 때는 “거짓말! 아니야!” 잠수를 배워서 물이 눈에 들어가도 끄떡없어요.</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>반쪽 레몬을 늘 손에 들고 다니며 할짝할짝 핥아 먹는 막내(레몬·자두·파인애플처럼 신 과일이 제일 좋아요). 누나 괴롭히기가 취미인 막내(사실은 누나가 좋아서). 혼자 노는 것 같아도 가족 말을 다 듣고 있고, 틀려도 일단 소리 지르며 우기다가 들키면 머리를 긁적긁적. “맛있는 거 죠!”가 입버릇이고, 누나랑 같이 좋아하는 마블 영웅(스파이더맨, 판타스틱 4, 어벤져스)도 태오식으로 불러요(블루베리, 쉬터맨, 스테잌로저…). 블랙 위도우랑 수가 제일 예쁘대요. 제일 좋아하는 놀이는 어벤져스로 타노스랑 싸우기! 모든 호칭은 태오 기준이라, 누가 “재이야” 하면 “재이 누나야!” 하고 고쳐 줘요. 요즘은 화가 나면 뾰족한 말이 튀어나오지만, “나 화났어!” 주문을 연습 중이에요.</t>
+          <t>반쪽 레몬을 늘 손에 들고 다니며 할짝할짝 핥아 먹는 막내(레몬·자두·파인애플처럼 신 과일이 제일 좋아요). 누나 괴롭히기가 취미인 막내(사실은 누나가 좋아서). 혼자 노는 것 같아도 가족 말을 다 듣고 있고, 틀려도 일단 소리 지르며 우기다가 들키면 머리를 긁적긁적. “맛있는 거 죠!”가 입버릇이고, 누나랑 같이 좋아하는 마블 영웅(스파이더맨, 판타스틱 4, 어벤져스)도 태오식으로 불러요(블루베리, 쉬터맨, 스테잌로저…). 블랙 위도우랑 수가 제일 예쁘대요. 제일 좋아하는 놀이는 어벤져스로 타노스랑 싸우기! 모든 호칭은 태오 기준이라, 누가 “재이야” 하면 “재이 누나야!” 하고 고쳐 줘요. 요즘은 화가 나면 뾰족한 말이 튀어나오지만, “나 화났어!” 주문을 연습 중이에요. 물이 눈에 들어가는 걸 엄청 무서워하고, 이 닦기를 제일 싫어해서 아침저녁으로 도망 다니고 바닥을 기어 다니며 엄마 아빠를 고생시켜요.</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>“머리 감을 시간이야.” “거짓말! 아니야!” 재이 누나가 기분 나쁘거나 하기 싫을 때 꺼내는 말. 그 뒤에 숨은 진짜 마음은 뭐였을까?</t>
+          <t>“씻을 시간이야.” “거짓말! 아니야!” 재이 누나가 하기 싫을 때 꺼내는 말. 그리고 물이 눈에 들어가는 게 세상에서 제일 무서운 태오.</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -1727,26 +1727,26 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>“머리 감을 시간이야.” “거짓말! 아니야!” “시계가 거짓말이야!” / 태오도 “거짓말! 아니야!” 따라 하고 “이거 내 말이야!” / 마지막엔 태오가 누나 말을 도로 가져가 “김태오!”</t>
+          <t>“씻을 시간이야.” “거짓말! 아니야!” “시계가 거짓말이야!” (그림을 더 그리고 싶어서) / 물이 눈에 들어갈까 봐 부르르 떠는 태오도 “거짓말! 아니야! 안 무서워!!” / 마지막엔 “김태오!! 그건 내 말이야!!”</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>‘아니야’ 뒤에 숨은 마음: 눈에 물 들어가는 게 무서워 / 엄마 ‘말해 줘서 고마워’, 아빠 수건으로 눈 가리기, 태오 레몬 냄새 응원</t>
+          <t>‘아니야’ 뒤에 숨은 마음을 말하는 재이 / 잠수를 배운 누나가 “태오도 할 수 있어. 누나가 손 잡아 줄게.” / 수건 + 레몬 냄새 + 누나 손으로 “조금은 안 무서웠어!”</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>“아니야” 뒤에는 마음이 숨어 있어요. 이유를 말하면 가족이 도와줄 수 있어요.</t>
+          <t>“아니야” 뒤에는 마음이 숨어 있어요. 무서운 건 사람마다 달라서, 잘하는 사람이 손을 잡아 주면 돼요.</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>나는 하기 싫을 때 어떤 말을 하나요? 그 말 뒤에는 어떤 마음이 숨어 있을까요?</t>
+          <t>나는 하기 싫을 때 어떤 말을 하나요? 무서운 걸 도와준 가족이 있나요?</t>
         </is>
       </c>
       <c r="I23" s="5" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
@@ -1755,20 +1755,50 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="n">
+      <c r="A24" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="7" t="n"/>
-      <c r="C24" s="7" t="n"/>
-      <c r="D24" s="7" t="n"/>
-      <c r="E24" s="7" t="n"/>
-      <c r="F24" s="7" t="n"/>
-      <c r="G24" s="7" t="n"/>
-      <c r="H24" s="7" t="n"/>
-      <c r="I24" s="7" t="n"/>
-      <c r="J24" s="7" t="inlineStr">
-        <is>
-          <t>기획 중</t>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>이 닦기 대작전</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>아침에도 도망, 저녁에도 도망. 바닥을 기어서라도 이 닦기는 싫은 태오. 오늘도 엄마 아빠의 대작전이 시작됐다.</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>재이, 엄마, 아빠, 태오</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>아침 7시 30분 “이 안 닦아! 싫어!!” 도망, 식탁·소파 밑을 기어서 숨기 / 저녁에도 또 도망 → 엄마 아빠 판다 눈 / “나와라 타노스! 어벤져스 칫솔!” → 아빠 “거품 공격에 졌다!” / 다음 날 아침 또 도망</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>“누나는 누나니까!”라던 태오가 타노스 놀이로 이를 다 닦는다 / 그래도 엄마 아빠는 아침에도, 저녁에도 오늘도 타노스가 된다</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>싫은 일도 놀이가 되면 할 수 있어요. 함께 웃으며 하면 더 쉬워져요.</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>우리 집에서 제일 하기 싫은 일은 뭐예요? 놀이로 바꾸면 어떻게 될까요?</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>완성</t>
         </is>
       </c>
     </row>
@@ -1808,13 +1838,31 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="7" t="n"/>
+      <c r="C27" s="7" t="n"/>
+      <c r="D27" s="7" t="n"/>
+      <c r="E27" s="7" t="n"/>
+      <c r="F27" s="7" t="n"/>
+      <c r="G27" s="7" t="n"/>
+      <c r="H27" s="7" t="n"/>
+      <c r="I27" s="7" t="n"/>
+      <c r="J27" s="7" t="inlineStr">
+        <is>
+          <t>기획 중</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:J23"/>
+  <autoFilter ref="A3:J24"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"아이디어,기획 중,콘티,완성"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1828,7 +1876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H356"/>
+  <dimension ref="A1:H374"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -12584,7 +12632,7 @@
       </c>
       <c r="D339" s="6" t="inlineStr">
         <is>
-          <t>거실(밤)</t>
+          <t>방</t>
         </is>
       </c>
       <c r="E339" s="6" t="inlineStr">
@@ -12594,12 +12642,12 @@
       </c>
       <c r="F339" s="6" t="inlineStr">
         <is>
-          <t>저녁 8시.</t>
+          <t>저녁 8시. 재이 누나는 그림 그리기에 푹 빠졌다.</t>
         </is>
       </c>
       <c r="G339" s="6" t="inlineStr">
         <is>
-          <t>재이야, 머리 감을 시간이야.</t>
+          <t>재이야, 씻을 시간이야.</t>
         </is>
       </c>
       <c r="H339" s="6" t="inlineStr"/>
@@ -12679,18 +12727,18 @@
       </c>
       <c r="D342" s="4" t="inlineStr">
         <is>
-          <t>부엌</t>
+          <t>효과: 반짝</t>
         </is>
       </c>
       <c r="E342" s="4" t="inlineStr">
         <is>
-          <t>아빠, 태오</t>
+          <t>엄마</t>
         </is>
       </c>
       <c r="F342" s="4" t="inlineStr"/>
       <c r="G342" s="4" t="inlineStr">
         <is>
-          <t>태오야, 이 닦자~</t>
+          <t>재이야, ‘거짓말! 아니야!’ 뒤에 뭐가 숨어 있는지 말해 줄 수 있어?</t>
         </is>
       </c>
       <c r="H342" s="4" t="inlineStr"/>
@@ -12709,18 +12757,18 @@
       </c>
       <c r="D343" s="6" t="inlineStr">
         <is>
-          <t>효과: 집중선</t>
+          <t>효과: 반짝</t>
         </is>
       </c>
       <c r="E343" s="6" t="inlineStr">
         <is>
-          <t>태오</t>
+          <t>재이</t>
         </is>
       </c>
       <c r="F343" s="6" t="inlineStr"/>
       <c r="G343" s="6" t="inlineStr">
         <is>
-          <t>거짓말! 아니야!!</t>
+          <t>(속삭임) …그림을 아직 다 못 그렸어. 조금만 더 그리고 싶어.</t>
         </is>
       </c>
       <c r="H343" s="6" t="inlineStr"/>
@@ -12739,19 +12787,18 @@
       </c>
       <c r="D344" s="4" t="inlineStr">
         <is>
-          <t>부엌</t>
+          <t>방</t>
         </is>
       </c>
       <c r="E344" s="4" t="inlineStr">
         <is>
-          <t>아빠, 태오</t>
+          <t>엄마, 재이</t>
         </is>
       </c>
       <c r="F344" s="4" t="inlineStr"/>
       <c r="G344" s="4" t="inlineStr">
         <is>
-          <t>누나 따라 하지 마~
-따라 아니야! 이거 내 말이야!</t>
+          <t>그랬구나. 10분만 더 그리고 씻자. 말해 줘서 고마워.</t>
         </is>
       </c>
       <c r="H344" s="4" t="inlineStr"/>
@@ -12770,25 +12817,29 @@
       </c>
       <c r="D345" s="6" t="inlineStr">
         <is>
-          <t>거실(밤)</t>
+          <t>bath</t>
         </is>
       </c>
       <c r="E345" s="6" t="inlineStr">
         <is>
-          <t>재이</t>
+          <t>태오, 아빠</t>
         </is>
       </c>
       <c r="F345" s="6" t="inlineStr">
         <is>
-          <t>하지만 재이 누나는 알고 있었다.</t>
+          <t>그리고 욕실. 태오는 벌써 부르르 떨고 있다.</t>
         </is>
       </c>
       <c r="G345" s="6" t="inlineStr">
         <is>
-          <t>(생각) (사실은 내 말이 맞는데…)</t>
-        </is>
-      </c>
-      <c r="H345" s="6" t="inlineStr"/>
+          <t>머리 감는 거 싫어! 눈에 물 들어가!</t>
+        </is>
+      </c>
+      <c r="H345" s="6" t="inlineStr">
+        <is>
+          <t>부들부들</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" s="3" t="n">
@@ -12804,18 +12855,18 @@
       </c>
       <c r="D346" s="4" t="inlineStr">
         <is>
-          <t>거실(밤)</t>
+          <t>효과: 집중선</t>
         </is>
       </c>
       <c r="E346" s="4" t="inlineStr">
         <is>
-          <t>엄마, 재이</t>
+          <t>태오</t>
         </is>
       </c>
       <c r="F346" s="4" t="inlineStr"/>
       <c r="G346" s="4" t="inlineStr">
         <is>
-          <t>재이가 하기 싫을 때 ‘거짓말! 아니야!’ 하는 거, 엄마 알아.</t>
+          <t>거짓말! 아니야! 안 무서워!!</t>
         </is>
       </c>
       <c r="H346" s="4" t="inlineStr"/>
@@ -12834,18 +12885,18 @@
       </c>
       <c r="D347" s="6" t="inlineStr">
         <is>
-          <t>효과: 반짝</t>
+          <t>bath</t>
         </is>
       </c>
       <c r="E347" s="6" t="inlineStr">
         <is>
-          <t>엄마</t>
+          <t>재이, 태오</t>
         </is>
       </c>
       <c r="F347" s="6" t="inlineStr"/>
       <c r="G347" s="6" t="inlineStr">
         <is>
-          <t>그 말 뒤에 뭐가 숨어 있는지 말해 줄 수 있어?</t>
+          <t>누나는 잠수도 배웠잖아. 눈에 물 들어가도 괜찮아. 봐 봐!</t>
         </is>
       </c>
       <c r="H347" s="6" t="inlineStr"/>
@@ -12864,7 +12915,7 @@
       </c>
       <c r="D348" s="4" t="inlineStr">
         <is>
-          <t>효과: 반짝</t>
+          <t>bath</t>
         </is>
       </c>
       <c r="E348" s="4" t="inlineStr">
@@ -12875,10 +12926,14 @@
       <c r="F348" s="4" t="inlineStr"/>
       <c r="G348" s="4" t="inlineStr">
         <is>
-          <t>(속삭임) …머리 헹굴 때 눈에 물 들어가는 게 무서워.</t>
-        </is>
-      </c>
-      <c r="H348" s="4" t="inlineStr"/>
+          <t>후~ 하나, 둘, 셋… 풍덩!</t>
+        </is>
+      </c>
+      <c r="H348" s="4" t="inlineStr">
+        <is>
+          <t>풍덩!</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" s="5" t="n">
@@ -12899,13 +12954,13 @@
       </c>
       <c r="E349" s="6" t="inlineStr">
         <is>
-          <t>엄마</t>
+          <t>태오</t>
         </is>
       </c>
       <c r="F349" s="6" t="inlineStr"/>
       <c r="G349" s="6" t="inlineStr">
         <is>
-          <t>아, 그래서 그랬구나. 말해 줘서 고마워. 같이 방법을 찾아보자.</t>
+          <t>누나 대단해…!</t>
         </is>
       </c>
       <c r="H349" s="6" t="inlineStr"/>
@@ -12929,13 +12984,13 @@
       </c>
       <c r="E350" s="4" t="inlineStr">
         <is>
-          <t>재이, 아빠, 태오</t>
+          <t>재이, 태오</t>
         </is>
       </c>
       <c r="F350" s="4" t="inlineStr"/>
       <c r="G350" s="4" t="inlineStr">
         <is>
-          <t>아빠가 수건으로 눈 가려 줄게. 절대 안 들어가!</t>
+          <t>태오도 할 수 있어. 누나가 손 잡아 줄게.</t>
         </is>
       </c>
       <c r="H350" s="4" t="inlineStr"/>
@@ -12959,16 +13014,20 @@
       </c>
       <c r="E351" s="6" t="inlineStr">
         <is>
-          <t>태오, 재이</t>
+          <t>아빠, 태오, 재이</t>
         </is>
       </c>
       <c r="F351" s="6" t="inlineStr"/>
       <c r="G351" s="6" t="inlineStr">
         <is>
-          <t>누나! 내 레몬 냄새 맡아 봐. 무서운 거 다 없어져!</t>
-        </is>
-      </c>
-      <c r="H351" s="6" t="inlineStr"/>
+          <t>수건으로 눈 가려 줄게. 절대 안 들어가!</t>
+        </is>
+      </c>
+      <c r="H351" s="6" t="inlineStr">
+        <is>
+          <t>꼬옥</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" s="3" t="n">
@@ -12984,25 +13043,21 @@
       </c>
       <c r="D352" s="4" t="inlineStr">
         <is>
-          <t>bath</t>
+          <t>효과: 반짝</t>
         </is>
       </c>
       <c r="E352" s="4" t="inlineStr">
         <is>
-          <t>재이</t>
+          <t>태오</t>
         </is>
       </c>
       <c r="F352" s="4" t="inlineStr"/>
       <c r="G352" s="4" t="inlineStr">
         <is>
-          <t>하나, 둘, 셋… 후~</t>
-        </is>
-      </c>
-      <c r="H352" s="4" t="inlineStr">
-        <is>
-          <t>쏴아~</t>
-        </is>
-      </c>
+          <t>…어? 조금은 안 무서웠어!</t>
+        </is>
+      </c>
+      <c r="H352" s="4" t="inlineStr"/>
     </row>
     <row r="353">
       <c r="A353" s="5" t="n">
@@ -13018,18 +13073,23 @@
       </c>
       <c r="D353" s="6" t="inlineStr">
         <is>
-          <t>효과: 반짝</t>
+          <t>거실(밤)</t>
         </is>
       </c>
       <c r="E353" s="6" t="inlineStr">
         <is>
-          <t>재이</t>
-        </is>
-      </c>
-      <c r="F353" s="6" t="inlineStr"/>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F353" s="6" t="inlineStr">
+        <is>
+          <t>그날 밤.</t>
+        </is>
+      </c>
       <c r="G353" s="6" t="inlineStr">
         <is>
-          <t>…어? 안 무서웠어!</t>
+          <t>이제 자야지~
+거짓말! 아니야!</t>
         </is>
       </c>
       <c r="H353" s="6" t="inlineStr"/>
@@ -13048,26 +13108,25 @@
       </c>
       <c r="D354" s="4" t="inlineStr">
         <is>
-          <t>거실(밤)</t>
+          <t>효과: 집중선</t>
         </is>
       </c>
       <c r="E354" s="4" t="inlineStr">
         <is>
-          <t>재이, 태오</t>
-        </is>
-      </c>
-      <c r="F354" s="4" t="inlineStr">
-        <is>
-          <t>그날 밤.</t>
-        </is>
-      </c>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F354" s="4" t="inlineStr"/>
       <c r="G354" s="4" t="inlineStr">
         <is>
-          <t>진짜야! 하나도 안 무서웠어!
-거짓말! 아니야!</t>
-        </is>
-      </c>
-      <c r="H354" s="4" t="inlineStr"/>
+          <t>김태오!! 그건 내 말이야!!</t>
+        </is>
+      </c>
+      <c r="H354" s="4" t="inlineStr">
+        <is>
+          <t>도망!</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" s="5" t="n">
@@ -13083,54 +13142,621 @@
       </c>
       <c r="D355" s="6" t="inlineStr">
         <is>
-          <t>효과: 집중선</t>
-        </is>
-      </c>
-      <c r="E355" s="6" t="inlineStr">
-        <is>
-          <t>재이</t>
-        </is>
-      </c>
-      <c r="F355" s="6" t="inlineStr"/>
-      <c r="G355" s="6" t="inlineStr">
-        <is>
-          <t>김태오!! 그건 내 말이야!!</t>
-        </is>
-      </c>
-      <c r="H355" s="6" t="inlineStr">
-        <is>
-          <t>도망!</t>
-        </is>
-      </c>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E355" s="6" t="inlineStr"/>
+      <c r="F355" s="6" t="inlineStr">
+        <is>
+          <t>무서운 건 사람마다 다르지만, / 손을 잡아 줄 누나는 하나뿐이다.</t>
+        </is>
+      </c>
+      <c r="G355" s="6" t="inlineStr"/>
+      <c r="H355" s="6" t="inlineStr"/>
     </row>
     <row r="356">
       <c r="A356" s="3" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B356" s="4" t="inlineStr">
         <is>
-          <t>거짓말! 아니야!</t>
+          <t>이 닦기 대작전</t>
         </is>
       </c>
       <c r="C356" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D356" s="4" t="inlineStr">
+        <is>
+          <t>부엌</t>
+        </is>
+      </c>
+      <c r="E356" s="4" t="inlineStr">
+        <is>
+          <t>아빠, 태오</t>
+        </is>
+      </c>
+      <c r="F356" s="4" t="inlineStr">
+        <is>
+          <t>아침 7시 30분.</t>
+        </is>
+      </c>
+      <c r="G356" s="4" t="inlineStr">
+        <is>
+          <t>태오야, 이 닦자~</t>
+        </is>
+      </c>
+      <c r="H356" s="4" t="inlineStr"/>
+    </row>
+    <row r="357">
+      <c r="A357" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B357" s="6" t="inlineStr">
+        <is>
+          <t>이 닦기 대작전</t>
+        </is>
+      </c>
+      <c r="C357" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D357" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E357" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F357" s="6" t="inlineStr"/>
+      <c r="G357" s="6" t="inlineStr">
+        <is>
+          <t>이 안 닦아! 싫어!!</t>
+        </is>
+      </c>
+      <c r="H357" s="6" t="inlineStr"/>
+    </row>
+    <row r="358">
+      <c r="A358" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B358" s="4" t="inlineStr">
+        <is>
+          <t>이 닦기 대작전</t>
+        </is>
+      </c>
+      <c r="C358" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D358" s="4" t="inlineStr">
+        <is>
+          <t>효과: 속도선</t>
+        </is>
+      </c>
+      <c r="E358" s="4" t="inlineStr">
+        <is>
+          <t>태오, 아빠</t>
+        </is>
+      </c>
+      <c r="F358" s="4" t="inlineStr"/>
+      <c r="G358" s="4" t="inlineStr">
+        <is>
+          <t>태오야 거기 서!</t>
+        </is>
+      </c>
+      <c r="H358" s="4" t="inlineStr">
+        <is>
+          <t>다다다다</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B359" s="6" t="inlineStr">
+        <is>
+          <t>이 닦기 대작전</t>
+        </is>
+      </c>
+      <c r="C359" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D359" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E359" s="6" t="inlineStr"/>
+      <c r="F359" s="6" t="inlineStr"/>
+      <c r="G359" s="6" t="inlineStr">
+        <is>
+          <t>(생각) (여기 숨으면 못 찾겠지…)</t>
+        </is>
+      </c>
+      <c r="H359" s="6" t="inlineStr">
+        <is>
+          <t>슬금슬금</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B360" s="4" t="inlineStr">
+        <is>
+          <t>이 닦기 대작전</t>
+        </is>
+      </c>
+      <c r="C360" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D360" s="4" t="inlineStr">
+        <is>
+          <t>부엌</t>
+        </is>
+      </c>
+      <c r="E360" s="4" t="inlineStr">
+        <is>
+          <t>엄마, 아빠</t>
+        </is>
+      </c>
+      <c r="F360" s="4" t="inlineStr"/>
+      <c r="G360" s="4" t="inlineStr">
+        <is>
+          <t>어디 갔지?
+…바닥에 발자국이 없는데?</t>
+        </is>
+      </c>
+      <c r="H360" s="4" t="inlineStr"/>
+    </row>
+    <row r="361">
+      <c r="A361" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B361" s="6" t="inlineStr">
+        <is>
+          <t>이 닦기 대작전</t>
+        </is>
+      </c>
+      <c r="C361" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D361" s="6" t="inlineStr">
+        <is>
+          <t>부엌</t>
+        </is>
+      </c>
+      <c r="E361" s="6" t="inlineStr"/>
+      <c r="F361" s="6" t="inlineStr"/>
+      <c r="G361" s="6" t="inlineStr">
+        <is>
+          <t>(속삭임) 헤헤…</t>
+        </is>
+      </c>
+      <c r="H361" s="6" t="inlineStr">
+        <is>
+          <t>기어기어</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B362" s="4" t="inlineStr">
+        <is>
+          <t>이 닦기 대작전</t>
+        </is>
+      </c>
+      <c r="C362" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D362" s="4" t="inlineStr">
+        <is>
+          <t>부엌</t>
+        </is>
+      </c>
+      <c r="E362" s="4" t="inlineStr">
+        <is>
+          <t>엄마, 아빠</t>
+        </is>
+      </c>
+      <c r="F362" s="4" t="inlineStr"/>
+      <c r="G362" s="4" t="inlineStr">
+        <is>
+          <t>잡았다! 식탁 밑에 파란 옷이 보이네~</t>
+        </is>
+      </c>
+      <c r="H362" s="4" t="inlineStr"/>
+    </row>
+    <row r="363">
+      <c r="A363" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B363" s="6" t="inlineStr">
+        <is>
+          <t>이 닦기 대작전</t>
+        </is>
+      </c>
+      <c r="C363" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D363" s="6" t="inlineStr">
+        <is>
+          <t>효과: 어두움</t>
+        </is>
+      </c>
+      <c r="E363" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F363" s="6" t="inlineStr"/>
+      <c r="G363" s="6" t="inlineStr">
+        <is>
+          <t>이 닦기 싫어어어~!</t>
+        </is>
+      </c>
+      <c r="H363" s="6" t="inlineStr"/>
+    </row>
+    <row r="364">
+      <c r="A364" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B364" s="4" t="inlineStr">
+        <is>
+          <t>이 닦기 대작전</t>
+        </is>
+      </c>
+      <c r="C364" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D364" s="4" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E364" s="4" t="inlineStr">
+        <is>
+          <t>엄마, 아빠</t>
+        </is>
+      </c>
+      <c r="F364" s="4" t="inlineStr">
+        <is>
+          <t>저녁 8시 30분. 어제도, 오늘도.</t>
+        </is>
+      </c>
+      <c r="G364" s="4" t="inlineStr">
+        <is>
+          <t>(속삭임) 아침에도 했는데…
+(속삭임) …또 도망갔다.</t>
+        </is>
+      </c>
+      <c r="H364" s="4" t="inlineStr">
+        <is>
+          <t>판다 눈</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B365" s="6" t="inlineStr">
+        <is>
+          <t>이 닦기 대작전</t>
+        </is>
+      </c>
+      <c r="C365" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D365" s="6" t="inlineStr">
+        <is>
+          <t>bath</t>
+        </is>
+      </c>
+      <c r="E365" s="6" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F365" s="6" t="inlineStr"/>
+      <c r="G365" s="6" t="inlineStr">
+        <is>
+          <t>누나는 혼자 닦아. 태오도 할 수 있어.</t>
+        </is>
+      </c>
+      <c r="H365" s="6" t="inlineStr"/>
+    </row>
+    <row r="366">
+      <c r="A366" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B366" s="4" t="inlineStr">
+        <is>
+          <t>이 닦기 대작전</t>
+        </is>
+      </c>
+      <c r="C366" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D366" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E366" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F366" s="4" t="inlineStr"/>
+      <c r="G366" s="4" t="inlineStr">
+        <is>
+          <t>누나는 누나니까!</t>
+        </is>
+      </c>
+      <c r="H366" s="4" t="inlineStr"/>
+    </row>
+    <row r="367">
+      <c r="A367" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B367" s="6" t="inlineStr">
+        <is>
+          <t>이 닦기 대작전</t>
+        </is>
+      </c>
+      <c r="C367" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D367" s="6" t="inlineStr">
+        <is>
+          <t>bath</t>
+        </is>
+      </c>
+      <c r="E367" s="6" t="inlineStr">
+        <is>
+          <t>아빠, 태오</t>
+        </is>
+      </c>
+      <c r="F367" s="6" t="inlineStr"/>
+      <c r="G367" s="6" t="inlineStr">
+        <is>
+          <t>어? 태오 이빨 속에 타노스가 숨어 있는데?</t>
+        </is>
+      </c>
+      <c r="H367" s="6" t="inlineStr"/>
+    </row>
+    <row r="368">
+      <c r="A368" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B368" s="4" t="inlineStr">
+        <is>
+          <t>이 닦기 대작전</t>
+        </is>
+      </c>
+      <c r="C368" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="D368" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E368" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F368" s="4" t="inlineStr"/>
+      <c r="G368" s="4" t="inlineStr">
+        <is>
+          <t>진짜?! 타노스?!</t>
+        </is>
+      </c>
+      <c r="H368" s="4" t="inlineStr"/>
+    </row>
+    <row r="369">
+      <c r="A369" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B369" s="6" t="inlineStr">
+        <is>
+          <t>이 닦기 대작전</t>
+        </is>
+      </c>
+      <c r="C369" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="D369" s="6" t="inlineStr">
+        <is>
+          <t>bath</t>
+        </is>
+      </c>
+      <c r="E369" s="6" t="inlineStr">
+        <is>
+          <t>태오, 아빠</t>
+        </is>
+      </c>
+      <c r="F369" s="6" t="inlineStr"/>
+      <c r="G369" s="6" t="inlineStr">
+        <is>
+          <t>나와라 타노스! 어벤져스 칫솔 받아라!</t>
+        </is>
+      </c>
+      <c r="H369" s="6" t="inlineStr">
+        <is>
+          <t>쓱싹쓱싹</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B370" s="4" t="inlineStr">
+        <is>
+          <t>이 닦기 대작전</t>
+        </is>
+      </c>
+      <c r="C370" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="D370" s="4" t="inlineStr">
+        <is>
+          <t>bath</t>
+        </is>
+      </c>
+      <c r="E370" s="4" t="inlineStr">
+        <is>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F370" s="4" t="inlineStr"/>
+      <c r="G370" s="4" t="inlineStr">
+        <is>
+          <t>으악! 거품 공격에 졌다!</t>
+        </is>
+      </c>
+      <c r="H370" s="4" t="inlineStr">
+        <is>
+          <t>보글보글</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B371" s="6" t="inlineStr">
+        <is>
+          <t>이 닦기 대작전</t>
+        </is>
+      </c>
+      <c r="C371" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="D371" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E371" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F371" s="6" t="inlineStr"/>
+      <c r="G371" s="6" t="inlineStr">
+        <is>
+          <t>나 이 다 닦았다! 나 잘해!</t>
+        </is>
+      </c>
+      <c r="H371" s="6" t="inlineStr"/>
+    </row>
+    <row r="372">
+      <c r="A372" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B372" s="4" t="inlineStr">
+        <is>
+          <t>이 닦기 대작전</t>
+        </is>
+      </c>
+      <c r="C372" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="D372" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E372" s="4" t="inlineStr">
+        <is>
+          <t>엄마, 아빠</t>
+        </is>
+      </c>
+      <c r="F372" s="4" t="inlineStr">
+        <is>
+          <t>다음 날 아침.</t>
+        </is>
+      </c>
+      <c r="G372" s="4" t="inlineStr">
+        <is>
+          <t>오늘은 한 번에 되려나?
+태오야, 이 닦자~</t>
+        </is>
+      </c>
+      <c r="H372" s="4" t="inlineStr"/>
+    </row>
+    <row r="373">
+      <c r="A373" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B373" s="6" t="inlineStr">
+        <is>
+          <t>이 닦기 대작전</t>
+        </is>
+      </c>
+      <c r="C373" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="D356" s="4" t="inlineStr">
+      <c r="D373" s="6" t="inlineStr">
+        <is>
+          <t>효과: 속도선</t>
+        </is>
+      </c>
+      <c r="E373" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F373" s="6" t="inlineStr"/>
+      <c r="G373" s="6" t="inlineStr">
+        <is>
+          <t>이 안 닦아! 싫어~!</t>
+        </is>
+      </c>
+      <c r="H373" s="6" t="inlineStr">
+        <is>
+          <t>다다다</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B374" s="4" t="inlineStr">
+        <is>
+          <t>이 닦기 대작전</t>
+        </is>
+      </c>
+      <c r="C374" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="D374" s="4" t="inlineStr">
         <is>
           <t>효과: 반짝</t>
         </is>
       </c>
-      <c r="E356" s="4" t="inlineStr"/>
-      <c r="F356" s="4" t="inlineStr">
-        <is>
-          <t>“아니야” 뒤에 숨은 마음을, / 이제 우리 집은 함께 찾아낸다.</t>
-        </is>
-      </c>
-      <c r="G356" s="4" t="inlineStr"/>
-      <c r="H356" s="4" t="inlineStr"/>
+      <c r="E374" s="4" t="inlineStr"/>
+      <c r="F374" s="4" t="inlineStr">
+        <is>
+          <t>그래도 엄마 아빠는 오늘도 타노스가 된다. / 아침에도, 저녁에도.</t>
+        </is>
+      </c>
+      <c r="G374" s="4" t="inlineStr"/>
+      <c r="H374" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:H356"/>
+  <autoFilter ref="A3:H374"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -13871,7 +14497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -14240,13 +14866,13 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>엄마 인누와~</t>
+          <t>이 안 닦아! 싫어!</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr"/>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>밤에 자다 깨서 (엄마가 옆에서 재워 줄 때까지)</t>
+          <t>아침저녁 이 닦을 때 (도망 다니고 바닥을 기어요)</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr"/>
@@ -14262,13 +14888,13 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>왜 놀려! 놀리지 마!</t>
+          <t>누나 대단해!</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr"/>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>“태오는 글씨·숫자 잘 몰라” 소리를 들으면 (손가락질하며)</t>
+          <t>누나가 잠수를 보여 줬을 때</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr"/>
@@ -14279,18 +14905,18 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>아니야!</t>
+          <t>엄마 인누와~</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr"/>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>하루에도 제일 많이 하는 말</t>
+          <t>밤에 자다 깨서 (엄마가 옆에서 재워 줄 때까지)</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr"/>
@@ -14301,18 +14927,18 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>거짓말! 아니야!</t>
+          <t>왜 놀려! 놀리지 마!</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr"/>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>기분 나쁘거나 하기 싫을 때</t>
+          <t>“태오는 글씨·숫자 잘 몰라” 소리를 들으면 (손가락질하며)</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr"/>
@@ -14328,13 +14954,13 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>맛있는데 지금은 먹기 싫어.</t>
+          <t>아니야!</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr"/>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>누가 음식을 권하면</t>
+          <t>하루에도 제일 많이 하는 말</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr"/>
@@ -14350,13 +14976,13 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>치즈 냄새 극혐!</t>
+          <t>거짓말! 아니야!</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr"/>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>치즈만 보면 (냄새는 더더욱)</t>
+          <t>기분 나쁘거나 하기 싫을 때</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr"/>
@@ -14372,13 +14998,13 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>김태오!</t>
+          <t>맛있는데 지금은 먹기 싫어.</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr"/>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+          <t>누가 음식을 권하면</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr"/>
@@ -14389,22 +15015,18 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>짐방</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>김서방</t>
-        </is>
-      </c>
+          <t>치즈 냄새 극혐!</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr"/>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+          <t>치즈만 보면 (냄새는 더더욱)</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr"/>
@@ -14415,22 +15037,18 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>꿍끙이</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>뿡뿡이</t>
-        </is>
-      </c>
+          <t>김태오!</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr"/>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr"/>
@@ -14439,20 +15057,52 @@
       <c r="A27" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="B27" s="6" t="inlineStr"/>
-      <c r="C27" s="6" t="inlineStr"/>
-      <c r="D27" s="6" t="inlineStr"/>
-      <c r="E27" s="6" t="inlineStr"/>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>짐방</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>김서방</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+        </is>
+      </c>
       <c r="F27" s="6" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="B28" s="4" t="inlineStr"/>
-      <c r="C28" s="4" t="inlineStr"/>
-      <c r="D28" s="4" t="inlineStr"/>
-      <c r="E28" s="4" t="inlineStr"/>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>꿍끙이</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>뿡뿡이</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+        </is>
+      </c>
       <c r="F28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
@@ -14585,8 +15235,28 @@
       <c r="E41" s="6" t="inlineStr"/>
       <c r="F41" s="6" t="inlineStr"/>
     </row>
+    <row r="42">
+      <c r="A42" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" s="4" t="inlineStr"/>
+      <c r="C42" s="4" t="inlineStr"/>
+      <c r="D42" s="4" t="inlineStr"/>
+      <c r="E42" s="4" t="inlineStr"/>
+      <c r="F42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" s="6" t="inlineStr"/>
+      <c r="C43" s="6" t="inlineStr"/>
+      <c r="D43" s="6" t="inlineStr"/>
+      <c r="E43" s="6" t="inlineStr"/>
+      <c r="F43" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F41"/>
+  <autoFilter ref="A3:F43"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add episode 22 "치앗촤! 가족 어벤져스" and Taeo's fight words
More of Taeo's Avengers play: he always opens with "어벤져스 캐릭터로
싸우자!", shouts "치앗촤 / 지앗 / 치앗차" while fighting, and says
"블랙 위도우 예뻐! 핀타스틱포 쑤우 예뻐!". Added to his dictionary
(치앗촤 · 지앗 · 치앗차, 핀타스틱포, 쑤우) and sayings; the beauty
line is now in his own words.

Episode 22: Taeo directs a family Avengers game, casts Jaei as Black
Widow and Mom as Sue, and fights Dad's Thanos to protect them; Jaei and
Mom answer that pretty heroes can fight too, and all three win. The
roles for Mom, Grandpa and Grandma are invented. Excel adds episode 22.
Cache v198.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$374</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$45</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$392</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1806,17 +1806,47 @@
       <c r="A25" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="B25" s="7" t="n"/>
-      <c r="C25" s="7" t="n"/>
-      <c r="D25" s="7" t="n"/>
-      <c r="E25" s="7" t="n"/>
-      <c r="F25" s="7" t="n"/>
-      <c r="G25" s="7" t="n"/>
-      <c r="H25" s="7" t="n"/>
-      <c r="I25" s="7" t="n"/>
-      <c r="J25" s="7" t="inlineStr">
-        <is>
-          <t>기획 중</t>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>치앗촤! 가족 어벤져스</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>“어벤져스 캐릭터로 싸우자! 치앗촤!” 태오가 감독이 된 가족 어벤져스 놀이. 가장 예쁜 영웅 둘은 반드시 지켜야 한다!</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>재이, 할머니, 엄마, 아빠, 할아버지, 태오</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>“어벤져스 캐릭터로 싸우자! 치앗촤!” 감독 태오가 역할 정하기 / 누나는 블랙 위도우, 엄마는 핀타스틱포 쑤우, 둘 다 “예뻐!” / 아빠 타노스 “아임 인에비터블” → 오늘도 패배</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>예뻐서 지키겠다던 태오에게 누나와 엄마가 “우리도 싸울 수 있어!” — 서로 지켜 주는 가족</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>지켜 주고 싶은 마음은 힘이 세요. 그리고 서로 지켜 주는 가족이 진짜 어벤져스예요.</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>우리 가족 어벤져스에서 나는 누구일까요? 내가 지켜 주고 싶은 사람은 누구예요?</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="J25" s="6" t="inlineStr">
+        <is>
+          <t>완성</t>
         </is>
       </c>
     </row>
@@ -1856,13 +1886,31 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" s="7" t="n"/>
+      <c r="C28" s="7" t="n"/>
+      <c r="D28" s="7" t="n"/>
+      <c r="E28" s="7" t="n"/>
+      <c r="F28" s="7" t="n"/>
+      <c r="G28" s="7" t="n"/>
+      <c r="H28" s="7" t="n"/>
+      <c r="I28" s="7" t="n"/>
+      <c r="J28" s="7" t="inlineStr">
+        <is>
+          <t>기획 중</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:J24"/>
+  <autoFilter ref="A3:J25"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"아이디어,기획 중,콘티,완성"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1876,7 +1924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H374"/>
+  <dimension ref="A1:H392"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -13755,8 +13803,586 @@
       <c r="G374" s="4" t="inlineStr"/>
       <c r="H374" s="4" t="inlineStr"/>
     </row>
+    <row r="375">
+      <c r="A375" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B375" s="6" t="inlineStr">
+        <is>
+          <t>치앗촤! 가족 어벤져스</t>
+        </is>
+      </c>
+      <c r="C375" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D375" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E375" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F375" s="6" t="inlineStr">
+        <is>
+          <t>토요일 오후, 거실.</t>
+        </is>
+      </c>
+      <c r="G375" s="6" t="inlineStr">
+        <is>
+          <t>어벤져스 캐릭터로 싸우자! 치앗촤!</t>
+        </is>
+      </c>
+      <c r="H375" s="6" t="inlineStr">
+        <is>
+          <t>휙!</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B376" s="4" t="inlineStr">
+        <is>
+          <t>치앗촤! 가족 어벤져스</t>
+        </is>
+      </c>
+      <c r="C376" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D376" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E376" s="4" t="inlineStr">
+        <is>
+          <t>재이, 엄마</t>
+        </is>
+      </c>
+      <c r="F376" s="4" t="inlineStr"/>
+      <c r="G376" s="4" t="inlineStr">
+        <is>
+          <t>그래. 누가 누구 할까?</t>
+        </is>
+      </c>
+      <c r="H376" s="4" t="inlineStr"/>
+    </row>
+    <row r="377">
+      <c r="A377" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B377" s="6" t="inlineStr">
+        <is>
+          <t>치앗촤! 가족 어벤져스</t>
+        </is>
+      </c>
+      <c r="C377" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D377" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E377" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F377" s="6" t="inlineStr"/>
+      <c r="G377" s="6" t="inlineStr">
+        <is>
+          <t>내가 감독이야! 역할을 정해 줄게!</t>
+        </is>
+      </c>
+      <c r="H377" s="6" t="inlineStr"/>
+    </row>
+    <row r="378">
+      <c r="A378" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B378" s="4" t="inlineStr">
+        <is>
+          <t>치앗촤! 가족 어벤져스</t>
+        </is>
+      </c>
+      <c r="C378" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D378" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E378" s="4" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="F378" s="4" t="inlineStr"/>
+      <c r="G378" s="4" t="inlineStr">
+        <is>
+          <t>누나는 블랙 위도우! 제일 예뻐!</t>
+        </is>
+      </c>
+      <c r="H378" s="4" t="inlineStr">
+        <is>
+          <t>반짝</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B379" s="6" t="inlineStr">
+        <is>
+          <t>치앗촤! 가족 어벤져스</t>
+        </is>
+      </c>
+      <c r="C379" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D379" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E379" s="6" t="inlineStr">
+        <is>
+          <t>태오, 엄마</t>
+        </is>
+      </c>
+      <c r="F379" s="6" t="inlineStr"/>
+      <c r="G379" s="6" t="inlineStr">
+        <is>
+          <t>엄마는 핀타스틱포 쑤우! 쑤우 예뻐!</t>
+        </is>
+      </c>
+      <c r="H379" s="6" t="inlineStr">
+        <is>
+          <t>반짝</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B380" s="4" t="inlineStr">
+        <is>
+          <t>치앗촤! 가족 어벤져스</t>
+        </is>
+      </c>
+      <c r="C380" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D380" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E380" s="4" t="inlineStr">
+        <is>
+          <t>엄마, 재이</t>
+        </is>
+      </c>
+      <c r="F380" s="4" t="inlineStr"/>
+      <c r="G380" s="4" t="inlineStr">
+        <is>
+          <t>어머, 엄마가 쑤우래.
+…아니야. 좋은데?</t>
+        </is>
+      </c>
+      <c r="H380" s="4" t="inlineStr"/>
+    </row>
+    <row r="381">
+      <c r="A381" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B381" s="6" t="inlineStr">
+        <is>
+          <t>치앗촤! 가족 어벤져스</t>
+        </is>
+      </c>
+      <c r="C381" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="D381" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E381" s="6" t="inlineStr">
+        <is>
+          <t>할아버지, 할머니, 태오</t>
+        </is>
+      </c>
+      <c r="F381" s="6" t="inlineStr"/>
+      <c r="G381" s="6" t="inlineStr">
+        <is>
+          <t>할아버지는 우엉! 할머니는… 맛있는 거 주는 영웅!</t>
+        </is>
+      </c>
+      <c r="H381" s="6" t="inlineStr"/>
+    </row>
+    <row r="382">
+      <c r="A382" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B382" s="4" t="inlineStr">
+        <is>
+          <t>치앗촤! 가족 어벤져스</t>
+        </is>
+      </c>
+      <c r="C382" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D382" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E382" s="4" t="inlineStr">
+        <is>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F382" s="4" t="inlineStr"/>
+      <c r="G382" s="4" t="inlineStr">
+        <is>
+          <t>그럼 아빠는 당연히…</t>
+        </is>
+      </c>
+      <c r="H382" s="4" t="inlineStr">
+        <is>
+          <t>크크크</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B383" s="6" t="inlineStr">
+        <is>
+          <t>치앗촤! 가족 어벤져스</t>
+        </is>
+      </c>
+      <c r="C383" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="D383" s="6" t="inlineStr">
+        <is>
+          <t>효과: 어두움</t>
+        </is>
+      </c>
+      <c r="E383" s="6" t="inlineStr">
+        <is>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F383" s="6" t="inlineStr"/>
+      <c r="G383" s="6" t="inlineStr">
+        <is>
+          <t>아임… 인에비터블.</t>
+        </is>
+      </c>
+      <c r="H383" s="6" t="inlineStr"/>
+    </row>
+    <row r="384">
+      <c r="A384" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B384" s="4" t="inlineStr">
+        <is>
+          <t>치앗촤! 가족 어벤져스</t>
+        </is>
+      </c>
+      <c r="C384" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D384" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E384" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F384" s="4" t="inlineStr"/>
+      <c r="G384" s="4" t="inlineStr">
+        <is>
+          <t>치앗촤!! 타노스 나와라!!</t>
+        </is>
+      </c>
+      <c r="H384" s="4" t="inlineStr">
+        <is>
+          <t>지앗!, 치앗차!</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B385" s="6" t="inlineStr">
+        <is>
+          <t>치앗촤! 가족 어벤져스</t>
+        </is>
+      </c>
+      <c r="C385" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="D385" s="6" t="inlineStr">
+        <is>
+          <t>효과: 속도선</t>
+        </is>
+      </c>
+      <c r="E385" s="6" t="inlineStr">
+        <is>
+          <t>태오, 아빠</t>
+        </is>
+      </c>
+      <c r="F385" s="6" t="inlineStr"/>
+      <c r="G385" s="6" t="inlineStr">
+        <is>
+          <t>블랙 위도우랑 쑤우는 내가 지킨다! 치앗촤!</t>
+        </is>
+      </c>
+      <c r="H385" s="6" t="inlineStr">
+        <is>
+          <t>퍽!</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B386" s="4" t="inlineStr">
+        <is>
+          <t>치앗촤! 가족 어벤져스</t>
+        </is>
+      </c>
+      <c r="C386" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D386" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E386" s="4" t="inlineStr">
+        <is>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F386" s="4" t="inlineStr"/>
+      <c r="G386" s="4" t="inlineStr">
+        <is>
+          <t>으악! 타노스가 졌다!</t>
+        </is>
+      </c>
+      <c r="H386" s="4" t="inlineStr">
+        <is>
+          <t>쿵</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B387" s="6" t="inlineStr">
+        <is>
+          <t>치앗촤! 가족 어벤져스</t>
+        </is>
+      </c>
+      <c r="C387" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="D387" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E387" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F387" s="6" t="inlineStr"/>
+      <c r="G387" s="6" t="inlineStr">
+        <is>
+          <t>이겼다! 타노스 끝! 치앗촤!</t>
+        </is>
+      </c>
+      <c r="H387" s="6" t="inlineStr"/>
+    </row>
+    <row r="388">
+      <c r="A388" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B388" s="4" t="inlineStr">
+        <is>
+          <t>치앗촤! 가족 어벤져스</t>
+        </is>
+      </c>
+      <c r="C388" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="D388" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E388" s="4" t="inlineStr">
+        <is>
+          <t>재이, 엄마</t>
+        </is>
+      </c>
+      <c r="F388" s="4" t="inlineStr"/>
+      <c r="G388" s="4" t="inlineStr">
+        <is>
+          <t>태오만 싸우는 게 아니야!
+블랙 위도우랑 쑤우도 싸울 수 있어!</t>
+        </is>
+      </c>
+      <c r="H388" s="4" t="inlineStr">
+        <is>
+          <t>얍!</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B389" s="6" t="inlineStr">
+        <is>
+          <t>치앗촤! 가족 어벤져스</t>
+        </is>
+      </c>
+      <c r="C389" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="D389" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E389" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F389" s="6" t="inlineStr"/>
+      <c r="G389" s="6" t="inlineStr">
+        <is>
+          <t>…예쁜데 센 영웅이었어?</t>
+        </is>
+      </c>
+      <c r="H389" s="6" t="inlineStr"/>
+    </row>
+    <row r="390">
+      <c r="A390" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B390" s="4" t="inlineStr">
+        <is>
+          <t>치앗촤! 가족 어벤져스</t>
+        </is>
+      </c>
+      <c r="C390" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="D390" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E390" s="4" t="inlineStr">
+        <is>
+          <t>태오, 재이, 엄마</t>
+        </is>
+      </c>
+      <c r="F390" s="4" t="inlineStr"/>
+      <c r="G390" s="4" t="inlineStr">
+        <is>
+          <t>그럼 다 같이 싸우자! 치앗촤!</t>
+        </is>
+      </c>
+      <c r="H390" s="4" t="inlineStr"/>
+    </row>
+    <row r="391">
+      <c r="A391" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B391" s="6" t="inlineStr">
+        <is>
+          <t>치앗촤! 가족 어벤져스</t>
+        </is>
+      </c>
+      <c r="C391" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="D391" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E391" s="6" t="inlineStr">
+        <is>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F391" s="6" t="inlineStr">
+        <is>
+          <t>그렇게 타노스는 또 졌다.</t>
+        </is>
+      </c>
+      <c r="G391" s="6" t="inlineStr">
+        <is>
+          <t>(속삭임) …아빠 오늘도 졌네. 그래도 행복하다.</t>
+        </is>
+      </c>
+      <c r="H391" s="6" t="inlineStr"/>
+    </row>
+    <row r="392">
+      <c r="A392" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B392" s="4" t="inlineStr">
+        <is>
+          <t>치앗촤! 가족 어벤져스</t>
+        </is>
+      </c>
+      <c r="C392" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="D392" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E392" s="4" t="inlineStr"/>
+      <c r="F392" s="4" t="inlineStr">
+        <is>
+          <t>예뻐서 지키고 싶었던 마음은, / 알고 보니 서로 지켜 주는 마음이었다.</t>
+        </is>
+      </c>
+      <c r="G392" s="4" t="inlineStr"/>
+      <c r="H392" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:H374"/>
+  <autoFilter ref="A3:H392"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -13770,7 +14396,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -14288,17 +14914,17 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>어벤져스에 가년~</t>
+          <t>치앗촤 · 지앗 · 치앗차</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>어벤져스에 가면~</t>
+          <t>이얍! (기합)</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>‘시장에 가면’ 놀이의 태오판. 누구누구 있는지 이어 말하기</t>
+          <t>어벤져스로 싸울 때 지르는 기합 소리</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr"/>
@@ -14308,9 +14934,21 @@
       <c r="A26" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="B26" s="4" t="inlineStr"/>
-      <c r="C26" s="4" t="inlineStr"/>
-      <c r="D26" s="4" t="inlineStr"/>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>핀타스틱포</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>판타스틱 4</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>마블 영웅 팀</t>
+        </is>
+      </c>
       <c r="E26" s="4" t="inlineStr"/>
       <c r="F26" s="4" t="inlineStr"/>
     </row>
@@ -14318,9 +14956,21 @@
       <c r="A27" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="B27" s="6" t="inlineStr"/>
-      <c r="C27" s="6" t="inlineStr"/>
-      <c r="D27" s="6" t="inlineStr"/>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>쑤우</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>수 (판타스틱 4)</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>“쑤우 예뻐!”</t>
+        </is>
+      </c>
       <c r="E27" s="6" t="inlineStr"/>
       <c r="F27" s="6" t="inlineStr"/>
     </row>
@@ -14328,9 +14978,21 @@
       <c r="A28" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="B28" s="4" t="inlineStr"/>
-      <c r="C28" s="4" t="inlineStr"/>
-      <c r="D28" s="4" t="inlineStr"/>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>어벤져스에 가년~</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>어벤져스에 가면~</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>‘시장에 가면’ 놀이의 태오판. 누구누구 있는지 이어 말하기</t>
+        </is>
+      </c>
       <c r="E28" s="4" t="inlineStr"/>
       <c r="F28" s="4" t="inlineStr"/>
     </row>
@@ -14504,8 +15166,38 @@
       <c r="E45" s="6" t="inlineStr"/>
       <c r="F45" s="6" t="inlineStr"/>
     </row>
+    <row r="46">
+      <c r="A46" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="B46" s="4" t="inlineStr"/>
+      <c r="C46" s="4" t="inlineStr"/>
+      <c r="D46" s="4" t="inlineStr"/>
+      <c r="E46" s="4" t="inlineStr"/>
+      <c r="F46" s="4" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" s="6" t="inlineStr"/>
+      <c r="C47" s="6" t="inlineStr"/>
+      <c r="D47" s="6" t="inlineStr"/>
+      <c r="E47" s="6" t="inlineStr"/>
+      <c r="F47" s="6" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" s="4" t="inlineStr"/>
+      <c r="C48" s="4" t="inlineStr"/>
+      <c r="D48" s="4" t="inlineStr"/>
+      <c r="E48" s="4" t="inlineStr"/>
+      <c r="F48" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F45"/>
+  <autoFilter ref="A3:F48"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -14519,7 +15211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -14712,7 +15404,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>블랙 위도우랑 수가 제일 예뻐!</t>
+          <t>블랙 위도우 예뻐! 핀타스틱포 쑤우 예뻐!</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr"/>
@@ -14822,13 +15514,13 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>싸우자! 타노스 나와라!</t>
+          <t>어벤져스 캐릭터로 싸우자! 치앗촤!</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr"/>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>제일 좋아하는 놀이, 어벤져스로 타노스랑 싸우기 (타노스는 늘 아빠, 건틀렛 끼고 “아임 인에비터블”)</t>
+          <t>놀자고 할 때 제일 먼저 하는 말 (발차기 기합과 함께)</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr"/>
@@ -14844,13 +15536,13 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>너라고 하지 마라! 나도 엄마 아빠한테 너라고 한다!</t>
+          <t>싸우자! 타노스 나와라!</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr"/>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>“너 엄마 아빠 말 잘 들어” 소리를 들으면</t>
+          <t>제일 좋아하는 놀이, 어벤져스로 타노스랑 싸우기 (타노스는 늘 아빠, 건틀렛 끼고 “아임 인에비터블”)</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr"/>
@@ -14866,13 +15558,13 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>재이 아니야! 재이 누나야!</t>
+          <t>너라고 하지 마라! 나도 엄마 아빠한테 너라고 한다!</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr"/>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>누가 누나를 “재이야” 하고 부르면 (모든 호칭은 태오 기준)</t>
+          <t>“너 엄마 아빠 말 잘 들어” 소리를 들으면</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr"/>
@@ -14888,13 +15580,13 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>이 안 닦아! 싫어!</t>
+          <t>재이 아니야! 재이 누나야!</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr"/>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>아침저녁 이 닦을 때 (도망 다니고 바닥을 기어요)</t>
+          <t>누가 누나를 “재이야” 하고 부르면 (모든 호칭은 태오 기준)</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr"/>
@@ -14910,13 +15602,13 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>누나 대단해!</t>
+          <t>이 안 닦아! 싫어!</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr"/>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>누나가 잠수를 보여 줬을 때</t>
+          <t>아침저녁 이 닦을 때 (도망 다니고 바닥을 기어요)</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr"/>
@@ -14932,13 +15624,13 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>엄마 인누와~</t>
+          <t>누나 대단해!</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr"/>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>밤에 자다 깨서 (엄마가 옆에서 재워 줄 때까지)</t>
+          <t>누나가 잠수를 보여 줬을 때</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr"/>
@@ -14954,13 +15646,13 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>왜 놀려! 놀리지 마!</t>
+          <t>엄마 인누와~</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr"/>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>“태오는 글씨·숫자 잘 몰라” 소리를 들으면 (손가락질하며)</t>
+          <t>밤에 자다 깨서 (엄마가 옆에서 재워 줄 때까지)</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr"/>
@@ -14971,18 +15663,18 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>아니야!</t>
+          <t>왜 놀려! 놀리지 마!</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr"/>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>하루에도 제일 많이 하는 말</t>
+          <t>“태오는 글씨·숫자 잘 몰라” 소리를 들으면 (손가락질하며)</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr"/>
@@ -14998,13 +15690,13 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>거짓말! 아니야!</t>
+          <t>아니야!</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr"/>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>기분 나쁘거나 하기 싫을 때</t>
+          <t>하루에도 제일 많이 하는 말</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr"/>
@@ -15020,13 +15712,13 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>맛있는데 지금은 먹기 싫어.</t>
+          <t>거짓말! 아니야!</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr"/>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>누가 음식을 권하면</t>
+          <t>기분 나쁘거나 하기 싫을 때</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr"/>
@@ -15042,13 +15734,13 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>치즈 냄새 극혐!</t>
+          <t>맛있는데 지금은 먹기 싫어.</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr"/>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>치즈만 보면 (냄새는 더더욱)</t>
+          <t>누가 음식을 권하면</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr"/>
@@ -15064,13 +15756,13 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>김태오!</t>
+          <t>치즈 냄새 극혐!</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr"/>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+          <t>치즈만 보면 (냄새는 더더욱)</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr"/>
@@ -15081,22 +15773,18 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>짐방</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>김서방</t>
-        </is>
-      </c>
+          <t>김태오!</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr"/>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr"/>
@@ -15112,17 +15800,17 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>꿍끙이</t>
+          <t>짐방</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>뿡뿡이</t>
+          <t>김서방</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr"/>
@@ -15131,10 +15819,26 @@
       <c r="A29" s="5" t="n">
         <v>26</v>
       </c>
-      <c r="B29" s="6" t="inlineStr"/>
-      <c r="C29" s="6" t="inlineStr"/>
-      <c r="D29" s="6" t="inlineStr"/>
-      <c r="E29" s="6" t="inlineStr"/>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>꿍끙이</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>뿡뿡이</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+        </is>
+      </c>
       <c r="F29" s="6" t="inlineStr"/>
     </row>
     <row r="30">
@@ -15277,8 +15981,18 @@
       <c r="E43" s="6" t="inlineStr"/>
       <c r="F43" s="6" t="inlineStr"/>
     </row>
+    <row r="44">
+      <c r="A44" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" s="4" t="inlineStr"/>
+      <c r="C44" s="4" t="inlineStr"/>
+      <c r="D44" s="4" t="inlineStr"/>
+      <c r="E44" s="4" t="inlineStr"/>
+      <c r="F44" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F43"/>
+  <autoFilter ref="A3:F44"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add episode 23: 아기 아니야, 내 친구야 (Taeo and the relativity of names)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$392</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$409</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$48</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>반쪽 레몬을 늘 손에 들고 다니며 할짝할짝 핥아 먹는 막내(레몬·자두·파인애플처럼 신 과일이 제일 좋아요). 누나 괴롭히기가 취미인 막내(사실은 누나가 좋아서). 혼자 노는 것 같아도 가족 말을 다 듣고 있고, 틀려도 일단 소리 지르며 우기다가 들키면 머리를 긁적긁적. “맛있는 거 죠!”가 입버릇이고, 누나랑 같이 좋아하는 마블 영웅(스파이더맨, 판타스틱 4, 어벤져스)도 태오식으로 불러요(블루베리, 쉬터맨, 스테잌로저…). 블랙 위도우랑 수가 제일 예쁘대요. 제일 좋아하는 놀이는 어벤져스로 타노스랑 싸우기! 모든 호칭은 태오 기준이라, 누가 “재이야” 하면 “재이 누나야!” 하고 고쳐 줘요. 요즘은 화가 나면 뾰족한 말이 튀어나오지만, “나 화났어!” 주문을 연습 중이에요. 물이 눈에 들어가는 걸 엄청 무서워하고, 이 닦기를 제일 싫어해서 아침저녁으로 도망 다니고 바닥을 기어 다니며 엄마 아빠를 고생시켜요.</t>
+          <t>반쪽 레몬을 늘 손에 들고 다니며 할짝할짝 핥아 먹는 막내(레몬·자두·파인애플처럼 신 과일이 제일 좋아요). 누나 괴롭히기가 취미인 막내(사실은 누나가 좋아서). 혼자 노는 것 같아도 가족 말을 다 듣고 있고, 틀려도 일단 소리 지르며 우기다가 들키면 머리를 긁적긁적. “맛있는 거 죠!”가 입버릇이고, 누나랑 같이 좋아하는 마블 영웅(스파이더맨, 판타스틱 4, 어벤져스)도 태오식으로 불러요(블루베리, 쉬터맨, 스테잌로저…). 블랙 위도우랑 수가 제일 예쁘대요. 제일 좋아하는 놀이는 어벤져스로 타노스랑 싸우기! 모든 호칭은 태오 기준이라, 누가 “재이야” 하면 “재이 누나야!” 하고 고쳐 줘요. 요즘은 화가 나면 뾰족한 말이 튀어나오지만, “나 화났어!” 주문을 연습 중이에요. 물이 눈에 들어가는 걸 엄청 무서워하고, 이 닦기를 제일 싫어해서 아침저녁으로 도망 다니고 바닥을 기어 다니며 엄마 아빠를 고생시켜요. 어린이집 친구가 놀림 받으면 “왜 내 친구를 놀려! 슬프잖아!” 하고 친구 편을 들어요.</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1851,20 +1851,50 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="n">
+      <c r="A26" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="B26" s="7" t="n"/>
-      <c r="C26" s="7" t="n"/>
-      <c r="D26" s="7" t="n"/>
-      <c r="E26" s="7" t="n"/>
-      <c r="F26" s="7" t="n"/>
-      <c r="G26" s="7" t="n"/>
-      <c r="H26" s="7" t="n"/>
-      <c r="I26" s="7" t="n"/>
-      <c r="J26" s="7" t="inlineStr">
-        <is>
-          <t>기획 중</t>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>아기 아니야, 내 친구야</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>“어린이집에 기저귀 하는 친구 있어?” 태오가 친구를 놀리는 말에 발끈! 그런데 “너는 형님이잖아”에도 발끈한다. 이름은 누가 기준일까?</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>재이, 엄마, 아빠, 태오</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>“하늘이는 아기네~” → “왜 내 친구를 놀려!” / “형님이잖아” → “너라고 하지 마라! 나도 아빠한테 너라고 한다!” (칭찬한 건데…) / 재이의 설명에 “태오는 태오인데?”</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>슬프잖아, 하며 친구 편을 드는 마음 / 다음 날 친구 손을 꼭 잡고 놀이터로 / 헷갈려도 마음은 벌써 형님</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>놀리지 않는 마음이 먼저예요. 부르는 이름은 천천히 배우면 돼요.</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>나는 누구에게는 동생이고, 누구에게는 형·언니·누나일 수 있어요. 나를 부르는 이름은 모두 몇 개일까요?</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>완성</t>
         </is>
       </c>
     </row>
@@ -1904,13 +1934,31 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" s="7" t="n"/>
+      <c r="C29" s="7" t="n"/>
+      <c r="D29" s="7" t="n"/>
+      <c r="E29" s="7" t="n"/>
+      <c r="F29" s="7" t="n"/>
+      <c r="G29" s="7" t="n"/>
+      <c r="H29" s="7" t="n"/>
+      <c r="I29" s="7" t="n"/>
+      <c r="J29" s="7" t="inlineStr">
+        <is>
+          <t>기획 중</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:J25"/>
+  <autoFilter ref="A3:J26"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"아이디어,기획 중,콘티,완성"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1924,7 +1972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H392"/>
+  <dimension ref="A1:H409"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -14381,8 +14429,541 @@
       <c r="G392" s="4" t="inlineStr"/>
       <c r="H392" s="4" t="inlineStr"/>
     </row>
+    <row r="393">
+      <c r="A393" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B393" s="6" t="inlineStr">
+        <is>
+          <t>아기 아니야, 내 친구야</t>
+        </is>
+      </c>
+      <c r="C393" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D393" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E393" s="6" t="inlineStr">
+        <is>
+          <t>아빠, 태오</t>
+        </is>
+      </c>
+      <c r="F393" s="6" t="inlineStr">
+        <is>
+          <t>저녁, 거실.</t>
+        </is>
+      </c>
+      <c r="G393" s="6" t="inlineStr">
+        <is>
+          <t>태오야, 어린이집에 기저귀 하는 친구 있어?</t>
+        </is>
+      </c>
+      <c r="H393" s="6" t="inlineStr"/>
+    </row>
+    <row r="394">
+      <c r="A394" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B394" s="4" t="inlineStr">
+        <is>
+          <t>아기 아니야, 내 친구야</t>
+        </is>
+      </c>
+      <c r="C394" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D394" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E394" s="4" t="inlineStr">
+        <is>
+          <t>태오, 아빠</t>
+        </is>
+      </c>
+      <c r="F394" s="4" t="inlineStr"/>
+      <c r="G394" s="4" t="inlineStr">
+        <is>
+          <t>응! 하늘이가 기저귀 해!
+오~ 하늘이는 아기네~</t>
+        </is>
+      </c>
+      <c r="H394" s="4" t="inlineStr"/>
+    </row>
+    <row r="395">
+      <c r="A395" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B395" s="6" t="inlineStr">
+        <is>
+          <t>아기 아니야, 내 친구야</t>
+        </is>
+      </c>
+      <c r="C395" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D395" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E395" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F395" s="6" t="inlineStr"/>
+      <c r="G395" s="6" t="inlineStr">
+        <is>
+          <t>왜 내 친구를 놀려!!</t>
+        </is>
+      </c>
+      <c r="H395" s="6" t="inlineStr">
+        <is>
+          <t>버럭!</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B396" s="4" t="inlineStr">
+        <is>
+          <t>아기 아니야, 내 친구야</t>
+        </is>
+      </c>
+      <c r="C396" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D396" s="4" t="inlineStr">
+        <is>
+          <t>효과: 어두움</t>
+        </is>
+      </c>
+      <c r="E396" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F396" s="4" t="inlineStr"/>
+      <c r="G396" s="4" t="inlineStr">
+        <is>
+          <t>하늘이가 슬프잖아!</t>
+        </is>
+      </c>
+      <c r="H396" s="4" t="inlineStr"/>
+    </row>
+    <row r="397">
+      <c r="A397" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B397" s="6" t="inlineStr">
+        <is>
+          <t>아기 아니야, 내 친구야</t>
+        </is>
+      </c>
+      <c r="C397" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D397" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E397" s="6" t="inlineStr">
+        <is>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F397" s="6" t="inlineStr">
+        <is>
+          <t>아빠는 얼른 사과하고, / 수습하려고 이렇게 말했다.</t>
+        </is>
+      </c>
+      <c r="G397" s="6" t="inlineStr">
+        <is>
+          <t>미안, 미안! 아빠가 잘못했어.</t>
+        </is>
+      </c>
+      <c r="H397" s="6" t="inlineStr"/>
+    </row>
+    <row r="398">
+      <c r="A398" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B398" s="4" t="inlineStr">
+        <is>
+          <t>아기 아니야, 내 친구야</t>
+        </is>
+      </c>
+      <c r="C398" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D398" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E398" s="4" t="inlineStr">
+        <is>
+          <t>아빠, 태오</t>
+        </is>
+      </c>
+      <c r="F398" s="4" t="inlineStr"/>
+      <c r="G398" s="4" t="inlineStr">
+        <is>
+          <t>태오는 기저귀 안 하니까 형님이잖아!</t>
+        </is>
+      </c>
+      <c r="H398" s="4" t="inlineStr"/>
+    </row>
+    <row r="399">
+      <c r="A399" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B399" s="6" t="inlineStr">
+        <is>
+          <t>아기 아니야, 내 친구야</t>
+        </is>
+      </c>
+      <c r="C399" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="D399" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E399" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F399" s="6" t="inlineStr"/>
+      <c r="G399" s="6" t="inlineStr">
+        <is>
+          <t>너라고 하지 마라!!</t>
+        </is>
+      </c>
+      <c r="H399" s="6" t="inlineStr">
+        <is>
+          <t>씩씩</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B400" s="4" t="inlineStr">
+        <is>
+          <t>아기 아니야, 내 친구야</t>
+        </is>
+      </c>
+      <c r="C400" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D400" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E400" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F400" s="4" t="inlineStr"/>
+      <c r="G400" s="4" t="inlineStr">
+        <is>
+          <t>나도 아빠한테 너라고 한다!</t>
+        </is>
+      </c>
+      <c r="H400" s="4" t="inlineStr"/>
+    </row>
+    <row r="401">
+      <c r="A401" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B401" s="6" t="inlineStr">
+        <is>
+          <t>아기 아니야, 내 친구야</t>
+        </is>
+      </c>
+      <c r="C401" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="D401" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E401" s="6" t="inlineStr">
+        <is>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F401" s="6" t="inlineStr">
+        <is>
+          <t>…형님이라고 한 건데?</t>
+        </is>
+      </c>
+      <c r="G401" s="6" t="inlineStr">
+        <is>
+          <t>(생각) (형님은 칭찬인데…)</t>
+        </is>
+      </c>
+      <c r="H401" s="6" t="inlineStr"/>
+    </row>
+    <row r="402">
+      <c r="A402" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B402" s="4" t="inlineStr">
+        <is>
+          <t>아기 아니야, 내 친구야</t>
+        </is>
+      </c>
+      <c r="C402" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D402" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E402" s="4" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F402" s="4" t="inlineStr"/>
+      <c r="G402" s="4" t="inlineStr">
+        <is>
+          <t>태오야, 태오는 나한테는 동생이고,</t>
+        </is>
+      </c>
+      <c r="H402" s="4" t="inlineStr"/>
+    </row>
+    <row r="403">
+      <c r="A403" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B403" s="6" t="inlineStr">
+        <is>
+          <t>아기 아니야, 내 친구야</t>
+        </is>
+      </c>
+      <c r="C403" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="D403" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E403" s="6" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F403" s="6" t="inlineStr"/>
+      <c r="G403" s="6" t="inlineStr">
+        <is>
+          <t>하늘이한테는 형님이고, 아빠한테는 아들이야.</t>
+        </is>
+      </c>
+      <c r="H403" s="6" t="inlineStr"/>
+    </row>
+    <row r="404">
+      <c r="A404" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B404" s="4" t="inlineStr">
+        <is>
+          <t>아기 아니야, 내 친구야</t>
+        </is>
+      </c>
+      <c r="C404" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D404" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E404" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F404" s="4" t="inlineStr"/>
+      <c r="G404" s="4" t="inlineStr">
+        <is>
+          <t>…태오는 태오인데?</t>
+        </is>
+      </c>
+      <c r="H404" s="4" t="inlineStr">
+        <is>
+          <t>갸웃</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B405" s="6" t="inlineStr">
+        <is>
+          <t>아기 아니야, 내 친구야</t>
+        </is>
+      </c>
+      <c r="C405" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="D405" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E405" s="6" t="inlineStr">
+        <is>
+          <t>엄마, 태오</t>
+        </is>
+      </c>
+      <c r="F405" s="6" t="inlineStr"/>
+      <c r="G405" s="6" t="inlineStr">
+        <is>
+          <t>하늘이도 곧 기저귀 졸업할 거야.
+엄마도 태오도 다 아기 때 했어.</t>
+        </is>
+      </c>
+      <c r="H405" s="6" t="inlineStr"/>
+    </row>
+    <row r="406">
+      <c r="A406" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B406" s="4" t="inlineStr">
+        <is>
+          <t>아기 아니야, 내 친구야</t>
+        </is>
+      </c>
+      <c r="C406" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="D406" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E406" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F406" s="4" t="inlineStr"/>
+      <c r="G406" s="4" t="inlineStr">
+        <is>
+          <t>그럼 내가 하늘이 지켜 줄 거야!</t>
+        </is>
+      </c>
+      <c r="H406" s="4" t="inlineStr"/>
+    </row>
+    <row r="407">
+      <c r="A407" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B407" s="6" t="inlineStr">
+        <is>
+          <t>아기 아니야, 내 친구야</t>
+        </is>
+      </c>
+      <c r="C407" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="D407" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E407" s="6" t="inlineStr">
+        <is>
+          <t>태오, 아빠</t>
+        </is>
+      </c>
+      <c r="F407" s="6" t="inlineStr">
+        <is>
+          <t>그리고 한마디 더.</t>
+        </is>
+      </c>
+      <c r="G407" s="6" t="inlineStr">
+        <is>
+          <t>형님이니까!
+…그래, 우리 형님.</t>
+        </is>
+      </c>
+      <c r="H407" s="6" t="inlineStr"/>
+    </row>
+    <row r="408">
+      <c r="A408" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B408" s="4" t="inlineStr">
+        <is>
+          <t>아기 아니야, 내 친구야</t>
+        </is>
+      </c>
+      <c r="C408" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="D408" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E408" s="4" t="inlineStr"/>
+      <c r="F408" s="4" t="inlineStr">
+        <is>
+          <t>다음 날 어린이집. / 태오는 친구 손을 꼭 잡고 놀이터로 갔대요.</t>
+        </is>
+      </c>
+      <c r="G408" s="4" t="inlineStr"/>
+      <c r="H408" s="4" t="inlineStr"/>
+    </row>
+    <row r="409">
+      <c r="A409" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B409" s="6" t="inlineStr">
+        <is>
+          <t>아기 아니야, 내 친구야</t>
+        </is>
+      </c>
+      <c r="C409" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="D409" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E409" s="6" t="inlineStr"/>
+      <c r="F409" s="6" t="inlineStr">
+        <is>
+          <t>누가 누구의 형님인지는 아직 헷갈려도, / 친구를 아끼는 마음은 벌써 형님이다.</t>
+        </is>
+      </c>
+      <c r="G409" s="6" t="inlineStr"/>
+      <c r="H409" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:H392"/>
+  <autoFilter ref="A3:H409"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -15211,7 +15792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -15685,18 +16266,18 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>아니야!</t>
+          <t>왜 내 친구를 놀려! 슬프잖아!</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr"/>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>하루에도 제일 많이 하는 말</t>
+          <t>어린이집 친구가 놀림 받는 것 같을 때 (친구 편이에요)</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr"/>
@@ -15712,13 +16293,13 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>거짓말! 아니야!</t>
+          <t>아니야!</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr"/>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>기분 나쁘거나 하기 싫을 때</t>
+          <t>하루에도 제일 많이 하는 말</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr"/>
@@ -15734,13 +16315,13 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>맛있는데 지금은 먹기 싫어.</t>
+          <t>거짓말! 아니야!</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr"/>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>누가 음식을 권하면</t>
+          <t>기분 나쁘거나 하기 싫을 때</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr"/>
@@ -15756,13 +16337,13 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>치즈 냄새 극혐!</t>
+          <t>맛있는데 지금은 먹기 싫어.</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr"/>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>치즈만 보면 (냄새는 더더욱)</t>
+          <t>누가 음식을 권하면</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr"/>
@@ -15778,13 +16359,13 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>김태오!</t>
+          <t>치즈 냄새 극혐!</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr"/>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+          <t>치즈만 보면 (냄새는 더더욱)</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr"/>
@@ -15795,22 +16376,18 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>짐방</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>김서방</t>
-        </is>
-      </c>
+          <t>김태오!</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr"/>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr"/>
@@ -15826,17 +16403,17 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>꿍끙이</t>
+          <t>짐방</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>뿡뿡이</t>
+          <t>김서방</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr"/>
@@ -15845,10 +16422,26 @@
       <c r="A30" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="B30" s="4" t="inlineStr"/>
-      <c r="C30" s="4" t="inlineStr"/>
-      <c r="D30" s="4" t="inlineStr"/>
-      <c r="E30" s="4" t="inlineStr"/>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>꿍끙이</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>뿡뿡이</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+        </is>
+      </c>
       <c r="F30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
@@ -15991,8 +16584,18 @@
       <c r="E44" s="4" t="inlineStr"/>
       <c r="F44" s="4" t="inlineStr"/>
     </row>
+    <row r="45">
+      <c r="A45" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="B45" s="6" t="inlineStr"/>
+      <c r="C45" s="6" t="inlineStr"/>
+      <c r="D45" s="6" t="inlineStr"/>
+      <c r="E45" s="6" t="inlineStr"/>
+      <c r="F45" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F44"/>
+  <autoFilter ref="A3:F45"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add Taeo-dictionary entries 닌재 and 놀래
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$409</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$50</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$10</definedName>
   </definedNames>
@@ -14977,7 +14977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -15581,9 +15581,21 @@
       <c r="A29" s="5" t="n">
         <v>26</v>
       </c>
-      <c r="B29" s="6" t="inlineStr"/>
-      <c r="C29" s="6" t="inlineStr"/>
-      <c r="D29" s="6" t="inlineStr"/>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>닌재</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>민재</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>어린이집 친구 이름</t>
+        </is>
+      </c>
       <c r="E29" s="6" t="inlineStr"/>
       <c r="F29" s="6" t="inlineStr"/>
     </row>
@@ -15591,9 +15603,21 @@
       <c r="A30" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="B30" s="4" t="inlineStr"/>
-      <c r="C30" s="4" t="inlineStr"/>
-      <c r="D30" s="4" t="inlineStr"/>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>놀래</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>놀려</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>“왜 내 친구를 놀래?” (놀리다 → 놀래다)</t>
+        </is>
+      </c>
       <c r="E30" s="4" t="inlineStr"/>
       <c r="F30" s="4" t="inlineStr"/>
     </row>
@@ -15777,8 +15801,28 @@
       <c r="E48" s="4" t="inlineStr"/>
       <c r="F48" s="4" t="inlineStr"/>
     </row>
+    <row r="49">
+      <c r="A49" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="B49" s="6" t="inlineStr"/>
+      <c r="C49" s="6" t="inlineStr"/>
+      <c r="D49" s="6" t="inlineStr"/>
+      <c r="E49" s="6" t="inlineStr"/>
+      <c r="F49" s="6" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="B50" s="4" t="inlineStr"/>
+      <c r="C50" s="4" t="inlineStr"/>
+      <c r="D50" s="4" t="inlineStr"/>
+      <c r="E50" s="4" t="inlineStr"/>
+      <c r="F50" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F48"/>
+  <autoFilter ref="A3:F50"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add episodes 24-25, 파라큘라 and favorite Marvel scenes to the family webtoon
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$409</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$50</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$435</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>반쪽 레몬을 늘 손에 들고 다니며 할짝할짝 핥아 먹는 막내(레몬·자두·파인애플처럼 신 과일이 제일 좋아요). 누나 괴롭히기가 취미인 막내(사실은 누나가 좋아서). 혼자 노는 것 같아도 가족 말을 다 듣고 있고, 틀려도 일단 소리 지르며 우기다가 들키면 머리를 긁적긁적. “맛있는 거 죠!”가 입버릇이고, 누나랑 같이 좋아하는 마블 영웅(스파이더맨, 판타스틱 4, 어벤져스)도 태오식으로 불러요(블루베리, 쉬터맨, 스테잌로저…). 블랙 위도우랑 수가 제일 예쁘대요. 제일 좋아하는 놀이는 어벤져스로 타노스랑 싸우기! 모든 호칭은 태오 기준이라, 누가 “재이야” 하면 “재이 누나야!” 하고 고쳐 줘요. 요즘은 화가 나면 뾰족한 말이 튀어나오지만, “나 화났어!” 주문을 연습 중이에요. 물이 눈에 들어가는 걸 엄청 무서워하고, 이 닦기를 제일 싫어해서 아침저녁으로 도망 다니고 바닥을 기어 다니며 엄마 아빠를 고생시켜요. 어린이집 친구가 놀림 받으면 “왜 내 친구를 놀려! 슬프잖아!” 하고 친구 편을 들어요.</t>
+          <t>반쪽 레몬을 늘 손에 들고 다니며 할짝할짝 핥아 먹는 막내(레몬·자두·파인애플처럼 신 과일이 제일 좋아요). 누나 괴롭히기가 취미인 막내(사실은 누나가 좋아서). 혼자 노는 것 같아도 가족 말을 다 듣고 있고, 틀려도 일단 소리 지르며 우기다가 들키면 머리를 긁적긁적. “맛있는 거 죠!”가 입버릇이고, 누나랑 같이 좋아하는 마블 영웅(스파이더맨, 판타스틱 4, 어벤져스)도 태오식으로 불러요(블루베리, 쉬터맨, 스테잌로저…). 블랙 위도우랑 수가 제일 예쁘대요. 제일 좋아하는 놀이는 어벤져스로 타노스랑 싸우기! 모든 호칭은 태오 기준이라, 누가 “재이야” 하면 “재이 누나야!” 하고 고쳐 줘요. 요즘은 화가 나면 뾰족한 말이 튀어나오지만, “나 화났어!” 주문을 연습 중이에요. 물이 눈에 들어가는 걸 엄청 무서워하고, 이 닦기를 제일 싫어해서 아침저녁으로 도망 다니고 바닥을 기어 다니며 엄마 아빠를 고생시켜요. 어린이집 친구가 놀림 받으면 “왜 내 친구를 놀려! 슬프잖아!” 하고 친구 편을 들어요. 캡틴 아메리카가 헬리콥터를 붙잡는 장면, 스파이더맨이 갈라지는 배를 거미줄로 버티는 장면을 제일 좋아하고, 드라큘라는 “파라큘라”, 무지개빛 망토와 또봇 Y가 갖고 싶대요.</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1902,35 +1902,95 @@
       <c r="A27" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="B27" s="7" t="n"/>
-      <c r="C27" s="7" t="n"/>
-      <c r="D27" s="7" t="n"/>
-      <c r="E27" s="7" t="n"/>
-      <c r="F27" s="7" t="n"/>
-      <c r="G27" s="7" t="n"/>
-      <c r="H27" s="7" t="n"/>
-      <c r="I27" s="7" t="n"/>
-      <c r="J27" s="7" t="inlineStr">
-        <is>
-          <t>기획 중</t>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>태오의 명장면 극장</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>“어벤져스… 어셈블!” 태오가 제일 좋아하는 장면만 모은 거실 극장이 열렸다. 헬리콥터도, 갈라지는 배도 우리 집에선 다 막아 낸다!</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>재이, 할머니, 엄마, 아빠, 할아버지, 태오</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>“어벤져스… 어셈블!” / 아빠가 헬리콥터가 되고 태오 캡틴이 팔을 잡아당겨 “못 날아가!” (아빠 팔 빠질 뻔) / 쪼개지는 배를 거미줄로 버티는 쉬터맨 / “와칸다 포에버!” 다 같이 달리기</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>혼자 버티던 태오에게 누나·할머니가 “나도 같이 잡을게!” / 헬리콥터 아빠도 끝까지 놀아 주는 사랑 / “우리 배는 안 갈라져!”</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>혼자 버티는 것보다 다 같이 붙잡는 게 힘이 세요. 함께라면 갈라지는 배도 가라앉지 않아요.</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>내가 제일 좋아하는 영화(만화) 장면은 뭐예요? 가족이랑 같이 따라 해 볼까요?</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="J27" s="6" t="inlineStr">
+        <is>
+          <t>완성</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="n">
+      <c r="A28" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="B28" s="7" t="n"/>
-      <c r="C28" s="7" t="n"/>
-      <c r="D28" s="7" t="n"/>
-      <c r="E28" s="7" t="n"/>
-      <c r="F28" s="7" t="n"/>
-      <c r="G28" s="7" t="n"/>
-      <c r="H28" s="7" t="n"/>
-      <c r="I28" s="7" t="n"/>
-      <c r="J28" s="7" t="inlineStr">
-        <is>
-          <t>기획 중</t>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>파라큘라와 무지개 망토</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>“엄마! 오늘 파라큘라 봤어!” 무지개빛 망토도, 또봇 Y도 갖고 싶은 태오. 할머니의 가위와 바늘이 소원 하나를 이뤄 준다.</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>재이, 할머니, 엄마, 아빠, 할아버지, 태오</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>“파라큘라 봤어!” “드라큘라?” “파라큘라야!!” / 파라큘라 흉내 내는 아빠에게 “아빠는 타노스잖아” / 무지개빛 망토 + 또봇 Y 갖고 싶다고 외침 / “…드라큘라야.”(누나)</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>할머니·할아버지가 자투리 천으로 밤새 만든 무지개 망토 / 또봇 Y는 “생일에 갖고 싶어!” 기다리는 마음을 배움</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>갖고 싶은 마음을 말하는 건 괜찮아요. 기다리는 마음, 손으로 만든 선물이 더 오래 반짝여요.</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>요즘 제일 갖고 싶은 건 뭐예요? 누군가 나를 위해 손으로 만들어 준 게 있나요?</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>완성</t>
         </is>
       </c>
     </row>
@@ -1952,13 +2012,49 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" s="7" t="n"/>
+      <c r="C30" s="7" t="n"/>
+      <c r="D30" s="7" t="n"/>
+      <c r="E30" s="7" t="n"/>
+      <c r="F30" s="7" t="n"/>
+      <c r="G30" s="7" t="n"/>
+      <c r="H30" s="7" t="n"/>
+      <c r="I30" s="7" t="n"/>
+      <c r="J30" s="7" t="inlineStr">
+        <is>
+          <t>기획 중</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" s="7" t="n"/>
+      <c r="C31" s="7" t="n"/>
+      <c r="D31" s="7" t="n"/>
+      <c r="E31" s="7" t="n"/>
+      <c r="F31" s="7" t="n"/>
+      <c r="G31" s="7" t="n"/>
+      <c r="H31" s="7" t="n"/>
+      <c r="I31" s="7" t="n"/>
+      <c r="J31" s="7" t="inlineStr">
+        <is>
+          <t>기획 중</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:J26"/>
+  <autoFilter ref="A3:J28"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"아이디어,기획 중,콘티,완성"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1972,7 +2068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H409"/>
+  <dimension ref="A1:H435"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -14962,8 +15058,849 @@
       <c r="G409" s="6" t="inlineStr"/>
       <c r="H409" s="6" t="inlineStr"/>
     </row>
+    <row r="410">
+      <c r="A410" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B410" s="4" t="inlineStr">
+        <is>
+          <t>태오의 명장면 극장</t>
+        </is>
+      </c>
+      <c r="C410" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D410" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E410" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F410" s="4" t="inlineStr">
+        <is>
+          <t>일요일 오후, 거실이 극장이 되었다.</t>
+        </is>
+      </c>
+      <c r="G410" s="4" t="inlineStr">
+        <is>
+          <t>오늘은 내가 제일 좋아하는 장면만 할 거야!</t>
+        </is>
+      </c>
+      <c r="H410" s="4" t="inlineStr"/>
+    </row>
+    <row r="411">
+      <c r="A411" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B411" s="6" t="inlineStr">
+        <is>
+          <t>태오의 명장면 극장</t>
+        </is>
+      </c>
+      <c r="C411" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D411" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E411" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F411" s="6" t="inlineStr"/>
+      <c r="G411" s="6" t="inlineStr">
+        <is>
+          <t>어벤져스… 어셈블!!</t>
+        </is>
+      </c>
+      <c r="H411" s="6" t="inlineStr">
+        <is>
+          <t>짜잔!</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B412" s="4" t="inlineStr">
+        <is>
+          <t>태오의 명장면 극장</t>
+        </is>
+      </c>
+      <c r="C412" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D412" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E412" s="4" t="inlineStr">
+        <is>
+          <t>재이, 엄마, 태오, 아빠, 할아버지</t>
+        </is>
+      </c>
+      <c r="F412" s="4" t="inlineStr"/>
+      <c r="G412" s="4" t="inlineStr">
+        <is>
+          <t>다 모여! 어셈블이야!</t>
+        </is>
+      </c>
+      <c r="H412" s="4" t="inlineStr"/>
+    </row>
+    <row r="413">
+      <c r="A413" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B413" s="6" t="inlineStr">
+        <is>
+          <t>태오의 명장면 극장</t>
+        </is>
+      </c>
+      <c r="C413" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D413" s="6" t="inlineStr">
+        <is>
+          <t>효과: 속도선</t>
+        </is>
+      </c>
+      <c r="E413" s="6" t="inlineStr">
+        <is>
+          <t>태오, 아빠</t>
+        </is>
+      </c>
+      <c r="F413" s="6" t="inlineStr">
+        <is>
+          <t>시빌 워. 아빠는 아이언맨 쪽이다.</t>
+        </is>
+      </c>
+      <c r="G413" s="6" t="inlineStr">
+        <is>
+          <t>왓 두 유 두, 캡틴~?
+위 파이트!!</t>
+        </is>
+      </c>
+      <c r="H413" s="6" t="inlineStr">
+        <is>
+          <t>쾅!</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B414" s="4" t="inlineStr">
+        <is>
+          <t>태오의 명장면 극장</t>
+        </is>
+      </c>
+      <c r="C414" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D414" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E414" s="4" t="inlineStr">
+        <is>
+          <t>아빠, 재이</t>
+        </is>
+      </c>
+      <c r="F414" s="4" t="inlineStr"/>
+      <c r="G414" s="4" t="inlineStr">
+        <is>
+          <t>나는 헬리콥터다~ 슈웅~ 날아간다~
+윙윙윙~ (프로펠러 소리 담당)</t>
+        </is>
+      </c>
+      <c r="H414" s="4" t="inlineStr">
+        <is>
+          <t>윙윙윙</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B415" s="6" t="inlineStr">
+        <is>
+          <t>태오의 명장면 극장</t>
+        </is>
+      </c>
+      <c r="C415" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D415" s="6" t="inlineStr">
+        <is>
+          <t>효과: 속도선</t>
+        </is>
+      </c>
+      <c r="E415" s="6" t="inlineStr">
+        <is>
+          <t>태오, 아빠</t>
+        </is>
+      </c>
+      <c r="F415" s="6" t="inlineStr"/>
+      <c r="G415" s="6" t="inlineStr">
+        <is>
+          <t>캡틴이 잡았다! 못 날아가!!</t>
+        </is>
+      </c>
+      <c r="H415" s="6" t="inlineStr">
+        <is>
+          <t>으아아!</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B416" s="4" t="inlineStr">
+        <is>
+          <t>태오의 명장면 극장</t>
+        </is>
+      </c>
+      <c r="C416" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D416" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E416" s="4" t="inlineStr">
+        <is>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="F416" s="4" t="inlineStr">
+        <is>
+          <t>6살 캡틴의 힘은 진짜였다.</t>
+        </is>
+      </c>
+      <c r="G416" s="4" t="inlineStr">
+        <is>
+          <t>(속삭임) 으윽… 팔이 빠지겠어…</t>
+        </is>
+      </c>
+      <c r="H416" s="4" t="inlineStr">
+        <is>
+          <t>부들부들</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B417" s="6" t="inlineStr">
+        <is>
+          <t>태오의 명장면 극장</t>
+        </is>
+      </c>
+      <c r="C417" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D417" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E417" s="6" t="inlineStr">
+        <is>
+          <t>엄마, 태오, 아빠</t>
+        </is>
+      </c>
+      <c r="F417" s="6" t="inlineStr">
+        <is>
+          <t>이번엔 스파이더맨. 배가 둘로 쪼개진다!</t>
+        </is>
+      </c>
+      <c r="G417" s="6" t="inlineStr">
+        <is>
+          <t>안 돼! 쉬터맨이 잡았다!!</t>
+        </is>
+      </c>
+      <c r="H417" s="6" t="inlineStr">
+        <is>
+          <t>슈욱!, 슈욱!</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B418" s="4" t="inlineStr">
+        <is>
+          <t>태오의 명장면 극장</t>
+        </is>
+      </c>
+      <c r="C418" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D418" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E418" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F418" s="4" t="inlineStr"/>
+      <c r="G418" s="4" t="inlineStr">
+        <is>
+          <t>으으으… 우리 배는 안 갈라져!!</t>
+        </is>
+      </c>
+      <c r="H418" s="4" t="inlineStr"/>
+    </row>
+    <row r="419">
+      <c r="A419" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B419" s="6" t="inlineStr">
+        <is>
+          <t>태오의 명장면 극장</t>
+        </is>
+      </c>
+      <c r="C419" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D419" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E419" s="6" t="inlineStr">
+        <is>
+          <t>재이, 태오, 할머니</t>
+        </is>
+      </c>
+      <c r="F419" s="6" t="inlineStr"/>
+      <c r="G419" s="6" t="inlineStr">
+        <is>
+          <t>나도 같이 잡을게!
+할머니도 거든다!</t>
+        </is>
+      </c>
+      <c r="H419" s="6" t="inlineStr"/>
+    </row>
+    <row r="420">
+      <c r="A420" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B420" s="4" t="inlineStr">
+        <is>
+          <t>태오의 명장면 극장</t>
+        </is>
+      </c>
+      <c r="C420" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D420" s="4" t="inlineStr">
+        <is>
+          <t>효과: 속도선</t>
+        </is>
+      </c>
+      <c r="E420" s="4" t="inlineStr">
+        <is>
+          <t>태오, 재이, 엄마, 아빠, 할머니</t>
+        </is>
+      </c>
+      <c r="F420" s="4" t="inlineStr">
+        <is>
+          <t>인피니티 워! 다 같이 달려간다!</t>
+        </is>
+      </c>
+      <c r="G420" s="4" t="inlineStr">
+        <is>
+          <t>와칸다 포에버!!!</t>
+        </is>
+      </c>
+      <c r="H420" s="4" t="inlineStr"/>
+    </row>
+    <row r="421">
+      <c r="A421" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B421" s="6" t="inlineStr">
+        <is>
+          <t>태오의 명장면 극장</t>
+        </is>
+      </c>
+      <c r="C421" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D421" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E421" s="6" t="inlineStr">
+        <is>
+          <t>태오, 재이, 엄마</t>
+        </is>
+      </c>
+      <c r="F421" s="6" t="inlineStr"/>
+      <c r="G421" s="6" t="inlineStr">
+        <is>
+          <t>블루베리가 알려 줬어! 이렇게 하는 거야!</t>
+        </is>
+      </c>
+      <c r="H421" s="6" t="inlineStr"/>
+    </row>
+    <row r="422">
+      <c r="A422" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B422" s="4" t="inlineStr">
+        <is>
+          <t>태오의 명장면 극장</t>
+        </is>
+      </c>
+      <c r="C422" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="D422" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E422" s="4" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F422" s="4" t="inlineStr"/>
+      <c r="G422" s="4" t="inlineStr">
+        <is>
+          <t>태오야, 오늘 제일 멋있었어.
+…진짜? 누나도!</t>
+        </is>
+      </c>
+      <c r="H422" s="4" t="inlineStr"/>
+    </row>
+    <row r="423">
+      <c r="A423" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B423" s="6" t="inlineStr">
+        <is>
+          <t>태오의 명장면 극장</t>
+        </is>
+      </c>
+      <c r="C423" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="D423" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E423" s="6" t="inlineStr"/>
+      <c r="F423" s="6" t="inlineStr">
+        <is>
+          <t>좋아하는 장면은 하나하나 달라도, / 우리 집은 오늘도 같은 장면 속에 있다.</t>
+        </is>
+      </c>
+      <c r="G423" s="6" t="inlineStr"/>
+      <c r="H423" s="6" t="inlineStr"/>
+    </row>
+    <row r="424">
+      <c r="A424" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B424" s="4" t="inlineStr">
+        <is>
+          <t>파라큘라와 무지개 망토</t>
+        </is>
+      </c>
+      <c r="C424" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D424" s="4" t="inlineStr">
+        <is>
+          <t>현관</t>
+        </is>
+      </c>
+      <c r="E424" s="4" t="inlineStr">
+        <is>
+          <t>태오, 엄마</t>
+        </is>
+      </c>
+      <c r="F424" s="4" t="inlineStr">
+        <is>
+          <t>10월. 어린이집에서 돌아온 저녁.</t>
+        </is>
+      </c>
+      <c r="G424" s="4" t="inlineStr">
+        <is>
+          <t>엄마! 오늘 파라큘라 봤어!
+파라큘라? 아~ 드라큘라?</t>
+        </is>
+      </c>
+      <c r="H424" s="4" t="inlineStr"/>
+    </row>
+    <row r="425">
+      <c r="A425" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="B425" s="6" t="inlineStr">
+        <is>
+          <t>파라큘라와 무지개 망토</t>
+        </is>
+      </c>
+      <c r="C425" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D425" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E425" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F425" s="6" t="inlineStr"/>
+      <c r="G425" s="6" t="inlineStr">
+        <is>
+          <t>파라큘라야!! 드라큘라 아니야!!</t>
+        </is>
+      </c>
+      <c r="H425" s="6" t="inlineStr"/>
+    </row>
+    <row r="426">
+      <c r="A426" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B426" s="4" t="inlineStr">
+        <is>
+          <t>파라큘라와 무지개 망토</t>
+        </is>
+      </c>
+      <c r="C426" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D426" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E426" s="4" t="inlineStr">
+        <is>
+          <t>아빠, 태오</t>
+        </is>
+      </c>
+      <c r="F426" s="4" t="inlineStr"/>
+      <c r="G426" s="4" t="inlineStr">
+        <is>
+          <t>나는 파라큘라다~ 피를 마시겠다~
+…아빠는 타노스잖아.</t>
+        </is>
+      </c>
+      <c r="H426" s="4" t="inlineStr"/>
+    </row>
+    <row r="427">
+      <c r="A427" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="B427" s="6" t="inlineStr">
+        <is>
+          <t>파라큘라와 무지개 망토</t>
+        </is>
+      </c>
+      <c r="C427" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D427" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E427" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F427" s="6" t="inlineStr"/>
+      <c r="G427" s="6" t="inlineStr">
+        <is>
+          <t>나 무지개빛 망토 갖고 싶어!!</t>
+        </is>
+      </c>
+      <c r="H427" s="6" t="inlineStr">
+        <is>
+          <t>반짝</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B428" s="4" t="inlineStr">
+        <is>
+          <t>파라큘라와 무지개 망토</t>
+        </is>
+      </c>
+      <c r="C428" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D428" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E428" s="4" t="inlineStr">
+        <is>
+          <t>엄마, 태오</t>
+        </is>
+      </c>
+      <c r="F428" s="4" t="inlineStr"/>
+      <c r="G428" s="4" t="inlineStr">
+        <is>
+          <t>그리고 또봇 Y도 갖고 싶어!!
+그건 생일 때 생각해 보자.</t>
+        </is>
+      </c>
+      <c r="H428" s="4" t="inlineStr"/>
+    </row>
+    <row r="429">
+      <c r="A429" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="B429" s="6" t="inlineStr">
+        <is>
+          <t>파라큘라와 무지개 망토</t>
+        </is>
+      </c>
+      <c r="C429" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D429" s="6" t="inlineStr">
+        <is>
+          <t>효과: 어두움</t>
+        </is>
+      </c>
+      <c r="E429" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F429" s="6" t="inlineStr"/>
+      <c r="G429" s="6" t="inlineStr">
+        <is>
+          <t>(속삭임) 지금 갖고 싶은데…</t>
+        </is>
+      </c>
+      <c r="H429" s="6" t="inlineStr">
+        <is>
+          <t>시무룩</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B430" s="4" t="inlineStr">
+        <is>
+          <t>파라큘라와 무지개 망토</t>
+        </is>
+      </c>
+      <c r="C430" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D430" s="4" t="inlineStr">
+        <is>
+          <t>할머니 댁</t>
+        </is>
+      </c>
+      <c r="E430" s="4" t="inlineStr">
+        <is>
+          <t>할머니, 할아버지</t>
+        </is>
+      </c>
+      <c r="F430" s="4" t="inlineStr">
+        <is>
+          <t>그날 밤, 할머니 집.</t>
+        </is>
+      </c>
+      <c r="G430" s="4" t="inlineStr">
+        <is>
+          <t>자투리 천 모아서 무지개를 만들어 볼까?
+허허, 실은 내가 잡아 줄게.</t>
+        </is>
+      </c>
+      <c r="H430" s="4" t="inlineStr"/>
+    </row>
+    <row r="431">
+      <c r="A431" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="B431" s="6" t="inlineStr">
+        <is>
+          <t>파라큘라와 무지개 망토</t>
+        </is>
+      </c>
+      <c r="C431" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D431" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E431" s="6" t="inlineStr"/>
+      <c r="F431" s="6" t="inlineStr">
+        <is>
+          <t>빨강, 주황, 노랑, 초록, 파랑, 보라. / 할머니는 밤새 바늘귀를 찾았다.</t>
+        </is>
+      </c>
+      <c r="G431" s="6" t="inlineStr"/>
+      <c r="H431" s="6" t="inlineStr"/>
+    </row>
+    <row r="432">
+      <c r="A432" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B432" s="4" t="inlineStr">
+        <is>
+          <t>파라큘라와 무지개 망토</t>
+        </is>
+      </c>
+      <c r="C432" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D432" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E432" s="4" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="F432" s="4" t="inlineStr"/>
+      <c r="G432" s="4" t="inlineStr">
+        <is>
+          <t>와! 무지개빛 망토다!!</t>
+        </is>
+      </c>
+      <c r="H432" s="4" t="inlineStr">
+        <is>
+          <t>휙!</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="B433" s="6" t="inlineStr">
+        <is>
+          <t>파라큘라와 무지개 망토</t>
+        </is>
+      </c>
+      <c r="C433" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D433" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E433" s="6" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="F433" s="6" t="inlineStr"/>
+      <c r="G433" s="6" t="inlineStr">
+        <is>
+          <t>파라큘라 나가신다!
+…드라큘라야.</t>
+        </is>
+      </c>
+      <c r="H433" s="6" t="inlineStr"/>
+    </row>
+    <row r="434">
+      <c r="A434" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B434" s="4" t="inlineStr">
+        <is>
+          <t>파라큘라와 무지개 망토</t>
+        </is>
+      </c>
+      <c r="C434" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D434" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E434" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F434" s="4" t="inlineStr"/>
+      <c r="G434" s="4" t="inlineStr">
+        <is>
+          <t>할머니 고마워. 또봇 Y는… 생일에 갖고 싶어!</t>
+        </is>
+      </c>
+      <c r="H434" s="4" t="inlineStr"/>
+    </row>
+    <row r="435">
+      <c r="A435" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="B435" s="6" t="inlineStr">
+        <is>
+          <t>파라큘라와 무지개 망토</t>
+        </is>
+      </c>
+      <c r="C435" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D435" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E435" s="6" t="inlineStr"/>
+      <c r="F435" s="6" t="inlineStr">
+        <is>
+          <t>갖고 싶은 건 아직 많지만, / 지금 두른 망토가 제일 따뜻했다.</t>
+        </is>
+      </c>
+      <c r="G435" s="6" t="inlineStr"/>
+      <c r="H435" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:H409"/>
+  <autoFilter ref="A3:H435"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -14977,7 +15914,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -15625,9 +16562,21 @@
       <c r="A31" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="B31" s="6" t="inlineStr"/>
-      <c r="C31" s="6" t="inlineStr"/>
-      <c r="D31" s="6" t="inlineStr"/>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>파라큘라</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>드라큘라</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>“드라큘라 아니야, 파라큘라야!”</t>
+        </is>
+      </c>
       <c r="E31" s="6" t="inlineStr"/>
       <c r="F31" s="6" t="inlineStr"/>
     </row>
@@ -15821,8 +16770,18 @@
       <c r="E50" s="4" t="inlineStr"/>
       <c r="F50" s="4" t="inlineStr"/>
     </row>
+    <row r="51">
+      <c r="A51" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B51" s="6" t="inlineStr"/>
+      <c r="C51" s="6" t="inlineStr"/>
+      <c r="D51" s="6" t="inlineStr"/>
+      <c r="E51" s="6" t="inlineStr"/>
+      <c r="F51" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F50"/>
+  <autoFilter ref="A3:F51"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -15836,7 +16795,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -16332,18 +17291,18 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>아니야!</t>
+          <t>나 무지개빛 망토 갖고 싶어!</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr"/>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>하루에도 제일 많이 하는 말</t>
+          <t>파라큘라를 본 날부터 (또봇 Y도 같이 갖고 싶어요!)</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr"/>
@@ -16354,18 +17313,18 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>거짓말! 아니야!</t>
+          <t>어벤져스… 어셈블!</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr"/>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>기분 나쁘거나 하기 싫을 때</t>
+          <t>엔드게임 마지막 장면을 따라 하며 가족을 다 모을 때</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr"/>
@@ -16376,18 +17335,18 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>맛있는데 지금은 먹기 싫어.</t>
+          <t>왓 두 유 두, 캡틴? 위 파이트!</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr"/>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>누가 음식을 권하면</t>
+          <t>시빌 워 싸움 장면 놀이를 할 때</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr"/>
@@ -16398,18 +17357,18 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>치즈 냄새 극혐!</t>
+          <t>와칸다 포에버!</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr"/>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>치즈만 보면 (냄새는 더더욱)</t>
+          <t>인피니티 워 장면처럼 다 같이 뛰어갈 때</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr"/>
@@ -16425,13 +17384,13 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>김태오!</t>
+          <t>아니야!</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr"/>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+          <t>하루에도 제일 많이 하는 말</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr"/>
@@ -16442,22 +17401,18 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>짐방</t>
-        </is>
-      </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>김서방</t>
-        </is>
-      </c>
+          <t>거짓말! 아니야!</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr"/>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+          <t>기분 나쁘거나 하기 싫을 때</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr"/>
@@ -16468,22 +17423,18 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>꿍끙이</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>뿡뿡이</t>
-        </is>
-      </c>
+          <t>맛있는데 지금은 먹기 싫어.</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr"/>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+          <t>누가 음식을 권하면</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr"/>
@@ -16492,40 +17443,96 @@
       <c r="A31" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="B31" s="6" t="inlineStr"/>
-      <c r="C31" s="6" t="inlineStr"/>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>재이 입버릇</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>치즈 냄새 극혐!</t>
+        </is>
+      </c>
       <c r="D31" s="6" t="inlineStr"/>
-      <c r="E31" s="6" t="inlineStr"/>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>치즈만 보면 (냄새는 더더욱)</t>
+        </is>
+      </c>
       <c r="F31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="B32" s="4" t="inlineStr"/>
-      <c r="C32" s="4" t="inlineStr"/>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>재이 입버릇</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>김태오!</t>
+        </is>
+      </c>
       <c r="D32" s="4" t="inlineStr"/>
-      <c r="E32" s="4" t="inlineStr"/>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+        </is>
+      </c>
       <c r="F32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="B33" s="6" t="inlineStr"/>
-      <c r="C33" s="6" t="inlineStr"/>
-      <c r="D33" s="6" t="inlineStr"/>
-      <c r="E33" s="6" t="inlineStr"/>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>짐방</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>김서방</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+        </is>
+      </c>
       <c r="F33" s="6" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="B34" s="4" t="inlineStr"/>
-      <c r="C34" s="4" t="inlineStr"/>
-      <c r="D34" s="4" t="inlineStr"/>
-      <c r="E34" s="4" t="inlineStr"/>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>꿍끙이</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>뿡뿡이</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+        </is>
+      </c>
       <c r="F34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
@@ -16638,8 +17645,48 @@
       <c r="E45" s="6" t="inlineStr"/>
       <c r="F45" s="6" t="inlineStr"/>
     </row>
+    <row r="46">
+      <c r="A46" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="B46" s="4" t="inlineStr"/>
+      <c r="C46" s="4" t="inlineStr"/>
+      <c r="D46" s="4" t="inlineStr"/>
+      <c r="E46" s="4" t="inlineStr"/>
+      <c r="F46" s="4" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" s="6" t="inlineStr"/>
+      <c r="C47" s="6" t="inlineStr"/>
+      <c r="D47" s="6" t="inlineStr"/>
+      <c r="E47" s="6" t="inlineStr"/>
+      <c r="F47" s="6" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" s="4" t="inlineStr"/>
+      <c r="C48" s="4" t="inlineStr"/>
+      <c r="D48" s="4" t="inlineStr"/>
+      <c r="E48" s="4" t="inlineStr"/>
+      <c r="F48" s="4" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="B49" s="6" t="inlineStr"/>
+      <c r="C49" s="6" t="inlineStr"/>
+      <c r="D49" s="6" t="inlineStr"/>
+      <c r="E49" s="6" t="inlineStr"/>
+      <c r="F49" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F45"/>
+  <autoFilter ref="A3:F49"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add episode 26: 오늘은 뽀로로 날!
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$435</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$448</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>반쪽 레몬을 늘 손에 들고 다니며 할짝할짝 핥아 먹는 막내(레몬·자두·파인애플처럼 신 과일이 제일 좋아요). 누나 괴롭히기가 취미인 막내(사실은 누나가 좋아서). 혼자 노는 것 같아도 가족 말을 다 듣고 있고, 틀려도 일단 소리 지르며 우기다가 들키면 머리를 긁적긁적. “맛있는 거 죠!”가 입버릇이고, 누나랑 같이 좋아하는 마블 영웅(스파이더맨, 판타스틱 4, 어벤져스)도 태오식으로 불러요(블루베리, 쉬터맨, 스테잌로저…). 블랙 위도우랑 수가 제일 예쁘대요. 제일 좋아하는 놀이는 어벤져스로 타노스랑 싸우기! 모든 호칭은 태오 기준이라, 누가 “재이야” 하면 “재이 누나야!” 하고 고쳐 줘요. 요즘은 화가 나면 뾰족한 말이 튀어나오지만, “나 화났어!” 주문을 연습 중이에요. 물이 눈에 들어가는 걸 엄청 무서워하고, 이 닦기를 제일 싫어해서 아침저녁으로 도망 다니고 바닥을 기어 다니며 엄마 아빠를 고생시켜요. 어린이집 친구가 놀림 받으면 “왜 내 친구를 놀려! 슬프잖아!” 하고 친구 편을 들어요. 캡틴 아메리카가 헬리콥터를 붙잡는 장면, 스파이더맨이 갈라지는 배를 거미줄로 버티는 장면을 제일 좋아하고, 드라큘라는 “파라큘라”, 무지개빛 망토와 또봇 Y가 갖고 싶대요.</t>
+          <t>반쪽 레몬을 늘 손에 들고 다니며 할짝할짝 핥아 먹는 막내(레몬·자두·파인애플처럼 신 과일이 제일 좋아요). 누나 괴롭히기가 취미인 막내(사실은 누나가 좋아서). 혼자 노는 것 같아도 가족 말을 다 듣고 있고, 틀려도 일단 소리 지르며 우기다가 들키면 머리를 긁적긁적. “맛있는 거 죠!”가 입버릇이고, 누나랑 같이 좋아하는 마블 영웅(스파이더맨, 판타스틱 4, 어벤져스)도 태오식으로 불러요(블루베리, 쉬터맨, 스테잌로저…). 블랙 위도우랑 수가 제일 예쁘대요. 제일 좋아하는 놀이는 어벤져스로 타노스랑 싸우기! 모든 호칭은 태오 기준이라, 누가 “재이야” 하면 “재이 누나야!” 하고 고쳐 줘요. 요즘은 화가 나면 뾰족한 말이 튀어나오지만, “나 화났어!” 주문을 연습 중이에요. 물이 눈에 들어가는 걸 엄청 무서워하고, 이 닦기를 제일 싫어해서 아침저녁으로 도망 다니고 바닥을 기어 다니며 엄마 아빠를 고생시켜요. 어린이집 친구가 놀림 받으면 “왜 내 친구를 놀려! 슬프잖아!” 하고 친구 편을 들어요. 캡틴 아메리카가 헬리콥터를 붙잡는 장면, 스파이더맨이 갈라지는 배를 거미줄로 버티는 장면을 제일 좋아하고, 드라큘라는 “파라큘라”, 무지개빛 망토와 또봇 Y가 갖고 싶대요. 아침마다 치카하기 싫어서 기어 다니고, 어린이집에 가기 싫어서 “데리러 올 거야?” 하고 몇 번씩 물어요. 태권도 가는 날은 “누나는 왜 학교만 가?” 하지만, 월요일은 태권도 안 가는 뽀로로 날!</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1998,17 +1998,47 @@
       <c r="A29" s="5" t="n">
         <v>26</v>
       </c>
-      <c r="B29" s="7" t="n"/>
-      <c r="C29" s="7" t="n"/>
-      <c r="D29" s="7" t="n"/>
-      <c r="E29" s="7" t="n"/>
-      <c r="F29" s="7" t="n"/>
-      <c r="G29" s="7" t="n"/>
-      <c r="H29" s="7" t="n"/>
-      <c r="I29" s="7" t="n"/>
-      <c r="J29" s="7" t="inlineStr">
-        <is>
-          <t>기획 중</t>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>오늘은 뽀로로 날!</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>“어린이집 가기 싫다. 누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?” 싫은 게 가득한 월요일 아침. 하지만 오늘은 뽀로로 날, 태권도 안 가는 날이다!</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>재이, 엄마, 아빠, 태오</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>치카 도망 → 어린이집 앞 “데리러 올 거야?” 몇 번씩 확인 / “누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?” → 누나 “나도 학원 가거든!” / 숫자·글씨는 몰라도 “뽀로로 날(월요일) = 태권도 안 가는 날” 정확히 앎</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>“제일 먼저 데리러 갈게” 약속 / 저녁에 엄마 보고 달려가는 태오 / “오늘은 어린이집 안 싫었어!”</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>싫은 날에도 “데리러 갈게”라는 약속이 있으면 힘이 나요. 지켜 주는 약속이 하루를 버티게 해요.</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>내가 기다리는 요일은 언제예요? 싫은 날을 이겨 내는 나만의 방법은 뭐예요?</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="J29" s="6" t="inlineStr">
+        <is>
+          <t>완성</t>
         </is>
       </c>
     </row>
@@ -2048,13 +2078,31 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" s="7" t="n"/>
+      <c r="C32" s="7" t="n"/>
+      <c r="D32" s="7" t="n"/>
+      <c r="E32" s="7" t="n"/>
+      <c r="F32" s="7" t="n"/>
+      <c r="G32" s="7" t="n"/>
+      <c r="H32" s="7" t="n"/>
+      <c r="I32" s="7" t="n"/>
+      <c r="J32" s="7" t="inlineStr">
+        <is>
+          <t>기획 중</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:J28"/>
+  <autoFilter ref="A3:J29"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"아이디어,기획 중,콘티,완성"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2068,7 +2116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H435"/>
+  <dimension ref="A1:H448"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -15899,8 +15947,434 @@
       <c r="G435" s="6" t="inlineStr"/>
       <c r="H435" s="6" t="inlineStr"/>
     </row>
+    <row r="436">
+      <c r="A436" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B436" s="4" t="inlineStr">
+        <is>
+          <t>오늘은 뽀로로 날!</t>
+        </is>
+      </c>
+      <c r="C436" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D436" s="4" t="inlineStr">
+        <is>
+          <t>bath</t>
+        </is>
+      </c>
+      <c r="E436" s="4" t="inlineStr">
+        <is>
+          <t>엄마</t>
+        </is>
+      </c>
+      <c r="F436" s="4" t="inlineStr">
+        <is>
+          <t>월요일 아침. / 오늘도 태오는 기어서 도망 중.</t>
+        </is>
+      </c>
+      <c r="G436" s="4" t="inlineStr">
+        <is>
+          <t>태오야~ 치카하자!</t>
+        </is>
+      </c>
+      <c r="H436" s="4" t="inlineStr"/>
+    </row>
+    <row r="437">
+      <c r="A437" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="B437" s="6" t="inlineStr">
+        <is>
+          <t>오늘은 뽀로로 날!</t>
+        </is>
+      </c>
+      <c r="C437" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D437" s="6" t="inlineStr">
+        <is>
+          <t>효과: 속도선</t>
+        </is>
+      </c>
+      <c r="E437" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F437" s="6" t="inlineStr"/>
+      <c r="G437" s="6" t="inlineStr">
+        <is>
+          <t>치카 싫어~!!</t>
+        </is>
+      </c>
+      <c r="H437" s="6" t="inlineStr">
+        <is>
+          <t>다다다</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B438" s="4" t="inlineStr">
+        <is>
+          <t>오늘은 뽀로로 날!</t>
+        </is>
+      </c>
+      <c r="C438" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D438" s="4" t="inlineStr">
+        <is>
+          <t>현관</t>
+        </is>
+      </c>
+      <c r="E438" s="4" t="inlineStr">
+        <is>
+          <t>엄마, 태오</t>
+        </is>
+      </c>
+      <c r="F438" s="4" t="inlineStr">
+        <is>
+          <t>어린이집 앞.</t>
+        </is>
+      </c>
+      <c r="G438" s="4" t="inlineStr">
+        <is>
+          <t>(속삭임) 어린이집 가기 싫다…
+그래도 가야지~</t>
+        </is>
+      </c>
+      <c r="H438" s="4" t="inlineStr"/>
+    </row>
+    <row r="439">
+      <c r="A439" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="B439" s="6" t="inlineStr">
+        <is>
+          <t>오늘은 뽀로로 날!</t>
+        </is>
+      </c>
+      <c r="C439" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D439" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E439" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F439" s="6" t="inlineStr"/>
+      <c r="G439" s="6" t="inlineStr">
+        <is>
+          <t>엄마… 어린이집에 데리러 올 거야?</t>
+        </is>
+      </c>
+      <c r="H439" s="6" t="inlineStr"/>
+    </row>
+    <row r="440">
+      <c r="A440" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B440" s="4" t="inlineStr">
+        <is>
+          <t>오늘은 뽀로로 날!</t>
+        </is>
+      </c>
+      <c r="C440" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D440" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E440" s="4" t="inlineStr">
+        <is>
+          <t>엄마</t>
+        </is>
+      </c>
+      <c r="F440" s="4" t="inlineStr"/>
+      <c r="G440" s="4" t="inlineStr">
+        <is>
+          <t>그럼! 제일 먼저 데리러 갈게.</t>
+        </is>
+      </c>
+      <c r="H440" s="4" t="inlineStr">
+        <is>
+          <t>꼬옥</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="B441" s="6" t="inlineStr">
+        <is>
+          <t>오늘은 뽀로로 날!</t>
+        </is>
+      </c>
+      <c r="C441" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D441" s="6" t="inlineStr">
+        <is>
+          <t>현관</t>
+        </is>
+      </c>
+      <c r="E441" s="6" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="F441" s="6" t="inlineStr"/>
+      <c r="G441" s="6" t="inlineStr">
+        <is>
+          <t>누나는 왜 학교만 가?! 나는 왜 태권도 가야 돼?!</t>
+        </is>
+      </c>
+      <c r="H441" s="6" t="inlineStr"/>
+    </row>
+    <row r="442">
+      <c r="A442" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B442" s="4" t="inlineStr">
+        <is>
+          <t>오늘은 뽀로로 날!</t>
+        </is>
+      </c>
+      <c r="C442" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D442" s="4" t="inlineStr">
+        <is>
+          <t>현관</t>
+        </is>
+      </c>
+      <c r="E442" s="4" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F442" s="4" t="inlineStr"/>
+      <c r="G442" s="4" t="inlineStr">
+        <is>
+          <t>아니야! 나도 학원 가거든!</t>
+        </is>
+      </c>
+      <c r="H442" s="4" t="inlineStr">
+        <is>
+          <t>움찔</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="B443" s="6" t="inlineStr">
+        <is>
+          <t>오늘은 뽀로로 날!</t>
+        </is>
+      </c>
+      <c r="C443" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D443" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E443" s="6" t="inlineStr">
+        <is>
+          <t>엄마</t>
+        </is>
+      </c>
+      <c r="F443" s="6" t="inlineStr">
+        <is>
+          <t>그런데 엄마가 휴대폰 달력을 보더니,</t>
+        </is>
+      </c>
+      <c r="G443" s="6" t="inlineStr">
+        <is>
+          <t>오늘이… 월요일이네?</t>
+        </is>
+      </c>
+      <c r="H443" s="6" t="inlineStr"/>
+    </row>
+    <row r="444">
+      <c r="A444" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B444" s="4" t="inlineStr">
+        <is>
+          <t>오늘은 뽀로로 날!</t>
+        </is>
+      </c>
+      <c r="C444" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D444" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E444" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F444" s="4" t="inlineStr"/>
+      <c r="G444" s="4" t="inlineStr">
+        <is>
+          <t>오늘은 뽀로로 날이다~!
+내가 싫어하는 태권도 안 가는 날이다~!</t>
+        </is>
+      </c>
+      <c r="H444" s="4" t="inlineStr">
+        <is>
+          <t>만세!</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="B445" s="6" t="inlineStr">
+        <is>
+          <t>오늘은 뽀로로 날!</t>
+        </is>
+      </c>
+      <c r="C445" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D445" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E445" s="6" t="inlineStr">
+        <is>
+          <t>재이, 아빠</t>
+        </is>
+      </c>
+      <c r="F445" s="6" t="inlineStr"/>
+      <c r="G445" s="6" t="inlineStr">
+        <is>
+          <t>…글씨도 숫자도 잘 모르면서.
+요일은 뽀로로가 알려 주나 봐.</t>
+        </is>
+      </c>
+      <c r="H445" s="6" t="inlineStr"/>
+    </row>
+    <row r="446">
+      <c r="A446" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B446" s="4" t="inlineStr">
+        <is>
+          <t>오늘은 뽀로로 날!</t>
+        </is>
+      </c>
+      <c r="C446" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D446" s="4" t="inlineStr">
+        <is>
+          <t>현관</t>
+        </is>
+      </c>
+      <c r="E446" s="4" t="inlineStr">
+        <is>
+          <t>엄마, 태오</t>
+        </is>
+      </c>
+      <c r="F446" s="4" t="inlineStr">
+        <is>
+          <t>저녁, 어린이집 앞.</t>
+        </is>
+      </c>
+      <c r="G446" s="4" t="inlineStr">
+        <is>
+          <t>엄마 왔다!!
+그럼, 약속했잖아.</t>
+        </is>
+      </c>
+      <c r="H446" s="4" t="inlineStr">
+        <is>
+          <t>다다다</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="B447" s="6" t="inlineStr">
+        <is>
+          <t>오늘은 뽀로로 날!</t>
+        </is>
+      </c>
+      <c r="C447" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D447" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E447" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F447" s="6" t="inlineStr"/>
+      <c r="G447" s="6" t="inlineStr">
+        <is>
+          <t>엄마 제일 먼저 왔다! 오늘은 어린이집 안 싫었어!</t>
+        </is>
+      </c>
+      <c r="H447" s="6" t="inlineStr"/>
+    </row>
+    <row r="448">
+      <c r="A448" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B448" s="4" t="inlineStr">
+        <is>
+          <t>오늘은 뽀로로 날!</t>
+        </is>
+      </c>
+      <c r="C448" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="D448" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E448" s="4" t="inlineStr"/>
+      <c r="F448" s="4" t="inlineStr">
+        <is>
+          <t>내일은 태권도 가는 날이지만, / 엄마가 데리러 온다니 괜찮다.</t>
+        </is>
+      </c>
+      <c r="G448" s="4" t="inlineStr"/>
+      <c r="H448" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:H435"/>
+  <autoFilter ref="A3:H448"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -16795,7 +17269,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -17379,18 +17853,18 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>아니야!</t>
+          <t>어린이집에 데리러 올 거야?</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr"/>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>하루에도 제일 많이 하는 말</t>
+          <t>어린이집 가기 싫은 아침에 (몇 번씩 확인해요)</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr"/>
@@ -17401,18 +17875,18 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>거짓말! 아니야!</t>
+          <t>어린이집 가기 싫다.</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr"/>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>기분 나쁘거나 하기 싫을 때</t>
+          <t>월·화·수… 아침마다</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr"/>
@@ -17423,18 +17897,18 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>맛있는데 지금은 먹기 싫어.</t>
+          <t>누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr"/>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>누가 음식을 권하면</t>
+          <t>싫은 태권도 가는 날</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr"/>
@@ -17445,18 +17919,18 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>치즈 냄새 극혐!</t>
+          <t>오늘은 뽀로로 날! 내가 싫어하는 태권도 안 가는 날이다~</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr"/>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>치즈만 보면 (냄새는 더더욱)</t>
+          <t>월요일 아침 (달력은 몰라도 뽀로로 날은 정확히 알아요)</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr"/>
@@ -17472,13 +17946,13 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>김태오!</t>
+          <t>아니야!</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr"/>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+          <t>하루에도 제일 많이 하는 말</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr"/>
@@ -17489,22 +17963,18 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>짐방</t>
-        </is>
-      </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>김서방</t>
-        </is>
-      </c>
+          <t>거짓말! 아니야!</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr"/>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+          <t>기분 나쁘거나 하기 싫을 때</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr"/>
@@ -17515,22 +17985,18 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>꿍끙이</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>뿡뿡이</t>
-        </is>
-      </c>
+          <t>맛있는데 지금은 먹기 싫어.</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr"/>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+          <t>누가 음식을 권하면</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr"/>
@@ -17539,40 +18005,96 @@
       <c r="A35" s="5" t="n">
         <v>32</v>
       </c>
-      <c r="B35" s="6" t="inlineStr"/>
-      <c r="C35" s="6" t="inlineStr"/>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>재이 입버릇</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>치즈 냄새 극혐!</t>
+        </is>
+      </c>
       <c r="D35" s="6" t="inlineStr"/>
-      <c r="E35" s="6" t="inlineStr"/>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>치즈만 보면 (냄새는 더더욱)</t>
+        </is>
+      </c>
       <c r="F35" s="6" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="B36" s="4" t="inlineStr"/>
-      <c r="C36" s="4" t="inlineStr"/>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>재이 입버릇</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>김태오!</t>
+        </is>
+      </c>
       <c r="D36" s="4" t="inlineStr"/>
-      <c r="E36" s="4" t="inlineStr"/>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+        </is>
+      </c>
       <c r="F36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n">
         <v>34</v>
       </c>
-      <c r="B37" s="6" t="inlineStr"/>
-      <c r="C37" s="6" t="inlineStr"/>
-      <c r="D37" s="6" t="inlineStr"/>
-      <c r="E37" s="6" t="inlineStr"/>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>짐방</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>김서방</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+        </is>
+      </c>
       <c r="F37" s="6" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="B38" s="4" t="inlineStr"/>
-      <c r="C38" s="4" t="inlineStr"/>
-      <c r="D38" s="4" t="inlineStr"/>
-      <c r="E38" s="4" t="inlineStr"/>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>꿍끙이</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>뿡뿡이</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+        </is>
+      </c>
       <c r="F38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
@@ -17685,8 +18207,48 @@
       <c r="E49" s="6" t="inlineStr"/>
       <c r="F49" s="6" t="inlineStr"/>
     </row>
+    <row r="50">
+      <c r="A50" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="B50" s="4" t="inlineStr"/>
+      <c r="C50" s="4" t="inlineStr"/>
+      <c r="D50" s="4" t="inlineStr"/>
+      <c r="E50" s="4" t="inlineStr"/>
+      <c r="F50" s="4" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B51" s="6" t="inlineStr"/>
+      <c r="C51" s="6" t="inlineStr"/>
+      <c r="D51" s="6" t="inlineStr"/>
+      <c r="E51" s="6" t="inlineStr"/>
+      <c r="F51" s="6" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="B52" s="4" t="inlineStr"/>
+      <c r="C52" s="4" t="inlineStr"/>
+      <c r="D52" s="4" t="inlineStr"/>
+      <c r="E52" s="4" t="inlineStr"/>
+      <c r="F52" s="4" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="B53" s="6" t="inlineStr"/>
+      <c r="C53" s="6" t="inlineStr"/>
+      <c r="D53" s="6" t="inlineStr"/>
+      <c r="E53" s="6" t="inlineStr"/>
+      <c r="F53" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F49"/>
+  <autoFilter ref="A3:F53"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add Taeo's Dinoster skill chant to the Taeo dictionary
New words 발싸 and the Dinoster skill names (안킬로해머, 스밀로클로, ...),
the 지앗차/이앗차 variants of his battle cry, and the full chant as a
daily saying. Ignore taeo-voice/ so raw recordings of the kids stay
off the public repo.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -18,8 +18,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$448</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16388,7 +16388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -16906,7 +16906,7 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>치앗촤 · 지앗 · 치앗차</t>
+          <t>치앗촤 · 지앗 · 치앗차 · 지앗차 · 이앗차</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -17058,9 +17058,21 @@
       <c r="A32" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="B32" s="4" t="inlineStr"/>
-      <c r="C32" s="4" t="inlineStr"/>
-      <c r="D32" s="4" t="inlineStr"/>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>발싸</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>발사</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>“스밀로클로 발싸!” 기술을 쏠 때</t>
+        </is>
+      </c>
       <c r="E32" s="4" t="inlineStr"/>
       <c r="F32" s="4" t="inlineStr"/>
     </row>
@@ -17068,9 +17080,21 @@
       <c r="A33" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="B33" s="6" t="inlineStr"/>
-      <c r="C33" s="6" t="inlineStr"/>
-      <c r="D33" s="6" t="inlineStr"/>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>안킬로해머 · 스밀로클로</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>다이노스터 기술</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>래터킥, 퀀텀해로우… 하나씩 외치고 “쓰구미~”</t>
+        </is>
+      </c>
       <c r="E33" s="6" t="inlineStr"/>
       <c r="F33" s="6" t="inlineStr"/>
     </row>
@@ -17254,8 +17278,28 @@
       <c r="E51" s="6" t="inlineStr"/>
       <c r="F51" s="6" t="inlineStr"/>
     </row>
+    <row r="52">
+      <c r="A52" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="B52" s="4" t="inlineStr"/>
+      <c r="C52" s="4" t="inlineStr"/>
+      <c r="D52" s="4" t="inlineStr"/>
+      <c r="E52" s="4" t="inlineStr"/>
+      <c r="F52" s="4" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="B53" s="6" t="inlineStr"/>
+      <c r="C53" s="6" t="inlineStr"/>
+      <c r="D53" s="6" t="inlineStr"/>
+      <c r="E53" s="6" t="inlineStr"/>
+      <c r="F53" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F51"/>
+  <autoFilter ref="A3:F53"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -17269,7 +17313,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -17594,13 +17638,13 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>싸우자! 타노스 나와라!</t>
+          <t>지앗차 지앗촤 쓰구미~ 래터킥 냅터킥 쓰구미~ 안킬로해머 스윔 쓰구미! 스밀로클로 발싸!</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr"/>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>제일 좋아하는 놀이, 어벤져스로 타노스랑 싸우기 (타노스는 늘 아빠, 건틀렛 끼고 “아임 인에비터블”)</t>
+          <t>다이노스터 기술을 줄줄이 외칠 때 (한 번 시작하면 1분 넘게)</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr"/>
@@ -17616,13 +17660,13 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>너라고 하지 마라! 나도 엄마 아빠한테 너라고 한다!</t>
+          <t>싸우자! 타노스 나와라!</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr"/>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>“너 엄마 아빠 말 잘 들어” 소리를 들으면</t>
+          <t>제일 좋아하는 놀이, 어벤져스로 타노스랑 싸우기 (타노스는 늘 아빠, 건틀렛 끼고 “아임 인에비터블”)</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr"/>
@@ -17638,13 +17682,13 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>재이 아니야! 재이 누나야!</t>
+          <t>너라고 하지 마라! 나도 엄마 아빠한테 너라고 한다!</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr"/>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>누가 누나를 “재이야” 하고 부르면 (모든 호칭은 태오 기준)</t>
+          <t>“너 엄마 아빠 말 잘 들어” 소리를 들으면</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr"/>
@@ -17660,13 +17704,13 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>이 안 닦아! 싫어!</t>
+          <t>재이 아니야! 재이 누나야!</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr"/>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>아침저녁 이 닦을 때 (도망 다니고 바닥을 기어요)</t>
+          <t>누가 누나를 “재이야” 하고 부르면 (모든 호칭은 태오 기준)</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr"/>
@@ -17682,13 +17726,13 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>누나 대단해!</t>
+          <t>이 안 닦아! 싫어!</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr"/>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>누나가 잠수를 보여 줬을 때</t>
+          <t>아침저녁 이 닦을 때 (도망 다니고 바닥을 기어요)</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr"/>
@@ -17704,13 +17748,13 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>엄마 인누와~</t>
+          <t>누나 대단해!</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr"/>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>밤에 자다 깨서 (엄마가 옆에서 재워 줄 때까지)</t>
+          <t>누나가 잠수를 보여 줬을 때</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr"/>
@@ -17726,13 +17770,13 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>왜 놀려! 놀리지 마!</t>
+          <t>엄마 인누와~</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr"/>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>“태오는 글씨·숫자 잘 몰라” 소리를 들으면 (손가락질하며)</t>
+          <t>밤에 자다 깨서 (엄마가 옆에서 재워 줄 때까지)</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr"/>
@@ -17748,13 +17792,13 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>왜 내 친구를 놀려! 슬프잖아!</t>
+          <t>왜 놀려! 놀리지 마!</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr"/>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>어린이집 친구가 놀림 받는 것 같을 때 (친구 편이에요)</t>
+          <t>“태오는 글씨·숫자 잘 몰라” 소리를 들으면 (손가락질하며)</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr"/>
@@ -17770,13 +17814,13 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>나 무지개빛 망토 갖고 싶어!</t>
+          <t>왜 내 친구를 놀려! 슬프잖아!</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr"/>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>파라큘라를 본 날부터 (또봇 Y도 같이 갖고 싶어요!)</t>
+          <t>어린이집 친구가 놀림 받는 것 같을 때 (친구 편이에요)</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr"/>
@@ -17792,13 +17836,13 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>어벤져스… 어셈블!</t>
+          <t>나 무지개빛 망토 갖고 싶어!</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr"/>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>엔드게임 마지막 장면을 따라 하며 가족을 다 모을 때</t>
+          <t>파라큘라를 본 날부터 (또봇 Y도 같이 갖고 싶어요!)</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr"/>
@@ -17814,13 +17858,13 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>왓 두 유 두, 캡틴? 위 파이트!</t>
+          <t>어벤져스… 어셈블!</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr"/>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>시빌 워 싸움 장면 놀이를 할 때</t>
+          <t>엔드게임 마지막 장면을 따라 하며 가족을 다 모을 때</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr"/>
@@ -17836,13 +17880,13 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>와칸다 포에버!</t>
+          <t>왓 두 유 두, 캡틴? 위 파이트!</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr"/>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>인피니티 워 장면처럼 다 같이 뛰어갈 때</t>
+          <t>시빌 워 싸움 장면 놀이를 할 때</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr"/>
@@ -17858,13 +17902,13 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>어린이집에 데리러 올 거야?</t>
+          <t>와칸다 포에버!</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr"/>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>어린이집 가기 싫은 아침에 (몇 번씩 확인해요)</t>
+          <t>인피니티 워 장면처럼 다 같이 뛰어갈 때</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr"/>
@@ -17880,13 +17924,13 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>어린이집 가기 싫다.</t>
+          <t>어린이집에 데리러 올 거야?</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr"/>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>월·화·수… 아침마다</t>
+          <t>어린이집 가기 싫은 아침에 (몇 번씩 확인해요)</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr"/>
@@ -17902,13 +17946,13 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?</t>
+          <t>어린이집 가기 싫다.</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr"/>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>싫은 태권도 가는 날</t>
+          <t>월·화·수… 아침마다</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr"/>
@@ -17924,13 +17968,13 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>오늘은 뽀로로 날! 내가 싫어하는 태권도 안 가는 날이다~</t>
+          <t>누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr"/>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>월요일 아침 (달력은 몰라도 뽀로로 날은 정확히 알아요)</t>
+          <t>싫은 태권도 가는 날</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr"/>
@@ -17941,18 +17985,18 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>아니야!</t>
+          <t>오늘은 뽀로로 날! 내가 싫어하는 태권도 안 가는 날이다~</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr"/>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>하루에도 제일 많이 하는 말</t>
+          <t>월요일 아침 (달력은 몰라도 뽀로로 날은 정확히 알아요)</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr"/>
@@ -17968,13 +18012,13 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>거짓말! 아니야!</t>
+          <t>아니야!</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr"/>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>기분 나쁘거나 하기 싫을 때</t>
+          <t>하루에도 제일 많이 하는 말</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr"/>
@@ -17990,13 +18034,13 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>맛있는데 지금은 먹기 싫어.</t>
+          <t>거짓말! 아니야!</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr"/>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>누가 음식을 권하면</t>
+          <t>기분 나쁘거나 하기 싫을 때</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr"/>
@@ -18012,13 +18056,13 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>치즈 냄새 극혐!</t>
+          <t>맛있는데 지금은 먹기 싫어.</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr"/>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>치즈만 보면 (냄새는 더더욱)</t>
+          <t>누가 음식을 권하면</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr"/>
@@ -18034,13 +18078,13 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>김태오!</t>
+          <t>치즈 냄새 극혐!</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr"/>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+          <t>치즈만 보면 (냄새는 더더욱)</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr"/>
@@ -18051,22 +18095,18 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>짐방</t>
-        </is>
-      </c>
-      <c r="D37" s="6" t="inlineStr">
-        <is>
-          <t>김서방</t>
-        </is>
-      </c>
+          <t>김태오!</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr"/>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr"/>
@@ -18082,17 +18122,17 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>꿍끙이</t>
+          <t>짐방</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>뿡뿡이</t>
+          <t>김서방</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr"/>
@@ -18101,10 +18141,26 @@
       <c r="A39" s="5" t="n">
         <v>36</v>
       </c>
-      <c r="B39" s="6" t="inlineStr"/>
-      <c r="C39" s="6" t="inlineStr"/>
-      <c r="D39" s="6" t="inlineStr"/>
-      <c r="E39" s="6" t="inlineStr"/>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>꿍끙이</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>뿡뿡이</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+        </is>
+      </c>
       <c r="F39" s="6" t="inlineStr"/>
     </row>
     <row r="40">
@@ -18247,8 +18303,18 @@
       <c r="E53" s="6" t="inlineStr"/>
       <c r="F53" s="6" t="inlineStr"/>
     </row>
+    <row r="54">
+      <c r="A54" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="B54" s="4" t="inlineStr"/>
+      <c r="C54" s="4" t="inlineStr"/>
+      <c r="D54" s="4" t="inlineStr"/>
+      <c r="E54" s="4" t="inlineStr"/>
+      <c r="F54" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F53"/>
+  <autoFilter ref="A3:F54"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add Taeo's Dinoster chants and card-game wishes to the games
Taeo dictionary: 다이아 (가이아) and his two card-game wishes.
Multiverse: Taeo's special shows a random Dinoster chant under his cry.
Sanguo: Taeo's bio mentions the chant. Cards: Taeo chants in the
intro scene (no extra line, scene length rule kept).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -18,8 +18,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$448</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16388,7 +16388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -17060,17 +17060,17 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>발싸</t>
+          <t>다이아</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>발사</t>
+          <t>가이아</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>“스밀로클로 발싸!” 기술을 쏠 때</t>
+          <t>그리스 로마 신화 카드게임에서 별 15개로 제일 센 카드. “다이아 제발!”</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr"/>
@@ -17082,17 +17082,17 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>안킬로해머 · 스밀로클로</t>
+          <t>발싸</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>다이노스터 기술</t>
+          <t>발사</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>래터킥, 퀀텀해로우… 하나씩 외치고 “쓰구미~”</t>
+          <t>“스밀로클로 발싸!” 기술을 쏠 때</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr"/>
@@ -17102,9 +17102,21 @@
       <c r="A34" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="B34" s="4" t="inlineStr"/>
-      <c r="C34" s="4" t="inlineStr"/>
-      <c r="D34" s="4" t="inlineStr"/>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>안킬로해머 · 스밀로클로</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>다이노스터 기술</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>래터킥, 퀀텀해로우… 하나씩 외치고 “쓰구미~”</t>
+        </is>
+      </c>
       <c r="E34" s="4" t="inlineStr"/>
       <c r="F34" s="4" t="inlineStr"/>
     </row>
@@ -17298,8 +17310,18 @@
       <c r="E53" s="6" t="inlineStr"/>
       <c r="F53" s="6" t="inlineStr"/>
     </row>
+    <row r="54">
+      <c r="A54" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="B54" s="4" t="inlineStr"/>
+      <c r="C54" s="4" t="inlineStr"/>
+      <c r="D54" s="4" t="inlineStr"/>
+      <c r="E54" s="4" t="inlineStr"/>
+      <c r="F54" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F53"/>
+  <autoFilter ref="A3:F54"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -17313,7 +17335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -17660,13 +17682,13 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>싸우자! 타노스 나와라!</t>
+          <t>다이아 제발!</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr"/>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>제일 좋아하는 놀이, 어벤져스로 타노스랑 싸우기 (타노스는 늘 아빠, 건틀렛 끼고 “아임 인에비터블”)</t>
+          <t>그리스 로마 신화 카드게임에서 별 15개짜리 제일 센 가이아 카드가 나오길 빌 때</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr"/>
@@ -17682,13 +17704,13 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>너라고 하지 마라! 나도 엄마 아빠한테 너라고 한다!</t>
+          <t>제발 오로라핑! 양핑은 싫어!</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr"/>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>“너 엄마 아빠 말 잘 들어” 소리를 들으면</t>
+          <t>티니핑 원카드에서 조커처럼 쓰는 오로라핑 카드를 간절히 기다릴 때</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr"/>
@@ -17704,13 +17726,13 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>재이 아니야! 재이 누나야!</t>
+          <t>싸우자! 타노스 나와라!</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr"/>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>누가 누나를 “재이야” 하고 부르면 (모든 호칭은 태오 기준)</t>
+          <t>제일 좋아하는 놀이, 어벤져스로 타노스랑 싸우기 (타노스는 늘 아빠, 건틀렛 끼고 “아임 인에비터블”)</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr"/>
@@ -17726,13 +17748,13 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>이 안 닦아! 싫어!</t>
+          <t>너라고 하지 마라! 나도 엄마 아빠한테 너라고 한다!</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr"/>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>아침저녁 이 닦을 때 (도망 다니고 바닥을 기어요)</t>
+          <t>“너 엄마 아빠 말 잘 들어” 소리를 들으면</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr"/>
@@ -17748,13 +17770,13 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>누나 대단해!</t>
+          <t>재이 아니야! 재이 누나야!</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr"/>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>누나가 잠수를 보여 줬을 때</t>
+          <t>누가 누나를 “재이야” 하고 부르면 (모든 호칭은 태오 기준)</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr"/>
@@ -17770,13 +17792,13 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>엄마 인누와~</t>
+          <t>이 안 닦아! 싫어!</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr"/>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>밤에 자다 깨서 (엄마가 옆에서 재워 줄 때까지)</t>
+          <t>아침저녁 이 닦을 때 (도망 다니고 바닥을 기어요)</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr"/>
@@ -17792,13 +17814,13 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>왜 놀려! 놀리지 마!</t>
+          <t>누나 대단해!</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr"/>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>“태오는 글씨·숫자 잘 몰라” 소리를 들으면 (손가락질하며)</t>
+          <t>누나가 잠수를 보여 줬을 때</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr"/>
@@ -17814,13 +17836,13 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>왜 내 친구를 놀려! 슬프잖아!</t>
+          <t>엄마 인누와~</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr"/>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>어린이집 친구가 놀림 받는 것 같을 때 (친구 편이에요)</t>
+          <t>밤에 자다 깨서 (엄마가 옆에서 재워 줄 때까지)</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr"/>
@@ -17836,13 +17858,13 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>나 무지개빛 망토 갖고 싶어!</t>
+          <t>왜 놀려! 놀리지 마!</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr"/>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>파라큘라를 본 날부터 (또봇 Y도 같이 갖고 싶어요!)</t>
+          <t>“태오는 글씨·숫자 잘 몰라” 소리를 들으면 (손가락질하며)</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr"/>
@@ -17858,13 +17880,13 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>어벤져스… 어셈블!</t>
+          <t>왜 내 친구를 놀려! 슬프잖아!</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr"/>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>엔드게임 마지막 장면을 따라 하며 가족을 다 모을 때</t>
+          <t>어린이집 친구가 놀림 받는 것 같을 때 (친구 편이에요)</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr"/>
@@ -17880,13 +17902,13 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>왓 두 유 두, 캡틴? 위 파이트!</t>
+          <t>나 무지개빛 망토 갖고 싶어!</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr"/>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>시빌 워 싸움 장면 놀이를 할 때</t>
+          <t>파라큘라를 본 날부터 (또봇 Y도 같이 갖고 싶어요!)</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr"/>
@@ -17902,13 +17924,13 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>와칸다 포에버!</t>
+          <t>어벤져스… 어셈블!</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr"/>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>인피니티 워 장면처럼 다 같이 뛰어갈 때</t>
+          <t>엔드게임 마지막 장면을 따라 하며 가족을 다 모을 때</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr"/>
@@ -17924,13 +17946,13 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>어린이집에 데리러 올 거야?</t>
+          <t>왓 두 유 두, 캡틴? 위 파이트!</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr"/>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>어린이집 가기 싫은 아침에 (몇 번씩 확인해요)</t>
+          <t>시빌 워 싸움 장면 놀이를 할 때</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr"/>
@@ -17946,13 +17968,13 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>어린이집 가기 싫다.</t>
+          <t>와칸다 포에버!</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr"/>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>월·화·수… 아침마다</t>
+          <t>인피니티 워 장면처럼 다 같이 뛰어갈 때</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr"/>
@@ -17968,13 +17990,13 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?</t>
+          <t>어린이집에 데리러 올 거야?</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr"/>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>싫은 태권도 가는 날</t>
+          <t>어린이집 가기 싫은 아침에 (몇 번씩 확인해요)</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr"/>
@@ -17990,13 +18012,13 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>오늘은 뽀로로 날! 내가 싫어하는 태권도 안 가는 날이다~</t>
+          <t>어린이집 가기 싫다.</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr"/>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>월요일 아침 (달력은 몰라도 뽀로로 날은 정확히 알아요)</t>
+          <t>월·화·수… 아침마다</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr"/>
@@ -18007,18 +18029,18 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>아니야!</t>
+          <t>누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr"/>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>하루에도 제일 많이 하는 말</t>
+          <t>싫은 태권도 가는 날</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr"/>
@@ -18029,18 +18051,18 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>거짓말! 아니야!</t>
+          <t>오늘은 뽀로로 날! 내가 싫어하는 태권도 안 가는 날이다~</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr"/>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>기분 나쁘거나 하기 싫을 때</t>
+          <t>월요일 아침 (달력은 몰라도 뽀로로 날은 정확히 알아요)</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr"/>
@@ -18056,13 +18078,13 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>맛있는데 지금은 먹기 싫어.</t>
+          <t>아니야!</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr"/>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>누가 음식을 권하면</t>
+          <t>하루에도 제일 많이 하는 말</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr"/>
@@ -18078,13 +18100,13 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>치즈 냄새 극혐!</t>
+          <t>거짓말! 아니야!</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr"/>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>치즈만 보면 (냄새는 더더욱)</t>
+          <t>기분 나쁘거나 하기 싫을 때</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr"/>
@@ -18100,13 +18122,13 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>김태오!</t>
+          <t>맛있는데 지금은 먹기 싫어.</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr"/>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+          <t>누가 음식을 권하면</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr"/>
@@ -18117,22 +18139,18 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>짐방</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>김서방</t>
-        </is>
-      </c>
+          <t>치즈 냄새 극혐!</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr"/>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+          <t>치즈만 보면 (냄새는 더더욱)</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr"/>
@@ -18143,22 +18161,18 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>꿍끙이</t>
-        </is>
-      </c>
-      <c r="D39" s="6" t="inlineStr">
-        <is>
-          <t>뿡뿡이</t>
-        </is>
-      </c>
+          <t>김태오!</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr"/>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr"/>
@@ -18167,20 +18181,52 @@
       <c r="A40" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="B40" s="4" t="inlineStr"/>
-      <c r="C40" s="4" t="inlineStr"/>
-      <c r="D40" s="4" t="inlineStr"/>
-      <c r="E40" s="4" t="inlineStr"/>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>짐방</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>김서방</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+        </is>
+      </c>
       <c r="F40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="B41" s="6" t="inlineStr"/>
-      <c r="C41" s="6" t="inlineStr"/>
-      <c r="D41" s="6" t="inlineStr"/>
-      <c r="E41" s="6" t="inlineStr"/>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>꿍끙이</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>뿡뿡이</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+        </is>
+      </c>
       <c r="F41" s="6" t="inlineStr"/>
     </row>
     <row r="42">
@@ -18313,8 +18359,28 @@
       <c r="E54" s="4" t="inlineStr"/>
       <c r="F54" s="4" t="inlineStr"/>
     </row>
+    <row r="55">
+      <c r="A55" s="5" t="n">
+        <v>52</v>
+      </c>
+      <c r="B55" s="6" t="inlineStr"/>
+      <c r="C55" s="6" t="inlineStr"/>
+      <c r="D55" s="6" t="inlineStr"/>
+      <c r="E55" s="6" t="inlineStr"/>
+      <c r="F55" s="6" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="n">
+        <v>53</v>
+      </c>
+      <c r="B56" s="4" t="inlineStr"/>
+      <c r="C56" s="4" t="inlineStr"/>
+      <c r="D56" s="4" t="inlineStr"/>
+      <c r="E56" s="4" t="inlineStr"/>
+      <c r="F56" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F54"/>
+  <autoFilter ref="A3:F56"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add 콩콩이차 and 둔쫀떡 to the Taeo dictionary, plus a mood-day episode idea
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -18,9 +18,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$448</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$54</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$56</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -16388,7 +16388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -17082,17 +17082,17 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>발싸</t>
+          <t>콩콩이차</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>발사</t>
+          <t>아우디 (자동차)</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>“스밀로클로 발싸!” 기술을 쏠 때</t>
+          <t>아우디 동그라미 로고를 보고. “나도 콩콩이차 타고 싶다~”</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr"/>
@@ -17104,17 +17104,17 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>안킬로해머 · 스밀로클로</t>
+          <t>둔쫀떡</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>다이노스터 기술</t>
+          <t>두바이 쫀득 찹쌀떡</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>래터킥, 퀀텀해로우… 하나씩 외치고 “쓰구미~”</t>
+          <t>아침에 먹으면 하루 종일 기분이 좋아져요</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr"/>
@@ -17124,9 +17124,21 @@
       <c r="A35" s="5" t="n">
         <v>32</v>
       </c>
-      <c r="B35" s="6" t="inlineStr"/>
-      <c r="C35" s="6" t="inlineStr"/>
-      <c r="D35" s="6" t="inlineStr"/>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>발싸</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>발사</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>“스밀로클로 발싸!” 기술을 쏠 때</t>
+        </is>
+      </c>
       <c r="E35" s="6" t="inlineStr"/>
       <c r="F35" s="6" t="inlineStr"/>
     </row>
@@ -17134,9 +17146,21 @@
       <c r="A36" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="B36" s="4" t="inlineStr"/>
-      <c r="C36" s="4" t="inlineStr"/>
-      <c r="D36" s="4" t="inlineStr"/>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>안킬로해머 · 스밀로클로</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>다이노스터 기술</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>래터킥, 퀀텀해로우… 하나씩 외치고 “쓰구미~”</t>
+        </is>
+      </c>
       <c r="E36" s="4" t="inlineStr"/>
       <c r="F36" s="4" t="inlineStr"/>
     </row>
@@ -17320,8 +17344,28 @@
       <c r="E54" s="4" t="inlineStr"/>
       <c r="F54" s="4" t="inlineStr"/>
     </row>
+    <row r="55">
+      <c r="A55" s="5" t="n">
+        <v>52</v>
+      </c>
+      <c r="B55" s="6" t="inlineStr"/>
+      <c r="C55" s="6" t="inlineStr"/>
+      <c r="D55" s="6" t="inlineStr"/>
+      <c r="E55" s="6" t="inlineStr"/>
+      <c r="F55" s="6" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="n">
+        <v>53</v>
+      </c>
+      <c r="B56" s="4" t="inlineStr"/>
+      <c r="C56" s="4" t="inlineStr"/>
+      <c r="D56" s="4" t="inlineStr"/>
+      <c r="E56" s="4" t="inlineStr"/>
+      <c r="F56" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F54"/>
+  <autoFilter ref="A3:F56"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -17335,7 +17379,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -17682,13 +17726,13 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>다이아 제발!</t>
+          <t>나도 콩콩이차 타고 싶다~</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr"/>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>그리스 로마 신화 카드게임에서 별 15개짜리 제일 센 가이아 카드가 나오길 빌 때</t>
+          <t>길에서 아우디 로고를 보면</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr"/>
@@ -17704,13 +17748,13 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>제발 오로라핑! 양핑은 싫어!</t>
+          <t>다이아 제발!</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr"/>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>티니핑 원카드에서 조커처럼 쓰는 오로라핑 카드를 간절히 기다릴 때</t>
+          <t>그리스 로마 신화 카드게임에서 별 15개짜리 제일 센 가이아 카드가 나오길 빌 때</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr"/>
@@ -17726,13 +17770,13 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>싸우자! 타노스 나와라!</t>
+          <t>제발 오로라핑! 양핑은 싫어!</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr"/>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>제일 좋아하는 놀이, 어벤져스로 타노스랑 싸우기 (타노스는 늘 아빠, 건틀렛 끼고 “아임 인에비터블”)</t>
+          <t>티니핑 원카드에서 조커처럼 쓰는 오로라핑 카드를 간절히 기다릴 때</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr"/>
@@ -17748,13 +17792,13 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>너라고 하지 마라! 나도 엄마 아빠한테 너라고 한다!</t>
+          <t>싸우자! 타노스 나와라!</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr"/>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>“너 엄마 아빠 말 잘 들어” 소리를 들으면</t>
+          <t>제일 좋아하는 놀이, 어벤져스로 타노스랑 싸우기 (타노스는 늘 아빠, 건틀렛 끼고 “아임 인에비터블”)</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr"/>
@@ -17770,13 +17814,13 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>재이 아니야! 재이 누나야!</t>
+          <t>너라고 하지 마라! 나도 엄마 아빠한테 너라고 한다!</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr"/>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>누가 누나를 “재이야” 하고 부르면 (모든 호칭은 태오 기준)</t>
+          <t>“너 엄마 아빠 말 잘 들어” 소리를 들으면</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr"/>
@@ -17792,13 +17836,13 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>이 안 닦아! 싫어!</t>
+          <t>재이 아니야! 재이 누나야!</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr"/>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>아침저녁 이 닦을 때 (도망 다니고 바닥을 기어요)</t>
+          <t>누가 누나를 “재이야” 하고 부르면 (모든 호칭은 태오 기준)</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr"/>
@@ -17814,13 +17858,13 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>누나 대단해!</t>
+          <t>이 안 닦아! 싫어!</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr"/>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>누나가 잠수를 보여 줬을 때</t>
+          <t>아침저녁 이 닦을 때 (도망 다니고 바닥을 기어요)</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr"/>
@@ -17836,13 +17880,13 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>엄마 인누와~</t>
+          <t>누나 대단해!</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr"/>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>밤에 자다 깨서 (엄마가 옆에서 재워 줄 때까지)</t>
+          <t>누나가 잠수를 보여 줬을 때</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr"/>
@@ -17858,13 +17902,13 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>왜 놀려! 놀리지 마!</t>
+          <t>엄마 인누와~</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr"/>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>“태오는 글씨·숫자 잘 몰라” 소리를 들으면 (손가락질하며)</t>
+          <t>밤에 자다 깨서 (엄마가 옆에서 재워 줄 때까지)</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr"/>
@@ -17880,13 +17924,13 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>왜 내 친구를 놀려! 슬프잖아!</t>
+          <t>왜 놀려! 놀리지 마!</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr"/>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>어린이집 친구가 놀림 받는 것 같을 때 (친구 편이에요)</t>
+          <t>“태오는 글씨·숫자 잘 몰라” 소리를 들으면 (손가락질하며)</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr"/>
@@ -17902,13 +17946,13 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>나 무지개빛 망토 갖고 싶어!</t>
+          <t>왜 내 친구를 놀려! 슬프잖아!</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr"/>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>파라큘라를 본 날부터 (또봇 Y도 같이 갖고 싶어요!)</t>
+          <t>어린이집 친구가 놀림 받는 것 같을 때 (친구 편이에요)</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr"/>
@@ -17924,13 +17968,13 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>어벤져스… 어셈블!</t>
+          <t>나 무지개빛 망토 갖고 싶어!</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr"/>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>엔드게임 마지막 장면을 따라 하며 가족을 다 모을 때</t>
+          <t>파라큘라를 본 날부터 (또봇 Y도 같이 갖고 싶어요!)</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr"/>
@@ -17946,13 +17990,13 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>왓 두 유 두, 캡틴? 위 파이트!</t>
+          <t>어벤져스… 어셈블!</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr"/>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>시빌 워 싸움 장면 놀이를 할 때</t>
+          <t>엔드게임 마지막 장면을 따라 하며 가족을 다 모을 때</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr"/>
@@ -17968,13 +18012,13 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>와칸다 포에버!</t>
+          <t>왓 두 유 두, 캡틴? 위 파이트!</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr"/>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>인피니티 워 장면처럼 다 같이 뛰어갈 때</t>
+          <t>시빌 워 싸움 장면 놀이를 할 때</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr"/>
@@ -17990,13 +18034,13 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>어린이집에 데리러 올 거야?</t>
+          <t>와칸다 포에버!</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr"/>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>어린이집 가기 싫은 아침에 (몇 번씩 확인해요)</t>
+          <t>인피니티 워 장면처럼 다 같이 뛰어갈 때</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr"/>
@@ -18012,13 +18056,13 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>어린이집 가기 싫다.</t>
+          <t>어린이집에 데리러 올 거야?</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr"/>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>월·화·수… 아침마다</t>
+          <t>어린이집 가기 싫은 아침에 (몇 번씩 확인해요)</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr"/>
@@ -18034,13 +18078,13 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?</t>
+          <t>어린이집 가기 싫다.</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr"/>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>싫은 태권도 가는 날</t>
+          <t>월·화·수… 아침마다</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr"/>
@@ -18056,13 +18100,13 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>오늘은 뽀로로 날! 내가 싫어하는 태권도 안 가는 날이다~</t>
+          <t>누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr"/>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>월요일 아침 (달력은 몰라도 뽀로로 날은 정확히 알아요)</t>
+          <t>싫은 태권도 가는 날</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr"/>
@@ -18073,18 +18117,18 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>아니야!</t>
+          <t>오늘은 뽀로로 날! 내가 싫어하는 태권도 안 가는 날이다~</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr"/>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>하루에도 제일 많이 하는 말</t>
+          <t>월요일 아침 (달력은 몰라도 뽀로로 날은 정확히 알아요)</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr"/>
@@ -18100,13 +18144,13 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>거짓말! 아니야!</t>
+          <t>아니야!</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr"/>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>기분 나쁘거나 하기 싫을 때</t>
+          <t>하루에도 제일 많이 하는 말</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr"/>
@@ -18122,13 +18166,13 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>맛있는데 지금은 먹기 싫어.</t>
+          <t>거짓말! 아니야!</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr"/>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>누가 음식을 권하면</t>
+          <t>기분 나쁘거나 하기 싫을 때</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr"/>
@@ -18144,13 +18188,13 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>치즈 냄새 극혐!</t>
+          <t>맛있는데 지금은 먹기 싫어.</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr"/>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>치즈만 보면 (냄새는 더더욱)</t>
+          <t>누가 음식을 권하면</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr"/>
@@ -18166,13 +18210,13 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>김태오!</t>
+          <t>치즈 냄새 극혐!</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr"/>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+          <t>치즈만 보면 (냄새는 더더욱)</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr"/>
@@ -18183,22 +18227,18 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>짐방</t>
-        </is>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>김서방</t>
-        </is>
-      </c>
+          <t>김태오!</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr"/>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr"/>
@@ -18214,17 +18254,17 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>꿍끙이</t>
+          <t>짐방</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>뿡뿡이</t>
+          <t>김서방</t>
         </is>
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr"/>
@@ -18233,10 +18273,26 @@
       <c r="A42" s="3" t="n">
         <v>39</v>
       </c>
-      <c r="B42" s="4" t="inlineStr"/>
-      <c r="C42" s="4" t="inlineStr"/>
-      <c r="D42" s="4" t="inlineStr"/>
-      <c r="E42" s="4" t="inlineStr"/>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>꿍끙이</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>뿡뿡이</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+        </is>
+      </c>
       <c r="F42" s="4" t="inlineStr"/>
     </row>
     <row r="43">
@@ -18379,8 +18435,18 @@
       <c r="E56" s="4" t="inlineStr"/>
       <c r="F56" s="4" t="inlineStr"/>
     </row>
+    <row r="57">
+      <c r="A57" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="B57" s="6" t="inlineStr"/>
+      <c r="C57" s="6" t="inlineStr"/>
+      <c r="D57" s="6" t="inlineStr"/>
+      <c r="E57" s="6" t="inlineStr"/>
+      <c r="F57" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F56"/>
+  <autoFilter ref="A3:F57"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -18399,7 +18465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -18575,11 +18641,31 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr"/>
-      <c r="B9" s="6" t="inlineStr"/>
-      <c r="C9" s="6" t="inlineStr"/>
-      <c r="D9" s="6" t="inlineStr"/>
-      <c r="E9" s="6" t="inlineStr"/>
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>기분파 태오의 둔쫀떡 아침</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>(가족 제보) 아침에 둔쫀떡을 먹은 태오는 기분이 최고! 누나 학교 가는 길에 안아 달라는 말도 없이 빠른 걸음으로 씩씩하게 걷는다. 가다가 아우디 로고를 보고는 “콩콩이차다! 나도 콩콩이차 타고 싶다~”</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>작은 기쁨 하나가 하루를 씩씩하게 만들어요.</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>아이디어</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr"/>
@@ -18588,8 +18674,15 @@
       <c r="D10" s="4" t="inlineStr"/>
       <c r="E10" s="4" t="inlineStr"/>
     </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr"/>
+      <c r="B11" s="6" t="inlineStr"/>
+      <c r="C11" s="6" t="inlineStr"/>
+      <c r="D11" s="6" t="inlineStr"/>
+      <c r="E11" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:E10"/>
+  <autoFilter ref="A3:E11"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add webtoon episode 27: 둔쫀떡 먹은 날, 콩콩이차
New car and rings props, a morning street background, spreadsheet rows,
episode count in the hub card.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -16,8 +16,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$448</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$461</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$11</definedName>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2043,20 +2043,50 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="n">
+      <c r="A30" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="B30" s="7" t="n"/>
-      <c r="C30" s="7" t="n"/>
-      <c r="D30" s="7" t="n"/>
-      <c r="E30" s="7" t="n"/>
-      <c r="F30" s="7" t="n"/>
-      <c r="G30" s="7" t="n"/>
-      <c r="H30" s="7" t="n"/>
-      <c r="I30" s="7" t="n"/>
-      <c r="J30" s="7" t="inlineStr">
-        <is>
-          <t>기획 중</t>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>둔쫀떡 먹은 날, 콩콩이차</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>아침에 둔쫀떡을 먹은 태오는 기분이 하늘 끝까지! 누나 학교 가는 길에 안아 달라는 말도 없이 씽씽 걷다가, 동그라미 네 개 로고를 보고 외쳤다. “콩콩이차다!”</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>재이, 엄마, 태오</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>둔쫀떡 먹고 “맛있는 거 죠!” / 아우디 로고를 보고 “콩콩이차다!” “나도 콩콩이차 타고 싶다~” / 누나 학교 가는 길에 안아 달라는 말도 없이 빠른 걸음</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>기분이 좋으면 걸음도 가벼워지는 태오 / 누나·엄마와 콩콩콩 뛰어서 가는 아침</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>작은 기쁨 하나가 하루를 씩씩하게 만들어요. 기분 좋은 마음은 걸음도 가볍게 해 줘요.</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>오늘 아침 나를 기분 좋게 한 건 뭐였어요? 타 보고 싶은 차가 있나요?</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>완성</t>
         </is>
       </c>
     </row>
@@ -2096,13 +2126,31 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" s="7" t="n"/>
+      <c r="C33" s="7" t="n"/>
+      <c r="D33" s="7" t="n"/>
+      <c r="E33" s="7" t="n"/>
+      <c r="F33" s="7" t="n"/>
+      <c r="G33" s="7" t="n"/>
+      <c r="H33" s="7" t="n"/>
+      <c r="I33" s="7" t="n"/>
+      <c r="J33" s="7" t="inlineStr">
+        <is>
+          <t>기획 중</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:J29"/>
+  <autoFilter ref="A3:J30"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"아이디어,기획 중,콘티,완성"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2116,7 +2164,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H448"/>
+  <dimension ref="A1:H461"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -16373,8 +16421,430 @@
       <c r="G448" s="4" t="inlineStr"/>
       <c r="H448" s="4" t="inlineStr"/>
     </row>
+    <row r="449">
+      <c r="A449" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="B449" s="6" t="inlineStr">
+        <is>
+          <t>둔쫀떡 먹은 날, 콩콩이차</t>
+        </is>
+      </c>
+      <c r="C449" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D449" s="6" t="inlineStr">
+        <is>
+          <t>부엌</t>
+        </is>
+      </c>
+      <c r="E449" s="6" t="inlineStr">
+        <is>
+          <t>태오, 엄마</t>
+        </is>
+      </c>
+      <c r="F449" s="6" t="inlineStr">
+        <is>
+          <t>아침, 식탁 위에 둔쫀떡.</t>
+        </is>
+      </c>
+      <c r="G449" s="6" t="inlineStr">
+        <is>
+          <t>두바이 쫀득 찹쌀떡이야.</t>
+        </is>
+      </c>
+      <c r="H449" s="6" t="inlineStr"/>
+    </row>
+    <row r="450">
+      <c r="A450" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B450" s="4" t="inlineStr">
+        <is>
+          <t>둔쫀떡 먹은 날, 콩콩이차</t>
+        </is>
+      </c>
+      <c r="C450" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D450" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E450" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F450" s="4" t="inlineStr"/>
+      <c r="G450" s="4" t="inlineStr">
+        <is>
+          <t>둔쫀떡! 맛있는 거 죠!</t>
+        </is>
+      </c>
+      <c r="H450" s="4" t="inlineStr">
+        <is>
+          <t>쫀득쫀득</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="B451" s="6" t="inlineStr">
+        <is>
+          <t>둔쫀떡 먹은 날, 콩콩이차</t>
+        </is>
+      </c>
+      <c r="C451" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D451" s="6" t="inlineStr">
+        <is>
+          <t>현관</t>
+        </is>
+      </c>
+      <c r="E451" s="6" t="inlineStr">
+        <is>
+          <t>엄마, 태오, 재이</t>
+        </is>
+      </c>
+      <c r="F451" s="6" t="inlineStr">
+        <is>
+          <t>누나 학교 가는 시간.</t>
+        </is>
+      </c>
+      <c r="G451" s="6" t="inlineStr">
+        <is>
+          <t>태오야, 안아 줄까?
+안 안아도 돼!</t>
+        </is>
+      </c>
+      <c r="H451" s="6" t="inlineStr"/>
+    </row>
+    <row r="452">
+      <c r="A452" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B452" s="4" t="inlineStr">
+        <is>
+          <t>둔쫀떡 먹은 날, 콩콩이차</t>
+        </is>
+      </c>
+      <c r="C452" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D452" s="4" t="inlineStr">
+        <is>
+          <t>퇴근길</t>
+        </is>
+      </c>
+      <c r="E452" s="4" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="F452" s="4" t="inlineStr">
+        <is>
+          <t>그러더니 빠른 걸음으로 씽씽!</t>
+        </is>
+      </c>
+      <c r="G452" s="4" t="inlineStr">
+        <is>
+          <t>얼른 와~!</t>
+        </is>
+      </c>
+      <c r="H452" s="4" t="inlineStr">
+        <is>
+          <t>씽씽</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="B453" s="6" t="inlineStr">
+        <is>
+          <t>둔쫀떡 먹은 날, 콩콩이차</t>
+        </is>
+      </c>
+      <c r="C453" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D453" s="6" t="inlineStr">
+        <is>
+          <t>퇴근길</t>
+        </is>
+      </c>
+      <c r="E453" s="6" t="inlineStr">
+        <is>
+          <t>재이, 엄마</t>
+        </is>
+      </c>
+      <c r="F453" s="6" t="inlineStr"/>
+      <c r="G453" s="6" t="inlineStr">
+        <is>
+          <t>태오가 안아 달라는 말을 안 하네?
+둔쫀떡 효과인가 봐.</t>
+        </is>
+      </c>
+      <c r="H453" s="6" t="inlineStr"/>
+    </row>
+    <row r="454">
+      <c r="A454" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B454" s="4" t="inlineStr">
+        <is>
+          <t>둔쫀떡 먹은 날, 콩콩이차</t>
+        </is>
+      </c>
+      <c r="C454" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D454" s="4" t="inlineStr">
+        <is>
+          <t>퇴근길</t>
+        </is>
+      </c>
+      <c r="E454" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F454" s="4" t="inlineStr">
+        <is>
+          <t>기분파 태오, 오늘은 기분이 최고!</t>
+        </is>
+      </c>
+      <c r="G454" s="4" t="inlineStr">
+        <is>
+          <t>둔쫀떡 먹으니까 기분 좋다~</t>
+        </is>
+      </c>
+      <c r="H454" s="4" t="inlineStr"/>
+    </row>
+    <row r="455">
+      <c r="A455" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="B455" s="6" t="inlineStr">
+        <is>
+          <t>둔쫀떡 먹은 날, 콩콩이차</t>
+        </is>
+      </c>
+      <c r="C455" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="D455" s="6" t="inlineStr">
+        <is>
+          <t>퇴근길</t>
+        </is>
+      </c>
+      <c r="E455" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F455" s="6" t="inlineStr"/>
+      <c r="G455" s="6" t="inlineStr">
+        <is>
+          <t>어!! 저기 봐!</t>
+        </is>
+      </c>
+      <c r="H455" s="6" t="inlineStr">
+        <is>
+          <t>번쩍</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B456" s="4" t="inlineStr">
+        <is>
+          <t>둔쫀떡 먹은 날, 콩콩이차</t>
+        </is>
+      </c>
+      <c r="C456" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D456" s="4" t="inlineStr">
+        <is>
+          <t>단색</t>
+        </is>
+      </c>
+      <c r="E456" s="4" t="inlineStr"/>
+      <c r="F456" s="4" t="inlineStr">
+        <is>
+          <t>동그라미가 하나, 둘, 셋, 넷. / 차 앞에 달린 은빛 동그라미 로고.</t>
+        </is>
+      </c>
+      <c r="G456" s="4" t="inlineStr"/>
+      <c r="H456" s="4" t="inlineStr"/>
+    </row>
+    <row r="457">
+      <c r="A457" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="B457" s="6" t="inlineStr">
+        <is>
+          <t>둔쫀떡 먹은 날, 콩콩이차</t>
+        </is>
+      </c>
+      <c r="C457" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="D457" s="6" t="inlineStr">
+        <is>
+          <t>퇴근길</t>
+        </is>
+      </c>
+      <c r="E457" s="6" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="F457" s="6" t="inlineStr"/>
+      <c r="G457" s="6" t="inlineStr">
+        <is>
+          <t>콩콩이차다!!
+아우디야.</t>
+        </is>
+      </c>
+      <c r="H457" s="6" t="inlineStr"/>
+    </row>
+    <row r="458">
+      <c r="A458" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B458" s="4" t="inlineStr">
+        <is>
+          <t>둔쫀떡 먹은 날, 콩콩이차</t>
+        </is>
+      </c>
+      <c r="C458" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D458" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E458" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F458" s="4" t="inlineStr"/>
+      <c r="G458" s="4" t="inlineStr">
+        <is>
+          <t>나도 콩콩이차 타고 싶다~</t>
+        </is>
+      </c>
+      <c r="H458" s="4" t="inlineStr">
+        <is>
+          <t>콩콩</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="B459" s="6" t="inlineStr">
+        <is>
+          <t>둔쫀떡 먹은 날, 콩콩이차</t>
+        </is>
+      </c>
+      <c r="C459" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="D459" s="6" t="inlineStr">
+        <is>
+          <t>퇴근길</t>
+        </is>
+      </c>
+      <c r="E459" s="6" t="inlineStr">
+        <is>
+          <t>엄마, 재이</t>
+        </is>
+      </c>
+      <c r="F459" s="6" t="inlineStr"/>
+      <c r="G459" s="6" t="inlineStr">
+        <is>
+          <t>그럼 우리 오늘은 신나게 걸어서 갈까?
+콩콩콩 뛰는 차처럼!</t>
+        </is>
+      </c>
+      <c r="H459" s="6" t="inlineStr"/>
+    </row>
+    <row r="460">
+      <c r="A460" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B460" s="4" t="inlineStr">
+        <is>
+          <t>둔쫀떡 먹은 날, 콩콩이차</t>
+        </is>
+      </c>
+      <c r="C460" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D460" s="4" t="inlineStr">
+        <is>
+          <t>퇴근길</t>
+        </is>
+      </c>
+      <c r="E460" s="4" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="F460" s="4" t="inlineStr">
+        <is>
+          <t>콩콩, 콩콩!</t>
+        </is>
+      </c>
+      <c r="G460" s="4" t="inlineStr"/>
+      <c r="H460" s="4" t="inlineStr">
+        <is>
+          <t>콩콩콩</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="B461" s="6" t="inlineStr">
+        <is>
+          <t>둔쫀떡 먹은 날, 콩콩이차</t>
+        </is>
+      </c>
+      <c r="C461" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="D461" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E461" s="6" t="inlineStr"/>
+      <c r="F461" s="6" t="inlineStr">
+        <is>
+          <t>안아 달라는 말도 잊은 아침. / 작은 기쁨이 태오의 걸음을 가볍게 했다.</t>
+        </is>
+      </c>
+      <c r="G461" s="6" t="inlineStr"/>
+      <c r="H461" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:H448"/>
+  <autoFilter ref="A3:H461"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -18663,7 +19133,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>아이디어</t>
+          <t>완성</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Episode 27: mom is away on a business trip, dad walks them to school
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -2053,12 +2053,12 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>아침에 둔쫀떡을 먹은 태오는 기분이 하늘 끝까지! 누나 학교 가는 길에 안아 달라는 말도 없이 씽씽 걷다가, 동그라미 네 개 로고를 보고 외쳤다. “콩콩이차다!”</t>
+          <t>엄마가 출장 간 아침, 아빠와 함께 둔쫀떡을 먹은 태오는 기분이 하늘 끝까지! 누나 학교 가는 길에 안아 달라는 말도 없이 씽씽 걷다가, 동그라미 네 개 로고를 보고 외쳤다. “콩콩이차다!”</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>재이, 엄마, 태오</t>
+          <t>재이, 아빠, 태오</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
@@ -2068,12 +2068,12 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>기분이 좋으면 걸음도 가벼워지는 태오 / 누나·엄마와 콩콩콩 뛰어서 가는 아침</t>
+          <t>기분이 좋으면 걸음도 가벼워지는 태오 / 엄마 없는 아침, 아빠·누나와 콩콩콩 뛰어서 가는 길</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>작은 기쁨 하나가 하루를 씩씩하게 만들어요. 기분 좋은 마음은 걸음도 가볍게 해 줘요.</t>
+          <t>엄마가 없는 아침에도 작은 기쁨 하나가 하루를 씩씩하게 만들어요. 기분 좋은 마음은 걸음도 가볍게 해 줘요.</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
@@ -16440,12 +16440,12 @@
       </c>
       <c r="E449" s="6" t="inlineStr">
         <is>
-          <t>태오, 엄마</t>
+          <t>태오, 아빠</t>
         </is>
       </c>
       <c r="F449" s="6" t="inlineStr">
         <is>
-          <t>아침, 식탁 위에 둔쫀떡.</t>
+          <t>엄마가 출장 간 아침. / 식탁 위에 둔쫀떡.</t>
         </is>
       </c>
       <c r="G449" s="6" t="inlineStr">
@@ -16508,12 +16508,12 @@
       </c>
       <c r="E451" s="6" t="inlineStr">
         <is>
-          <t>엄마, 태오, 재이</t>
+          <t>아빠, 태오, 재이</t>
         </is>
       </c>
       <c r="F451" s="6" t="inlineStr">
         <is>
-          <t>누나 학교 가는 시간.</t>
+          <t>엄마 대신 아빠가 누나 학교 데려다주는 시간.</t>
         </is>
       </c>
       <c r="G451" s="6" t="inlineStr">
@@ -16581,7 +16581,7 @@
       </c>
       <c r="E453" s="6" t="inlineStr">
         <is>
-          <t>재이, 엄마</t>
+          <t>재이, 아빠</t>
         </is>
       </c>
       <c r="F453" s="6" t="inlineStr"/>
@@ -16771,7 +16771,7 @@
       </c>
       <c r="E459" s="6" t="inlineStr">
         <is>
-          <t>엄마, 재이</t>
+          <t>아빠, 재이</t>
         </is>
       </c>
       <c r="F459" s="6" t="inlineStr"/>
@@ -19118,12 +19118,12 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>태오, 재이</t>
+          <t>태오, 재이, 아빠</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>(가족 제보) 아침에 둔쫀떡을 먹은 태오는 기분이 최고! 누나 학교 가는 길에 안아 달라는 말도 없이 빠른 걸음으로 씩씩하게 걷는다. 가다가 아우디 로고를 보고는 “콩콩이차다! 나도 콩콩이차 타고 싶다~”</t>
+          <t>(가족 제보) 엄마가 출장 간 아침, 아빠·재이와 함께 학교에 걸어가는 길. 둔쫀떡을 먹은 태오는 기분이 최고! 누나 학교 가는 길에 안아 달라는 말도 없이 빠른 걸음으로 씩씩하게 걷는다. 가다가 아우디 로고를 보고는 “콩콩이차다! 나도 콩콩이차 타고 싶다~”</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Add 카레슘마그네슘 to the Taeo dictionary
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$461</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$11</definedName>
   </definedNames>
@@ -16858,7 +16858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -17552,17 +17552,17 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>콩콩이차</t>
+          <t>카레슘마그네슘</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>아우디 (자동차)</t>
+          <t>칼슘마그네슘</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>아우디 동그라미 로고를 보고. “나도 콩콩이차 타고 싶다~”</t>
+          <t>매일 먹는 영양제 이름</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr"/>
@@ -17574,17 +17574,17 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>둔쫀떡</t>
+          <t>콩콩이차</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>두바이 쫀득 찹쌀떡</t>
+          <t>아우디 (자동차)</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>아침에 먹으면 하루 종일 기분이 좋아져요</t>
+          <t>아우디 동그라미 로고를 보고. “나도 콩콩이차 타고 싶다~”</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr"/>
@@ -17596,17 +17596,17 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>발싸</t>
+          <t>둔쫀떡</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>발사</t>
+          <t>두바이 쫀득 찹쌀떡</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>“스밀로클로 발싸!” 기술을 쏠 때</t>
+          <t>아침에 먹으면 하루 종일 기분이 좋아져요</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr"/>
@@ -17618,17 +17618,17 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>안킬로해머 · 스밀로클로</t>
+          <t>발싸</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>다이노스터 기술</t>
+          <t>발사</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>래터킥, 퀀텀해로우… 하나씩 외치고 “쓰구미~”</t>
+          <t>“스밀로클로 발싸!” 기술을 쏠 때</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr"/>
@@ -17638,9 +17638,21 @@
       <c r="A37" s="5" t="n">
         <v>34</v>
       </c>
-      <c r="B37" s="6" t="inlineStr"/>
-      <c r="C37" s="6" t="inlineStr"/>
-      <c r="D37" s="6" t="inlineStr"/>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>안킬로해머 · 스밀로클로</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>다이노스터 기술</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>래터킥, 퀀텀해로우… 하나씩 외치고 “쓰구미~”</t>
+        </is>
+      </c>
       <c r="E37" s="6" t="inlineStr"/>
       <c r="F37" s="6" t="inlineStr"/>
     </row>
@@ -17834,8 +17846,18 @@
       <c r="E56" s="4" t="inlineStr"/>
       <c r="F56" s="4" t="inlineStr"/>
     </row>
+    <row r="57">
+      <c r="A57" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="B57" s="6" t="inlineStr"/>
+      <c r="C57" s="6" t="inlineStr"/>
+      <c r="D57" s="6" t="inlineStr"/>
+      <c r="E57" s="6" t="inlineStr"/>
+      <c r="F57" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F56"/>
+  <autoFilter ref="A3:F57"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add 두쫀쿠 (heard for 국중박) to the Taeo dictionary
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$461</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$58</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$11</definedName>
   </definedNames>
@@ -16858,7 +16858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -17552,17 +17552,17 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>카레슘마그네슘</t>
+          <t>두쫀쿠</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>칼슘마그네슘</t>
+          <t>국중박 (국립중앙박물관)</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>매일 먹는 영양제 이름</t>
+          <t>“내일 국중박 간대” 했더니 “두쫀쿠에 간다고?” 줄임말이 아직 낯설어요 (두쫀쿠는 두바이 쫀득 쿠키)</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr"/>
@@ -17574,17 +17574,17 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>콩콩이차</t>
+          <t>카레슘마그네슘</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>아우디 (자동차)</t>
+          <t>칼슘마그네슘</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>아우디 동그라미 로고를 보고. “나도 콩콩이차 타고 싶다~”</t>
+          <t>매일 먹는 영양제 이름</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr"/>
@@ -17596,17 +17596,17 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>둔쫀떡</t>
+          <t>콩콩이차</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>두바이 쫀득 찹쌀떡</t>
+          <t>아우디 (자동차)</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>아침에 먹으면 하루 종일 기분이 좋아져요</t>
+          <t>아우디 동그라미 로고를 보고. “나도 콩콩이차 타고 싶다~”</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr"/>
@@ -17618,17 +17618,17 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>발싸</t>
+          <t>둔쫀떡</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>발사</t>
+          <t>두바이 쫀득 찹쌀떡</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>“스밀로클로 발싸!” 기술을 쏠 때</t>
+          <t>아침에 먹으면 하루 종일 기분이 좋아져요</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr"/>
@@ -17640,17 +17640,17 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>안킬로해머 · 스밀로클로</t>
+          <t>발싸</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>다이노스터 기술</t>
+          <t>발사</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>래터킥, 퀀텀해로우… 하나씩 외치고 “쓰구미~”</t>
+          <t>“스밀로클로 발싸!” 기술을 쏠 때</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr"/>
@@ -17660,9 +17660,21 @@
       <c r="A38" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="B38" s="4" t="inlineStr"/>
-      <c r="C38" s="4" t="inlineStr"/>
-      <c r="D38" s="4" t="inlineStr"/>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>안킬로해머 · 스밀로클로</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>다이노스터 기술</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>래터킥, 퀀텀해로우… 하나씩 외치고 “쓰구미~”</t>
+        </is>
+      </c>
       <c r="E38" s="4" t="inlineStr"/>
       <c r="F38" s="4" t="inlineStr"/>
     </row>
@@ -17856,8 +17868,18 @@
       <c r="E57" s="6" t="inlineStr"/>
       <c r="F57" s="6" t="inlineStr"/>
     </row>
+    <row r="58">
+      <c r="A58" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="B58" s="4" t="inlineStr"/>
+      <c r="C58" s="4" t="inlineStr"/>
+      <c r="D58" s="4" t="inlineStr"/>
+      <c r="E58" s="4" t="inlineStr"/>
+      <c r="F58" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F57"/>
+  <autoFilter ref="A3:F58"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add Taeo sayings: pine needles are 두쫀쿠, measuring height after one spoonful
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$461</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$58</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17893,7 +17893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18284,13 +18284,13 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>제발 오로라핑! 양핑은 싫어!</t>
+          <t>두쫀쿠 안에 들어가는 거다!</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr"/>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>티니핑 원카드에서 조커처럼 쓰는 오로라핑 카드를 간절히 기다릴 때</t>
+          <t>바닥에 떨어진 소나무잎을 보고 (두쫀쿠가 머릿속에서 떠나질 않아요)</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr"/>
@@ -18306,13 +18306,13 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>싸우자! 타노스 나와라!</t>
+          <t>엄마, 나 두쫀쿠 먹고 싶어~</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr"/>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>제일 좋아하는 놀이, 어벤져스로 타노스랑 싸우기 (타노스는 늘 아빠, 건틀렛 끼고 “아임 인에비터블”)</t>
+          <t>요즘 틈만 나면</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr"/>
@@ -18328,13 +18328,13 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>너라고 하지 마라! 나도 엄마 아빠한테 너라고 한다!</t>
+          <t>밥 한 숟가락 먹고 키 재 봐야지~</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr"/>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>“너 엄마 아빠 말 잘 들어” 소리를 들으면</t>
+          <t>밥 먹으면 키가 클까 봐 (한 숟가락 먹고 벽으로 달려가요)</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr"/>
@@ -18350,13 +18350,13 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>재이 아니야! 재이 누나야!</t>
+          <t>여기야? 오늘은 작아졌네</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr"/>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>누가 누나를 “재이야” 하고 부르면 (모든 호칭은 태오 기준)</t>
+          <t>벽에 붙인 키 재는 표에서 95cm 눈금을 보면서</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr"/>
@@ -18372,13 +18372,13 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>이 안 닦아! 싫어!</t>
+          <t>제발 오로라핑! 양핑은 싫어!</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr"/>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>아침저녁 이 닦을 때 (도망 다니고 바닥을 기어요)</t>
+          <t>티니핑 원카드에서 조커처럼 쓰는 오로라핑 카드를 간절히 기다릴 때</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr"/>
@@ -18394,13 +18394,13 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>누나 대단해!</t>
+          <t>싸우자! 타노스 나와라!</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr"/>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>누나가 잠수를 보여 줬을 때</t>
+          <t>제일 좋아하는 놀이, 어벤져스로 타노스랑 싸우기 (타노스는 늘 아빠, 건틀렛 끼고 “아임 인에비터블”)</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr"/>
@@ -18416,13 +18416,13 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>엄마 인누와~</t>
+          <t>너라고 하지 마라! 나도 엄마 아빠한테 너라고 한다!</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr"/>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>밤에 자다 깨서 (엄마가 옆에서 재워 줄 때까지)</t>
+          <t>“너 엄마 아빠 말 잘 들어” 소리를 들으면</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr"/>
@@ -18438,13 +18438,13 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>왜 놀려! 놀리지 마!</t>
+          <t>재이 아니야! 재이 누나야!</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr"/>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>“태오는 글씨·숫자 잘 몰라” 소리를 들으면 (손가락질하며)</t>
+          <t>누가 누나를 “재이야” 하고 부르면 (모든 호칭은 태오 기준)</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr"/>
@@ -18460,13 +18460,13 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>왜 내 친구를 놀려! 슬프잖아!</t>
+          <t>이 안 닦아! 싫어!</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr"/>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>어린이집 친구가 놀림 받는 것 같을 때 (친구 편이에요)</t>
+          <t>아침저녁 이 닦을 때 (도망 다니고 바닥을 기어요)</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr"/>
@@ -18482,13 +18482,13 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>나 무지개빛 망토 갖고 싶어!</t>
+          <t>누나 대단해!</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr"/>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>파라큘라를 본 날부터 (또봇 Y도 같이 갖고 싶어요!)</t>
+          <t>누나가 잠수를 보여 줬을 때</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr"/>
@@ -18504,13 +18504,13 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>어벤져스… 어셈블!</t>
+          <t>엄마 인누와~</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr"/>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>엔드게임 마지막 장면을 따라 하며 가족을 다 모을 때</t>
+          <t>밤에 자다 깨서 (엄마가 옆에서 재워 줄 때까지)</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr"/>
@@ -18526,13 +18526,13 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>왓 두 유 두, 캡틴? 위 파이트!</t>
+          <t>왜 놀려! 놀리지 마!</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr"/>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>시빌 워 싸움 장면 놀이를 할 때</t>
+          <t>“태오는 글씨·숫자 잘 몰라” 소리를 들으면 (손가락질하며)</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr"/>
@@ -18548,13 +18548,13 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>와칸다 포에버!</t>
+          <t>왜 내 친구를 놀려! 슬프잖아!</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr"/>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>인피니티 워 장면처럼 다 같이 뛰어갈 때</t>
+          <t>어린이집 친구가 놀림 받는 것 같을 때 (친구 편이에요)</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr"/>
@@ -18570,13 +18570,13 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>어린이집에 데리러 올 거야?</t>
+          <t>나 무지개빛 망토 갖고 싶어!</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr"/>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>어린이집 가기 싫은 아침에 (몇 번씩 확인해요)</t>
+          <t>파라큘라를 본 날부터 (또봇 Y도 같이 갖고 싶어요!)</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr"/>
@@ -18592,13 +18592,13 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>어린이집 가기 싫다.</t>
+          <t>어벤져스… 어셈블!</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr"/>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>월·화·수… 아침마다</t>
+          <t>엔드게임 마지막 장면을 따라 하며 가족을 다 모을 때</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr"/>
@@ -18614,13 +18614,13 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?</t>
+          <t>왓 두 유 두, 캡틴? 위 파이트!</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr"/>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>싫은 태권도 가는 날</t>
+          <t>시빌 워 싸움 장면 놀이를 할 때</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr"/>
@@ -18636,13 +18636,13 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>오늘은 뽀로로 날! 내가 싫어하는 태권도 안 가는 날이다~</t>
+          <t>와칸다 포에버!</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr"/>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>월요일 아침 (달력은 몰라도 뽀로로 날은 정확히 알아요)</t>
+          <t>인피니티 워 장면처럼 다 같이 뛰어갈 때</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr"/>
@@ -18653,18 +18653,18 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>아니야!</t>
+          <t>어린이집에 데리러 올 거야?</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr"/>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>하루에도 제일 많이 하는 말</t>
+          <t>어린이집 가기 싫은 아침에 (몇 번씩 확인해요)</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr"/>
@@ -18675,18 +18675,18 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>거짓말! 아니야!</t>
+          <t>어린이집 가기 싫다.</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr"/>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>기분 나쁘거나 하기 싫을 때</t>
+          <t>월·화·수… 아침마다</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr"/>
@@ -18697,18 +18697,18 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>맛있는데 지금은 먹기 싫어.</t>
+          <t>누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr"/>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>누가 음식을 권하면</t>
+          <t>싫은 태권도 가는 날</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr"/>
@@ -18719,18 +18719,18 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>치즈 냄새 극혐!</t>
+          <t>오늘은 뽀로로 날! 내가 싫어하는 태권도 안 가는 날이다~</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr"/>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>치즈만 보면 (냄새는 더더욱)</t>
+          <t>월요일 아침 (달력은 몰라도 뽀로로 날은 정확히 알아요)</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr"/>
@@ -18746,13 +18746,13 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>김태오!</t>
+          <t>아니야!</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr"/>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+          <t>하루에도 제일 많이 하는 말</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr"/>
@@ -18763,22 +18763,18 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>짐방</t>
-        </is>
-      </c>
-      <c r="D41" s="6" t="inlineStr">
-        <is>
-          <t>김서방</t>
-        </is>
-      </c>
+          <t>거짓말! 아니야!</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr"/>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+          <t>기분 나쁘거나 하기 싫을 때</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr"/>
@@ -18789,22 +18785,18 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>꿍끙이</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>뿡뿡이</t>
-        </is>
-      </c>
+          <t>맛있는데 지금은 먹기 싫어.</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr"/>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+          <t>누가 음식을 권하면</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr"/>
@@ -18813,40 +18805,96 @@
       <c r="A43" s="5" t="n">
         <v>40</v>
       </c>
-      <c r="B43" s="6" t="inlineStr"/>
-      <c r="C43" s="6" t="inlineStr"/>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>재이 입버릇</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>치즈 냄새 극혐!</t>
+        </is>
+      </c>
       <c r="D43" s="6" t="inlineStr"/>
-      <c r="E43" s="6" t="inlineStr"/>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>치즈만 보면 (냄새는 더더욱)</t>
+        </is>
+      </c>
       <c r="F43" s="6" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n">
         <v>41</v>
       </c>
-      <c r="B44" s="4" t="inlineStr"/>
-      <c r="C44" s="4" t="inlineStr"/>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>재이 입버릇</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>김태오!</t>
+        </is>
+      </c>
       <c r="D44" s="4" t="inlineStr"/>
-      <c r="E44" s="4" t="inlineStr"/>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+        </is>
+      </c>
       <c r="F44" s="4" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="n">
         <v>42</v>
       </c>
-      <c r="B45" s="6" t="inlineStr"/>
-      <c r="C45" s="6" t="inlineStr"/>
-      <c r="D45" s="6" t="inlineStr"/>
-      <c r="E45" s="6" t="inlineStr"/>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>짐방</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>김서방</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+        </is>
+      </c>
       <c r="F45" s="6" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n">
         <v>43</v>
       </c>
-      <c r="B46" s="4" t="inlineStr"/>
-      <c r="C46" s="4" t="inlineStr"/>
-      <c r="D46" s="4" t="inlineStr"/>
-      <c r="E46" s="4" t="inlineStr"/>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>꿍끙이</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>뿡뿡이</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+        </is>
+      </c>
       <c r="F46" s="4" t="inlineStr"/>
     </row>
     <row r="47">
@@ -18959,8 +19007,48 @@
       <c r="E57" s="6" t="inlineStr"/>
       <c r="F57" s="6" t="inlineStr"/>
     </row>
+    <row r="58">
+      <c r="A58" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="B58" s="4" t="inlineStr"/>
+      <c r="C58" s="4" t="inlineStr"/>
+      <c r="D58" s="4" t="inlineStr"/>
+      <c r="E58" s="4" t="inlineStr"/>
+      <c r="F58" s="4" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="B59" s="6" t="inlineStr"/>
+      <c r="C59" s="6" t="inlineStr"/>
+      <c r="D59" s="6" t="inlineStr"/>
+      <c r="E59" s="6" t="inlineStr"/>
+      <c r="F59" s="6" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="B60" s="4" t="inlineStr"/>
+      <c r="C60" s="4" t="inlineStr"/>
+      <c r="D60" s="4" t="inlineStr"/>
+      <c r="E60" s="4" t="inlineStr"/>
+      <c r="F60" s="4" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="B61" s="6" t="inlineStr"/>
+      <c r="C61" s="6" t="inlineStr"/>
+      <c r="D61" s="6" t="inlineStr"/>
+      <c r="E61" s="6" t="inlineStr"/>
+      <c r="F61" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F57"/>
+  <autoFilter ref="A3:F61"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Fix the height-measuring sayings: he turns around and reads the number at eye level
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -18334,7 +18334,7 @@
       <c r="D21" s="6" t="inlineStr"/>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>밥 먹으면 키가 클까 봐 (한 숟가락 먹고 벽으로 달려가요)</t>
+          <t>밥 먹으면 키가 클까 봐 (한 숟가락 먹고 바로 키를 재러 가요)</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr"/>
@@ -18356,7 +18356,7 @@
       <c r="D22" s="4" t="inlineStr"/>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>벽에 붙인 키 재는 표에서 95cm 눈금을 보면서</t>
+          <t>정수리에 손을 대고 재야 하는데, 뒤돌아서 눈앞에 있는 95cm 숫자를 가리키면서 (눈높이 숫자라 늘 작아져요)</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Add Taeo's 자음춤 song to the dictionary and sayings
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -18,8 +18,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$461</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$58</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$62</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16858,7 +16858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -17574,17 +17574,17 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>카레슘마그네슘</t>
+          <t>쭈룹쫩 쭈룹쫩 쭈룹쫩쫩</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>칼슘마그네슘</t>
+          <t>자음춤 노래의 후렴 (원래 가사는 아직 몰라요)</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>매일 먹는 영양제 이름</t>
+          <t>어린이집에서 새로 배워 온 노래. “ㄱ ㄴ ㄷ ㄹ 자음춤을 춰봐요~”</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr"/>
@@ -17596,17 +17596,17 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>콩콩이차</t>
+          <t>카레슘마그네슘</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>아우디 (자동차)</t>
+          <t>칼슘마그네슘</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>아우디 동그라미 로고를 보고. “나도 콩콩이차 타고 싶다~”</t>
+          <t>매일 먹는 영양제 이름</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr"/>
@@ -17618,17 +17618,17 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>둔쫀떡</t>
+          <t>콩콩이차</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>두바이 쫀득 찹쌀떡</t>
+          <t>아우디 (자동차)</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>아침에 먹으면 하루 종일 기분이 좋아져요</t>
+          <t>아우디 동그라미 로고를 보고. “나도 콩콩이차 타고 싶다~”</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr"/>
@@ -17640,17 +17640,17 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>발싸</t>
+          <t>둔쫀떡</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>발사</t>
+          <t>두바이 쫀득 찹쌀떡</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>“스밀로클로 발싸!” 기술을 쏠 때</t>
+          <t>아침에 먹으면 하루 종일 기분이 좋아져요</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr"/>
@@ -17662,17 +17662,17 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>안킬로해머 · 스밀로클로</t>
+          <t>발싸</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>다이노스터 기술</t>
+          <t>발사</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>래터킥, 퀀텀해로우… 하나씩 외치고 “쓰구미~”</t>
+          <t>“스밀로클로 발싸!” 기술을 쏠 때</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr"/>
@@ -17682,9 +17682,21 @@
       <c r="A39" s="5" t="n">
         <v>36</v>
       </c>
-      <c r="B39" s="6" t="inlineStr"/>
-      <c r="C39" s="6" t="inlineStr"/>
-      <c r="D39" s="6" t="inlineStr"/>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>안킬로해머 · 스밀로클로</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>다이노스터 기술</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>래터킥, 퀀텀해로우… 하나씩 외치고 “쓰구미~”</t>
+        </is>
+      </c>
       <c r="E39" s="6" t="inlineStr"/>
       <c r="F39" s="6" t="inlineStr"/>
     </row>
@@ -17878,8 +17890,18 @@
       <c r="E58" s="4" t="inlineStr"/>
       <c r="F58" s="4" t="inlineStr"/>
     </row>
+    <row r="59">
+      <c r="A59" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="B59" s="6" t="inlineStr"/>
+      <c r="C59" s="6" t="inlineStr"/>
+      <c r="D59" s="6" t="inlineStr"/>
+      <c r="E59" s="6" t="inlineStr"/>
+      <c r="F59" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F58"/>
+  <autoFilter ref="A3:F59"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -17893,7 +17915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18284,13 +18306,13 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>두쫀쿠 안에 들어가는 거다!</t>
+          <t>아빠 그게 아니야! 자음춤을 춰보자야~ 쭈룹쫩 쭈룹쫩</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr"/>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>바닥에 떨어진 소나무잎을 보고 (두쫀쿠가 머릿속에서 떠나질 않아요)</t>
+          <t>어린이집에서 새로 배운 자음춤 노래를 아빠가 엉뚱하게 따라 부를 때</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr"/>
@@ -18306,13 +18328,13 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>엄마, 나 두쫀쿠 먹고 싶어~</t>
+          <t>두쫀쿠 안에 들어가는 거다!</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr"/>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>요즘 틈만 나면</t>
+          <t>바닥에 떨어진 소나무잎을 보고 (두쫀쿠가 머릿속에서 떠나질 않아요)</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr"/>
@@ -18328,13 +18350,13 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>밥 한 숟가락 먹고 키 재 봐야지~</t>
+          <t>엄마, 나 두쫀쿠 먹고 싶어~</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr"/>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>밥 먹으면 키가 클까 봐 (한 숟가락 먹고 바로 키를 재러 가요)</t>
+          <t>요즘 틈만 나면</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr"/>
@@ -18350,13 +18372,13 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>여기야? 오늘은 작아졌네</t>
+          <t>밥 한 숟가락 먹고 키 재 봐야지~</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr"/>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>정수리에 손을 대고 재야 하는데, 뒤돌아서 눈앞에 있는 95cm 숫자를 가리키면서 (눈높이 숫자라 늘 작아져요)</t>
+          <t>밥 먹으면 키가 클까 봐 (한 숟가락 먹고 바로 키를 재러 가요)</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr"/>
@@ -18372,13 +18394,13 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>제발 오로라핑! 양핑은 싫어!</t>
+          <t>여기야? 오늘은 작아졌네</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr"/>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>티니핑 원카드에서 조커처럼 쓰는 오로라핑 카드를 간절히 기다릴 때</t>
+          <t>정수리에 손을 대고 재야 하는데, 뒤돌아서 눈앞에 있는 95cm 숫자를 가리키면서 (눈높이 숫자라 늘 작아져요)</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr"/>
@@ -18394,13 +18416,13 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>싸우자! 타노스 나와라!</t>
+          <t>제발 오로라핑! 양핑은 싫어!</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr"/>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>제일 좋아하는 놀이, 어벤져스로 타노스랑 싸우기 (타노스는 늘 아빠, 건틀렛 끼고 “아임 인에비터블”)</t>
+          <t>티니핑 원카드에서 조커처럼 쓰는 오로라핑 카드를 간절히 기다릴 때</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr"/>
@@ -18416,13 +18438,13 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>너라고 하지 마라! 나도 엄마 아빠한테 너라고 한다!</t>
+          <t>싸우자! 타노스 나와라!</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr"/>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>“너 엄마 아빠 말 잘 들어” 소리를 들으면</t>
+          <t>제일 좋아하는 놀이, 어벤져스로 타노스랑 싸우기 (타노스는 늘 아빠, 건틀렛 끼고 “아임 인에비터블”)</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr"/>
@@ -18438,13 +18460,13 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>재이 아니야! 재이 누나야!</t>
+          <t>너라고 하지 마라! 나도 엄마 아빠한테 너라고 한다!</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr"/>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>누가 누나를 “재이야” 하고 부르면 (모든 호칭은 태오 기준)</t>
+          <t>“너 엄마 아빠 말 잘 들어” 소리를 들으면</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr"/>
@@ -18460,13 +18482,13 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>이 안 닦아! 싫어!</t>
+          <t>재이 아니야! 재이 누나야!</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr"/>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>아침저녁 이 닦을 때 (도망 다니고 바닥을 기어요)</t>
+          <t>누가 누나를 “재이야” 하고 부르면 (모든 호칭은 태오 기준)</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr"/>
@@ -18482,13 +18504,13 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>누나 대단해!</t>
+          <t>이 안 닦아! 싫어!</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr"/>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>누나가 잠수를 보여 줬을 때</t>
+          <t>아침저녁 이 닦을 때 (도망 다니고 바닥을 기어요)</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr"/>
@@ -18504,13 +18526,13 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>엄마 인누와~</t>
+          <t>누나 대단해!</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr"/>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>밤에 자다 깨서 (엄마가 옆에서 재워 줄 때까지)</t>
+          <t>누나가 잠수를 보여 줬을 때</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr"/>
@@ -18526,13 +18548,13 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>왜 놀려! 놀리지 마!</t>
+          <t>엄마 인누와~</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr"/>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>“태오는 글씨·숫자 잘 몰라” 소리를 들으면 (손가락질하며)</t>
+          <t>밤에 자다 깨서 (엄마가 옆에서 재워 줄 때까지)</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr"/>
@@ -18548,13 +18570,13 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>왜 내 친구를 놀려! 슬프잖아!</t>
+          <t>왜 놀려! 놀리지 마!</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr"/>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>어린이집 친구가 놀림 받는 것 같을 때 (친구 편이에요)</t>
+          <t>“태오는 글씨·숫자 잘 몰라” 소리를 들으면 (손가락질하며)</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr"/>
@@ -18570,13 +18592,13 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>나 무지개빛 망토 갖고 싶어!</t>
+          <t>왜 내 친구를 놀려! 슬프잖아!</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr"/>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>파라큘라를 본 날부터 (또봇 Y도 같이 갖고 싶어요!)</t>
+          <t>어린이집 친구가 놀림 받는 것 같을 때 (친구 편이에요)</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr"/>
@@ -18592,13 +18614,13 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>어벤져스… 어셈블!</t>
+          <t>나 무지개빛 망토 갖고 싶어!</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr"/>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>엔드게임 마지막 장면을 따라 하며 가족을 다 모을 때</t>
+          <t>파라큘라를 본 날부터 (또봇 Y도 같이 갖고 싶어요!)</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr"/>
@@ -18614,13 +18636,13 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>왓 두 유 두, 캡틴? 위 파이트!</t>
+          <t>어벤져스… 어셈블!</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr"/>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>시빌 워 싸움 장면 놀이를 할 때</t>
+          <t>엔드게임 마지막 장면을 따라 하며 가족을 다 모을 때</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr"/>
@@ -18636,13 +18658,13 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>와칸다 포에버!</t>
+          <t>왓 두 유 두, 캡틴? 위 파이트!</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr"/>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>인피니티 워 장면처럼 다 같이 뛰어갈 때</t>
+          <t>시빌 워 싸움 장면 놀이를 할 때</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr"/>
@@ -18658,13 +18680,13 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>어린이집에 데리러 올 거야?</t>
+          <t>와칸다 포에버!</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr"/>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>어린이집 가기 싫은 아침에 (몇 번씩 확인해요)</t>
+          <t>인피니티 워 장면처럼 다 같이 뛰어갈 때</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr"/>
@@ -18680,13 +18702,13 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>어린이집 가기 싫다.</t>
+          <t>어린이집에 데리러 올 거야?</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr"/>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>월·화·수… 아침마다</t>
+          <t>어린이집 가기 싫은 아침에 (몇 번씩 확인해요)</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr"/>
@@ -18702,13 +18724,13 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?</t>
+          <t>어린이집 가기 싫다.</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr"/>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>싫은 태권도 가는 날</t>
+          <t>월·화·수… 아침마다</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr"/>
@@ -18724,13 +18746,13 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>오늘은 뽀로로 날! 내가 싫어하는 태권도 안 가는 날이다~</t>
+          <t>누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr"/>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>월요일 아침 (달력은 몰라도 뽀로로 날은 정확히 알아요)</t>
+          <t>싫은 태권도 가는 날</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr"/>
@@ -18741,18 +18763,18 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>아니야!</t>
+          <t>오늘은 뽀로로 날! 내가 싫어하는 태권도 안 가는 날이다~</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr"/>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>하루에도 제일 많이 하는 말</t>
+          <t>월요일 아침 (달력은 몰라도 뽀로로 날은 정확히 알아요)</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr"/>
@@ -18768,13 +18790,13 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>거짓말! 아니야!</t>
+          <t>아니야!</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr"/>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>기분 나쁘거나 하기 싫을 때</t>
+          <t>하루에도 제일 많이 하는 말</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr"/>
@@ -18790,13 +18812,13 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>맛있는데 지금은 먹기 싫어.</t>
+          <t>거짓말! 아니야!</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr"/>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>누가 음식을 권하면</t>
+          <t>기분 나쁘거나 하기 싫을 때</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr"/>
@@ -18812,13 +18834,13 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>치즈 냄새 극혐!</t>
+          <t>맛있는데 지금은 먹기 싫어.</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr"/>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>치즈만 보면 (냄새는 더더욱)</t>
+          <t>누가 음식을 권하면</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr"/>
@@ -18834,13 +18856,13 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>김태오!</t>
+          <t>치즈 냄새 극혐!</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr"/>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+          <t>치즈만 보면 (냄새는 더더욱)</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr"/>
@@ -18851,22 +18873,18 @@
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>짐방</t>
-        </is>
-      </c>
-      <c r="D45" s="6" t="inlineStr">
-        <is>
-          <t>김서방</t>
-        </is>
-      </c>
+          <t>김태오!</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr"/>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr"/>
@@ -18882,17 +18900,17 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>꿍끙이</t>
+          <t>짐방</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>뿡뿡이</t>
+          <t>김서방</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr"/>
@@ -18901,10 +18919,26 @@
       <c r="A47" s="5" t="n">
         <v>44</v>
       </c>
-      <c r="B47" s="6" t="inlineStr"/>
-      <c r="C47" s="6" t="inlineStr"/>
-      <c r="D47" s="6" t="inlineStr"/>
-      <c r="E47" s="6" t="inlineStr"/>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>꿍끙이</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>뿡뿡이</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+        </is>
+      </c>
       <c r="F47" s="6" t="inlineStr"/>
     </row>
     <row r="48">
@@ -19047,8 +19081,18 @@
       <c r="E61" s="6" t="inlineStr"/>
       <c r="F61" s="6" t="inlineStr"/>
     </row>
+    <row r="62">
+      <c r="A62" s="3" t="n">
+        <v>59</v>
+      </c>
+      <c r="B62" s="4" t="inlineStr"/>
+      <c r="C62" s="4" t="inlineStr"/>
+      <c r="D62" s="4" t="inlineStr"/>
+      <c r="E62" s="4" t="inlineStr"/>
+      <c r="F62" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F61"/>
+  <autoFilter ref="A3:F62"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add 스테고테라쉴드 (Oz's shield skill, unverified) to the Taeo dictionary
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$461</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$60</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$62</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$11</definedName>
   </definedNames>
@@ -16858,7 +16858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -17684,17 +17684,17 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>안킬로해머 · 스밀로클로</t>
+          <t>스테고테라쉴드</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>다이노스터 기술</t>
+          <t>오즈의 방패 기술 이름 (추정, 확인 중)</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>래터킥, 퀀텀해로우… 하나씩 외치고 “쓰구미~”</t>
+          <t>다이노스터 오즈의 스테고 지프 방패 기술. 스테고 + 방패(쉴드)라서 오즈 거예요</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr"/>
@@ -17704,9 +17704,21 @@
       <c r="A40" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="B40" s="4" t="inlineStr"/>
-      <c r="C40" s="4" t="inlineStr"/>
-      <c r="D40" s="4" t="inlineStr"/>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>안킬로해머 · 스밀로클로</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>다이노스터 기술</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>래터킥, 퀀텀해로우… 하나씩 외치고 “쓰구미~”</t>
+        </is>
+      </c>
       <c r="E40" s="4" t="inlineStr"/>
       <c r="F40" s="4" t="inlineStr"/>
     </row>
@@ -17900,8 +17912,18 @@
       <c r="E59" s="6" t="inlineStr"/>
       <c r="F59" s="6" t="inlineStr"/>
     </row>
+    <row r="60">
+      <c r="A60" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="B60" s="4" t="inlineStr"/>
+      <c r="C60" s="4" t="inlineStr"/>
+      <c r="D60" s="4" t="inlineStr"/>
+      <c r="E60" s="4" t="inlineStr"/>
+      <c r="F60" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F59"/>
+  <autoFilter ref="A3:F60"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Remove Oz's skill from the Taeo dictionary: Taeo does not know Oz's skills
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$461</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$59</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$62</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$11</definedName>
   </definedNames>
@@ -16858,7 +16858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -17684,17 +17684,17 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>스테고테라쉴드</t>
+          <t>안킬로해머 · 스밀로클로</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>스테고쉴드 스트라이크 (오즈)</t>
+          <t>다이노스터 기술</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>오즈의 방패 기술. 방패가 깨지면 조각이 양쪽 팔꿈치에 붙어 주먹이 되고, 이어서 스테고너클 스트라이크!</t>
+          <t>래터킥, 퀀텀해로우… 하나씩 외치고 “쓰구미~”</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr"/>
@@ -17704,21 +17704,9 @@
       <c r="A40" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>안킬로해머 · 스밀로클로</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>다이노스터 기술</t>
-        </is>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>래터킥, 퀀텀해로우… 하나씩 외치고 “쓰구미~”</t>
-        </is>
-      </c>
+      <c r="B40" s="4" t="inlineStr"/>
+      <c r="C40" s="4" t="inlineStr"/>
+      <c r="D40" s="4" t="inlineStr"/>
       <c r="E40" s="4" t="inlineStr"/>
       <c r="F40" s="4" t="inlineStr"/>
     </row>
@@ -17912,18 +17900,8 @@
       <c r="E59" s="6" t="inlineStr"/>
       <c r="F59" s="6" t="inlineStr"/>
     </row>
-    <row r="60">
-      <c r="A60" s="3" t="n">
-        <v>57</v>
-      </c>
-      <c r="B60" s="4" t="inlineStr"/>
-      <c r="C60" s="4" t="inlineStr"/>
-      <c r="D60" s="4" t="inlineStr"/>
-      <c r="E60" s="4" t="inlineStr"/>
-      <c r="F60" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A3:F60"/>
+  <autoFilter ref="A3:F59"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add Taeo's height-measuring saying (106, will be 100)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$461</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$63</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17915,7 +17915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18394,13 +18394,13 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>여기야? 오늘은 작아졌네</t>
+          <t>오늘도 키 재 봐야지~ 너 키 몇이야? 106! 밥 많이 먹어서 100 될 거다~</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr"/>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>정수리에 손을 대고 재야 하는데, 뒤돌아서 눈앞에 있는 95cm 숫자를 가리키면서 (눈높이 숫자라 늘 작아져요)</t>
+          <t>키를 재면서 혼자 묻고 답할 때</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr"/>
@@ -18416,13 +18416,13 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>제발 오로라핑! 양핑은 싫어!</t>
+          <t>여기야? 오늘은 작아졌네</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr"/>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>티니핑 원카드에서 조커처럼 쓰는 오로라핑 카드를 간절히 기다릴 때</t>
+          <t>정수리에 손을 대고 재야 하는데, 뒤돌아서 눈앞에 있는 95cm 숫자를 가리키면서 (눈높이 숫자라 늘 작아져요)</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr"/>
@@ -18438,13 +18438,13 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>싸우자! 타노스 나와라!</t>
+          <t>제발 오로라핑! 양핑은 싫어!</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr"/>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>제일 좋아하는 놀이, 어벤져스로 타노스랑 싸우기 (타노스는 늘 아빠, 건틀렛 끼고 “아임 인에비터블”)</t>
+          <t>티니핑 원카드에서 조커처럼 쓰는 오로라핑 카드를 간절히 기다릴 때</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr"/>
@@ -18460,13 +18460,13 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>너라고 하지 마라! 나도 엄마 아빠한테 너라고 한다!</t>
+          <t>싸우자! 타노스 나와라!</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr"/>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>“너 엄마 아빠 말 잘 들어” 소리를 들으면</t>
+          <t>제일 좋아하는 놀이, 어벤져스로 타노스랑 싸우기 (타노스는 늘 아빠, 건틀렛 끼고 “아임 인에비터블”)</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr"/>
@@ -18482,13 +18482,13 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>재이 아니야! 재이 누나야!</t>
+          <t>너라고 하지 마라! 나도 엄마 아빠한테 너라고 한다!</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr"/>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>누가 누나를 “재이야” 하고 부르면 (모든 호칭은 태오 기준)</t>
+          <t>“너 엄마 아빠 말 잘 들어” 소리를 들으면</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr"/>
@@ -18504,13 +18504,13 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>이 안 닦아! 싫어!</t>
+          <t>재이 아니야! 재이 누나야!</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr"/>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>아침저녁 이 닦을 때 (도망 다니고 바닥을 기어요)</t>
+          <t>누가 누나를 “재이야” 하고 부르면 (모든 호칭은 태오 기준)</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr"/>
@@ -18526,13 +18526,13 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>누나 대단해!</t>
+          <t>이 안 닦아! 싫어!</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr"/>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>누나가 잠수를 보여 줬을 때</t>
+          <t>아침저녁 이 닦을 때 (도망 다니고 바닥을 기어요)</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr"/>
@@ -18548,13 +18548,13 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>엄마 인누와~</t>
+          <t>누나 대단해!</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr"/>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>밤에 자다 깨서 (엄마가 옆에서 재워 줄 때까지)</t>
+          <t>누나가 잠수를 보여 줬을 때</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr"/>
@@ -18570,13 +18570,13 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>왜 놀려! 놀리지 마!</t>
+          <t>엄마 인누와~</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr"/>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>“태오는 글씨·숫자 잘 몰라” 소리를 들으면 (손가락질하며)</t>
+          <t>밤에 자다 깨서 (엄마가 옆에서 재워 줄 때까지)</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr"/>
@@ -18592,13 +18592,13 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>왜 내 친구를 놀려! 슬프잖아!</t>
+          <t>왜 놀려! 놀리지 마!</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr"/>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>어린이집 친구가 놀림 받는 것 같을 때 (친구 편이에요)</t>
+          <t>“태오는 글씨·숫자 잘 몰라” 소리를 들으면 (손가락질하며)</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr"/>
@@ -18614,13 +18614,13 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>나 무지개빛 망토 갖고 싶어!</t>
+          <t>왜 내 친구를 놀려! 슬프잖아!</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr"/>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>파라큘라를 본 날부터 (또봇 Y도 같이 갖고 싶어요!)</t>
+          <t>어린이집 친구가 놀림 받는 것 같을 때 (친구 편이에요)</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr"/>
@@ -18636,13 +18636,13 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>어벤져스… 어셈블!</t>
+          <t>나 무지개빛 망토 갖고 싶어!</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr"/>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>엔드게임 마지막 장면을 따라 하며 가족을 다 모을 때</t>
+          <t>파라큘라를 본 날부터 (또봇 Y도 같이 갖고 싶어요!)</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr"/>
@@ -18658,13 +18658,13 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>왓 두 유 두, 캡틴? 위 파이트!</t>
+          <t>어벤져스… 어셈블!</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr"/>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>시빌 워 싸움 장면 놀이를 할 때</t>
+          <t>엔드게임 마지막 장면을 따라 하며 가족을 다 모을 때</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr"/>
@@ -18680,13 +18680,13 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>와칸다 포에버!</t>
+          <t>왓 두 유 두, 캡틴? 위 파이트!</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr"/>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>인피니티 워 장면처럼 다 같이 뛰어갈 때</t>
+          <t>시빌 워 싸움 장면 놀이를 할 때</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr"/>
@@ -18702,13 +18702,13 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>어린이집에 데리러 올 거야?</t>
+          <t>와칸다 포에버!</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr"/>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>어린이집 가기 싫은 아침에 (몇 번씩 확인해요)</t>
+          <t>인피니티 워 장면처럼 다 같이 뛰어갈 때</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr"/>
@@ -18724,13 +18724,13 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>어린이집 가기 싫다.</t>
+          <t>어린이집에 데리러 올 거야?</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr"/>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>월·화·수… 아침마다</t>
+          <t>어린이집 가기 싫은 아침에 (몇 번씩 확인해요)</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr"/>
@@ -18746,13 +18746,13 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?</t>
+          <t>어린이집 가기 싫다.</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr"/>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>싫은 태권도 가는 날</t>
+          <t>월·화·수… 아침마다</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr"/>
@@ -18768,13 +18768,13 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>오늘은 뽀로로 날! 내가 싫어하는 태권도 안 가는 날이다~</t>
+          <t>누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr"/>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>월요일 아침 (달력은 몰라도 뽀로로 날은 정확히 알아요)</t>
+          <t>싫은 태권도 가는 날</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr"/>
@@ -18785,18 +18785,18 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>아니야!</t>
+          <t>오늘은 뽀로로 날! 내가 싫어하는 태권도 안 가는 날이다~</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr"/>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>하루에도 제일 많이 하는 말</t>
+          <t>월요일 아침 (달력은 몰라도 뽀로로 날은 정확히 알아요)</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr"/>
@@ -18812,13 +18812,13 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>거짓말! 아니야!</t>
+          <t>아니야!</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr"/>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>기분 나쁘거나 하기 싫을 때</t>
+          <t>하루에도 제일 많이 하는 말</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr"/>
@@ -18834,13 +18834,13 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>맛있는데 지금은 먹기 싫어.</t>
+          <t>거짓말! 아니야!</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr"/>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>누가 음식을 권하면</t>
+          <t>기분 나쁘거나 하기 싫을 때</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr"/>
@@ -18856,13 +18856,13 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>치즈 냄새 극혐!</t>
+          <t>맛있는데 지금은 먹기 싫어.</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr"/>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>치즈만 보면 (냄새는 더더욱)</t>
+          <t>누가 음식을 권하면</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr"/>
@@ -18878,13 +18878,13 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>김태오!</t>
+          <t>치즈 냄새 극혐!</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr"/>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+          <t>치즈만 보면 (냄새는 더더욱)</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr"/>
@@ -18895,22 +18895,18 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>짐방</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>김서방</t>
-        </is>
-      </c>
+          <t>김태오!</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr"/>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr"/>
@@ -18926,17 +18922,17 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>꿍끙이</t>
+          <t>짐방</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>뿡뿡이</t>
+          <t>김서방</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr"/>
@@ -18945,10 +18941,26 @@
       <c r="A48" s="3" t="n">
         <v>45</v>
       </c>
-      <c r="B48" s="4" t="inlineStr"/>
-      <c r="C48" s="4" t="inlineStr"/>
-      <c r="D48" s="4" t="inlineStr"/>
-      <c r="E48" s="4" t="inlineStr"/>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>꿍끙이</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>뿡뿡이</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+        </is>
+      </c>
       <c r="F48" s="4" t="inlineStr"/>
     </row>
     <row r="49">
@@ -19091,8 +19103,18 @@
       <c r="E62" s="4" t="inlineStr"/>
       <c r="F62" s="4" t="inlineStr"/>
     </row>
+    <row r="63">
+      <c r="A63" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="B63" s="6" t="inlineStr"/>
+      <c r="C63" s="6" t="inlineStr"/>
+      <c r="D63" s="6" t="inlineStr"/>
+      <c r="E63" s="6" t="inlineStr"/>
+      <c r="F63" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F62"/>
+  <autoFilter ref="A3:F63"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add webtoon episode 28: 키 재는 날, 106과 100
New wall height-chart prop, hub card says 28 episodes. Draft was reviewed
with Gemini; the unknown reason for "100" is left as Taeo's secret.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -16,8 +16,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$461</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$475</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$59</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$63</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$11</definedName>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2094,17 +2094,47 @@
       <c r="A31" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="B31" s="7" t="n"/>
-      <c r="C31" s="7" t="n"/>
-      <c r="D31" s="7" t="n"/>
-      <c r="E31" s="7" t="n"/>
-      <c r="F31" s="7" t="n"/>
-      <c r="G31" s="7" t="n"/>
-      <c r="H31" s="7" t="n"/>
-      <c r="I31" s="7" t="n"/>
-      <c r="J31" s="7" t="inlineStr">
-        <is>
-          <t>기획 중</t>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>키 재는 날, 106과 100</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>밥 한 숟가락 먹고 달려가 키를 재는 태오. 정수리에 손을 올려야 하는데 뒤돌아서 눈앞의 숫자를 가리키며 “오늘은 작아졌네!” 그리고 다른 날엔 “106! 밥 많이 먹어서 100 될 거다~”</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>재이, 아빠, 태오</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>“밥 한 숟가락 먹고 키 재 봐야지~” 바로 달려감 / 정수리에 손을 대고 재야 하는데 뒤돌아서 눈앞의 95를 가리키며 “여기야? 오늘은 작아졌네” / “너 키 몇이야? 106! 밥 많이 먹어서 100 될 거다~” (106이 실제 키, 100 이유는 태오만 앎)</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>도와주는 아빠·재이 / 106cm를 확인하고 뿌듯한 태오 / “태오만 아는 비밀인가 봐” — 이유를 캐묻지 않고 받아 주는 가족</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>얼른 크고 싶은 마음은 밥 한 숟가락도 힘이 나게 해요. 키만큼 마음도 쑥쑥 자라요.</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>요즘 얼른 크고 싶은 만큼 내가 해 보는 일은 뭐예요? 우리 집 벽에서 가장 높은 곳은 어디일까요?</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="J31" s="6" t="inlineStr">
+        <is>
+          <t>완성</t>
         </is>
       </c>
     </row>
@@ -2144,13 +2174,31 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" s="7" t="n"/>
+      <c r="C34" s="7" t="n"/>
+      <c r="D34" s="7" t="n"/>
+      <c r="E34" s="7" t="n"/>
+      <c r="F34" s="7" t="n"/>
+      <c r="G34" s="7" t="n"/>
+      <c r="H34" s="7" t="n"/>
+      <c r="I34" s="7" t="n"/>
+      <c r="J34" s="7" t="inlineStr">
+        <is>
+          <t>기획 중</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:J30"/>
+  <autoFilter ref="A3:J31"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"아이디어,기획 중,콘티,완성"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2164,7 +2212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H461"/>
+  <dimension ref="A1:H475"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -16843,8 +16891,474 @@
       <c r="G461" s="6" t="inlineStr"/>
       <c r="H461" s="6" t="inlineStr"/>
     </row>
+    <row r="462">
+      <c r="A462" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B462" s="4" t="inlineStr">
+        <is>
+          <t>키 재는 날, 106과 100</t>
+        </is>
+      </c>
+      <c r="C462" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D462" s="4" t="inlineStr">
+        <is>
+          <t>부엌</t>
+        </is>
+      </c>
+      <c r="E462" s="4" t="inlineStr">
+        <is>
+          <t>태오, 아빠</t>
+        </is>
+      </c>
+      <c r="F462" s="4" t="inlineStr">
+        <is>
+          <t>저녁 식탁, 태오의 요즘 일과.</t>
+        </is>
+      </c>
+      <c r="G462" s="4" t="inlineStr">
+        <is>
+          <t>밥 한 숟가락 먹고 키 재 봐야지~</t>
+        </is>
+      </c>
+      <c r="H462" s="4" t="inlineStr">
+        <is>
+          <t>냠</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="B463" s="6" t="inlineStr">
+        <is>
+          <t>키 재는 날, 106과 100</t>
+        </is>
+      </c>
+      <c r="C463" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D463" s="6" t="inlineStr">
+        <is>
+          <t>효과: 속도선</t>
+        </is>
+      </c>
+      <c r="E463" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F463" s="6" t="inlineStr"/>
+      <c r="G463" s="6" t="inlineStr">
+        <is>
+          <t>키 재러 간다~!</t>
+        </is>
+      </c>
+      <c r="H463" s="6" t="inlineStr">
+        <is>
+          <t>우다다</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B464" s="4" t="inlineStr">
+        <is>
+          <t>키 재는 날, 106과 100</t>
+        </is>
+      </c>
+      <c r="C464" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D464" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E464" s="4" t="inlineStr">
+        <is>
+          <t>태오, 아빠</t>
+        </is>
+      </c>
+      <c r="F464" s="4" t="inlineStr">
+        <is>
+          <t>키는 정수리에 손을 대고 재야 하는데…</t>
+        </is>
+      </c>
+      <c r="G464" s="4" t="inlineStr">
+        <is>
+          <t>태오야, 정수리에 손을 올려 줄게~</t>
+        </is>
+      </c>
+      <c r="H464" s="4" t="inlineStr"/>
+    </row>
+    <row r="465">
+      <c r="A465" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="B465" s="6" t="inlineStr">
+        <is>
+          <t>키 재는 날, 106과 100</t>
+        </is>
+      </c>
+      <c r="C465" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D465" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E465" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F465" s="6" t="inlineStr">
+        <is>
+          <t>뒤돌아선 태오. 눈앞에 있는 숫자를 가리킨다.</t>
+        </is>
+      </c>
+      <c r="G465" s="6" t="inlineStr">
+        <is>
+          <t>여기야?</t>
+        </is>
+      </c>
+      <c r="H465" s="6" t="inlineStr">
+        <is>
+          <t>콕!</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B466" s="4" t="inlineStr">
+        <is>
+          <t>키 재는 날, 106과 100</t>
+        </is>
+      </c>
+      <c r="C466" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D466" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E466" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F466" s="4" t="inlineStr"/>
+      <c r="G466" s="4" t="inlineStr">
+        <is>
+          <t>오늘은 작아졌네…</t>
+        </is>
+      </c>
+      <c r="H466" s="4" t="inlineStr">
+        <is>
+          <t>쪼옥</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="B467" s="6" t="inlineStr">
+        <is>
+          <t>키 재는 날, 106과 100</t>
+        </is>
+      </c>
+      <c r="C467" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D467" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E467" s="6" t="inlineStr">
+        <is>
+          <t>재이, 아빠</t>
+        </is>
+      </c>
+      <c r="F467" s="6" t="inlineStr"/>
+      <c r="G467" s="6" t="inlineStr">
+        <is>
+          <t>아니야, 그건 눈높이 숫자야.
+키는 정수리! 자, 다시.</t>
+        </is>
+      </c>
+      <c r="H467" s="6" t="inlineStr"/>
+    </row>
+    <row r="468">
+      <c r="A468" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B468" s="4" t="inlineStr">
+        <is>
+          <t>키 재는 날, 106과 100</t>
+        </is>
+      </c>
+      <c r="C468" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D468" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E468" s="4" t="inlineStr">
+        <is>
+          <t>아빠, 태오</t>
+        </is>
+      </c>
+      <c r="F468" s="4" t="inlineStr"/>
+      <c r="G468" s="4" t="inlineStr">
+        <is>
+          <t>106cm! 우리 태오 많이 컸다.</t>
+        </is>
+      </c>
+      <c r="H468" s="4" t="inlineStr">
+        <is>
+          <t>쑤욱</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="B469" s="6" t="inlineStr">
+        <is>
+          <t>키 재는 날, 106과 100</t>
+        </is>
+      </c>
+      <c r="C469" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D469" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E469" s="6" t="inlineStr"/>
+      <c r="F469" s="6" t="inlineStr">
+        <is>
+          <t>다른 날. / 오늘도 키 재는 시간.</t>
+        </is>
+      </c>
+      <c r="G469" s="6" t="inlineStr"/>
+      <c r="H469" s="6" t="inlineStr"/>
+    </row>
+    <row r="470">
+      <c r="A470" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B470" s="4" t="inlineStr">
+        <is>
+          <t>키 재는 날, 106과 100</t>
+        </is>
+      </c>
+      <c r="C470" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D470" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E470" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F470" s="4" t="inlineStr"/>
+      <c r="G470" s="4" t="inlineStr">
+        <is>
+          <t>오늘도 키 재 봐야지~</t>
+        </is>
+      </c>
+      <c r="H470" s="4" t="inlineStr">
+        <is>
+          <t>콩콩</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="B471" s="6" t="inlineStr">
+        <is>
+          <t>키 재는 날, 106과 100</t>
+        </is>
+      </c>
+      <c r="C471" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D471" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E471" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F471" s="6" t="inlineStr">
+        <is>
+          <t>혼자 묻고,</t>
+        </is>
+      </c>
+      <c r="G471" s="6" t="inlineStr">
+        <is>
+          <t>너 키 몇이야?</t>
+        </is>
+      </c>
+      <c r="H471" s="6" t="inlineStr"/>
+    </row>
+    <row r="472">
+      <c r="A472" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B472" s="4" t="inlineStr">
+        <is>
+          <t>키 재는 날, 106과 100</t>
+        </is>
+      </c>
+      <c r="C472" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D472" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E472" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F472" s="4" t="inlineStr">
+        <is>
+          <t>혼자 대답한다.</t>
+        </is>
+      </c>
+      <c r="G472" s="4" t="inlineStr">
+        <is>
+          <t>106!</t>
+        </is>
+      </c>
+      <c r="H472" s="4" t="inlineStr">
+        <is>
+          <t>으쓱!</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="B473" s="6" t="inlineStr">
+        <is>
+          <t>키 재는 날, 106과 100</t>
+        </is>
+      </c>
+      <c r="C473" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D473" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E473" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F473" s="6" t="inlineStr"/>
+      <c r="G473" s="6" t="inlineStr">
+        <is>
+          <t>밥 많이 먹어서 100 될 거다~</t>
+        </is>
+      </c>
+      <c r="H473" s="6" t="inlineStr">
+        <is>
+          <t>꾹!</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B474" s="4" t="inlineStr">
+        <is>
+          <t>키 재는 날, 106과 100</t>
+        </is>
+      </c>
+      <c r="C474" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="D474" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E474" s="4" t="inlineStr">
+        <is>
+          <t>재이, 아빠</t>
+        </is>
+      </c>
+      <c r="F474" s="4" t="inlineStr"/>
+      <c r="G474" s="4" t="inlineStr">
+        <is>
+          <t>106인데… 왜 100이 돼?
+글쎄, 태오만 아는 비밀인가 봐.</t>
+        </is>
+      </c>
+      <c r="H474" s="4" t="inlineStr"/>
+    </row>
+    <row r="475">
+      <c r="A475" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="B475" s="6" t="inlineStr">
+        <is>
+          <t>키 재는 날, 106과 100</t>
+        </is>
+      </c>
+      <c r="C475" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="D475" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E475" s="6" t="inlineStr"/>
+      <c r="F475" s="6" t="inlineStr">
+        <is>
+          <t>벽의 자에는 오늘도 106이 새겨졌다. / 태오의 ‘100’은 아직 비밀!</t>
+        </is>
+      </c>
+      <c r="G475" s="6" t="inlineStr"/>
+      <c r="H475" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:H461"/>
+  <autoFilter ref="A3:H475"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add 태리토터 (Harry Potter) to the Taeo dictionary
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$475</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$60</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$63</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$11</definedName>
   </definedNames>
@@ -17372,7 +17372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18132,17 +18132,17 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>콩콩이차</t>
+          <t>태리토터</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>아우디 (자동차)</t>
+          <t>해리포터</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>아우디 동그라미 로고를 보고. “나도 콩콩이차 타고 싶다~”</t>
+          <t>TV에서 ‘해리포터와 아즈카반의 죄수’에 나오는 괴수를 보고 무서워해요</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr"/>
@@ -18154,17 +18154,17 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>둔쫀떡</t>
+          <t>콩콩이차</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>두바이 쫀득 찹쌀떡</t>
+          <t>아우디 (자동차)</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>아침에 먹으면 하루 종일 기분이 좋아져요</t>
+          <t>아우디 동그라미 로고를 보고. “나도 콩콩이차 타고 싶다~”</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr"/>
@@ -18176,17 +18176,17 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>발싸</t>
+          <t>둔쫀떡</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>발사</t>
+          <t>두바이 쫀득 찹쌀떡</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>“스밀로클로 발싸!” 기술을 쏠 때</t>
+          <t>아침에 먹으면 하루 종일 기분이 좋아져요</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr"/>
@@ -18198,17 +18198,17 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>안킬로해머 · 스밀로클로</t>
+          <t>발싸</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>다이노스터 기술</t>
+          <t>발사</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>래터킥, 퀀텀해로우… 하나씩 외치고 “쓰구미~”</t>
+          <t>“스밀로클로 발싸!” 기술을 쏠 때</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr"/>
@@ -18218,9 +18218,21 @@
       <c r="A40" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="B40" s="4" t="inlineStr"/>
-      <c r="C40" s="4" t="inlineStr"/>
-      <c r="D40" s="4" t="inlineStr"/>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>안킬로해머 · 스밀로클로</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>다이노스터 기술</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>래터킥, 퀀텀해로우… 하나씩 외치고 “쓰구미~”</t>
+        </is>
+      </c>
       <c r="E40" s="4" t="inlineStr"/>
       <c r="F40" s="4" t="inlineStr"/>
     </row>
@@ -18414,8 +18426,18 @@
       <c r="E59" s="6" t="inlineStr"/>
       <c r="F59" s="6" t="inlineStr"/>
     </row>
+    <row r="60">
+      <c r="A60" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="B60" s="4" t="inlineStr"/>
+      <c r="C60" s="4" t="inlineStr"/>
+      <c r="D60" s="4" t="inlineStr"/>
+      <c r="E60" s="4" t="inlineStr"/>
+      <c r="F60" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F59"/>
+  <autoFilter ref="A3:F60"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add episode 28: 루돌푸를 만났다 and 루돌푸 to the Taeo dictionary
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$461</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$471</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$63</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2094,17 +2094,47 @@
       <c r="A31" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="B31" s="7" t="n"/>
-      <c r="C31" s="7" t="n"/>
-      <c r="D31" s="7" t="n"/>
-      <c r="E31" s="7" t="n"/>
-      <c r="F31" s="7" t="n"/>
-      <c r="G31" s="7" t="n"/>
-      <c r="H31" s="7" t="n"/>
-      <c r="I31" s="7" t="n"/>
-      <c r="J31" s="7" t="inlineStr">
-        <is>
-          <t>기획 중</t>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>루돌푸를 만났다</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>디즈니랜드 캘리포니아에서 눈사람을 본 태오. “루돌푸다!” 이름은 틀려도 반가운 마음은 정확하다. 누나의 정정, 아빠의 사슴 이야기, 그리고 따뜻한 포옹.</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>재이, 엄마, 아빠, 태오</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>눈사람을 보고 “루돌푸다!” → 누나 “올라프야” → “아니야! 루돌푸야!!” / 아빠의 “루돌프는 빨간 코 사슴” → “…루돌푸 코 당근이야.” / 밤에 “루돌푸… 안녕…”</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>쑥스러워하며 “안아 줘도 돼?” → 따뜻한 포옹 / 이름은 틀려도 반가운 마음은 정확</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>이름은 틀려도 괜찮아요. 반갑다는 마음이 먼저 닿으면 돼요.</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>여행에서 제일 기억에 남는 장면은 뭐예요? 처음 만났을 때 이름을 틀리게 부른 적 있어요?</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="J31" s="6" t="inlineStr">
+        <is>
+          <t>완성</t>
         </is>
       </c>
     </row>
@@ -2144,13 +2174,31 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" s="7" t="n"/>
+      <c r="C34" s="7" t="n"/>
+      <c r="D34" s="7" t="n"/>
+      <c r="E34" s="7" t="n"/>
+      <c r="F34" s="7" t="n"/>
+      <c r="G34" s="7" t="n"/>
+      <c r="H34" s="7" t="n"/>
+      <c r="I34" s="7" t="n"/>
+      <c r="J34" s="7" t="inlineStr">
+        <is>
+          <t>기획 중</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:J30"/>
+  <autoFilter ref="A3:J31"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"아이디어,기획 중,콘티,완성"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2164,7 +2212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H461"/>
+  <dimension ref="A1:H471"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -16843,8 +16891,328 @@
       <c r="G461" s="6" t="inlineStr"/>
       <c r="H461" s="6" t="inlineStr"/>
     </row>
+    <row r="462">
+      <c r="A462" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B462" s="4" t="inlineStr">
+        <is>
+          <t>루돌푸를 만났다</t>
+        </is>
+      </c>
+      <c r="C462" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D462" s="4" t="inlineStr">
+        <is>
+          <t>단색</t>
+        </is>
+      </c>
+      <c r="E462" s="4" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="F462" s="4" t="inlineStr">
+        <is>
+          <t>디즈니랜드 캘리포니아. 햇볕이 쨍쨍한 날.</t>
+        </is>
+      </c>
+      <c r="G462" s="4" t="inlineStr">
+        <is>
+          <t>누나, 여기 진짜 신기하다!</t>
+        </is>
+      </c>
+      <c r="H462" s="4" t="inlineStr"/>
+    </row>
+    <row r="463">
+      <c r="A463" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="B463" s="6" t="inlineStr">
+        <is>
+          <t>루돌푸를 만났다</t>
+        </is>
+      </c>
+      <c r="C463" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D463" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E463" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F463" s="6" t="inlineStr"/>
+      <c r="G463" s="6" t="inlineStr">
+        <is>
+          <t>루돌푸다!!!</t>
+        </is>
+      </c>
+      <c r="H463" s="6" t="inlineStr">
+        <is>
+          <t>두둥!</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B464" s="4" t="inlineStr">
+        <is>
+          <t>루돌푸를 만났다</t>
+        </is>
+      </c>
+      <c r="C464" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D464" s="4" t="inlineStr">
+        <is>
+          <t>단색</t>
+        </is>
+      </c>
+      <c r="E464" s="4" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F464" s="4" t="inlineStr"/>
+      <c r="G464" s="4" t="inlineStr">
+        <is>
+          <t>태오야, 루돌푸가 아니라 올라프야.
+아니야! 루돌푸야!!</t>
+        </is>
+      </c>
+      <c r="H464" s="4" t="inlineStr"/>
+    </row>
+    <row r="465">
+      <c r="A465" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="B465" s="6" t="inlineStr">
+        <is>
+          <t>루돌푸를 만났다</t>
+        </is>
+      </c>
+      <c r="C465" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D465" s="6" t="inlineStr">
+        <is>
+          <t>단색</t>
+        </is>
+      </c>
+      <c r="E465" s="6" t="inlineStr">
+        <is>
+          <t>아빠, 태오</t>
+        </is>
+      </c>
+      <c r="F465" s="6" t="inlineStr"/>
+      <c r="G465" s="6" t="inlineStr">
+        <is>
+          <t>루돌프는 빨간 코 사슴인데~ 눈사람은 당근 코야.
+…루돌푸 코 당근이야.</t>
+        </is>
+      </c>
+      <c r="H465" s="6" t="inlineStr"/>
+    </row>
+    <row r="466">
+      <c r="A466" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B466" s="4" t="inlineStr">
+        <is>
+          <t>루돌푸를 만났다</t>
+        </is>
+      </c>
+      <c r="C466" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D466" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E466" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F466" s="4" t="inlineStr"/>
+      <c r="G466" s="4" t="inlineStr">
+        <is>
+          <t>루돌푸는 루돌푸라고 부를 거야!</t>
+        </is>
+      </c>
+      <c r="H466" s="4" t="inlineStr"/>
+    </row>
+    <row r="467">
+      <c r="A467" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="B467" s="6" t="inlineStr">
+        <is>
+          <t>루돌푸를 만났다</t>
+        </is>
+      </c>
+      <c r="C467" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D467" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E467" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F467" s="6" t="inlineStr">
+        <is>
+          <t>그래도 가까이 가니까, 조금 쑥스럽다.</t>
+        </is>
+      </c>
+      <c r="G467" s="6" t="inlineStr">
+        <is>
+          <t>(속삭임) …루돌푸, 안아 줘도 돼?</t>
+        </is>
+      </c>
+      <c r="H467" s="6" t="inlineStr"/>
+    </row>
+    <row r="468">
+      <c r="A468" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B468" s="4" t="inlineStr">
+        <is>
+          <t>루돌푸를 만났다</t>
+        </is>
+      </c>
+      <c r="C468" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D468" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E468" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F468" s="4" t="inlineStr">
+        <is>
+          <t>따뜻한 포옹이다.</t>
+        </is>
+      </c>
+      <c r="G468" s="4" t="inlineStr">
+        <is>
+          <t>루돌푸는 안 차가워. 따뜻해!</t>
+        </is>
+      </c>
+      <c r="H468" s="4" t="inlineStr"/>
+    </row>
+    <row r="469">
+      <c r="A469" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="B469" s="6" t="inlineStr">
+        <is>
+          <t>루돌푸를 만났다</t>
+        </is>
+      </c>
+      <c r="C469" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D469" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E469" s="6" t="inlineStr">
+        <is>
+          <t>엄마, 태오</t>
+        </is>
+      </c>
+      <c r="F469" s="6" t="inlineStr">
+        <is>
+          <t>그날 밤, 호텔 방.</t>
+        </is>
+      </c>
+      <c r="G469" s="6" t="inlineStr">
+        <is>
+          <t>오늘 제일 좋았던 게 뭐였어?
+루돌푸 안아 준 거!</t>
+        </is>
+      </c>
+      <c r="H469" s="6" t="inlineStr"/>
+    </row>
+    <row r="470">
+      <c r="A470" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B470" s="4" t="inlineStr">
+        <is>
+          <t>루돌푸를 만났다</t>
+        </is>
+      </c>
+      <c r="C470" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D470" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E470" s="4" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F470" s="4" t="inlineStr"/>
+      <c r="G470" s="4" t="inlineStr">
+        <is>
+          <t>(속삭임) …올라프야.
+(속삭임) 루돌푸… 안녕…</t>
+        </is>
+      </c>
+      <c r="H470" s="4" t="inlineStr"/>
+    </row>
+    <row r="471">
+      <c r="A471" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="B471" s="6" t="inlineStr">
+        <is>
+          <t>루돌푸를 만났다</t>
+        </is>
+      </c>
+      <c r="C471" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D471" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E471" s="6" t="inlineStr"/>
+      <c r="F471" s="6" t="inlineStr">
+        <is>
+          <t>이름은 조금 달라도, / 반갑다는 마음은 정확하게 전해졌다.</t>
+        </is>
+      </c>
+      <c r="G471" s="6" t="inlineStr"/>
+      <c r="H471" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:H461"/>
+  <autoFilter ref="A3:H471"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -16858,7 +17226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -17662,17 +18030,17 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>발싸</t>
+          <t>루돌푸</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>발사</t>
+          <t>올라프</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>“스밀로클로 발싸!” 기술을 쏠 때</t>
+          <t>디즈니랜드 캘리포니아에서 만난 눈사람 친구</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr"/>
@@ -17684,17 +18052,17 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>안킬로해머 · 스밀로클로</t>
+          <t>발싸</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>다이노스터 기술</t>
+          <t>발사</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>래터킥, 퀀텀해로우… 하나씩 외치고 “쓰구미~”</t>
+          <t>“스밀로클로 발싸!” 기술을 쏠 때</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr"/>
@@ -17704,9 +18072,21 @@
       <c r="A40" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="B40" s="4" t="inlineStr"/>
-      <c r="C40" s="4" t="inlineStr"/>
-      <c r="D40" s="4" t="inlineStr"/>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>안킬로해머 · 스밀로클로</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>다이노스터 기술</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>래터킥, 퀀텀해로우… 하나씩 외치고 “쓰구미~”</t>
+        </is>
+      </c>
       <c r="E40" s="4" t="inlineStr"/>
       <c r="F40" s="4" t="inlineStr"/>
     </row>
@@ -17900,8 +18280,18 @@
       <c r="E59" s="6" t="inlineStr"/>
       <c r="F59" s="6" t="inlineStr"/>
     </row>
+    <row r="60">
+      <c r="A60" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="B60" s="4" t="inlineStr"/>
+      <c r="C60" s="4" t="inlineStr"/>
+      <c r="D60" s="4" t="inlineStr"/>
+      <c r="E60" s="4" t="inlineStr"/>
+      <c r="F60" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F59"/>
+  <autoFilter ref="A3:F60"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -17915,7 +18305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18680,13 +19070,13 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>와칸다 포에버!</t>
+          <t>루돌푸다! 루돌푸는 루돌푸라고 부를 거야!</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr"/>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>인피니티 워 장면처럼 다 같이 뛰어갈 때</t>
+          <t>누나가 “올라프야” 하고 고쳐 줘도 (디즈니랜드에서)</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr"/>
@@ -18702,13 +19092,13 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>어린이집에 데리러 올 거야?</t>
+          <t>와칸다 포에버!</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr"/>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>어린이집 가기 싫은 아침에 (몇 번씩 확인해요)</t>
+          <t>인피니티 워 장면처럼 다 같이 뛰어갈 때</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr"/>
@@ -18724,13 +19114,13 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>어린이집 가기 싫다.</t>
+          <t>어린이집에 데리러 올 거야?</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr"/>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>월·화·수… 아침마다</t>
+          <t>어린이집 가기 싫은 아침에 (몇 번씩 확인해요)</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr"/>
@@ -18746,13 +19136,13 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?</t>
+          <t>어린이집 가기 싫다.</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr"/>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>싫은 태권도 가는 날</t>
+          <t>월·화·수… 아침마다</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr"/>
@@ -18768,13 +19158,13 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>오늘은 뽀로로 날! 내가 싫어하는 태권도 안 가는 날이다~</t>
+          <t>누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr"/>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>월요일 아침 (달력은 몰라도 뽀로로 날은 정확히 알아요)</t>
+          <t>싫은 태권도 가는 날</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr"/>
@@ -18785,18 +19175,18 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>아니야!</t>
+          <t>오늘은 뽀로로 날! 내가 싫어하는 태권도 안 가는 날이다~</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr"/>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>하루에도 제일 많이 하는 말</t>
+          <t>월요일 아침 (달력은 몰라도 뽀로로 날은 정확히 알아요)</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr"/>
@@ -18812,13 +19202,13 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>거짓말! 아니야!</t>
+          <t>아니야!</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr"/>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>기분 나쁘거나 하기 싫을 때</t>
+          <t>하루에도 제일 많이 하는 말</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr"/>
@@ -18834,13 +19224,13 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>맛있는데 지금은 먹기 싫어.</t>
+          <t>거짓말! 아니야!</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr"/>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>누가 음식을 권하면</t>
+          <t>기분 나쁘거나 하기 싫을 때</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr"/>
@@ -18856,13 +19246,13 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>치즈 냄새 극혐!</t>
+          <t>맛있는데 지금은 먹기 싫어.</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr"/>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>치즈만 보면 (냄새는 더더욱)</t>
+          <t>누가 음식을 권하면</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr"/>
@@ -18878,13 +19268,13 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>김태오!</t>
+          <t>치즈 냄새 극혐!</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr"/>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+          <t>치즈만 보면 (냄새는 더더욱)</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr"/>
@@ -18895,22 +19285,18 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>짐방</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>김서방</t>
-        </is>
-      </c>
+          <t>김태오!</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr"/>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr"/>
@@ -18926,17 +19312,17 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>꿍끙이</t>
+          <t>짐방</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>뿡뿡이</t>
+          <t>김서방</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr"/>
@@ -18945,10 +19331,26 @@
       <c r="A48" s="3" t="n">
         <v>45</v>
       </c>
-      <c r="B48" s="4" t="inlineStr"/>
-      <c r="C48" s="4" t="inlineStr"/>
-      <c r="D48" s="4" t="inlineStr"/>
-      <c r="E48" s="4" t="inlineStr"/>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>꿍끙이</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>뿡뿡이</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+        </is>
+      </c>
       <c r="F48" s="4" t="inlineStr"/>
     </row>
     <row r="49">
@@ -19091,8 +19493,18 @@
       <c r="E62" s="4" t="inlineStr"/>
       <c r="F62" s="4" t="inlineStr"/>
     </row>
+    <row r="63">
+      <c r="A63" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="B63" s="6" t="inlineStr"/>
+      <c r="C63" s="6" t="inlineStr"/>
+      <c r="D63" s="6" t="inlineStr"/>
+      <c r="E63" s="6" t="inlineStr"/>
+      <c r="F63" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F62"/>
+  <autoFilter ref="A3:F63"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add episode 29: 누나도 무서운 게 있다 (Orlando rides)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$471</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$483</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$60</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$64</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -551,7 +551,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>“아니야!”가 입버릇인 누나. 방은 늘 반듯하게 정리해 두고, 학교 숙제는 미리 다 해 놓고 노는 게 좋아요. 음식을 권하면 “맛있는데 지금은 먹기 싫어.” 치즈는 싫고 치즈 냄새는 극혐! 티니핑, 위시캣, 그리고 스파이더맨·판타스틱 4·어벤져스 같은 마블 영웅은 태오랑 둘 다 좋아해요. 동생이 괴롭혀도 참고 또 참다가, 폭발하면… “김태오!” 엉덩이 찰싹! 기분 나쁘거나 하기 싫을 때는 “거짓말! 아니야!” 잠수를 배워서 물이 눈에 들어가도 끄떡없어요.</t>
+          <t>“아니야!”가 입버릇인 누나. 방은 늘 반듯하게 정리해 두고, 학교 숙제는 미리 다 해 놓고 노는 게 좋아요. 음식을 권하면 “맛있는데 지금은 먹기 싫어.” 치즈는 싫고 치즈 냄새는 극혐! 티니핑, 위시캣, 그리고 스파이더맨·판타스틱 4·어벤져스 같은 마블 영웅은 태오랑 둘 다 좋아해요. 동생이 괴롭혀도 참고 또 참다가, 폭발하면… “김태오!” 엉덩이 찰싹! 기분 나쁘거나 하기 싫을 때는 “거짓말! 아니야!” 잠수를 배워서 물이 눈에 들어가도 끄떡없어요. 올랜도에서 스타워즈 놀이기구는 신나게 탔지만 가디언즈 오브 갤럭시는 너무 무서워서, 이제 떨어지는 건 안 타요.</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2139,20 +2139,50 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="n">
+      <c r="A32" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="B32" s="7" t="n"/>
-      <c r="C32" s="7" t="n"/>
-      <c r="D32" s="7" t="n"/>
-      <c r="E32" s="7" t="n"/>
-      <c r="F32" s="7" t="n"/>
-      <c r="G32" s="7" t="n"/>
-      <c r="H32" s="7" t="n"/>
-      <c r="I32" s="7" t="n"/>
-      <c r="J32" s="7" t="inlineStr">
-        <is>
-          <t>기획 중</t>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>누나도 무서운 게 있다</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>올랜도 디즈니 월드에서 스타워즈는 신나게, 가디언즈는 비명 속에. “나 이제 떨어지는 건 안 탈 거야.” 그날 용감한 동생은 누나에게 반쪽 레몬을 내밀었다.</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>스타워즈 줄에서 “치앗촤!” / 가디언즈 “아니야, 하나도 안 무서워.” → 비명 / 신난 태오 “누나 시끄러워~ 또 타자!” / “아니야! 안 무서웠어!” → 태오 “거짓말! 아니야!”(누나 말투 되돌려 주기) / 반쪽 레몬을 내밀며 “튼튼해져!”</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>무서워서 이제 떨어지는 건 안 탄다는 누나를 놀리지 않고 “태오가 탈게, 누나는 손 흔들어 줘” / 동생이 누나 편이 되는 날</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>무서운 건 부끄러운 게 아니에요. 무섭다고 말하면 손 잡아 주는 사람이 생겨요.</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>내가 제일 무서웠던 건 뭐예요? 무서울 때 누가 옆에 있어 주면 좋아요?</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>완성</t>
         </is>
       </c>
     </row>
@@ -2192,13 +2222,31 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="B35" s="7" t="n"/>
+      <c r="C35" s="7" t="n"/>
+      <c r="D35" s="7" t="n"/>
+      <c r="E35" s="7" t="n"/>
+      <c r="F35" s="7" t="n"/>
+      <c r="G35" s="7" t="n"/>
+      <c r="H35" s="7" t="n"/>
+      <c r="I35" s="7" t="n"/>
+      <c r="J35" s="7" t="inlineStr">
+        <is>
+          <t>기획 중</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:J31"/>
+  <autoFilter ref="A3:J32"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"아이디어,기획 중,콘티,완성"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2212,7 +2260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H471"/>
+  <dimension ref="A1:H483"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -17211,8 +17259,391 @@
       <c r="G471" s="6" t="inlineStr"/>
       <c r="H471" s="6" t="inlineStr"/>
     </row>
+    <row r="472">
+      <c r="A472" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B472" s="4" t="inlineStr">
+        <is>
+          <t>누나도 무서운 게 있다</t>
+        </is>
+      </c>
+      <c r="C472" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D472" s="4" t="inlineStr">
+        <is>
+          <t>단색</t>
+        </is>
+      </c>
+      <c r="E472" s="4" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="F472" s="4" t="inlineStr">
+        <is>
+          <t>올랜도 디즈니 월드. 스타워즈 라이즈 오브 레지스탕스 줄.</t>
+        </is>
+      </c>
+      <c r="G472" s="4" t="inlineStr">
+        <is>
+          <t>누나, 이거 우주 전쟁이야! 치앗촤!</t>
+        </is>
+      </c>
+      <c r="H472" s="4" t="inlineStr"/>
+    </row>
+    <row r="473">
+      <c r="A473" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="B473" s="6" t="inlineStr">
+        <is>
+          <t>누나도 무서운 게 있다</t>
+        </is>
+      </c>
+      <c r="C473" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D473" s="6" t="inlineStr">
+        <is>
+          <t>효과: 속도선</t>
+        </is>
+      </c>
+      <c r="E473" s="6" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="F473" s="6" t="inlineStr"/>
+      <c r="G473" s="6" t="inlineStr">
+        <is>
+          <t>또 타자! 또 타자!
+재밌다~! 이건 괜찮아!</t>
+        </is>
+      </c>
+      <c r="H473" s="6" t="inlineStr">
+        <is>
+          <t>슝~</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B474" s="4" t="inlineStr">
+        <is>
+          <t>누나도 무서운 게 있다</t>
+        </is>
+      </c>
+      <c r="C474" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D474" s="4" t="inlineStr">
+        <is>
+          <t>단색</t>
+        </is>
+      </c>
+      <c r="E474" s="4" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F474" s="4" t="inlineStr">
+        <is>
+          <t>다음은 가디언즈 오브 갤럭시.</t>
+        </is>
+      </c>
+      <c r="G474" s="4" t="inlineStr">
+        <is>
+          <t>아니야, 하나도 안 무서워.</t>
+        </is>
+      </c>
+      <c r="H474" s="4" t="inlineStr"/>
+    </row>
+    <row r="475">
+      <c r="A475" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="B475" s="6" t="inlineStr">
+        <is>
+          <t>누나도 무서운 게 있다</t>
+        </is>
+      </c>
+      <c r="C475" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D475" s="6" t="inlineStr">
+        <is>
+          <t>효과: 속도선</t>
+        </is>
+      </c>
+      <c r="E475" s="6" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F475" s="6" t="inlineStr"/>
+      <c r="G475" s="6" t="inlineStr">
+        <is>
+          <t>으아아아아악!!!</t>
+        </is>
+      </c>
+      <c r="H475" s="6" t="inlineStr">
+        <is>
+          <t>쉬이잉!, 덜컹</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B476" s="4" t="inlineStr">
+        <is>
+          <t>누나도 무서운 게 있다</t>
+        </is>
+      </c>
+      <c r="C476" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D476" s="4" t="inlineStr">
+        <is>
+          <t>효과: 속도선</t>
+        </is>
+      </c>
+      <c r="E476" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F476" s="4" t="inlineStr"/>
+      <c r="G476" s="4" t="inlineStr">
+        <is>
+          <t>누나 시끄러워~! 또 타자~!</t>
+        </is>
+      </c>
+      <c r="H476" s="4" t="inlineStr"/>
+    </row>
+    <row r="477">
+      <c r="A477" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="B477" s="6" t="inlineStr">
+        <is>
+          <t>누나도 무서운 게 있다</t>
+        </is>
+      </c>
+      <c r="C477" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D477" s="6" t="inlineStr">
+        <is>
+          <t>효과: 어두움</t>
+        </is>
+      </c>
+      <c r="E477" s="6" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F477" s="6" t="inlineStr"/>
+      <c r="G477" s="6" t="inlineStr">
+        <is>
+          <t>(속삭임) …나 이제 떨어지는 건 안 탈 거야.</t>
+        </is>
+      </c>
+      <c r="H477" s="6" t="inlineStr"/>
+    </row>
+    <row r="478">
+      <c r="A478" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B478" s="4" t="inlineStr">
+        <is>
+          <t>누나도 무서운 게 있다</t>
+        </is>
+      </c>
+      <c r="C478" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D478" s="4" t="inlineStr">
+        <is>
+          <t>단색</t>
+        </is>
+      </c>
+      <c r="E478" s="4" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="F478" s="4" t="inlineStr"/>
+      <c r="G478" s="4" t="inlineStr">
+        <is>
+          <t>누나 무서웠지?
+아니야! 안 무서웠어!</t>
+        </is>
+      </c>
+      <c r="H478" s="4" t="inlineStr"/>
+    </row>
+    <row r="479">
+      <c r="A479" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="B479" s="6" t="inlineStr">
+        <is>
+          <t>누나도 무서운 게 있다</t>
+        </is>
+      </c>
+      <c r="C479" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D479" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E479" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F479" s="6" t="inlineStr"/>
+      <c r="G479" s="6" t="inlineStr">
+        <is>
+          <t>거짓말! 아니야!!</t>
+        </is>
+      </c>
+      <c r="H479" s="6" t="inlineStr">
+        <is>
+          <t>찌릿</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B480" s="4" t="inlineStr">
+        <is>
+          <t>누나도 무서운 게 있다</t>
+        </is>
+      </c>
+      <c r="C480" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D480" s="4" t="inlineStr">
+        <is>
+          <t>단색</t>
+        </is>
+      </c>
+      <c r="E480" s="4" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="F480" s="4" t="inlineStr"/>
+      <c r="G480" s="4" t="inlineStr">
+        <is>
+          <t>누나, 레몬 먹어! 튼튼해져!</t>
+        </is>
+      </c>
+      <c r="H480" s="4" t="inlineStr"/>
+    </row>
+    <row r="481">
+      <c r="A481" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="B481" s="6" t="inlineStr">
+        <is>
+          <t>누나도 무서운 게 있다</t>
+        </is>
+      </c>
+      <c r="C481" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D481" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E481" s="6" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F481" s="6" t="inlineStr"/>
+      <c r="G481" s="6" t="inlineStr">
+        <is>
+          <t>으엑, 셔!!</t>
+        </is>
+      </c>
+      <c r="H481" s="6" t="inlineStr">
+        <is>
+          <t>찌잉</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B482" s="4" t="inlineStr">
+        <is>
+          <t>누나도 무서운 게 있다</t>
+        </is>
+      </c>
+      <c r="C482" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D482" s="4" t="inlineStr">
+        <is>
+          <t>단색</t>
+        </is>
+      </c>
+      <c r="E482" s="4" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F482" s="4" t="inlineStr"/>
+      <c r="G482" s="4" t="inlineStr">
+        <is>
+          <t>…고마워. 그래도 떨어지는 건 안 탈래.
+알았어! 태오가 탈게. 누나는 손 흔들어 줘!</t>
+        </is>
+      </c>
+      <c r="H482" s="4" t="inlineStr"/>
+    </row>
+    <row r="483">
+      <c r="A483" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="B483" s="6" t="inlineStr">
+        <is>
+          <t>누나도 무서운 게 있다</t>
+        </is>
+      </c>
+      <c r="C483" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D483" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E483" s="6" t="inlineStr"/>
+      <c r="F483" s="6" t="inlineStr">
+        <is>
+          <t>누나도 무서운 게 있고, / 동생이 누나 편이 되는 날도 있다.</t>
+        </is>
+      </c>
+      <c r="G483" s="6" t="inlineStr"/>
+      <c r="H483" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:H471"/>
+  <autoFilter ref="A3:H483"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -18305,7 +18736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -19290,13 +19721,13 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>김태오!</t>
+          <t>나 이제 떨어지는 건 안 탈 거야.</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr"/>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+          <t>올랜도 디즈니 월드에서 가디언즈 오브 갤럭시를 타고 너무 무서웠던 뒤로</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr"/>
@@ -19307,22 +19738,18 @@
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>짐방</t>
-        </is>
-      </c>
-      <c r="D47" s="6" t="inlineStr">
-        <is>
-          <t>김서방</t>
-        </is>
-      </c>
+          <t>김태오!</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr"/>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr"/>
@@ -19338,17 +19765,17 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>꿍끙이</t>
+          <t>짐방</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>뿡뿡이</t>
+          <t>김서방</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr"/>
@@ -19357,10 +19784,26 @@
       <c r="A49" s="5" t="n">
         <v>46</v>
       </c>
-      <c r="B49" s="6" t="inlineStr"/>
-      <c r="C49" s="6" t="inlineStr"/>
-      <c r="D49" s="6" t="inlineStr"/>
-      <c r="E49" s="6" t="inlineStr"/>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>꿍끙이</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>뿡뿡이</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+        </is>
+      </c>
       <c r="F49" s="6" t="inlineStr"/>
     </row>
     <row r="50">
@@ -19503,8 +19946,18 @@
       <c r="E63" s="6" t="inlineStr"/>
       <c r="F63" s="6" t="inlineStr"/>
     </row>
+    <row r="64">
+      <c r="A64" s="3" t="n">
+        <v>61</v>
+      </c>
+      <c r="B64" s="4" t="inlineStr"/>
+      <c r="C64" s="4" t="inlineStr"/>
+      <c r="D64" s="4" t="inlineStr"/>
+      <c r="E64" s="4" t="inlineStr"/>
+      <c r="F64" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F63"/>
+  <autoFilter ref="A3:F64"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add episode 30: 누나 또 하자! (One Card, 3-6-9 and tangled words)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$483</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$499</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$60</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>반쪽 레몬을 늘 손에 들고 다니며 할짝할짝 핥아 먹는 막내(레몬·자두·파인애플처럼 신 과일이 제일 좋아요). 누나 괴롭히기가 취미인 막내(사실은 누나가 좋아서). 혼자 노는 것 같아도 가족 말을 다 듣고 있고, 틀려도 일단 소리 지르며 우기다가 들키면 머리를 긁적긁적. “맛있는 거 죠!”가 입버릇이고, 누나랑 같이 좋아하는 마블 영웅(스파이더맨, 판타스틱 4, 어벤져스)도 태오식으로 불러요(블루베리, 쉬터맨, 스테잌로저…). 블랙 위도우랑 수가 제일 예쁘대요. 제일 좋아하는 놀이는 어벤져스로 타노스랑 싸우기! 모든 호칭은 태오 기준이라, 누가 “재이야” 하면 “재이 누나야!” 하고 고쳐 줘요. 요즘은 화가 나면 뾰족한 말이 튀어나오지만, “나 화났어!” 주문을 연습 중이에요. 물이 눈에 들어가는 걸 엄청 무서워하고, 이 닦기를 제일 싫어해서 아침저녁으로 도망 다니고 바닥을 기어 다니며 엄마 아빠를 고생시켜요. 어린이집 친구가 놀림 받으면 “왜 내 친구를 놀려! 슬프잖아!” 하고 친구 편을 들어요. 캡틴 아메리카가 헬리콥터를 붙잡는 장면, 스파이더맨이 갈라지는 배를 거미줄로 버티는 장면을 제일 좋아하고, 드라큘라는 “파라큘라”, 무지개빛 망토와 또봇 Y가 갖고 싶대요. 아침마다 치카하기 싫어서 기어 다니고, 어린이집에 가기 싫어서 “데리러 올 거야?” 하고 몇 번씩 물어요. 태권도 가는 날은 “누나는 왜 학교만 가?” 하지만, 월요일은 태권도 안 가는 뽀로로 날!</t>
+          <t>반쪽 레몬을 늘 손에 들고 다니며 할짝할짝 핥아 먹는 막내(레몬·자두·파인애플처럼 신 과일이 제일 좋아요). 누나 괴롭히기가 취미인 막내(사실은 누나가 좋아서). 혼자 노는 것 같아도 가족 말을 다 듣고 있고, 틀려도 일단 소리 지르며 우기다가 들키면 머리를 긁적긁적. “맛있는 거 죠!”가 입버릇이고, 누나랑 같이 좋아하는 마블 영웅(스파이더맨, 판타스틱 4, 어벤져스)도 태오식으로 불러요(블루베리, 쉬터맨, 스테잌로저…). 블랙 위도우랑 수가 제일 예쁘대요. 제일 좋아하는 놀이는 어벤져스로 타노스랑 싸우기! 모든 호칭은 태오 기준이라, 누가 “재이야” 하면 “재이 누나야!” 하고 고쳐 줘요. 요즘은 화가 나면 뾰족한 말이 튀어나오지만, “나 화났어!” 주문을 연습 중이에요. 물이 눈에 들어가는 걸 엄청 무서워하고, 이 닦기를 제일 싫어해서 아침저녁으로 도망 다니고 바닥을 기어 다니며 엄마 아빠를 고생시켜요. 어린이집 친구가 놀림 받으면 “왜 내 친구를 놀려! 슬프잖아!” 하고 친구 편을 들어요. 캡틴 아메리카가 헬리콥터를 붙잡는 장면, 스파이더맨이 갈라지는 배를 거미줄로 버티는 장면을 제일 좋아하고, 드라큘라는 “파라큘라”, 무지개빛 망토와 또봇 Y가 갖고 싶대요. 아침마다 치카하기 싫어서 기어 다니고, 어린이집에 가기 싫어서 “데리러 올 거야?” 하고 몇 번씩 물어요. 태권도 가는 날은 “누나는 왜 학교만 가?” 하지만, 월요일은 태권도 안 가는 뽀로로 날! 제일 좋아하는 게임은 원카드라 누나가 지겨워해도 “또 하자!”, 요즘은 3·6·9 박수도 멈추지 않아요. 혼잣말하다 말이 꼬이면 버럭 화를 내요.</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2190,17 +2190,47 @@
       <c r="A33" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="B33" s="7" t="n"/>
-      <c r="C33" s="7" t="n"/>
-      <c r="D33" s="7" t="n"/>
-      <c r="E33" s="7" t="n"/>
-      <c r="F33" s="7" t="n"/>
-      <c r="G33" s="7" t="n"/>
-      <c r="H33" s="7" t="n"/>
-      <c r="I33" s="7" t="n"/>
-      <c r="J33" s="7" t="inlineStr">
-        <is>
-          <t>기획 중</t>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>누나 또 하자!</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>렌터카를 기다리는 동안 원카드만 열 판 넘게. “난 한 번도 못 이겼단 말이야!” 차 안에서는 3·6·9 박수가 멈추지 않고, 말이 꼬이면 버럭. 그래도 누나는 한 판 더 해 준다.</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>재이, 엄마, 아빠, 태오</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>렌터카 줄에서 원카드 열 판 넘게 → 누나 “지겨워…” → “난 한 번도 못 이겼단 말이야!!” / 차 안 3·6·9 “하나, 둘, 짝!” → 4에도 짝! 30분 박수 / 혼잣말하다 “왜 말이 안 나와!!” → 생각난 말은 “원카드!”</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>지겨워도 “딱 한 판만 더” 해 주는 누나 / “천천히 해도 돼” 기다려 주는 엄마 / 열한 번째 판 결과는 비밀</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>져도 “또 하자” 말하는 건 용기예요. 지겨워도 한 판 더 해 주는 건 사랑이에요.</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr">
+        <is>
+          <t>우리 가족이 제일 좋아하는 게임은 뭐예요? 계속 져서 속상했던 적 있어요?</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>완성</t>
         </is>
       </c>
     </row>
@@ -2240,13 +2270,31 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="B36" s="7" t="n"/>
+      <c r="C36" s="7" t="n"/>
+      <c r="D36" s="7" t="n"/>
+      <c r="E36" s="7" t="n"/>
+      <c r="F36" s="7" t="n"/>
+      <c r="G36" s="7" t="n"/>
+      <c r="H36" s="7" t="n"/>
+      <c r="I36" s="7" t="n"/>
+      <c r="J36" s="7" t="inlineStr">
+        <is>
+          <t>기획 중</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:J32"/>
+  <autoFilter ref="A3:J33"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"아이디어,기획 중,콘티,완성"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2260,7 +2308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H483"/>
+  <dimension ref="A1:H499"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -17642,8 +17690,518 @@
       <c r="G483" s="6" t="inlineStr"/>
       <c r="H483" s="6" t="inlineStr"/>
     </row>
+    <row r="484">
+      <c r="A484" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B484" s="4" t="inlineStr">
+        <is>
+          <t>누나 또 하자!</t>
+        </is>
+      </c>
+      <c r="C484" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D484" s="4" t="inlineStr">
+        <is>
+          <t>단색</t>
+        </is>
+      </c>
+      <c r="E484" s="4" t="inlineStr">
+        <is>
+          <t>아빠, 태오</t>
+        </is>
+      </c>
+      <c r="F484" s="4" t="inlineStr">
+        <is>
+          <t>렌터카 빌리는 줄. 기다림이 길다.</t>
+        </is>
+      </c>
+      <c r="G484" s="4" t="inlineStr">
+        <is>
+          <t>누나! 원카드 하자!
+(생각) (아직 한참 남았네…)</t>
+        </is>
+      </c>
+      <c r="H484" s="4" t="inlineStr"/>
+    </row>
+    <row r="485">
+      <c r="A485" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="B485" s="6" t="inlineStr">
+        <is>
+          <t>누나 또 하자!</t>
+        </is>
+      </c>
+      <c r="C485" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D485" s="6" t="inlineStr">
+        <is>
+          <t>단색</t>
+        </is>
+      </c>
+      <c r="E485" s="6" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="F485" s="6" t="inlineStr"/>
+      <c r="G485" s="6" t="inlineStr">
+        <is>
+          <t>원카드!
+어? 어?!</t>
+        </is>
+      </c>
+      <c r="H485" s="6" t="inlineStr"/>
+    </row>
+    <row r="486">
+      <c r="A486" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B486" s="4" t="inlineStr">
+        <is>
+          <t>누나 또 하자!</t>
+        </is>
+      </c>
+      <c r="C486" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D486" s="4" t="inlineStr">
+        <is>
+          <t>단색</t>
+        </is>
+      </c>
+      <c r="E486" s="4" t="inlineStr"/>
+      <c r="F486" s="4" t="inlineStr">
+        <is>
+          <t>한 판 더. 또 한 판 더. / 그리고 또, 또, 또…</t>
+        </is>
+      </c>
+      <c r="G486" s="4" t="inlineStr"/>
+      <c r="H486" s="4" t="inlineStr">
+        <is>
+          <t>3판, 7판, 10판!</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="B487" s="6" t="inlineStr">
+        <is>
+          <t>누나 또 하자!</t>
+        </is>
+      </c>
+      <c r="C487" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D487" s="6" t="inlineStr">
+        <is>
+          <t>효과: 어두움</t>
+        </is>
+      </c>
+      <c r="E487" s="6" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F487" s="6" t="inlineStr"/>
+      <c r="G487" s="6" t="inlineStr">
+        <is>
+          <t>(속삭임) 태오야… 벌써 열 번 넘게 했어. 지겨워…</t>
+        </is>
+      </c>
+      <c r="H487" s="6" t="inlineStr"/>
+    </row>
+    <row r="488">
+      <c r="A488" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B488" s="4" t="inlineStr">
+        <is>
+          <t>누나 또 하자!</t>
+        </is>
+      </c>
+      <c r="C488" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D488" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E488" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F488" s="4" t="inlineStr"/>
+      <c r="G488" s="4" t="inlineStr">
+        <is>
+          <t>난 한 번도 못 이겼단 말이야!!</t>
+        </is>
+      </c>
+      <c r="H488" s="4" t="inlineStr">
+        <is>
+          <t>버럭!</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="B489" s="6" t="inlineStr">
+        <is>
+          <t>누나 또 하자!</t>
+        </is>
+      </c>
+      <c r="C489" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D489" s="6" t="inlineStr">
+        <is>
+          <t>단색</t>
+        </is>
+      </c>
+      <c r="E489" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F489" s="6" t="inlineStr"/>
+      <c r="G489" s="6" t="inlineStr">
+        <is>
+          <t>누나… 또 하자…</t>
+        </is>
+      </c>
+      <c r="H489" s="6" t="inlineStr"/>
+    </row>
+    <row r="490">
+      <c r="A490" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B490" s="4" t="inlineStr">
+        <is>
+          <t>누나 또 하자!</t>
+        </is>
+      </c>
+      <c r="C490" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D490" s="4" t="inlineStr">
+        <is>
+          <t>단색</t>
+        </is>
+      </c>
+      <c r="E490" s="4" t="inlineStr">
+        <is>
+          <t>재이, 아빠</t>
+        </is>
+      </c>
+      <c r="F490" s="4" t="inlineStr"/>
+      <c r="G490" s="4" t="inlineStr">
+        <is>
+          <t>…딱 한 판만 더.
+차 나왔다~! 출발!</t>
+        </is>
+      </c>
+      <c r="H490" s="4" t="inlineStr"/>
+    </row>
+    <row r="491">
+      <c r="A491" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="B491" s="6" t="inlineStr">
+        <is>
+          <t>누나 또 하자!</t>
+        </is>
+      </c>
+      <c r="C491" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D491" s="6" t="inlineStr">
+        <is>
+          <t>효과: 속도선</t>
+        </is>
+      </c>
+      <c r="E491" s="6" t="inlineStr">
+        <is>
+          <t>아빠, 태오</t>
+        </is>
+      </c>
+      <c r="F491" s="6" t="inlineStr">
+        <is>
+          <t>렌터카 안. 아빠가 새 게임을 알려 준다.</t>
+        </is>
+      </c>
+      <c r="G491" s="6" t="inlineStr">
+        <is>
+          <t>3, 6, 9가 나오면 박수 치는 거야!
+박수?!</t>
+        </is>
+      </c>
+      <c r="H491" s="6" t="inlineStr"/>
+    </row>
+    <row r="492">
+      <c r="A492" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B492" s="4" t="inlineStr">
+        <is>
+          <t>누나 또 하자!</t>
+        </is>
+      </c>
+      <c r="C492" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D492" s="4" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E492" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F492" s="4" t="inlineStr"/>
+      <c r="G492" s="4" t="inlineStr">
+        <is>
+          <t>하나, 둘, 짝!</t>
+        </is>
+      </c>
+      <c r="H492" s="4" t="inlineStr">
+        <is>
+          <t>짝!</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="B493" s="6" t="inlineStr">
+        <is>
+          <t>누나 또 하자!</t>
+        </is>
+      </c>
+      <c r="C493" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D493" s="6" t="inlineStr">
+        <is>
+          <t>효과: 속도선</t>
+        </is>
+      </c>
+      <c r="E493" s="6" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F493" s="6" t="inlineStr">
+        <is>
+          <t>그 뒤로 30분 동안 박수가 멈추지 않았다.</t>
+        </is>
+      </c>
+      <c r="G493" s="6" t="inlineStr">
+        <is>
+          <t>태오야, 4는 박수 아니야!
+짝! 짝! 짝!</t>
+        </is>
+      </c>
+      <c r="H493" s="6" t="inlineStr">
+        <is>
+          <t>짝!, 짝!</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B494" s="4" t="inlineStr">
+        <is>
+          <t>누나 또 하자!</t>
+        </is>
+      </c>
+      <c r="C494" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D494" s="4" t="inlineStr">
+        <is>
+          <t>단색</t>
+        </is>
+      </c>
+      <c r="E494" s="4" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F494" s="4" t="inlineStr"/>
+      <c r="G494" s="4" t="inlineStr">
+        <is>
+          <t>(속삭임) 그러니까… 그거… 그… 우와 그… 뭐지…</t>
+        </is>
+      </c>
+      <c r="H494" s="4" t="inlineStr"/>
+    </row>
+    <row r="495">
+      <c r="A495" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="B495" s="6" t="inlineStr">
+        <is>
+          <t>누나 또 하자!</t>
+        </is>
+      </c>
+      <c r="C495" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D495" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E495" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F495" s="6" t="inlineStr"/>
+      <c r="G495" s="6" t="inlineStr">
+        <is>
+          <t>아 진짜! 왜 말이 안 나와!!</t>
+        </is>
+      </c>
+      <c r="H495" s="6" t="inlineStr">
+        <is>
+          <t>부글부글</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B496" s="4" t="inlineStr">
+        <is>
+          <t>누나 또 하자!</t>
+        </is>
+      </c>
+      <c r="C496" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="D496" s="4" t="inlineStr">
+        <is>
+          <t>효과: 속도선</t>
+        </is>
+      </c>
+      <c r="E496" s="4" t="inlineStr">
+        <is>
+          <t>엄마, 태오</t>
+        </is>
+      </c>
+      <c r="F496" s="4" t="inlineStr"/>
+      <c r="G496" s="4" t="inlineStr">
+        <is>
+          <t>천천히 해도 돼. 생각나면 말해 줘.
+…흥.</t>
+        </is>
+      </c>
+      <c r="H496" s="4" t="inlineStr"/>
+    </row>
+    <row r="497">
+      <c r="A497" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="B497" s="6" t="inlineStr">
+        <is>
+          <t>누나 또 하자!</t>
+        </is>
+      </c>
+      <c r="C497" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="D497" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E497" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F497" s="6" t="inlineStr"/>
+      <c r="G497" s="6" t="inlineStr">
+        <is>
+          <t>생각났다! 원카드! 원카드 또 하고 싶다고!</t>
+        </is>
+      </c>
+      <c r="H497" s="6" t="inlineStr"/>
+    </row>
+    <row r="498">
+      <c r="A498" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B498" s="4" t="inlineStr">
+        <is>
+          <t>누나 또 하자!</t>
+        </is>
+      </c>
+      <c r="C498" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="D498" s="4" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E498" s="4" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F498" s="4" t="inlineStr"/>
+      <c r="G498" s="4" t="inlineStr">
+        <is>
+          <t>…알았어. 숙소 가서 한 판 더.</t>
+        </is>
+      </c>
+      <c r="H498" s="4" t="inlineStr"/>
+    </row>
+    <row r="499">
+      <c r="A499" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="B499" s="6" t="inlineStr">
+        <is>
+          <t>누나 또 하자!</t>
+        </is>
+      </c>
+      <c r="C499" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="D499" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E499" s="6" t="inlineStr"/>
+      <c r="F499" s="6" t="inlineStr">
+        <is>
+          <t>열한 번째 판의 결과는, / 아직도 비밀이다.</t>
+        </is>
+      </c>
+      <c r="G499" s="6" t="inlineStr"/>
+      <c r="H499" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:H483"/>
+  <autoFilter ref="A3:H499"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -18736,7 +19294,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:F67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -19523,13 +20081,13 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>와칸다 포에버!</t>
+          <t>난 한 번도 못 이겼단 말이야! 누나 또 하자!</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr"/>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>인피니티 워 장면처럼 다 같이 뛰어갈 때</t>
+          <t>제일 좋아하는 원카드를 열 판 넘게 하고도 (누나가 지겨워해도)</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr"/>
@@ -19545,13 +20103,13 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>어린이집에 데리러 올 거야?</t>
+          <t>짝! 짝! 짝!</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr"/>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>어린이집 가기 싫은 아침에 (몇 번씩 확인해요)</t>
+          <t>3·6·9 게임을 배운 뒤로 차 안에서 계속 (아무 숫자에나 박수)</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr"/>
@@ -19567,13 +20125,13 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>어린이집 가기 싫다.</t>
+          <t>아 진짜! 왜 말이 안 나와!</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr"/>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>월·화·수… 아침마다</t>
+          <t>혼잣말하다가 단어가 생각 안 나거나 말이 꼬일 때</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr"/>
@@ -19589,13 +20147,13 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?</t>
+          <t>와칸다 포에버!</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr"/>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>싫은 태권도 가는 날</t>
+          <t>인피니티 워 장면처럼 다 같이 뛰어갈 때</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr"/>
@@ -19611,13 +20169,13 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>오늘은 뽀로로 날! 내가 싫어하는 태권도 안 가는 날이다~</t>
+          <t>어린이집에 데리러 올 거야?</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr"/>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>월요일 아침 (달력은 몰라도 뽀로로 날은 정확히 알아요)</t>
+          <t>어린이집 가기 싫은 아침에 (몇 번씩 확인해요)</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr"/>
@@ -19628,18 +20186,18 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>아니야!</t>
+          <t>어린이집 가기 싫다.</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr"/>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>하루에도 제일 많이 하는 말</t>
+          <t>월·화·수… 아침마다</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr"/>
@@ -19650,18 +20208,18 @@
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>거짓말! 아니야!</t>
+          <t>누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr"/>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>기분 나쁘거나 하기 싫을 때</t>
+          <t>싫은 태권도 가는 날</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr"/>
@@ -19672,18 +20230,18 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>맛있는데 지금은 먹기 싫어.</t>
+          <t>오늘은 뽀로로 날! 내가 싫어하는 태권도 안 가는 날이다~</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr"/>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>누가 음식을 권하면</t>
+          <t>월요일 아침 (달력은 몰라도 뽀로로 날은 정확히 알아요)</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr"/>
@@ -19699,13 +20257,13 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>치즈 냄새 극혐!</t>
+          <t>아니야!</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr"/>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>치즈만 보면 (냄새는 더더욱)</t>
+          <t>하루에도 제일 많이 하는 말</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr"/>
@@ -19721,13 +20279,13 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>나 이제 떨어지는 건 안 탈 거야.</t>
+          <t>거짓말! 아니야!</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr"/>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>올랜도 디즈니 월드에서 가디언즈 오브 갤럭시를 타고 너무 무서웠던 뒤로</t>
+          <t>기분 나쁘거나 하기 싫을 때</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr"/>
@@ -19743,13 +20301,13 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>김태오!</t>
+          <t>맛있는데 지금은 먹기 싫어.</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr"/>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+          <t>누가 음식을 권하면</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr"/>
@@ -19760,22 +20318,18 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>짐방</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>김서방</t>
-        </is>
-      </c>
+          <t>치즈 냄새 극혐!</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr"/>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+          <t>치즈만 보면 (냄새는 더더욱)</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr"/>
@@ -19786,22 +20340,18 @@
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>꿍끙이</t>
-        </is>
-      </c>
-      <c r="D49" s="6" t="inlineStr">
-        <is>
-          <t>뿡뿡이</t>
-        </is>
-      </c>
+          <t>나 이제 떨어지는 건 안 탈 거야.</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr"/>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+          <t>올랜도 디즈니 월드에서 가디언즈 오브 갤럭시를 타고 너무 무서웠던 뒤로</t>
         </is>
       </c>
       <c r="F49" s="6" t="inlineStr"/>
@@ -19810,30 +20360,74 @@
       <c r="A50" s="3" t="n">
         <v>47</v>
       </c>
-      <c r="B50" s="4" t="inlineStr"/>
-      <c r="C50" s="4" t="inlineStr"/>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>재이 입버릇</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>김태오!</t>
+        </is>
+      </c>
       <c r="D50" s="4" t="inlineStr"/>
-      <c r="E50" s="4" t="inlineStr"/>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+        </is>
+      </c>
       <c r="F50" s="4" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n">
         <v>48</v>
       </c>
-      <c r="B51" s="6" t="inlineStr"/>
-      <c r="C51" s="6" t="inlineStr"/>
-      <c r="D51" s="6" t="inlineStr"/>
-      <c r="E51" s="6" t="inlineStr"/>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>짐방</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>김서방</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+        </is>
+      </c>
       <c r="F51" s="6" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n">
         <v>49</v>
       </c>
-      <c r="B52" s="4" t="inlineStr"/>
-      <c r="C52" s="4" t="inlineStr"/>
-      <c r="D52" s="4" t="inlineStr"/>
-      <c r="E52" s="4" t="inlineStr"/>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>꿍끙이</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>뿡뿡이</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+        </is>
+      </c>
       <c r="F52" s="4" t="inlineStr"/>
     </row>
     <row r="53">
@@ -19956,8 +20550,38 @@
       <c r="E64" s="4" t="inlineStr"/>
       <c r="F64" s="4" t="inlineStr"/>
     </row>
+    <row r="65">
+      <c r="A65" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="B65" s="6" t="inlineStr"/>
+      <c r="C65" s="6" t="inlineStr"/>
+      <c r="D65" s="6" t="inlineStr"/>
+      <c r="E65" s="6" t="inlineStr"/>
+      <c r="F65" s="6" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="B66" s="4" t="inlineStr"/>
+      <c r="C66" s="4" t="inlineStr"/>
+      <c r="D66" s="4" t="inlineStr"/>
+      <c r="E66" s="4" t="inlineStr"/>
+      <c r="F66" s="4" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="B67" s="6" t="inlineStr"/>
+      <c r="C67" s="6" t="inlineStr"/>
+      <c r="D67" s="6" t="inlineStr"/>
+      <c r="E67" s="6" t="inlineStr"/>
+      <c r="F67" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F64"/>
+  <autoFilter ref="A3:F67"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Episode 31: Jaei and Taeo shout 하나 together and call 찌찌뽕
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -17,9 +17,9 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$514</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$516</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$61</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$70</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2245,7 +2245,7 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>31화니까 배스킨라빈스 31 게임! 아니, 태오식으로는 “배스틴라빈스”. 31을 외치고 신난 태오, 라스베가스 게임도 하자, 3·6·9에서는 “박수 한 번만 치고 싶어!”</t>
+          <t>31화니까 배스킨라빈스 31 게임! 아니, 태오식으로는 “배스틴라빈스”. 31을 외치고 신난 태오, 라스베가스 게임도 하자, 3·6·9에서는 누나랑 “하나!” 동시에 외치고 찌찌뽕, 그리고 “박수 한 번만 치고 싶어!”</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>“배스틴라빈스 하자!” “배스킨라빈스야.” “아니야!” / “넷, 다섯, 서른하나!! 내가 31 말했다!” → 지는 거야 → “이번 건 연습이야!” / 엄마가 몰래 숫자 알려 주기 → 아빠 타노스 또 패배 / “라스베가스 게임 하자!” / 3·6·9 “박수 한 번만 치고 싶어! 짝!”</t>
+          <t>“배스틴라빈스 하자!” “배스킨라빈스야.” “아니야!” / “넷, 다섯, 서른하나!! 내가 31 말했다!” → 지는 거야 → “이번 건 연습이야!” / 엄마가 몰래 숫자 알려 주기 → 아빠 타노스 또 패배 / “라스베가스 게임 하자!” / “계속 3·6·9 하자~~” → 누나랑 동시에 “하나!” → “찌찌뽕!!” / “박수 한 번만 치고 싶어! 짝!”</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
@@ -2274,7 +2274,7 @@
         </is>
       </c>
       <c r="I34" s="3" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
@@ -2356,7 +2356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H514"/>
+  <dimension ref="A1:H516"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -18596,7 +18596,7 @@
       <c r="G510" s="4" t="inlineStr">
         <is>
           <t>라스베가스는 내일 하자. 이제 잘 시간.
-그럼 3·6·9 딱 한 번만!</t>
+그럼 3·6·9 하자~~ 계속 3·6·9 하자~~</t>
         </is>
       </c>
       <c r="H510" s="4" t="inlineStr"/>
@@ -18623,18 +18623,18 @@
           <t>재이, 태오</t>
         </is>
       </c>
-      <c r="F511" s="6" t="inlineStr"/>
+      <c r="F511" s="6" t="inlineStr">
+        <is>
+          <t>시작하자마자, 둘이 동시에.</t>
+        </is>
+      </c>
       <c r="G511" s="6" t="inlineStr">
         <is>
           <t>하나!
-박수 한 번만 치고 싶어! 짝!</t>
-        </is>
-      </c>
-      <c r="H511" s="6" t="inlineStr">
-        <is>
-          <t>짝!</t>
-        </is>
-      </c>
+하나!</t>
+        </is>
+      </c>
+      <c r="H511" s="6" t="inlineStr"/>
     </row>
     <row r="512">
       <c r="A512" s="3" t="n">
@@ -18650,7 +18650,7 @@
       </c>
       <c r="D512" s="4" t="inlineStr">
         <is>
-          <t>거실(밤)</t>
+          <t>효과: 집중선</t>
         </is>
       </c>
       <c r="E512" s="4" t="inlineStr">
@@ -18661,13 +18661,12 @@
       <c r="F512" s="4" t="inlineStr"/>
       <c r="G512" s="4" t="inlineStr">
         <is>
-          <t>1은 박수 아니야!
-한 번만! 짝! 한 번만! 짝!</t>
+          <t>찌찌뽕!!</t>
         </is>
       </c>
       <c r="H512" s="4" t="inlineStr">
         <is>
-          <t>짝!</t>
+          <t>뽕!</t>
         </is>
       </c>
     </row>
@@ -18685,23 +18684,24 @@
       </c>
       <c r="D513" s="6" t="inlineStr">
         <is>
-          <t>방(밤)</t>
+          <t>거실(밤)</t>
         </is>
       </c>
       <c r="E513" s="6" t="inlineStr">
         <is>
-          <t>태오</t>
+          <t>재이, 태오</t>
         </is>
       </c>
       <c r="F513" s="6" t="inlineStr"/>
       <c r="G513" s="6" t="inlineStr">
         <is>
-          <t>(속삭임) …짝… 한 번만…</t>
+          <t>…둘!
+박수 한 번만 치고 싶어! 짝!</t>
         </is>
       </c>
       <c r="H513" s="6" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>짝!</t>
         </is>
       </c>
     </row>
@@ -18719,20 +18719,89 @@
       </c>
       <c r="D514" s="4" t="inlineStr">
         <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E514" s="4" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F514" s="4" t="inlineStr"/>
+      <c r="G514" s="4" t="inlineStr">
+        <is>
+          <t>2는 박수 아니야!
+한 번만! 짝! 한 번만! 짝!</t>
+        </is>
+      </c>
+      <c r="H514" s="4" t="inlineStr">
+        <is>
+          <t>짝!</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="B515" s="6" t="inlineStr">
+        <is>
+          <t>배스틴라빈스 하자!</t>
+        </is>
+      </c>
+      <c r="C515" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="D515" s="6" t="inlineStr">
+        <is>
+          <t>방(밤)</t>
+        </is>
+      </c>
+      <c r="E515" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F515" s="6" t="inlineStr"/>
+      <c r="G515" s="6" t="inlineStr">
+        <is>
+          <t>(속삭임) …짝… 한 번만…</t>
+        </is>
+      </c>
+      <c r="H515" s="6" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B516" s="4" t="inlineStr">
+        <is>
+          <t>배스틴라빈스 하자!</t>
+        </is>
+      </c>
+      <c r="C516" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="D516" s="4" t="inlineStr">
+        <is>
           <t>효과: 반짝</t>
         </is>
       </c>
-      <c r="E514" s="4" t="inlineStr"/>
-      <c r="F514" s="4" t="inlineStr">
+      <c r="E516" s="4" t="inlineStr"/>
+      <c r="F516" s="4" t="inlineStr">
         <is>
           <t>오늘 밤 태오의 “한 번만” 박수는, / 꼭 서른한 번이었다.</t>
         </is>
       </c>
-      <c r="G514" s="4" t="inlineStr"/>
-      <c r="H514" s="4" t="inlineStr"/>
+      <c r="G516" s="4" t="inlineStr"/>
+      <c r="H516" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:H514"/>
+  <autoFilter ref="A3:H516"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -19847,7 +19916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -20722,13 +20791,13 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>박수 한 번만 치고 싶어!</t>
+          <t>계속 3·6·9 하자~~</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr"/>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>3·6·9 게임을 하면서 계속 (박수 차례가 아니어도)</t>
+          <t>3·6·9를 배운 뒤로 틈만 나면 (누나랑 “하나!” 같이 외치면 찌찌뽕!)</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr"/>
@@ -20744,13 +20813,13 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>와칸다 포에버!</t>
+          <t>박수 한 번만 치고 싶어!</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr"/>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>인피니티 워 장면처럼 다 같이 뛰어갈 때</t>
+          <t>3·6·9 게임을 하면서 계속 (박수 차례가 아니어도)</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr"/>
@@ -20766,13 +20835,13 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>어린이집에 데리러 올 거야?</t>
+          <t>와칸다 포에버!</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr"/>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>어린이집 가기 싫은 아침에 (몇 번씩 확인해요)</t>
+          <t>인피니티 워 장면처럼 다 같이 뛰어갈 때</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr"/>
@@ -20788,13 +20857,13 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>어린이집 가기 싫다.</t>
+          <t>어린이집에 데리러 올 거야?</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr"/>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>월·화·수… 아침마다</t>
+          <t>어린이집 가기 싫은 아침에 (몇 번씩 확인해요)</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr"/>
@@ -20810,13 +20879,13 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?</t>
+          <t>어린이집 가기 싫다.</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr"/>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>싫은 태권도 가는 날</t>
+          <t>월·화·수… 아침마다</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr"/>
@@ -20832,13 +20901,13 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>오늘은 뽀로로 날! 내가 싫어하는 태권도 안 가는 날이다~</t>
+          <t>누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr"/>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>월요일 아침 (달력은 몰라도 뽀로로 날은 정확히 알아요)</t>
+          <t>싫은 태권도 가는 날</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr"/>
@@ -20849,18 +20918,18 @@
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>아니야!</t>
+          <t>오늘은 뽀로로 날! 내가 싫어하는 태권도 안 가는 날이다~</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr"/>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>하루에도 제일 많이 하는 말</t>
+          <t>월요일 아침 (달력은 몰라도 뽀로로 날은 정확히 알아요)</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr"/>
@@ -20876,13 +20945,13 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>거짓말! 아니야!</t>
+          <t>아니야!</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr"/>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>기분 나쁘거나 하기 싫을 때</t>
+          <t>하루에도 제일 많이 하는 말</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr"/>
@@ -20898,13 +20967,13 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>맛있는데 지금은 먹기 싫어.</t>
+          <t>거짓말! 아니야!</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr"/>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>누가 음식을 권하면</t>
+          <t>기분 나쁘거나 하기 싫을 때</t>
         </is>
       </c>
       <c r="F49" s="6" t="inlineStr"/>
@@ -20920,13 +20989,13 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>치즈 냄새 극혐!</t>
+          <t>맛있는데 지금은 먹기 싫어.</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr"/>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>치즈만 보면 (냄새는 더더욱)</t>
+          <t>누가 음식을 권하면</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr"/>
@@ -20942,13 +21011,13 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>나 이제 떨어지는 건 안 탈 거야.</t>
+          <t>치즈 냄새 극혐!</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr"/>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>올랜도 디즈니 월드에서 가디언즈 오브 갤럭시를 타고 너무 무서웠던 뒤로</t>
+          <t>치즈만 보면 (냄새는 더더욱)</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr"/>
@@ -20964,13 +21033,13 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>김태오!</t>
+          <t>나 이제 떨어지는 건 안 탈 거야.</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr"/>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+          <t>올랜도 디즈니 월드에서 가디언즈 오브 갤럭시를 타고 너무 무서웠던 뒤로</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr"/>
@@ -20981,22 +21050,18 @@
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>짐방</t>
-        </is>
-      </c>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>김서방</t>
-        </is>
-      </c>
+          <t>김태오!</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr"/>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
         </is>
       </c>
       <c r="F53" s="6" t="inlineStr"/>
@@ -21012,17 +21077,17 @@
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>꿍끙이</t>
+          <t>짐방</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>뿡뿡이</t>
+          <t>김서방</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr"/>
@@ -21031,10 +21096,26 @@
       <c r="A55" s="5" t="n">
         <v>52</v>
       </c>
-      <c r="B55" s="6" t="inlineStr"/>
-      <c r="C55" s="6" t="inlineStr"/>
-      <c r="D55" s="6" t="inlineStr"/>
-      <c r="E55" s="6" t="inlineStr"/>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>꿍끙이</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>뿡뿡이</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+        </is>
+      </c>
       <c r="F55" s="6" t="inlineStr"/>
     </row>
     <row r="56">
@@ -21177,8 +21258,18 @@
       <c r="E69" s="6" t="inlineStr"/>
       <c r="F69" s="6" t="inlineStr"/>
     </row>
+    <row r="70">
+      <c r="A70" s="3" t="n">
+        <v>67</v>
+      </c>
+      <c r="B70" s="4" t="inlineStr"/>
+      <c r="C70" s="4" t="inlineStr"/>
+      <c r="D70" s="4" t="inlineStr"/>
+      <c r="E70" s="4" t="inlineStr"/>
+      <c r="F70" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F69"/>
+  <autoFilter ref="A3:F70"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Episode 31: after 찌찌뽕 nobody may talk until someone says 뽕뽕찌
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -17,9 +17,9 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$516</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$520</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$61</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2245,7 +2245,7 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>31화니까 배스킨라빈스 31 게임! 아니, 태오식으로는 “배스틴라빈스”. 31을 외치고 신난 태오, 라스베가스 게임도 하자, 3·6·9에서는 누나랑 “하나!” 동시에 외치고 찌찌뽕, 그리고 “박수 한 번만 치고 싶어!”</t>
+          <t>31화니까 배스킨라빈스 31 게임! 아니, 태오식으로는 “배스틴라빈스”. 31을 외치고 신난 태오, 라스베가스 게임도 하자, 3·6·9에서는 누나랑 “하나!” 동시에 외치고 찌찌뽕(뽕뽕찌 할 때까지 입 꾹!), 그리고 “박수 한 번만 치고 싶어!”</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>“배스틴라빈스 하자!” “배스킨라빈스야.” “아니야!” / “넷, 다섯, 서른하나!! 내가 31 말했다!” → 지는 거야 → “이번 건 연습이야!” / 엄마가 몰래 숫자 알려 주기 → 아빠 타노스 또 패배 / “라스베가스 게임 하자!” / “계속 3·6·9 하자~~” → 누나랑 동시에 “하나!” → “찌찌뽕!!” / “박수 한 번만 치고 싶어! 짝!”</t>
+          <t>“배스틴라빈스 하자!” “배스킨라빈스야.” “아니야!” / “넷, 다섯, 서른하나!! 내가 31 말했다!” → 지는 거야 → “이번 건 연습이야!” / 엄마가 몰래 숫자 알려 주기 → 아빠 타노스 또 패배 / “라스베가스 게임 하자!” / “계속 3·6·9 하자~~” → 누나랑 동시에 “하나!” → “찌찌뽕!!” → 뽕뽕찌 해 줄 때까지 둘 다 입 꾹 (태오는 박수 치고 싶어서 부들부들) → 엄마 “뽕뽕찌!” → “푸하!” / “박수 한 번만 치고 싶어! 짝!”</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
@@ -2274,7 +2274,7 @@
         </is>
       </c>
       <c r="I34" s="3" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
@@ -2356,7 +2356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H516"/>
+  <dimension ref="A1:H520"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -18692,16 +18692,20 @@
           <t>재이, 태오</t>
         </is>
       </c>
-      <c r="F513" s="6" t="inlineStr"/>
+      <c r="F513" s="6" t="inlineStr">
+        <is>
+          <t>찌찌뽕을 하면, 누가 “뽕뽕찌” 해 줄 때까지 말하면 안 된다.</t>
+        </is>
+      </c>
       <c r="G513" s="6" t="inlineStr">
         <is>
-          <t>…둘!
-박수 한 번만 치고 싶어! 짝!</t>
+          <t>(생각) (……)
+(생각) (……)</t>
         </is>
       </c>
       <c r="H513" s="6" t="inlineStr">
         <is>
-          <t>짝!</t>
+          <t>읍!</t>
         </is>
       </c>
     </row>
@@ -18719,24 +18723,23 @@
       </c>
       <c r="D514" s="4" t="inlineStr">
         <is>
-          <t>거실(밤)</t>
+          <t>효과: 집중선</t>
         </is>
       </c>
       <c r="E514" s="4" t="inlineStr">
         <is>
-          <t>재이, 태오</t>
+          <t>태오</t>
         </is>
       </c>
       <c r="F514" s="4" t="inlineStr"/>
       <c r="G514" s="4" t="inlineStr">
         <is>
-          <t>2는 박수 아니야!
-한 번만! 짝! 한 번만! 짝!</t>
+          <t>(생각) (박수 치고 싶은데… 말하고 싶은데…!)</t>
         </is>
       </c>
       <c r="H514" s="4" t="inlineStr">
         <is>
-          <t>짝!</t>
+          <t>읍읍읍, 부들</t>
         </is>
       </c>
     </row>
@@ -18754,25 +18757,25 @@
       </c>
       <c r="D515" s="6" t="inlineStr">
         <is>
-          <t>방(밤)</t>
+          <t>거실(밤)</t>
         </is>
       </c>
       <c r="E515" s="6" t="inlineStr">
         <is>
-          <t>태오</t>
-        </is>
-      </c>
-      <c r="F515" s="6" t="inlineStr"/>
+          <t>엄마</t>
+        </is>
+      </c>
+      <c r="F515" s="6" t="inlineStr">
+        <is>
+          <t>엄마가 한참 웃다가 겨우 풀어 준다.</t>
+        </is>
+      </c>
       <c r="G515" s="6" t="inlineStr">
         <is>
-          <t>(속삭임) …짝… 한 번만…</t>
-        </is>
-      </c>
-      <c r="H515" s="6" t="inlineStr">
-        <is>
-          <t>Z</t>
-        </is>
-      </c>
+          <t>뽕뽕찌!</t>
+        </is>
+      </c>
+      <c r="H515" s="6" t="inlineStr"/>
     </row>
     <row r="516">
       <c r="A516" s="3" t="n">
@@ -18788,20 +18791,154 @@
       </c>
       <c r="D516" s="4" t="inlineStr">
         <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E516" s="4" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F516" s="4" t="inlineStr"/>
+      <c r="G516" s="4" t="inlineStr">
+        <is>
+          <t>푸하! 이제 말할 수 있다!</t>
+        </is>
+      </c>
+      <c r="H516" s="4" t="inlineStr"/>
+    </row>
+    <row r="517">
+      <c r="A517" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="B517" s="6" t="inlineStr">
+        <is>
+          <t>배스틴라빈스 하자!</t>
+        </is>
+      </c>
+      <c r="C517" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="D517" s="6" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E517" s="6" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F517" s="6" t="inlineStr"/>
+      <c r="G517" s="6" t="inlineStr">
+        <is>
+          <t>…둘!
+박수 한 번만 치고 싶어! 짝!</t>
+        </is>
+      </c>
+      <c r="H517" s="6" t="inlineStr">
+        <is>
+          <t>짝!</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B518" s="4" t="inlineStr">
+        <is>
+          <t>배스틴라빈스 하자!</t>
+        </is>
+      </c>
+      <c r="C518" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="D518" s="4" t="inlineStr">
+        <is>
+          <t>거실(밤)</t>
+        </is>
+      </c>
+      <c r="E518" s="4" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F518" s="4" t="inlineStr"/>
+      <c r="G518" s="4" t="inlineStr">
+        <is>
+          <t>2는 박수 아니야!
+한 번만! 짝! 한 번만! 짝!</t>
+        </is>
+      </c>
+      <c r="H518" s="4" t="inlineStr">
+        <is>
+          <t>짝!</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="B519" s="6" t="inlineStr">
+        <is>
+          <t>배스틴라빈스 하자!</t>
+        </is>
+      </c>
+      <c r="C519" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="D519" s="6" t="inlineStr">
+        <is>
+          <t>방(밤)</t>
+        </is>
+      </c>
+      <c r="E519" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F519" s="6" t="inlineStr"/>
+      <c r="G519" s="6" t="inlineStr">
+        <is>
+          <t>(속삭임) …짝… 한 번만…</t>
+        </is>
+      </c>
+      <c r="H519" s="6" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B520" s="4" t="inlineStr">
+        <is>
+          <t>배스틴라빈스 하자!</t>
+        </is>
+      </c>
+      <c r="C520" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="D520" s="4" t="inlineStr">
+        <is>
           <t>효과: 반짝</t>
         </is>
       </c>
-      <c r="E516" s="4" t="inlineStr"/>
-      <c r="F516" s="4" t="inlineStr">
+      <c r="E520" s="4" t="inlineStr"/>
+      <c r="F520" s="4" t="inlineStr">
         <is>
           <t>오늘 밤 태오의 “한 번만” 박수는, / 꼭 서른한 번이었다.</t>
         </is>
       </c>
-      <c r="G516" s="4" t="inlineStr"/>
-      <c r="H516" s="4" t="inlineStr"/>
+      <c r="G520" s="4" t="inlineStr"/>
+      <c r="H520" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:H516"/>
+  <autoFilter ref="A3:H520"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -19916,7 +20053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:F71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -20813,13 +20950,13 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>박수 한 번만 치고 싶어!</t>
+          <t>찌찌뽕!</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr"/>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>3·6·9 게임을 하면서 계속 (박수 차례가 아니어도)</t>
+          <t>누나랑 같은 말을 동시에 했을 때 (누가 “뽕뽕찌” 해 줄 때까지 말을 못 하고 꾹 참아요)</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr"/>
@@ -20835,13 +20972,13 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>와칸다 포에버!</t>
+          <t>박수 한 번만 치고 싶어!</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr"/>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>인피니티 워 장면처럼 다 같이 뛰어갈 때</t>
+          <t>3·6·9 게임을 하면서 계속 (박수 차례가 아니어도)</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr"/>
@@ -20857,13 +20994,13 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>어린이집에 데리러 올 거야?</t>
+          <t>와칸다 포에버!</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr"/>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>어린이집 가기 싫은 아침에 (몇 번씩 확인해요)</t>
+          <t>인피니티 워 장면처럼 다 같이 뛰어갈 때</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr"/>
@@ -20879,13 +21016,13 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>어린이집 가기 싫다.</t>
+          <t>어린이집에 데리러 올 거야?</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr"/>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>월·화·수… 아침마다</t>
+          <t>어린이집 가기 싫은 아침에 (몇 번씩 확인해요)</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr"/>
@@ -20901,13 +21038,13 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?</t>
+          <t>어린이집 가기 싫다.</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr"/>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>싫은 태권도 가는 날</t>
+          <t>월·화·수… 아침마다</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr"/>
@@ -20923,13 +21060,13 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>오늘은 뽀로로 날! 내가 싫어하는 태권도 안 가는 날이다~</t>
+          <t>누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr"/>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>월요일 아침 (달력은 몰라도 뽀로로 날은 정확히 알아요)</t>
+          <t>싫은 태권도 가는 날</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr"/>
@@ -20940,18 +21077,18 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>아니야!</t>
+          <t>오늘은 뽀로로 날! 내가 싫어하는 태권도 안 가는 날이다~</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr"/>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>하루에도 제일 많이 하는 말</t>
+          <t>월요일 아침 (달력은 몰라도 뽀로로 날은 정확히 알아요)</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr"/>
@@ -20967,13 +21104,13 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>거짓말! 아니야!</t>
+          <t>아니야!</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr"/>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>기분 나쁘거나 하기 싫을 때</t>
+          <t>하루에도 제일 많이 하는 말</t>
         </is>
       </c>
       <c r="F49" s="6" t="inlineStr"/>
@@ -20989,13 +21126,13 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>맛있는데 지금은 먹기 싫어.</t>
+          <t>거짓말! 아니야!</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr"/>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>누가 음식을 권하면</t>
+          <t>기분 나쁘거나 하기 싫을 때</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr"/>
@@ -21011,13 +21148,13 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>치즈 냄새 극혐!</t>
+          <t>맛있는데 지금은 먹기 싫어.</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr"/>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>치즈만 보면 (냄새는 더더욱)</t>
+          <t>누가 음식을 권하면</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr"/>
@@ -21033,13 +21170,13 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>나 이제 떨어지는 건 안 탈 거야.</t>
+          <t>치즈 냄새 극혐!</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr"/>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>올랜도 디즈니 월드에서 가디언즈 오브 갤럭시를 타고 너무 무서웠던 뒤로</t>
+          <t>치즈만 보면 (냄새는 더더욱)</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr"/>
@@ -21055,13 +21192,13 @@
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>김태오!</t>
+          <t>나 이제 떨어지는 건 안 탈 거야.</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr"/>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+          <t>올랜도 디즈니 월드에서 가디언즈 오브 갤럭시를 타고 너무 무서웠던 뒤로</t>
         </is>
       </c>
       <c r="F53" s="6" t="inlineStr"/>
@@ -21072,22 +21209,18 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>짐방</t>
-        </is>
-      </c>
-      <c r="D54" s="4" t="inlineStr">
-        <is>
-          <t>김서방</t>
-        </is>
-      </c>
+          <t>김태오!</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr"/>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr"/>
@@ -21103,17 +21236,17 @@
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>꿍끙이</t>
+          <t>짐방</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>뿡뿡이</t>
+          <t>김서방</t>
         </is>
       </c>
       <c r="E55" s="6" t="inlineStr">
         <is>
-          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
         </is>
       </c>
       <c r="F55" s="6" t="inlineStr"/>
@@ -21122,10 +21255,26 @@
       <c r="A56" s="3" t="n">
         <v>53</v>
       </c>
-      <c r="B56" s="4" t="inlineStr"/>
-      <c r="C56" s="4" t="inlineStr"/>
-      <c r="D56" s="4" t="inlineStr"/>
-      <c r="E56" s="4" t="inlineStr"/>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>꿍끙이</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>뿡뿡이</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+        </is>
+      </c>
       <c r="F56" s="4" t="inlineStr"/>
     </row>
     <row r="57">
@@ -21268,8 +21417,18 @@
       <c r="E70" s="4" t="inlineStr"/>
       <c r="F70" s="4" t="inlineStr"/>
     </row>
+    <row r="71">
+      <c r="A71" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="B71" s="6" t="inlineStr"/>
+      <c r="C71" s="6" t="inlineStr"/>
+      <c r="D71" s="6" t="inlineStr"/>
+      <c r="E71" s="6" t="inlineStr"/>
+      <c r="F71" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F70"/>
+  <autoFilter ref="A3:F71"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add episode 33: 가윌 가게 오픈! and 가윌 to the Taeo dictionary
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgYJfYKNHdeLAeBso6ziaf
</commit_message>
<xml_diff>
--- a/webtoon/planning/오늘도우리집_기획표.xlsx
+++ b/webtoon/planning/오늘도우리집_기획표.xlsx
@@ -16,10 +16,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'등장인물'!$A$3:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$35</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$531</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$61</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'에피소드'!$A$3:$J$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'컷 대본'!$A$3:$H$545</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'태오어 사전'!$A$3:$F$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'우리 집 말 모음'!$A$3:$F$74</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'다음 화 아이디어'!$A$3:$E$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2331,20 +2331,50 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="5" t="n">
+      <c r="A36" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="B36" s="7" t="n"/>
-      <c r="C36" s="7" t="n"/>
-      <c r="D36" s="7" t="n"/>
-      <c r="E36" s="7" t="n"/>
-      <c r="F36" s="7" t="n"/>
-      <c r="G36" s="7" t="n"/>
-      <c r="H36" s="7" t="n"/>
-      <c r="I36" s="7" t="n"/>
-      <c r="J36" s="7" t="inlineStr">
-        <is>
-          <t>기획 중</t>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>가윌 가게 오픈!</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>“우리 가게 놀이 할까?” “우리 가윌 없잖아!” 과일 없는 과일 가게를 살린 건 그림 과일, 할머니 바구니, 그리고 절대 안 파는 반쪽 레몬.</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>재이, 할머니, 엄마, 아빠, 할아버지, 태오</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>“우리 가게 놀이 할까?” “우리 가윌 없잖아!” / 그림 가윌 + 할머니 바구니로 ‘태오 가윌 가게’ 오픈 / 아빠 “그 레몬 주세요” → “이건 안 팔아! 태오 레몬이야!” / 엄마는 아빠 쉬는 쿠폰으로 계산, 값은 “맛있는 거 죠!”</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>돈 없는 할아버지에게 “공짜! 가족이니까!” / 다 먹으면 또 그리면 된다 / 문 닫을 때 누나에게만 레몬 한 번 핥게 해 주기</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>없는 건 같이 만들면 돼요. 나누는 가게가 제일 부자예요.</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>우리 집 가게 놀이를 한다면 무엇을 팔고 싶어요? 돈 대신 무엇을 받으면 좋을까요?</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>완성</t>
         </is>
       </c>
     </row>
@@ -2384,13 +2414,31 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" s="7" t="n"/>
+      <c r="C39" s="7" t="n"/>
+      <c r="D39" s="7" t="n"/>
+      <c r="E39" s="7" t="n"/>
+      <c r="F39" s="7" t="n"/>
+      <c r="G39" s="7" t="n"/>
+      <c r="H39" s="7" t="n"/>
+      <c r="I39" s="7" t="n"/>
+      <c r="J39" s="7" t="inlineStr">
+        <is>
+          <t>기획 중</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:J35"/>
+  <autoFilter ref="A3:J36"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"아이디어,기획 중,콘티,완성"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2404,7 +2452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H531"/>
+  <dimension ref="A1:H545"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -19357,8 +19405,442 @@
       <c r="G531" s="6" t="inlineStr"/>
       <c r="H531" s="6" t="inlineStr"/>
     </row>
+    <row r="532">
+      <c r="A532" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B532" s="4" t="inlineStr">
+        <is>
+          <t>가윌 가게 오픈!</t>
+        </is>
+      </c>
+      <c r="C532" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D532" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E532" s="4" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F532" s="4" t="inlineStr">
+        <is>
+          <t>비 오는 주말 오후.</t>
+        </is>
+      </c>
+      <c r="G532" s="4" t="inlineStr">
+        <is>
+          <t>우리 가게 놀이 할까?</t>
+        </is>
+      </c>
+      <c r="H532" s="4" t="inlineStr"/>
+    </row>
+    <row r="533">
+      <c r="A533" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="B533" s="6" t="inlineStr">
+        <is>
+          <t>가윌 가게 오픈!</t>
+        </is>
+      </c>
+      <c r="C533" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D533" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E533" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F533" s="6" t="inlineStr"/>
+      <c r="G533" s="6" t="inlineStr">
+        <is>
+          <t>우리 가윌 없잖아!</t>
+        </is>
+      </c>
+      <c r="H533" s="6" t="inlineStr"/>
+    </row>
+    <row r="534">
+      <c r="A534" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B534" s="4" t="inlineStr">
+        <is>
+          <t>가윌 가게 오픈!</t>
+        </is>
+      </c>
+      <c r="C534" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D534" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E534" s="4" t="inlineStr">
+        <is>
+          <t>재이, 태오</t>
+        </is>
+      </c>
+      <c r="F534" s="4" t="inlineStr"/>
+      <c r="G534" s="4" t="inlineStr">
+        <is>
+          <t>…가윌? 아, 과일?
+가윌! 가윌 가게 할 거야!</t>
+        </is>
+      </c>
+      <c r="H534" s="4" t="inlineStr"/>
+    </row>
+    <row r="535">
+      <c r="A535" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="B535" s="6" t="inlineStr">
+        <is>
+          <t>가윌 가게 오픈!</t>
+        </is>
+      </c>
+      <c r="C535" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D535" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E535" s="6" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F535" s="6" t="inlineStr">
+        <is>
+          <t>재이는 종이에 과일을 그려 오려 냈다.</t>
+        </is>
+      </c>
+      <c r="G535" s="6" t="inlineStr">
+        <is>
+          <t>수박, 포도, 딸기… 그림 가윌!</t>
+        </is>
+      </c>
+      <c r="H535" s="6" t="inlineStr"/>
+    </row>
+    <row r="536">
+      <c r="A536" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B536" s="4" t="inlineStr">
+        <is>
+          <t>가윌 가게 오픈!</t>
+        </is>
+      </c>
+      <c r="C536" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D536" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E536" s="4" t="inlineStr">
+        <is>
+          <t>할머니, 태오</t>
+        </is>
+      </c>
+      <c r="F536" s="4" t="inlineStr"/>
+      <c r="G536" s="4" t="inlineStr">
+        <is>
+          <t>진짜 가윌도 있다~
+우와! 할머니 가윌!</t>
+        </is>
+      </c>
+      <c r="H536" s="4" t="inlineStr"/>
+    </row>
+    <row r="537">
+      <c r="A537" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="B537" s="6" t="inlineStr">
+        <is>
+          <t>가윌 가게 오픈!</t>
+        </is>
+      </c>
+      <c r="C537" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D537" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E537" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F537" s="6" t="inlineStr"/>
+      <c r="G537" s="6" t="inlineStr">
+        <is>
+          <t>어서 오세요! 맛있는 가윌 있어요!</t>
+        </is>
+      </c>
+      <c r="H537" s="6" t="inlineStr"/>
+    </row>
+    <row r="538">
+      <c r="A538" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B538" s="4" t="inlineStr">
+        <is>
+          <t>가윌 가게 오픈!</t>
+        </is>
+      </c>
+      <c r="C538" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D538" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E538" s="4" t="inlineStr">
+        <is>
+          <t>아빠, 태오</t>
+        </is>
+      </c>
+      <c r="F538" s="4" t="inlineStr"/>
+      <c r="G538" s="4" t="inlineStr">
+        <is>
+          <t>사장님, 그 레몬 하나 주세요~
+이건 안 팔아!</t>
+        </is>
+      </c>
+      <c r="H538" s="4" t="inlineStr"/>
+    </row>
+    <row r="539">
+      <c r="A539" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="B539" s="6" t="inlineStr">
+        <is>
+          <t>가윌 가게 오픈!</t>
+        </is>
+      </c>
+      <c r="C539" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D539" s="6" t="inlineStr">
+        <is>
+          <t>효과: 집중선</t>
+        </is>
+      </c>
+      <c r="E539" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F539" s="6" t="inlineStr"/>
+      <c r="G539" s="6" t="inlineStr">
+        <is>
+          <t>이건 태오 레몬이야! 가게 거 아니야!</t>
+        </is>
+      </c>
+      <c r="H539" s="6" t="inlineStr"/>
+    </row>
+    <row r="540">
+      <c r="A540" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B540" s="4" t="inlineStr">
+        <is>
+          <t>가윌 가게 오픈!</t>
+        </is>
+      </c>
+      <c r="C540" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D540" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E540" s="4" t="inlineStr">
+        <is>
+          <t>엄마, 태오</t>
+        </is>
+      </c>
+      <c r="F540" s="4" t="inlineStr"/>
+      <c r="G540" s="4" t="inlineStr">
+        <is>
+          <t>딸기 주세요. 얼마예요?
+음… 맛있는 거 죠!</t>
+        </is>
+      </c>
+      <c r="H540" s="4" t="inlineStr"/>
+    </row>
+    <row r="541">
+      <c r="A541" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="B541" s="6" t="inlineStr">
+        <is>
+          <t>가윌 가게 오픈!</t>
+        </is>
+      </c>
+      <c r="C541" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D541" s="6" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E541" s="6" t="inlineStr">
+        <is>
+          <t>할아버지, 태오</t>
+        </is>
+      </c>
+      <c r="F541" s="6" t="inlineStr"/>
+      <c r="G541" s="6" t="inlineStr">
+        <is>
+          <t>할아버지는 돈이 없는데…
+그럼 공짜! 가족이니까!</t>
+        </is>
+      </c>
+      <c r="H541" s="6" t="inlineStr"/>
+    </row>
+    <row r="542">
+      <c r="A542" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B542" s="4" t="inlineStr">
+        <is>
+          <t>가윌 가게 오픈!</t>
+        </is>
+      </c>
+      <c r="C542" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D542" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E542" s="4" t="inlineStr">
+        <is>
+          <t>재이</t>
+        </is>
+      </c>
+      <c r="F542" s="4" t="inlineStr"/>
+      <c r="G542" s="4" t="inlineStr">
+        <is>
+          <t>태오야, 다 공짜로 주면 가게 망해!</t>
+        </is>
+      </c>
+      <c r="H542" s="4" t="inlineStr"/>
+    </row>
+    <row r="543">
+      <c r="A543" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="B543" s="6" t="inlineStr">
+        <is>
+          <t>가윌 가게 오픈!</t>
+        </is>
+      </c>
+      <c r="C543" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D543" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E543" s="6" t="inlineStr">
+        <is>
+          <t>태오</t>
+        </is>
+      </c>
+      <c r="F543" s="6" t="inlineStr"/>
+      <c r="G543" s="6" t="inlineStr">
+        <is>
+          <t>괜찮아! 다 먹으면 또 가윌 그리면 돼!</t>
+        </is>
+      </c>
+      <c r="H543" s="6" t="inlineStr"/>
+    </row>
+    <row r="544">
+      <c r="A544" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B544" s="4" t="inlineStr">
+        <is>
+          <t>가윌 가게 오픈!</t>
+        </is>
+      </c>
+      <c r="C544" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="D544" s="4" t="inlineStr">
+        <is>
+          <t>거실</t>
+        </is>
+      </c>
+      <c r="E544" s="4" t="inlineStr">
+        <is>
+          <t>태오, 재이</t>
+        </is>
+      </c>
+      <c r="F544" s="4" t="inlineStr">
+        <is>
+          <t>가게 문 닫을 시간. 남은 건 반쪽 레몬 하나.</t>
+        </is>
+      </c>
+      <c r="G544" s="4" t="inlineStr">
+        <is>
+          <t>(속삭임) …누나만 한 번 핥아도 돼.
+아니야, 괜찮아!</t>
+        </is>
+      </c>
+      <c r="H544" s="4" t="inlineStr"/>
+    </row>
+    <row r="545">
+      <c r="A545" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="B545" s="6" t="inlineStr">
+        <is>
+          <t>가윌 가게 오픈!</t>
+        </is>
+      </c>
+      <c r="C545" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="D545" s="6" t="inlineStr">
+        <is>
+          <t>효과: 반짝</t>
+        </is>
+      </c>
+      <c r="E545" s="6" t="inlineStr"/>
+      <c r="F545" s="6" t="inlineStr">
+        <is>
+          <t>가윌 가게는 오늘도 적자. / 그래도 우리 집에서 제일 부자 가게다.</t>
+        </is>
+      </c>
+      <c r="G545" s="6" t="inlineStr"/>
+      <c r="H545" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:H531"/>
+  <autoFilter ref="A3:H545"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -19372,7 +19854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -20198,17 +20680,17 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>루돌푸</t>
+          <t>가윌</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>올라프</t>
+          <t>과일</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>디즈니랜드 캘리포니아에서 만난 눈사람 친구</t>
+          <t>“우리 가윌 없잖아!” 가게 놀이 하자고 하면</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr"/>
@@ -20220,17 +20702,17 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>발싸</t>
+          <t>루돌푸</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>발사</t>
+          <t>올라프</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>“스밀로클로 발싸!” 기술을 쏠 때</t>
+          <t>디즈니랜드 캘리포니아에서 만난 눈사람 친구</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr"/>
@@ -20242,17 +20724,17 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>안킬로해머 · 스밀로클로</t>
+          <t>발싸</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>다이노스터 기술</t>
+          <t>발사</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>래터킥, 퀀텀해로우… 하나씩 외치고 “쓰구미~”</t>
+          <t>“스밀로클로 발싸!” 기술을 쏠 때</t>
         </is>
       </c>
       <c r="E41" s="6" t="inlineStr"/>
@@ -20262,9 +20744,21 @@
       <c r="A42" s="3" t="n">
         <v>39</v>
       </c>
-      <c r="B42" s="4" t="inlineStr"/>
-      <c r="C42" s="4" t="inlineStr"/>
-      <c r="D42" s="4" t="inlineStr"/>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>안킬로해머 · 스밀로클로</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>다이노스터 기술</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>래터킥, 퀀텀해로우… 하나씩 외치고 “쓰구미~”</t>
+        </is>
+      </c>
       <c r="E42" s="4" t="inlineStr"/>
       <c r="F42" s="4" t="inlineStr"/>
     </row>
@@ -20458,8 +20952,18 @@
       <c r="E61" s="6" t="inlineStr"/>
       <c r="F61" s="6" t="inlineStr"/>
     </row>
+    <row r="62">
+      <c r="A62" s="3" t="n">
+        <v>59</v>
+      </c>
+      <c r="B62" s="4" t="inlineStr"/>
+      <c r="C62" s="4" t="inlineStr"/>
+      <c r="D62" s="4" t="inlineStr"/>
+      <c r="E62" s="4" t="inlineStr"/>
+      <c r="F62" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F61"/>
+  <autoFilter ref="A3:F62"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -20473,7 +20977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -21370,13 +21874,13 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>흥!</t>
+          <t>우리 가게 놀이 할까?</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr"/>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>화나면 한 발을 번쩍 들었다가 쾅! 내리치면서</t>
+          <t>심심할 때 (그런데 “우리 가윌 없잖아!”가 바로 따라 나와요)</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr"/>
@@ -21392,13 +21896,13 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>(엉덩이 씰룩씰룩 춤)</t>
+          <t>흥!</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr"/>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>기분이 좋으면 엉덩이를 양쪽으로 흔들며 춤춰요</t>
+          <t>화나면 한 발을 번쩍 들었다가 쾅! 내리치면서</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr"/>
@@ -21414,13 +21918,13 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>찌찌뽕!</t>
+          <t>(엉덩이 씰룩씰룩 춤)</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr"/>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>누나랑 같은 말을 동시에 했을 때 (누가 “뽕뽕찌” 해 줄 때까지 말을 못 하고 꾹 참아요)</t>
+          <t>기분이 좋으면 엉덩이를 양쪽으로 흔들며 춤춰요</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr"/>
@@ -21436,13 +21940,13 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>박수 한 번만 치고 싶어!</t>
+          <t>찌찌뽕!</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr"/>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>3·6·9 게임을 하면서 계속 (박수 차례가 아니어도)</t>
+          <t>누나랑 같은 말을 동시에 했을 때 (누가 “뽕뽕찌” 해 줄 때까지 말을 못 하고 꾹 참아요)</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr"/>
@@ -21458,13 +21962,13 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>와칸다 포에버!</t>
+          <t>박수 한 번만 치고 싶어!</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr"/>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>인피니티 워 장면처럼 다 같이 뛰어갈 때</t>
+          <t>3·6·9 게임을 하면서 계속 (박수 차례가 아니어도)</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr"/>
@@ -21480,13 +21984,13 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>어린이집에 데리러 올 거야?</t>
+          <t>와칸다 포에버!</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr"/>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>어린이집 가기 싫은 아침에 (몇 번씩 확인해요)</t>
+          <t>인피니티 워 장면처럼 다 같이 뛰어갈 때</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr"/>
@@ -21502,13 +22006,13 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>어린이집 가기 싫다.</t>
+          <t>어린이집에 데리러 올 거야?</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr"/>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>월·화·수… 아침마다</t>
+          <t>어린이집 가기 싫은 아침에 (몇 번씩 확인해요)</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr"/>
@@ -21524,13 +22028,13 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?</t>
+          <t>어린이집 가기 싫다.</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr"/>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>싫은 태권도 가는 날</t>
+          <t>월·화·수… 아침마다</t>
         </is>
       </c>
       <c r="F49" s="6" t="inlineStr"/>
@@ -21546,13 +22050,13 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>오늘은 뽀로로 날! 내가 싫어하는 태권도 안 가는 날이다~</t>
+          <t>누나는 왜 학교만 가? 나는 왜 태권도 가야 돼?</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr"/>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>월요일 아침 (달력은 몰라도 뽀로로 날은 정확히 알아요)</t>
+          <t>싫은 태권도 가는 날</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr"/>
@@ -21563,18 +22067,18 @@
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>재이 입버릇</t>
+          <t>태오 입버릇</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>아니야!</t>
+          <t>오늘은 뽀로로 날! 내가 싫어하는 태권도 안 가는 날이다~</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr"/>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>하루에도 제일 많이 하는 말</t>
+          <t>월요일 아침 (달력은 몰라도 뽀로로 날은 정확히 알아요)</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr"/>
@@ -21590,13 +22094,13 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>거짓말! 아니야!</t>
+          <t>아니야!</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr"/>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>기분 나쁘거나 하기 싫을 때</t>
+          <t>하루에도 제일 많이 하는 말</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr"/>
@@ -21612,13 +22116,13 @@
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>맛있는데 지금은 먹기 싫어.</t>
+          <t>거짓말! 아니야!</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr"/>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>누가 음식을 권하면</t>
+          <t>기분 나쁘거나 하기 싫을 때</t>
         </is>
       </c>
       <c r="F53" s="6" t="inlineStr"/>
@@ -21634,13 +22138,13 @@
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>치즈 냄새 극혐!</t>
+          <t>맛있는데 지금은 먹기 싫어.</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr"/>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>치즈만 보면 (냄새는 더더욱)</t>
+          <t>누가 음식을 권하면</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr"/>
@@ -21656,13 +22160,13 @@
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>나 이제 떨어지는 건 안 탈 거야.</t>
+          <t>치즈 냄새 극혐!</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr"/>
       <c r="E55" s="6" t="inlineStr">
         <is>
-          <t>올랜도 디즈니 월드에서 가디언즈 오브 갤럭시를 타고 너무 무서웠던 뒤로</t>
+          <t>치즈만 보면 (냄새는 더더욱)</t>
         </is>
       </c>
       <c r="F55" s="6" t="inlineStr"/>
@@ -21678,13 +22182,13 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>김태오!</t>
+          <t>나 이제 떨어지는 건 안 탈 거야.</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr"/>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
+          <t>올랜도 디즈니 월드에서 가디언즈 오브 갤럭시를 타고 너무 무서웠던 뒤로</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr"/>
@@ -21695,22 +22199,18 @@
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>재이 아기 말</t>
+          <t>재이 입버릇</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>짐방</t>
-        </is>
-      </c>
-      <c r="D57" s="6" t="inlineStr">
-        <is>
-          <t>김서방</t>
-        </is>
-      </c>
+          <t>김태오!</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr"/>
       <c r="E57" s="6" t="inlineStr">
         <is>
-          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
+          <t>참고 참다가 폭발했을 때 (그다음은 엉덩이 찰싹!)</t>
         </is>
       </c>
       <c r="F57" s="6" t="inlineStr"/>
@@ -21726,17 +22226,17 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>꿍끙이</t>
+          <t>짐방</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>뿡뿡이</t>
+          <t>김서방</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+          <t>할머니가 아빠를 “김서방~” 하고 부르시는 걸 따라서 아빠를 부른 말</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr"/>
@@ -21745,10 +22245,26 @@
       <c r="A59" s="5" t="n">
         <v>56</v>
       </c>
-      <c r="B59" s="6" t="inlineStr"/>
-      <c r="C59" s="6" t="inlineStr"/>
-      <c r="D59" s="6" t="inlineStr"/>
-      <c r="E59" s="6" t="inlineStr"/>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>재이 아기 말</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>꿍끙이</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>뿡뿡이</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>‘방귀대장 뿡뿡이’를 부르던 말</t>
+        </is>
+      </c>
       <c r="F59" s="6" t="inlineStr"/>
     </row>
     <row r="60">
@@ -21891,8 +22407,18 @@
       <c r="E73" s="6" t="inlineStr"/>
       <c r="F73" s="6" t="inlineStr"/>
     </row>
+    <row r="74">
+      <c r="A74" s="3" t="n">
+        <v>71</v>
+      </c>
+      <c r="B74" s="4" t="inlineStr"/>
+      <c r="C74" s="4" t="inlineStr"/>
+      <c r="D74" s="4" t="inlineStr"/>
+      <c r="E74" s="4" t="inlineStr"/>
+      <c r="F74" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F73"/>
+  <autoFilter ref="A3:F74"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>